<commit_message>
[IMP] tables: import table styles in xlsx
Task: 3789612
</commit_message>
<xml_diff>
--- a/tests/__xlsx__/xlsx_demo_data.xlsx
+++ b/tests/__xlsx__/xlsx_demo_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Adrien\odoo\spreadsheet\tests\__xlsx__\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{676AF7E1-BB07-416E-B55F-CE934DA012B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60269A66-F8A2-476A-97C7-A95174A5895C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="419">
   <si>
     <t>CF =42</t>
   </si>
@@ -1298,12 +1298,21 @@
   </si>
   <si>
     <t>'sheet!'!R[1]C[1]</t>
+  </si>
+  <si>
+    <t>CustomStyle</t>
+  </si>
+  <si>
+    <t>Column1</t>
+  </si>
+  <si>
+    <t>Column2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <numFmts count="7">
     <numFmt numFmtId="164" formatCode="m/d/yyyy"/>
     <numFmt numFmtId="165" formatCode="m/d/yyyy\ hh:mm:ss"/>
@@ -2209,7 +2218,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{1493241F-B85D-4F84-BBA0-86191B8FD032}"/>
   </cellStyles>
-  <dxfs count="44">
+  <dxfs count="46">
     <dxf>
       <fill>
         <patternFill>
@@ -2220,165 +2229,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-        <strike/>
-        <u/>
-        <color theme="7"/>
-      </font>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <fill>
-        <patternFill patternType="lightTrellis">
-          <fgColor theme="4"/>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE06666"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFB6D7A8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF9900"/>
+          <bgColor theme="5"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2764,8 +2615,185 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+        <strike/>
+        <u/>
+        <color theme="7"/>
+      </font>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <fill>
+        <patternFill patternType="lightTrellis">
+          <fgColor theme="4"/>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE06666"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFB6D7A8"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
+    <tableStyle name="MyCustomTableStyle" pivot="0" count="2" xr9:uid="{DDE0F8F2-27C1-476B-B1FE-0502518857F6}">
+      <tableStyleElement type="wholeTable" dxfId="1"/>
+      <tableStyleElement type="headerRow" dxfId="0"/>
+    </tableStyle>
+  </tableStyles>
   <colors>
     <mruColors>
       <color rgb="FF000000"/>
@@ -6247,7 +6275,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{09C35CC7-7259-4A97-8FEA-EDB47375DF08}" name="Table3" displayName="Table3" ref="C3:J6" totalsRowCount="1" headerRowDxfId="20" dataDxfId="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{09C35CC7-7259-4A97-8FEA-EDB47375DF08}" name="Table3" displayName="Table3" ref="C3:J6" totalsRowCount="1" headerRowDxfId="45" dataDxfId="44">
   <autoFilter ref="C3:J5" xr:uid="{09C35CC7-7259-4A97-8FEA-EDB47375DF08}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -6259,26 +6287,37 @@
     <filterColumn colId="7" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{C4EE018E-238B-42BA-9035-DB01FA5420D3}" name="Name" totalsRowLabel="Total" dataDxfId="18" totalsRowDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{C1F6911F-9482-4C98-BBFB-21D9CAA66DA4}" name="Age" totalsRowFunction="sum" dataDxfId="16" totalsRowDxfId="15"/>
-    <tableColumn id="5" xr3:uid="{3CE9F5DA-0A57-4696-B4E0-53601C3B7798}" name="Rank" totalsRowFunction="sum" dataDxfId="14" totalsRowDxfId="13"/>
-    <tableColumn id="6" xr3:uid="{34912838-665C-4472-B558-25990E5B148D}" name="Rank+Age =E4+D4" totalsRowFunction="sum" dataDxfId="12" totalsRowDxfId="11">
+    <tableColumn id="1" xr3:uid="{C4EE018E-238B-42BA-9035-DB01FA5420D3}" name="Name" totalsRowLabel="Total" dataDxfId="43" totalsRowDxfId="42"/>
+    <tableColumn id="2" xr3:uid="{C1F6911F-9482-4C98-BBFB-21D9CAA66DA4}" name="Age" totalsRowFunction="sum" dataDxfId="41" totalsRowDxfId="40"/>
+    <tableColumn id="5" xr3:uid="{3CE9F5DA-0A57-4696-B4E0-53601C3B7798}" name="Rank" totalsRowFunction="sum" dataDxfId="39" totalsRowDxfId="38"/>
+    <tableColumn id="6" xr3:uid="{34912838-665C-4472-B558-25990E5B148D}" name="Rank+Age =E4+D4" totalsRowFunction="sum" dataDxfId="37" totalsRowDxfId="36">
       <calculatedColumnFormula>Table3[[#This Row],[Rank]]+Table3[[#This Row],[Age]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{89D90022-7073-4067-BAF8-1587D27C4AFB}" name="Data =SUM(E4:E5)" totalsRowFunction="sum" dataDxfId="10" totalsRowDxfId="9">
+    <tableColumn id="7" xr3:uid="{89D90022-7073-4067-BAF8-1587D27C4AFB}" name="Data =SUM(E4:E5)" totalsRowFunction="sum" dataDxfId="35" totalsRowDxfId="34">
       <calculatedColumnFormula>SUM(Table3[Rank])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{B2A7E5BB-A379-492B-9484-72F2FD1FF3A0}" name="All =SUM(E3:E6)" totalsRowFunction="sum" dataDxfId="8" totalsRowDxfId="7">
+    <tableColumn id="8" xr3:uid="{B2A7E5BB-A379-492B-9484-72F2FD1FF3A0}" name="All =SUM(E3:E6)" totalsRowFunction="sum" dataDxfId="33" totalsRowDxfId="32">
       <calculatedColumnFormula>SUM(Table3[[#All],[Rank]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{3C532A69-E4BC-4A20-A922-4BCAA0D3FEC9}" name="Totals =E6" totalsRowFunction="sum" dataDxfId="6" totalsRowDxfId="5">
+    <tableColumn id="9" xr3:uid="{3C532A69-E4BC-4A20-A922-4BCAA0D3FEC9}" name="Totals =E6" totalsRowFunction="sum" dataDxfId="31" totalsRowDxfId="30">
       <calculatedColumnFormula>Table3[[#Totals],[Rank]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{35E9E9C3-9148-468A-85B6-19290CEB6F00}" name="Headers =E3" totalsRowFunction="sum" dataDxfId="4" totalsRowDxfId="3">
+    <tableColumn id="10" xr3:uid="{35E9E9C3-9148-468A-85B6-19290CEB6F00}" name="Headers =E3" totalsRowFunction="sum" dataDxfId="29" totalsRowDxfId="28">
       <calculatedColumnFormula>Table3[[#Headers],[Rank]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight10" showFirstColumn="1" showLastColumn="1" showRowStripes="0" showColumnStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B96C8832-8BF1-48C8-B9E9-9E059A81B5EF}" name="Table2" displayName="Table2" ref="C34:D35" insertRow="1" totalsRowShown="0">
+  <autoFilter ref="C34:D35" xr:uid="{B96C8832-8BF1-48C8-B9E9-9E059A81B5EF}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{0CD8A320-6EED-46F6-8606-8C017A8A7672}" name="Column1"/>
+    <tableColumn id="2" xr3:uid="{4EDBDF5C-3A86-4C30-807B-5FBD3E92A53B}" name="Column2"/>
+  </tableColumns>
+  <tableStyleInfo name="MyCustomTableStyle" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -7071,7 +7110,7 @@
     <mergeCell ref="K3:K8"/>
   </mergeCells>
   <conditionalFormatting sqref="C1:C100 B21">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="27" priority="1" operator="equal">
       <formula>42</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9014,7 +9053,7 @@
       </c>
       <c r="B100" s="20">
         <f ca="1">NOW()</f>
-        <v>45359.413205787037</v>
+        <v>45359.41589340278</v>
       </c>
       <c r="D100" s="2">
         <f ca="1">IF(ISNUMBER(B100),1,0)</f>
@@ -10018,10 +10057,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="D1:D180">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="26" priority="1" operator="equal">
       <formula>1</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="25" priority="2" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11267,67 +11306,67 @@
   </sheetData>
   <phoneticPr fontId="21" type="noConversion"/>
   <conditionalFormatting sqref="B3:C3">
-    <cfRule type="beginsWith" dxfId="43" priority="73" operator="beginsWith" text="rule">
+    <cfRule type="beginsWith" dxfId="24" priority="73" operator="beginsWith" text="rule">
       <formula>LEFT(B3,LEN("rule"))="rule"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B4:C4">
-    <cfRule type="containsBlanks" dxfId="42" priority="71">
+    <cfRule type="containsBlanks" dxfId="23" priority="71">
       <formula>LEN(TRIM(B4))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B5:C5">
-    <cfRule type="containsErrors" dxfId="41" priority="70">
+    <cfRule type="containsErrors" dxfId="22" priority="70">
       <formula>ISERROR(B5)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:C6">
-    <cfRule type="containsText" dxfId="40" priority="69" operator="containsText" text="rule">
+    <cfRule type="containsText" dxfId="21" priority="69" operator="containsText" text="rule">
       <formula>NOT(ISERROR(SEARCH("rule",B6)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8:C8">
-    <cfRule type="endsWith" dxfId="39" priority="67" operator="endsWith" text="rule">
+    <cfRule type="endsWith" dxfId="20" priority="67" operator="endsWith" text="rule">
       <formula>RIGHT(B8,LEN("rule"))="rule"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B9:C9">
-    <cfRule type="notContainsBlanks" dxfId="38" priority="66">
+    <cfRule type="notContainsBlanks" dxfId="19" priority="66">
       <formula>LEN(TRIM(B9))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B10:C10">
-    <cfRule type="notContainsErrors" dxfId="37" priority="65">
+    <cfRule type="notContainsErrors" dxfId="18" priority="65">
       <formula>NOT(ISERROR(B10))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B11:C11">
-    <cfRule type="notContainsText" dxfId="36" priority="64" operator="notContains" text="rule">
+    <cfRule type="notContainsText" dxfId="17" priority="64" operator="notContains" text="rule">
       <formula>ISERROR(SEARCH("rule",B11))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12:C12">
-    <cfRule type="timePeriod" dxfId="35" priority="63" timePeriod="today">
+    <cfRule type="timePeriod" dxfId="16" priority="63" timePeriod="today">
       <formula>FLOOR(B12,1)=TODAY()</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B15">
-    <cfRule type="expression" dxfId="34" priority="58">
+    <cfRule type="expression" dxfId="15" priority="58">
       <formula>ODD(B15)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B17:C17">
-    <cfRule type="cellIs" dxfId="33" priority="56" operator="notEqual">
+    <cfRule type="cellIs" dxfId="14" priority="56" operator="notEqual">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B26:B27">
-    <cfRule type="cellIs" dxfId="32" priority="46" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="46" operator="equal">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B16:C16">
-    <cfRule type="cellIs" dxfId="31" priority="45" operator="equal">
+    <cfRule type="cellIs" dxfId="12" priority="45" operator="equal">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11493,10 +11532,10 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7:D7">
-    <cfRule type="duplicateValues" dxfId="30" priority="82"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="82"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B14:D14">
-    <cfRule type="uniqueValues" dxfId="29" priority="96"/>
+    <cfRule type="uniqueValues" dxfId="10" priority="96"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B24:C24">
     <cfRule type="dataBar" priority="100">
@@ -11513,10 +11552,10 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B2:C2">
-    <cfRule type="aboveAverage" dxfId="28" priority="114"/>
+    <cfRule type="aboveAverage" dxfId="9" priority="114"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B13:C13">
-    <cfRule type="top10" dxfId="27" priority="115" rank="1"/>
+    <cfRule type="top10" dxfId="8" priority="115" rank="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H21:K21">
     <cfRule type="iconSet" priority="18">
@@ -11613,33 +11652,33 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B18:C18">
-    <cfRule type="cellIs" dxfId="26" priority="6" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="7" priority="6" operator="greaterThan">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B19:C19">
-    <cfRule type="cellIs" dxfId="25" priority="5" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="6" priority="5" operator="greaterThanOrEqual">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B20:C20">
-    <cfRule type="cellIs" dxfId="24" priority="4" operator="lessThan">
+    <cfRule type="cellIs" dxfId="5" priority="4" operator="lessThan">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B21:C21">
-    <cfRule type="cellIs" dxfId="23" priority="3" operator="lessThanOrEqual">
+    <cfRule type="cellIs" dxfId="4" priority="3" operator="lessThanOrEqual">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B22:C22">
-    <cfRule type="cellIs" dxfId="22" priority="2" operator="between">
+    <cfRule type="cellIs" dxfId="3" priority="2" operator="between">
       <formula>2</formula>
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B23:C23">
-    <cfRule type="cellIs" dxfId="21" priority="1" operator="notBetween">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="notBetween">
       <formula>2</formula>
       <formula>4</formula>
     </cfRule>
@@ -11823,7 +11862,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDA2AD09-EFB1-4B74-862F-432090DD90CB}">
-  <dimension ref="A1:J32"/>
+  <dimension ref="A1:J34"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="17.28515625" customWidth="1"/>
@@ -12131,9 +12170,20 @@
         <v>408</v>
       </c>
     </row>
+    <row r="34" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B34" t="s">
+        <v>416</v>
+      </c>
+      <c r="C34" t="s">
+        <v>417</v>
+      </c>
+      <c r="D34" t="s">
+        <v>418</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="9">
+  <tableParts count="10">
     <tablePart r:id="rId1"/>
     <tablePart r:id="rId2"/>
     <tablePart r:id="rId3"/>
@@ -12143,6 +12193,7 @@
     <tablePart r:id="rId7"/>
     <tablePart r:id="rId8"/>
     <tablePart r:id="rId9"/>
+    <tablePart r:id="rId10"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
[IMP] charts: add radar chart
</commit_message>
<xml_diff>
--- a/tests/__xlsx__/xlsx_demo_data.xlsx
+++ b/tests/__xlsx__/xlsx_demo_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Adrien\odoo\spreadsheet\tests\__xlsx__\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E0F1A66-FDA3-41D2-8301-AC5DB36FDC80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5418097B-5455-451A-9833-8DDA204394AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,17 +34,6 @@
   <pivotCaches>
     <pivotCache cacheId="0" r:id="rId15"/>
   </pivotCaches>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
@@ -2208,25 +2197,11 @@
     </xf>
   </cellXfs>
   <cellStyles count="3">
-    <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
+    <cellStyle name="Lien hypertexte" xfId="2" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{1493241F-B85D-4F84-BBA0-86191B8FD032}"/>
   </cellStyles>
   <dxfs count="46">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -2781,11 +2756,25 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="Table Style 1" pivot="0" count="2" xr9:uid="{33B8EB55-D8D8-4B00-B5CF-C84A8AC9E775}">
-      <tableStyleElement type="wholeTable" dxfId="1"/>
-      <tableStyleElement type="firstRowStripe" dxfId="0"/>
+      <tableStyleElement type="wholeTable" dxfId="45"/>
+      <tableStyleElement type="firstRowStripe" dxfId="44"/>
     </tableStyle>
   </tableStyles>
   <colors>
@@ -2812,7 +2801,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="fr-FR"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -3413,7 +3402,7 @@
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="fr-FR"/>
   <c:roundedCorners val="0"/>
   <c:style val="2"/>
   <c:chart>
@@ -3841,7 +3830,7 @@
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="fr-FR"/>
   <c:roundedCorners val="0"/>
   <c:style val="2"/>
   <c:chart>
@@ -4459,7 +4448,7 @@
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="fr-FR"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -4825,7 +4814,7 @@
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="fr-FR"/>
   <c:roundedCorners val="1"/>
   <c:style val="2"/>
   <c:chart>
@@ -5124,7 +5113,7 @@
 <file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="fr-FR"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -5560,7 +5549,409 @@
 <file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="fr-FR"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr lvl="0">
+              <a:defRPr b="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="2200"/>
+              <a:t>radar chart</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:radarChart>
+        <c:radarStyle val="marker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln cmpd="sng">
+              <a:solidFill>
+                <a:srgbClr val="1F77B4"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet1!$A$27:$A$35</c:f>
+              <c:strCache>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>Emily Anderson (Emmy)</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Sophie Allen (Saffi)</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Chloe Adams</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Megan Alexander (Meg)</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Lucy Arnold (Lulu)</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Hannah Alvarez</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Jessica Alcock (Jess)</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Charlotte Anaya</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Lauren Anthony</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$B$27:$B$35</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>48</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>31</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>16</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-A060-40CF-8F7B-7D927B019D4E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:spPr>
+            <a:ln cmpd="sng">
+              <a:solidFill>
+                <a:srgbClr val="FF7F0E"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet1!$A$27:$A$35</c:f>
+              <c:strCache>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>Emily Anderson (Emmy)</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Sophie Allen (Saffi)</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Chloe Adams</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Megan Alexander (Meg)</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Lucy Arnold (Lulu)</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Hannah Alvarez</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Jessica Alcock (Jess)</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Charlotte Anaya</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Lauren Anthony</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$C$27:$C$35</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>27</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>43</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>16</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-A060-40CF-8F7B-7D927B019D4E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="17781237"/>
+        <c:axId val="88853993"/>
+      </c:radarChart>
+      <c:catAx>
+        <c:axId val="17781237"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln cmpd="sng">
+              <a:solidFill>
+                <a:srgbClr val="B7B7B7"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr lvl="0">
+                  <a:defRPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="1"/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr lvl="0">
+              <a:defRPr sz="1000" b="0" i="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="fr-FR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="88853993"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="1"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="88853993"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln cmpd="sng">
+              <a:solidFill>
+                <a:srgbClr val="B7B7B7"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr lvl="0">
+                  <a:defRPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="1"/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr lvl="0">
+              <a:defRPr sz="1000" b="0" i="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="fr-FR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="17781237"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="t"/>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr lvl="0">
+            <a:defRPr sz="1000" b="0" i="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="fr-FR"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="zero"/>
+    <c:showDLblsOverMax val="1"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln cmpd="sng">
+      <a:solidFill>
+        <a:srgbClr val="000000"/>
+      </a:solidFill>
+    </a:ln>
+  </c:spPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="fr-FR"/>
   <c:roundedCorners val="1"/>
   <c:style val="2"/>
   <c:chart>
@@ -6671,6 +7062,44 @@
     </xdr:graphicFrame>
     <xdr:clientData fLocksWithSheet="0"/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>47625</xdr:colOff>
+      <xdr:row>57</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>200025</xdr:colOff>
+      <xdr:row>70</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Chart 2" title="Chart">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2768A00C-0BD9-43E8-B0A0-2D9210A64EA6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -7080,7 +7509,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{09C35CC7-7259-4A97-8FEA-EDB47375DF08}" name="Table3" displayName="Table3" ref="C3:J6" totalsRowCount="1" headerRowDxfId="45" dataDxfId="44">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{09C35CC7-7259-4A97-8FEA-EDB47375DF08}" name="Table3" displayName="Table3" ref="C3:J6" totalsRowCount="1" headerRowDxfId="43" dataDxfId="42">
   <autoFilter ref="C3:J5" xr:uid="{09C35CC7-7259-4A97-8FEA-EDB47375DF08}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -7092,22 +7521,22 @@
     <filterColumn colId="7" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{C4EE018E-238B-42BA-9035-DB01FA5420D3}" name="Name" totalsRowLabel="Total" dataDxfId="43" totalsRowDxfId="42"/>
-    <tableColumn id="2" xr3:uid="{C1F6911F-9482-4C98-BBFB-21D9CAA66DA4}" name="Age" totalsRowFunction="sum" dataDxfId="41" totalsRowDxfId="40"/>
-    <tableColumn id="5" xr3:uid="{3CE9F5DA-0A57-4696-B4E0-53601C3B7798}" name="Rank" totalsRowFunction="sum" dataDxfId="39" totalsRowDxfId="38"/>
-    <tableColumn id="6" xr3:uid="{34912838-665C-4472-B558-25990E5B148D}" name="Rank+Age =E4+D4" totalsRowFunction="sum" dataDxfId="37" totalsRowDxfId="36">
+    <tableColumn id="1" xr3:uid="{C4EE018E-238B-42BA-9035-DB01FA5420D3}" name="Name" totalsRowLabel="Total" dataDxfId="41" totalsRowDxfId="40"/>
+    <tableColumn id="2" xr3:uid="{C1F6911F-9482-4C98-BBFB-21D9CAA66DA4}" name="Age" totalsRowFunction="sum" dataDxfId="39" totalsRowDxfId="38"/>
+    <tableColumn id="5" xr3:uid="{3CE9F5DA-0A57-4696-B4E0-53601C3B7798}" name="Rank" totalsRowFunction="sum" dataDxfId="37" totalsRowDxfId="36"/>
+    <tableColumn id="6" xr3:uid="{34912838-665C-4472-B558-25990E5B148D}" name="Rank+Age =E4+D4" totalsRowFunction="sum" dataDxfId="35" totalsRowDxfId="34">
       <calculatedColumnFormula>Table3[[#This Row],[Rank]]+Table3[[#This Row],[Age]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{89D90022-7073-4067-BAF8-1587D27C4AFB}" name="Data =SUM(E4:E5)" totalsRowFunction="sum" dataDxfId="35" totalsRowDxfId="34">
+    <tableColumn id="7" xr3:uid="{89D90022-7073-4067-BAF8-1587D27C4AFB}" name="Data =SUM(E4:E5)" totalsRowFunction="sum" dataDxfId="33" totalsRowDxfId="32">
       <calculatedColumnFormula>SUM(Table3[Rank])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{B2A7E5BB-A379-492B-9484-72F2FD1FF3A0}" name="All =SUM(E3:E6)" totalsRowFunction="sum" dataDxfId="33" totalsRowDxfId="32">
+    <tableColumn id="8" xr3:uid="{B2A7E5BB-A379-492B-9484-72F2FD1FF3A0}" name="All =SUM(E3:E6)" totalsRowFunction="sum" dataDxfId="31" totalsRowDxfId="30">
       <calculatedColumnFormula>SUM(Table3[[#All],[Rank]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{3C532A69-E4BC-4A20-A922-4BCAA0D3FEC9}" name="Totals =E6" totalsRowFunction="sum" dataDxfId="31" totalsRowDxfId="30">
+    <tableColumn id="9" xr3:uid="{3C532A69-E4BC-4A20-A922-4BCAA0D3FEC9}" name="Totals =E6" totalsRowFunction="sum" dataDxfId="29" totalsRowDxfId="28">
       <calculatedColumnFormula>Table3[[#Totals],[Rank]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{35E9E9C3-9148-468A-85B6-19290CEB6F00}" name="Headers =E3" totalsRowFunction="sum" dataDxfId="29" totalsRowDxfId="28">
+    <tableColumn id="10" xr3:uid="{35E9E9C3-9148-468A-85B6-19290CEB6F00}" name="Headers =E3" totalsRowFunction="sum" dataDxfId="27" totalsRowDxfId="26">
       <calculatedColumnFormula>Table3[[#Headers],[Rank]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -7217,9 +7646,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -7257,7 +7686,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -7363,7 +7792,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -7505,7 +7934,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -7514,7 +7943,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{385D5EBC-45F5-4C42-AA75-560DF70B9F2E}">
   <dimension ref="A1:L35"/>
-  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="13.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.28515625" customWidth="1"/>
     <col min="2" max="2" width="13.7109375" customWidth="1"/>
@@ -7914,7 +8343,7 @@
     <mergeCell ref="K3:K8"/>
   </mergeCells>
   <conditionalFormatting sqref="C1:C100 B21">
-    <cfRule type="cellIs" dxfId="27" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="25" priority="1" operator="equal">
       <formula>42</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7959,7 +8388,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F7A934C-2218-4A12-8B75-EE28D615D774}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -7968,7 +8397,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96301BE1-D86D-4D45-870D-85A75D53FC99}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -7977,7 +8406,7 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B10A8834-0E20-4F80-8813-3ACA5527B377}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="13.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="65.140625" customWidth="1"/>
     <col min="2" max="26" width="13.7109375" customWidth="1"/>
@@ -7994,7 +8423,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8004,7 +8433,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0630FA18-71FC-4ACD-8379-39A3603D1DD6}">
   <dimension ref="A1:R163"/>
-  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="13.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="26" width="13.7109375" customWidth="1"/>
   </cols>
@@ -9857,7 +10286,7 @@
       </c>
       <c r="B100" s="20">
         <f ca="1">NOW()</f>
-        <v>45398.580923148147</v>
+        <v>45450.649344444442</v>
       </c>
       <c r="D100" s="2">
         <f ca="1">IF(ISNUMBER(B100),1,0)</f>
@@ -10547,7 +10976,7 @@
       </c>
       <c r="B144" s="19">
         <f ca="1">TODAY()</f>
-        <v>45398</v>
+        <v>45450</v>
       </c>
       <c r="D144" s="2">
         <f ca="1">IF(ISNUMBER(B144),1,0)</f>
@@ -10861,10 +11290,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="D1:D180">
-    <cfRule type="cellIs" dxfId="26" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="24" priority="1" operator="equal">
       <formula>1</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="23" priority="2" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10878,7 +11307,7 @@
     <outlinePr summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:R18"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" outlineLevelRow="2" outlineLevelCol="2" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="12.75" outlineLevelRow="2" outlineLevelCol="2" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="0" hidden="1" customWidth="1"/>
     <col min="6" max="6" width="14.28515625" customWidth="1"/>
@@ -10961,7 +11390,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF68F2C0-1053-4FB6-BD74-8A11B0CAF123}">
   <dimension ref="A1:M30"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="17.7109375" customWidth="1"/>
     <col min="5" max="5" width="18.28515625" customWidth="1"/>
@@ -11347,7 +11776,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D919E811-4385-4D35-A19E-3B7E0E659A89}">
   <dimension ref="A1:L39"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.140625" customWidth="1"/>
     <col min="7" max="7" width="15.85546875" customWidth="1"/>
@@ -11576,7 +12005,7 @@
       </c>
       <c r="B12" s="40">
         <f ca="1">TODAY()</f>
-        <v>45398</v>
+        <v>45450</v>
       </c>
       <c r="C12" s="40">
         <f>DATE(2010,10,2)</f>
@@ -12110,104 +12539,104 @@
   </sheetData>
   <phoneticPr fontId="21" type="noConversion"/>
   <conditionalFormatting sqref="B15">
-    <cfRule type="expression" dxfId="24" priority="58">
+    <cfRule type="expression" dxfId="22" priority="58">
       <formula>ODD(B15)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B26:B27">
-    <cfRule type="cellIs" dxfId="23" priority="46" operator="equal">
+    <cfRule type="cellIs" dxfId="21" priority="46" operator="equal">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B2:C2">
-    <cfRule type="aboveAverage" dxfId="22" priority="114"/>
+    <cfRule type="aboveAverage" dxfId="20" priority="114"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:C3">
-    <cfRule type="beginsWith" dxfId="21" priority="73" operator="beginsWith" text="rule">
+    <cfRule type="beginsWith" dxfId="19" priority="73" operator="beginsWith" text="rule">
       <formula>LEFT(B3,LEN("rule"))="rule"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B4:C4">
-    <cfRule type="containsBlanks" dxfId="20" priority="71">
+    <cfRule type="containsBlanks" dxfId="18" priority="71">
       <formula>LEN(TRIM(B4))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B5:C5">
-    <cfRule type="containsErrors" dxfId="19" priority="70">
+    <cfRule type="containsErrors" dxfId="17" priority="70">
       <formula>ISERROR(B5)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:C6">
-    <cfRule type="containsText" dxfId="18" priority="69" operator="containsText" text="rule">
+    <cfRule type="containsText" dxfId="16" priority="69" operator="containsText" text="rule">
       <formula>NOT(ISERROR(SEARCH("rule",B6)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8:C8">
-    <cfRule type="endsWith" dxfId="17" priority="67" operator="endsWith" text="rule">
+    <cfRule type="endsWith" dxfId="15" priority="67" operator="endsWith" text="rule">
       <formula>RIGHT(B8,LEN("rule"))="rule"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B9:C9">
-    <cfRule type="notContainsBlanks" dxfId="16" priority="66">
+    <cfRule type="notContainsBlanks" dxfId="14" priority="66">
       <formula>LEN(TRIM(B9))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B10:C10">
-    <cfRule type="notContainsErrors" dxfId="15" priority="65">
+    <cfRule type="notContainsErrors" dxfId="13" priority="65">
       <formula>NOT(ISERROR(B10))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B11:C11">
-    <cfRule type="notContainsText" dxfId="14" priority="64" operator="notContains" text="rule">
+    <cfRule type="notContainsText" dxfId="12" priority="64" operator="notContains" text="rule">
       <formula>ISERROR(SEARCH("rule",B11))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12:C12">
-    <cfRule type="timePeriod" dxfId="13" priority="63" timePeriod="today">
+    <cfRule type="timePeriod" dxfId="11" priority="63" timePeriod="today">
       <formula>FLOOR(B12,1)=TODAY()</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B13:C13">
-    <cfRule type="top10" dxfId="12" priority="115" rank="1"/>
+    <cfRule type="top10" dxfId="10" priority="115" rank="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B16:C16">
-    <cfRule type="cellIs" dxfId="11" priority="45" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="45" operator="equal">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B17:C17">
-    <cfRule type="cellIs" dxfId="10" priority="56" operator="notEqual">
+    <cfRule type="cellIs" dxfId="8" priority="56" operator="notEqual">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B18:C18">
-    <cfRule type="cellIs" dxfId="9" priority="6" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="7" priority="6" operator="greaterThan">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B19:C19">
-    <cfRule type="cellIs" dxfId="8" priority="5" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="6" priority="5" operator="greaterThanOrEqual">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B20:C20">
-    <cfRule type="cellIs" dxfId="7" priority="4" operator="lessThan">
+    <cfRule type="cellIs" dxfId="5" priority="4" operator="lessThan">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B21:C21">
-    <cfRule type="cellIs" dxfId="6" priority="3" operator="lessThanOrEqual">
+    <cfRule type="cellIs" dxfId="4" priority="3" operator="lessThanOrEqual">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B22:C22">
-    <cfRule type="cellIs" dxfId="5" priority="2" operator="between">
+    <cfRule type="cellIs" dxfId="3" priority="2" operator="between">
       <formula>2</formula>
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B23:C23">
-    <cfRule type="cellIs" dxfId="4" priority="1" operator="notBetween">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="notBetween">
       <formula>2</formula>
       <formula>4</formula>
     </cfRule>
@@ -12241,10 +12670,10 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7:D7">
-    <cfRule type="duplicateValues" dxfId="3" priority="82"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="82"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B14:D14">
-    <cfRule type="uniqueValues" dxfId="2" priority="96"/>
+    <cfRule type="uniqueValues" dxfId="0" priority="96"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:J2">
     <cfRule type="colorScale" priority="44">
@@ -12667,7 +13096,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5CCC4B1-5C65-4837-AA26-56CCF06B63BB}">
   <dimension ref="A1:J34"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="17.28515625" customWidth="1"/>
     <col min="4" max="4" width="9.5703125" customWidth="1"/>
@@ -12999,7 +13428,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE9224F2-4D06-4586-886C-E51F5EBCA7B0}">
   <dimension ref="A1:L21"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="13.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.5703125" bestFit="1" customWidth="1"/>
@@ -13311,7 +13740,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C47BF70-BA80-4124-B359-67CBCB635390}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="13.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="65.140625" customWidth="1"/>
     <col min="2" max="26" width="13.7109375" customWidth="1"/>
@@ -13347,7 +13776,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FE31E21-0350-44E7-AF13-4CA140505B30}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:1" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A1" s="100" t="s">

</xml_diff>

<commit_message>
[FIX] xlsx: import new lines in sharedStrings
When implementing the multiline text feature, we forgot to change the
xlsx import, that explicitly removed new lines from the sharedStrings
because we didn't support it at the time.

There was also a bug where the whitespace was not preserved in the
sharedStrings, because we extracted the text from the `<si>` element
instead of the `<t>` element that had the attribute xml:space="preserve".

And for multi-line cells to be considered as such by Excel, they need
to have the style `wrapText="1"`.

Task: 4044862
</commit_message>
<xml_diff>
--- a/tests/__xlsx__/xlsx_demo_data.xlsx
+++ b/tests/__xlsx__/xlsx_demo_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27930"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Adrien\odoo\spreadsheet\tests\__xlsx__\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Odoo\spreadsheet\tests\__xlsx__\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{82EC8D04-FB30-4625-805F-DD659B4B146F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0219CD72-FC93-4738-B246-ADCEF801BFC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="5" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="5" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -30,9 +30,9 @@
   <externalReferences>
     <externalReference r:id="rId14"/>
   </externalReferences>
-  <calcPr calcId="191028" calcCompleted="0"/>
+  <calcPr calcId="191028"/>
   <pivotCaches>
-    <pivotCache cacheId="828" r:id="rId15"/>
+    <pivotCache cacheId="0" r:id="rId15"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="466" uniqueCount="417">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="467" uniqueCount="418">
   <si>
     <t>CF =42</t>
   </si>
@@ -1306,6 +1306,9 @@
   <si>
     <t>This text have
  a newLine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">      with whitespace before</t>
   </si>
 </sst>
 </file>
@@ -1321,7 +1324,7 @@
     <numFmt numFmtId="169" formatCode="#,##0&quot; EUR €&quot;"/>
     <numFmt numFmtId="170" formatCode="&quot;€&quot;#,##0.00\ &quot;€&quot;"/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="25" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -2198,6 +2201,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -2210,7 +2214,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
@@ -2218,157 +2221,6 @@
     <cellStyle name="Normal 2" xfId="1" xr:uid="{1493241F-B85D-4F84-BBA0-86191B8FD032}"/>
   </cellStyles>
   <dxfs count="46">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-        <strike/>
-        <u/>
-        <color theme="7"/>
-      </font>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <fill>
-        <patternFill patternType="lightTrellis">
-          <fgColor theme="4"/>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE06666"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFB6D7A8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -2775,6 +2627,157 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+        <strike/>
+        <u/>
+        <color theme="7"/>
+      </font>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <fill>
+        <patternFill patternType="lightTrellis">
+          <fgColor theme="4"/>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE06666"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFB6D7A8"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor theme="4"/>
         </patternFill>
       </fill>
@@ -2873,7 +2876,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="fr-FR"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -3195,7 +3198,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-US"/>
+              <a:endParaRPr lang="fr-FR"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -3228,7 +3231,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="en-US"/>
+            <a:endParaRPr lang="fr-FR"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="88853993"/>
@@ -3299,7 +3302,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-US"/>
+              <a:endParaRPr lang="fr-FR"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -3332,7 +3335,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="en-US"/>
+            <a:endParaRPr lang="fr-FR"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="17781237"/>
@@ -3376,7 +3379,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="fr-FR"/>
         </a:p>
       </c:txPr>
     </c:legend>
@@ -3404,7 +3407,7 @@
       <a:pPr>
         <a:defRPr/>
       </a:pPr>
-      <a:endParaRPr lang="en-US"/>
+      <a:endParaRPr lang="fr-FR"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
@@ -3731,7 +3734,7 @@
                 <a:latin typeface="+mn-lt"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="en-US"/>
+            <a:endParaRPr lang="fr-FR"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="88853993"/>
@@ -3793,7 +3796,7 @@
                 <a:latin typeface="+mn-lt"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="en-US"/>
+            <a:endParaRPr lang="fr-FR"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="17781237"/>
@@ -3821,7 +3824,7 @@
               <a:latin typeface="+mn-lt"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="fr-FR"/>
         </a:p>
       </c:txPr>
     </c:legend>
@@ -4439,7 +4442,7 @@
               <a:latin typeface="+mn-lt"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="fr-FR"/>
         </a:p>
       </c:txPr>
     </c:legend>
@@ -4805,7 +4808,7 @@
               <a:latin typeface="+mn-lt"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="fr-FR"/>
         </a:p>
       </c:txPr>
     </c:legend>
@@ -5017,7 +5020,7 @@
                 <a:latin typeface="+mn-lt"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="en-US"/>
+            <a:endParaRPr lang="fr-FR"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="88853993"/>
@@ -5076,7 +5079,7 @@
                 <a:latin typeface="+mn-lt"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="en-US"/>
+            <a:endParaRPr lang="fr-FR"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="17781237"/>
@@ -5104,7 +5107,7 @@
               <a:latin typeface="+mn-lt"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="fr-FR"/>
         </a:p>
       </c:txPr>
     </c:legend>
@@ -5450,7 +5453,7 @@
                 <a:latin typeface="+mn-lt"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="en-US"/>
+            <a:endParaRPr lang="fr-FR"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="88853993"/>
@@ -5512,7 +5515,7 @@
                 <a:latin typeface="+mn-lt"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="en-US"/>
+            <a:endParaRPr lang="fr-FR"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="17781237"/>
@@ -5540,7 +5543,7 @@
               <a:latin typeface="+mn-lt"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="fr-FR"/>
         </a:p>
       </c:txPr>
     </c:legend>
@@ -5867,7 +5870,7 @@
                 <a:latin typeface="+mn-lt"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="en-US"/>
+            <a:endParaRPr lang="fr-FR"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="344680958"/>
@@ -5943,7 +5946,7 @@
                 <a:latin typeface="+mn-lt"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="en-US"/>
+            <a:endParaRPr lang="fr-FR"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="998664793"/>
@@ -5966,7 +5969,7 @@
               <a:latin typeface="+mn-lt"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="fr-FR"/>
         </a:p>
       </c:txPr>
     </c:legend>
@@ -6942,7 +6945,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9B3CE3F5-58D8-48A3-B9C6-24D1506C9F5C}" name="PivotTable1" cacheId="828" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9B3CE3F5-58D8-48A3-B9C6-24D1506C9F5C}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="C3:L21" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="5">
     <pivotField axis="axisRow" showAll="0">
@@ -7092,7 +7095,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{09C35CC7-7259-4A97-8FEA-EDB47375DF08}" name="Table3" displayName="Table3" ref="C3:J6" totalsRowCount="1" headerRowDxfId="17" dataDxfId="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{09C35CC7-7259-4A97-8FEA-EDB47375DF08}" name="Table3" displayName="Table3" ref="C3:J6" totalsRowCount="1" headerRowDxfId="43" dataDxfId="42">
   <autoFilter ref="C3:J5" xr:uid="{09C35CC7-7259-4A97-8FEA-EDB47375DF08}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -7104,22 +7107,22 @@
     <filterColumn colId="7" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{C4EE018E-238B-42BA-9035-DB01FA5420D3}" name="Name" totalsRowLabel="Total" dataDxfId="14" totalsRowDxfId="15"/>
-    <tableColumn id="2" xr3:uid="{C1F6911F-9482-4C98-BBFB-21D9CAA66DA4}" name="Age" totalsRowFunction="sum" dataDxfId="12" totalsRowDxfId="13"/>
-    <tableColumn id="5" xr3:uid="{3CE9F5DA-0A57-4696-B4E0-53601C3B7798}" name="Rank" totalsRowFunction="sum" dataDxfId="10" totalsRowDxfId="11"/>
-    <tableColumn id="6" xr3:uid="{34912838-665C-4472-B558-25990E5B148D}" name="Rank+Age =E4+D4" totalsRowFunction="sum" dataDxfId="8" totalsRowDxfId="9">
+    <tableColumn id="1" xr3:uid="{C4EE018E-238B-42BA-9035-DB01FA5420D3}" name="Name" totalsRowLabel="Total" dataDxfId="41" totalsRowDxfId="40"/>
+    <tableColumn id="2" xr3:uid="{C1F6911F-9482-4C98-BBFB-21D9CAA66DA4}" name="Age" totalsRowFunction="sum" dataDxfId="39" totalsRowDxfId="38"/>
+    <tableColumn id="5" xr3:uid="{3CE9F5DA-0A57-4696-B4E0-53601C3B7798}" name="Rank" totalsRowFunction="sum" dataDxfId="37" totalsRowDxfId="36"/>
+    <tableColumn id="6" xr3:uid="{34912838-665C-4472-B558-25990E5B148D}" name="Rank+Age =E4+D4" totalsRowFunction="sum" dataDxfId="35" totalsRowDxfId="34">
       <calculatedColumnFormula>Table3[[#This Row],[Rank]]+Table3[[#This Row],[Age]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{89D90022-7073-4067-BAF8-1587D27C4AFB}" name="Data =SUM(E4:E5)" totalsRowFunction="sum" dataDxfId="6" totalsRowDxfId="7">
+    <tableColumn id="7" xr3:uid="{89D90022-7073-4067-BAF8-1587D27C4AFB}" name="Data =SUM(E4:E5)" totalsRowFunction="sum" dataDxfId="33" totalsRowDxfId="32">
       <calculatedColumnFormula>SUM(Table3[Rank])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{B2A7E5BB-A379-492B-9484-72F2FD1FF3A0}" name="All =SUM(E3:E6)" totalsRowFunction="sum" dataDxfId="4" totalsRowDxfId="5">
+    <tableColumn id="8" xr3:uid="{B2A7E5BB-A379-492B-9484-72F2FD1FF3A0}" name="All =SUM(E3:E6)" totalsRowFunction="sum" dataDxfId="31" totalsRowDxfId="30">
       <calculatedColumnFormula>SUM(Table3[[#All],[Rank]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{3C532A69-E4BC-4A20-A922-4BCAA0D3FEC9}" name="Totals =E6" totalsRowFunction="sum" dataDxfId="2" totalsRowDxfId="3">
+    <tableColumn id="9" xr3:uid="{3C532A69-E4BC-4A20-A922-4BCAA0D3FEC9}" name="Totals =E6" totalsRowFunction="sum" dataDxfId="29" totalsRowDxfId="28">
       <calculatedColumnFormula>Table3[[#Totals],[Rank]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{35E9E9C3-9148-468A-85B6-19290CEB6F00}" name="Headers =E3" totalsRowFunction="sum" dataDxfId="0" totalsRowDxfId="1">
+    <tableColumn id="10" xr3:uid="{35E9E9C3-9148-468A-85B6-19290CEB6F00}" name="Headers =E3" totalsRowFunction="sum" dataDxfId="27" totalsRowDxfId="26">
       <calculatedColumnFormula>Table3[[#Headers],[Rank]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -7229,9 +7232,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -7269,7 +7272,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -7375,7 +7378,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -7517,7 +7520,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -7526,7 +7529,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{385D5EBC-45F5-4C42-AA75-560DF70B9F2E}">
   <dimension ref="A1:L35"/>
-  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.28515625" customWidth="1"/>
     <col min="2" max="2" width="13.7109375" customWidth="1"/>
@@ -7535,7 +7538,7 @@
     <col min="6" max="26" width="13.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="38.25" customHeight="1">
+    <row r="1" spans="1:12" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="22"/>
       <c r="C1" s="1" t="s">
         <v>0</v>
@@ -7544,7 +7547,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="27.75">
+    <row r="2" spans="1:12" ht="27.75" x14ac:dyDescent="0.2">
       <c r="B2" s="23" t="s">
         <v>2</v>
       </c>
@@ -7557,25 +7560,25 @@
       <c r="H2" s="105" t="s">
         <v>4</v>
       </c>
-      <c r="I2" s="110"/>
+      <c r="I2" s="106"/>
       <c r="K2" s="4"/>
     </row>
-    <row r="3" spans="1:12" ht="17.25" customHeight="1">
+    <row r="3" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F3" s="5" t="s">
         <v>5</v>
       </c>
       <c r="G3" s="2">
         <v>8</v>
       </c>
-      <c r="H3" s="110"/>
-      <c r="I3" s="110"/>
+      <c r="H3" s="106"/>
+      <c r="I3" s="106"/>
       <c r="J3" s="6"/>
-      <c r="K3" s="106">
+      <c r="K3" s="107">
         <v>5</v>
       </c>
       <c r="L3" s="7"/>
     </row>
-    <row r="4" spans="1:12" ht="17.25" customHeight="1">
+    <row r="4" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="8" t="s">
         <v>6</v>
       </c>
@@ -7588,50 +7591,50 @@
       <c r="G4" s="2">
         <v>9</v>
       </c>
-      <c r="H4" s="110"/>
-      <c r="I4" s="110"/>
+      <c r="H4" s="106"/>
+      <c r="I4" s="106"/>
       <c r="J4" s="6"/>
-      <c r="K4" s="107"/>
+      <c r="K4" s="108"/>
       <c r="L4" s="7"/>
     </row>
-    <row r="5" spans="1:12" ht="17.25" customHeight="1">
+    <row r="5" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C5" s="2">
         <v>42</v>
       </c>
       <c r="G5" s="2">
         <v>15</v>
       </c>
-      <c r="H5" s="110"/>
-      <c r="I5" s="110"/>
+      <c r="H5" s="106"/>
+      <c r="I5" s="106"/>
       <c r="J5" s="6"/>
-      <c r="K5" s="107"/>
+      <c r="K5" s="108"/>
       <c r="L5" s="7"/>
     </row>
-    <row r="6" spans="1:12" ht="17.25" customHeight="1">
+    <row r="6" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="G6" s="2">
         <v>22</v>
       </c>
       <c r="J6" s="6"/>
-      <c r="K6" s="107"/>
+      <c r="K6" s="108"/>
       <c r="L6" s="7"/>
     </row>
-    <row r="7" spans="1:12" ht="17.25" customHeight="1">
+    <row r="7" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C7" s="2">
         <v>3</v>
       </c>
       <c r="J7" s="6"/>
-      <c r="K7" s="107"/>
+      <c r="K7" s="108"/>
       <c r="L7" s="7"/>
     </row>
-    <row r="8" spans="1:12" ht="17.25" customHeight="1">
+    <row r="8" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="G8" s="2">
         <v>30</v>
       </c>
       <c r="J8" s="6"/>
-      <c r="K8" s="108"/>
+      <c r="K8" s="109"/>
       <c r="L8" s="7"/>
     </row>
-    <row r="9" spans="1:12" ht="17.25" customHeight="1">
+    <row r="9" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="10" t="s">
         <v>8</v>
       </c>
@@ -7641,7 +7644,7 @@
       </c>
       <c r="K9" s="11"/>
     </row>
-    <row r="10" spans="1:12" ht="17.25" customHeight="1">
+    <row r="10" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C10" s="2">
         <f>SUM(C4:C7)</f>
         <v>57.4</v>
@@ -7650,13 +7653,13 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="17.25" customHeight="1">
+    <row r="11" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C11" s="2">
         <f>-(3+C7*SUM(C4:C7))</f>
         <v>-175.2</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="17.25" customHeight="1">
+    <row r="12" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C12" s="2">
         <f>SUM(C9:C11)</f>
         <v>-63.399999999999991</v>
@@ -7665,13 +7668,13 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="17.25" customHeight="1">
+    <row r="13" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="G13" s="2">
         <f>A1+A2+A3+A4+A5+A6+A7+A8+A9+A10+A11+A12+A13+A14+A15+A16+A17+A18</f>
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="17.25" customHeight="1">
+    <row r="14" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="12" t="s">
         <v>11</v>
       </c>
@@ -7680,32 +7683,32 @@
         <v>#CYCLE</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="17.25" customHeight="1">
+    <row r="15" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C15" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:12" ht="17.25" customHeight="1">
+    <row r="16" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C16" s="2" t="str">
         <f>C15</f>
         <v>=(+</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="17.25" customHeight="1">
+    <row r="17" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C17" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="17.25" customHeight="1">
+    <row r="18" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C18" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="17.25" customHeight="1">
+    <row r="19" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="E19" s="4"/>
       <c r="G19" s="4"/>
     </row>
-    <row r="20" spans="1:9" ht="17.25" customHeight="1">
+    <row r="20" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B20" s="6"/>
       <c r="C20" s="7" t="s">
         <v>15</v>
@@ -7719,7 +7722,7 @@
       </c>
       <c r="H20" s="7"/>
     </row>
-    <row r="21" spans="1:9" ht="17.25" customHeight="1">
+    <row r="21" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="14" t="s">
         <v>18</v>
       </c>
@@ -7729,7 +7732,7 @@
       </c>
       <c r="G21" s="11"/>
     </row>
-    <row r="23" spans="1:9" ht="17.25" customHeight="1">
+    <row r="23" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="14" t="s">
         <v>19</v>
       </c>
@@ -7743,7 +7746,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="17.25" customHeight="1">
+    <row r="24" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C24" s="17">
         <v>10</v>
       </c>
@@ -7754,7 +7757,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="17.25" customHeight="1">
+    <row r="25" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C25" s="17">
         <v>10.122999999999999</v>
       </c>
@@ -7765,7 +7768,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="17.25" customHeight="1">
+    <row r="26" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="2" t="s">
         <v>20</v>
       </c>
@@ -7779,7 +7782,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="17.25" customHeight="1">
+    <row r="27" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
         <v>22</v>
       </c>
@@ -7796,7 +7799,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="17.25" customHeight="1">
+    <row r="28" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
         <v>23</v>
       </c>
@@ -7813,7 +7816,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="17.25" customHeight="1">
+    <row r="29" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
         <v>24</v>
       </c>
@@ -7830,7 +7833,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="17.25" customHeight="1">
+    <row r="30" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
         <v>25</v>
       </c>
@@ -7847,7 +7850,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="17.25" customHeight="1">
+    <row r="31" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
         <v>26</v>
       </c>
@@ -7864,7 +7867,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="17.25" customHeight="1">
+    <row r="32" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
         <v>27</v>
       </c>
@@ -7881,7 +7884,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="17.25" customHeight="1">
+    <row r="33" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
         <v>28</v>
       </c>
@@ -7898,7 +7901,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="17.25" customHeight="1">
+    <row r="34" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
         <v>29</v>
       </c>
@@ -7909,7 +7912,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="35" spans="1:9" ht="17.25" customHeight="1">
+    <row r="35" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
         <v>30</v>
       </c>
@@ -7926,7 +7929,7 @@
     <mergeCell ref="K3:K8"/>
   </mergeCells>
   <conditionalFormatting sqref="C1:C100 B21">
-    <cfRule type="cellIs" dxfId="43" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="25" priority="1" operator="equal">
       <formula>42</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7971,7 +7974,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F7A934C-2218-4A12-8B75-EE28D615D774}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -7980,7 +7983,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96301BE1-D86D-4D45-870D-85A75D53FC99}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -7989,7 +7992,7 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B10A8834-0E20-4F80-8813-3ACA5527B377}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="65.140625" customWidth="1"/>
     <col min="2" max="26" width="13.7109375" customWidth="1"/>
@@ -8006,7 +8009,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8016,12 +8019,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0630FA18-71FC-4ACD-8379-39A3603D1DD6}">
   <dimension ref="A1:R163"/>
-  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="26" width="13.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="17.25" customHeight="1">
+    <row r="1" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>31</v>
       </c>
@@ -8056,7 +8059,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="17.25" customHeight="1">
+    <row r="2" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>41</v>
       </c>
@@ -8102,7 +8105,7 @@
         <v>1230.7</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="17.25" customHeight="1">
+    <row r="3" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>43</v>
       </c>
@@ -8148,7 +8151,7 @@
         <v>1217.7</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="17.25" customHeight="1">
+    <row r="4" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>45</v>
       </c>
@@ -8194,7 +8197,7 @@
         <v>1230.7</v>
       </c>
     </row>
-    <row r="5" spans="1:18" ht="17.25" customHeight="1">
+    <row r="5" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>47</v>
       </c>
@@ -8240,7 +8243,7 @@
         <v>1246.7</v>
       </c>
     </row>
-    <row r="6" spans="1:18" ht="17.25" customHeight="1">
+    <row r="6" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>49</v>
       </c>
@@ -8286,7 +8289,7 @@
         <v>1213.7</v>
       </c>
     </row>
-    <row r="7" spans="1:18" ht="17.25" customHeight="1">
+    <row r="7" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>52</v>
       </c>
@@ -8320,7 +8323,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:18" ht="17.25" customHeight="1">
+    <row r="8" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>54</v>
       </c>
@@ -8354,7 +8357,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:18" ht="17.25" customHeight="1">
+    <row r="9" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>56</v>
       </c>
@@ -8385,7 +8388,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="17.25" customHeight="1">
+    <row r="10" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>58</v>
       </c>
@@ -8401,7 +8404,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:18" ht="17.25" customHeight="1">
+    <row r="11" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>59</v>
       </c>
@@ -8420,7 +8423,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="12" spans="1:18" ht="17.25" customHeight="1">
+    <row r="12" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>61</v>
       </c>
@@ -8451,7 +8454,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="13" spans="1:18" ht="17.25" customHeight="1">
+    <row r="13" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>62</v>
       </c>
@@ -8482,7 +8485,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="14" spans="1:18" ht="17.25" customHeight="1">
+    <row r="14" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>67</v>
       </c>
@@ -8498,7 +8501,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:18" ht="17.25" customHeight="1">
+    <row r="15" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>68</v>
       </c>
@@ -8514,7 +8517,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:18" ht="17.25" customHeight="1">
+    <row r="16" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>69</v>
       </c>
@@ -8530,7 +8533,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="17.25" customHeight="1">
+    <row r="17" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>70</v>
       </c>
@@ -8546,7 +8549,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="17.25" customHeight="1">
+    <row r="18" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
         <v>71</v>
       </c>
@@ -8562,7 +8565,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="17.25" customHeight="1">
+    <row r="19" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>72</v>
       </c>
@@ -8578,7 +8581,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="17.25" customHeight="1">
+    <row r="20" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>73</v>
       </c>
@@ -8594,7 +8597,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="17.25" customHeight="1">
+    <row r="21" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>74</v>
       </c>
@@ -8610,7 +8613,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="17.25" customHeight="1">
+    <row r="22" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>76</v>
       </c>
@@ -8626,7 +8629,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="17.25" customHeight="1">
+    <row r="23" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
         <v>77</v>
       </c>
@@ -8642,7 +8645,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="17.25" customHeight="1">
+    <row r="24" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
         <v>78</v>
       </c>
@@ -8659,7 +8662,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="17.25" customHeight="1">
+    <row r="25" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>79</v>
       </c>
@@ -8675,7 +8678,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:4" ht="17.25" customHeight="1">
+    <row r="26" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
         <v>81</v>
       </c>
@@ -8691,7 +8694,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="17.25" customHeight="1">
+    <row r="27" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
         <v>82</v>
       </c>
@@ -8707,7 +8710,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="17.25" customHeight="1">
+    <row r="28" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
         <v>83</v>
       </c>
@@ -8724,7 +8727,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="17.25" customHeight="1">
+    <row r="29" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
         <v>84</v>
       </c>
@@ -8740,7 +8743,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:4" ht="17.25" customHeight="1">
+    <row r="30" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
         <v>85</v>
       </c>
@@ -8756,7 +8759,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:4" ht="17.25" customHeight="1">
+    <row r="31" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
         <v>86</v>
       </c>
@@ -8772,7 +8775,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:4" ht="17.25" customHeight="1">
+    <row r="32" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
         <v>87</v>
       </c>
@@ -8788,7 +8791,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:4" ht="17.25" customHeight="1">
+    <row r="33" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
         <v>88</v>
       </c>
@@ -8804,7 +8807,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:4" ht="17.25" customHeight="1">
+    <row r="34" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
         <v>89</v>
       </c>
@@ -8820,7 +8823,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:4" ht="17.25" customHeight="1">
+    <row r="35" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
         <v>90</v>
       </c>
@@ -8836,7 +8839,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:4" ht="17.25" customHeight="1">
+    <row r="36" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
         <v>91</v>
       </c>
@@ -8852,7 +8855,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:4" ht="17.25" customHeight="1">
+    <row r="37" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
         <v>92</v>
       </c>
@@ -8868,7 +8871,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:4" ht="17.25" customHeight="1">
+    <row r="38" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
         <v>93</v>
       </c>
@@ -8885,7 +8888,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:4" ht="17.25" customHeight="1">
+    <row r="39" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
         <v>94</v>
       </c>
@@ -8901,7 +8904,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:4" ht="17.25" customHeight="1">
+    <row r="40" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
         <v>95</v>
       </c>
@@ -8917,7 +8920,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:4" ht="17.25" customHeight="1">
+    <row r="41" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
         <v>96</v>
       </c>
@@ -8933,7 +8936,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:4" ht="17.25" customHeight="1">
+    <row r="42" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
         <v>97</v>
       </c>
@@ -8949,7 +8952,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:4" ht="17.25" customHeight="1">
+    <row r="43" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
         <v>98</v>
       </c>
@@ -8965,7 +8968,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:4" ht="17.25" customHeight="1">
+    <row r="44" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
         <v>99</v>
       </c>
@@ -8981,7 +8984,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:4" ht="17.25" customHeight="1">
+    <row r="45" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
         <v>100</v>
       </c>
@@ -8997,7 +9000,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:4" ht="17.25" customHeight="1">
+    <row r="46" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
         <v>101</v>
       </c>
@@ -9013,7 +9016,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:4" ht="17.25" customHeight="1">
+    <row r="47" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
         <v>102</v>
       </c>
@@ -9029,7 +9032,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:4" ht="17.25" customHeight="1">
+    <row r="48" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
         <v>103</v>
       </c>
@@ -9045,7 +9048,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:4" ht="17.25" customHeight="1">
+    <row r="49" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
         <v>104</v>
       </c>
@@ -9061,7 +9064,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:4" ht="17.25" customHeight="1">
+    <row r="50" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
         <v>105</v>
       </c>
@@ -9078,7 +9081,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:4" ht="17.25" customHeight="1">
+    <row r="51" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="2" t="s">
         <v>106</v>
       </c>
@@ -9095,7 +9098,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:4" ht="17.25" customHeight="1">
+    <row r="52" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
         <v>107</v>
       </c>
@@ -9111,7 +9114,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:4" ht="17.25" customHeight="1">
+    <row r="53" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="2" t="s">
         <v>108</v>
       </c>
@@ -9127,7 +9130,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:4" ht="17.25" customHeight="1">
+    <row r="54" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
         <v>109</v>
       </c>
@@ -9143,7 +9146,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:4" ht="17.25" customHeight="1">
+    <row r="55" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="2" t="s">
         <v>110</v>
       </c>
@@ -9159,7 +9162,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:4" ht="17.25" customHeight="1">
+    <row r="56" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="2" t="s">
         <v>111</v>
       </c>
@@ -9175,7 +9178,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:4" ht="17.25" customHeight="1">
+    <row r="57" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="2" t="s">
         <v>112</v>
       </c>
@@ -9191,7 +9194,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:4" ht="17.25" customHeight="1">
+    <row r="58" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="2" t="s">
         <v>113</v>
       </c>
@@ -9207,7 +9210,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:4" ht="17.25" customHeight="1">
+    <row r="59" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="2" t="s">
         <v>114</v>
       </c>
@@ -9223,7 +9226,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:4" ht="17.25" customHeight="1">
+    <row r="60" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="2" t="s">
         <v>115</v>
       </c>
@@ -9239,7 +9242,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:4" ht="17.25" customHeight="1">
+    <row r="61" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="2" t="s">
         <v>116</v>
       </c>
@@ -9255,7 +9258,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:4" ht="17.25" customHeight="1">
+    <row r="62" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="2" t="s">
         <v>117</v>
       </c>
@@ -9271,7 +9274,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:4" ht="17.25" customHeight="1">
+    <row r="63" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="2" t="s">
         <v>118</v>
       </c>
@@ -9287,7 +9290,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:4" ht="17.25" customHeight="1">
+    <row r="64" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="2" t="s">
         <v>119</v>
       </c>
@@ -9303,7 +9306,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:4" ht="17.25" customHeight="1">
+    <row r="65" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="2" t="s">
         <v>120</v>
       </c>
@@ -9319,7 +9322,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:4" ht="17.25" customHeight="1">
+    <row r="66" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="2" t="s">
         <v>121</v>
       </c>
@@ -9335,7 +9338,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:4" ht="17.25" customHeight="1">
+    <row r="67" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="2" t="s">
         <v>122</v>
       </c>
@@ -9351,7 +9354,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:4" ht="17.25" customHeight="1">
+    <row r="68" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="2" t="s">
         <v>123</v>
       </c>
@@ -9367,7 +9370,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:4" ht="17.25" customHeight="1">
+    <row r="69" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="2" t="s">
         <v>125</v>
       </c>
@@ -9383,7 +9386,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:4" ht="17.25" customHeight="1">
+    <row r="70" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="2" t="s">
         <v>127</v>
       </c>
@@ -9399,7 +9402,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:4" ht="17.25" customHeight="1">
+    <row r="71" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="2" t="s">
         <v>129</v>
       </c>
@@ -9415,7 +9418,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:4" ht="17.25" customHeight="1">
+    <row r="72" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="2" t="s">
         <v>130</v>
       </c>
@@ -9431,7 +9434,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:4" ht="17.25" customHeight="1">
+    <row r="73" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="2" t="s">
         <v>131</v>
       </c>
@@ -9447,7 +9450,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:4" ht="17.25" customHeight="1">
+    <row r="74" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="2" t="s">
         <v>132</v>
       </c>
@@ -9463,7 +9466,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:4" ht="17.25" customHeight="1">
+    <row r="75" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="2" t="s">
         <v>133</v>
       </c>
@@ -9479,7 +9482,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="1:4" ht="17.25" customHeight="1">
+    <row r="76" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="2" t="s">
         <v>134</v>
       </c>
@@ -9495,7 +9498,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:4" ht="17.25" customHeight="1">
+    <row r="77" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="2" t="s">
         <v>135</v>
       </c>
@@ -9511,7 +9514,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="78" spans="1:4" ht="17.25" customHeight="1">
+    <row r="78" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="2" t="s">
         <v>136</v>
       </c>
@@ -9527,7 +9530,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:4" ht="17.25" customHeight="1">
+    <row r="79" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="2" t="s">
         <v>137</v>
       </c>
@@ -9543,7 +9546,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="1:4" ht="17.25" customHeight="1">
+    <row r="80" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="2" t="s">
         <v>138</v>
       </c>
@@ -9559,7 +9562,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="1:4" ht="17.25" customHeight="1">
+    <row r="81" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="2" t="s">
         <v>139</v>
       </c>
@@ -9575,7 +9578,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:4" ht="17.25" customHeight="1">
+    <row r="82" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="2" t="s">
         <v>141</v>
       </c>
@@ -9591,7 +9594,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:4" ht="17.25" customHeight="1">
+    <row r="83" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="2" t="s">
         <v>142</v>
       </c>
@@ -9607,7 +9610,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="1:4" ht="17.25" customHeight="1">
+    <row r="84" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="2" t="s">
         <v>143</v>
       </c>
@@ -9623,7 +9626,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:4" ht="17.25" customHeight="1">
+    <row r="85" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="2" t="s">
         <v>144</v>
       </c>
@@ -9639,7 +9642,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="86" spans="1:4" ht="17.25" customHeight="1">
+    <row r="86" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="2" t="s">
         <v>146</v>
       </c>
@@ -9655,7 +9658,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="1:4" ht="17.25" customHeight="1">
+    <row r="87" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="2" t="s">
         <v>147</v>
       </c>
@@ -9671,7 +9674,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="1:4" ht="17.25" customHeight="1">
+    <row r="88" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="2" t="s">
         <v>148</v>
       </c>
@@ -9687,7 +9690,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="1:4" ht="17.25" customHeight="1">
+    <row r="89" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" s="2" t="s">
         <v>149</v>
       </c>
@@ -9703,7 +9706,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="90" spans="1:4" ht="17.25" customHeight="1">
+    <row r="90" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" s="2" t="s">
         <v>150</v>
       </c>
@@ -9719,7 +9722,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:4" ht="17.25" customHeight="1">
+    <row r="91" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" s="2" t="s">
         <v>151</v>
       </c>
@@ -9735,7 +9738,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="1:4" ht="17.25" customHeight="1">
+    <row r="92" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" s="2" t="s">
         <v>152</v>
       </c>
@@ -9751,7 +9754,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:4" ht="17.25" customHeight="1">
+    <row r="93" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="2" t="s">
         <v>153</v>
       </c>
@@ -9767,7 +9770,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="94" spans="1:4" ht="17.25" customHeight="1">
+    <row r="94" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" s="2" t="s">
         <v>154</v>
       </c>
@@ -9783,7 +9786,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="95" spans="1:4" ht="17.25" customHeight="1">
+    <row r="95" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" s="2" t="s">
         <v>155</v>
       </c>
@@ -9799,7 +9802,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="96" spans="1:4" ht="17.25" customHeight="1">
+    <row r="96" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" s="2" t="s">
         <v>156</v>
       </c>
@@ -9815,7 +9818,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="97" spans="1:4" ht="17.25" customHeight="1">
+    <row r="97" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" s="2" t="s">
         <v>157</v>
       </c>
@@ -9831,7 +9834,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="98" spans="1:4" ht="17.25" customHeight="1">
+    <row r="98" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" s="2" t="s">
         <v>158</v>
       </c>
@@ -9847,7 +9850,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="99" spans="1:4" ht="17.25" customHeight="1">
+    <row r="99" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" s="2" t="s">
         <v>159</v>
       </c>
@@ -9863,20 +9866,20 @@
         <v>1</v>
       </c>
     </row>
-    <row r="100" spans="1:4" ht="17.25" customHeight="1">
+    <row r="100" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" s="2" t="s">
         <v>160</v>
       </c>
       <c r="B100" s="20">
         <f ca="1">NOW()</f>
-        <v>45512.434189004627</v>
+        <v>45643.379599189815</v>
       </c>
       <c r="D100" s="2">
         <f ca="1">IF(ISNUMBER(B100),1,0)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="101" spans="1:4" ht="17.25" customHeight="1">
+    <row r="101" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" s="2" t="s">
         <v>161</v>
       </c>
@@ -9892,7 +9895,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="102" spans="1:4" ht="17.25" customHeight="1">
+    <row r="102" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A102" s="2" t="s">
         <v>162</v>
       </c>
@@ -9908,7 +9911,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="103" spans="1:4" ht="17.25" customHeight="1">
+    <row r="103" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A103" s="2" t="s">
         <v>163</v>
       </c>
@@ -9924,7 +9927,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="104" spans="1:4" ht="17.25" customHeight="1">
+    <row r="104" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104" s="2" t="s">
         <v>164</v>
       </c>
@@ -9940,7 +9943,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="105" spans="1:4" ht="17.25" customHeight="1">
+    <row r="105" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" s="2" t="s">
         <v>165</v>
       </c>
@@ -9956,7 +9959,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="106" spans="1:4" ht="17.25" customHeight="1">
+    <row r="106" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A106" s="2" t="s">
         <v>166</v>
       </c>
@@ -9972,7 +9975,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="107" spans="1:4" ht="17.25" customHeight="1">
+    <row r="107" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A107" s="2" t="s">
         <v>167</v>
       </c>
@@ -9988,7 +9991,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="1:4" ht="17.25" customHeight="1">
+    <row r="108" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" s="2" t="s">
         <v>168</v>
       </c>
@@ -10004,7 +10007,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="109" spans="1:4" ht="17.25" customHeight="1">
+    <row r="109" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" s="2" t="s">
         <v>169</v>
       </c>
@@ -10020,7 +10023,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="110" spans="1:4" ht="17.25" customHeight="1">
+    <row r="110" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" s="2" t="s">
         <v>170</v>
       </c>
@@ -10036,7 +10039,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="111" spans="1:4" ht="17.25" customHeight="1">
+    <row r="111" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A111" s="2" t="s">
         <v>171</v>
       </c>
@@ -10052,12 +10055,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="112" spans="1:4" ht="17.25" customHeight="1">
+    <row r="112" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A112" s="2"/>
       <c r="B112" s="2"/>
       <c r="D112" s="2"/>
     </row>
-    <row r="113" spans="1:4" ht="17.25" customHeight="1">
+    <row r="113" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A113" s="2" t="s">
         <v>172</v>
       </c>
@@ -10073,7 +10076,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="114" spans="1:4" ht="17.25" customHeight="1">
+    <row r="114" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A114" s="2" t="s">
         <v>173</v>
       </c>
@@ -10089,7 +10092,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="115" spans="1:4" ht="17.25" customHeight="1">
+    <row r="115" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A115" s="2" t="s">
         <v>175</v>
       </c>
@@ -10105,7 +10108,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="116" spans="1:4" ht="17.25" customHeight="1">
+    <row r="116" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" s="2" t="s">
         <v>177</v>
       </c>
@@ -10121,7 +10124,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="117" spans="1:4" ht="17.25" customHeight="1">
+    <row r="117" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A117" s="2" t="s">
         <v>178</v>
       </c>
@@ -10137,7 +10140,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="118" spans="1:4" ht="17.25" customHeight="1">
+    <row r="118" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A118" s="2" t="s">
         <v>179</v>
       </c>
@@ -10153,7 +10156,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="119" spans="1:4" ht="17.25" customHeight="1">
+    <row r="119" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A119" s="2" t="s">
         <v>180</v>
       </c>
@@ -10169,7 +10172,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="120" spans="1:4" ht="17.25" customHeight="1">
+    <row r="120" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A120" s="2" t="s">
         <v>181</v>
       </c>
@@ -10185,7 +10188,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="121" spans="1:4" ht="17.25" customHeight="1">
+    <row r="121" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A121" s="2" t="s">
         <v>182</v>
       </c>
@@ -10201,7 +10204,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="122" spans="1:4" ht="17.25" customHeight="1">
+    <row r="122" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A122" s="2" t="s">
         <v>183</v>
       </c>
@@ -10217,7 +10220,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="123" spans="1:4" ht="17.25" customHeight="1">
+    <row r="123" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A123" s="2" t="s">
         <v>184</v>
       </c>
@@ -10233,7 +10236,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="124" spans="1:4" ht="17.25" customHeight="1">
+    <row r="124" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A124" s="2" t="s">
         <v>185</v>
       </c>
@@ -10249,7 +10252,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="125" spans="1:4" ht="17.25" customHeight="1">
+    <row r="125" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A125" s="2" t="s">
         <v>186</v>
       </c>
@@ -10265,7 +10268,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="126" spans="1:4" ht="17.25" customHeight="1">
+    <row r="126" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A126" s="2" t="s">
         <v>187</v>
       </c>
@@ -10281,7 +10284,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="127" spans="1:4" ht="17.25" customHeight="1">
+    <row r="127" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A127" s="2" t="s">
         <v>188</v>
       </c>
@@ -10297,7 +10300,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="128" spans="1:4" ht="17.25" customHeight="1">
+    <row r="128" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A128" s="2" t="s">
         <v>189</v>
       </c>
@@ -10313,7 +10316,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="129" spans="1:4" ht="17.25" customHeight="1">
+    <row r="129" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A129" s="2" t="s">
         <v>190</v>
       </c>
@@ -10329,7 +10332,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="130" spans="1:4" ht="17.25" customHeight="1">
+    <row r="130" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A130" s="2" t="s">
         <v>191</v>
       </c>
@@ -10345,7 +10348,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="131" spans="1:4" ht="17.25" customHeight="1">
+    <row r="131" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A131" s="2" t="s">
         <v>192</v>
       </c>
@@ -10361,7 +10364,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="132" spans="1:4" ht="17.25" customHeight="1">
+    <row r="132" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A132" s="2" t="s">
         <v>193</v>
       </c>
@@ -10377,7 +10380,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="133" spans="1:4" ht="17.25" customHeight="1">
+    <row r="133" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A133" s="2" t="s">
         <v>194</v>
       </c>
@@ -10393,7 +10396,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="134" spans="1:4" ht="17.25" customHeight="1">
+    <row r="134" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A134" s="2" t="s">
         <v>195</v>
       </c>
@@ -10409,7 +10412,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="135" spans="1:4" ht="17.25" customHeight="1">
+    <row r="135" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A135" s="2" t="s">
         <v>196</v>
       </c>
@@ -10425,7 +10428,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="136" spans="1:4" ht="17.25" customHeight="1">
+    <row r="136" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A136" s="2" t="s">
         <v>198</v>
       </c>
@@ -10441,7 +10444,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="137" spans="1:4" ht="17.25" customHeight="1">
+    <row r="137" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A137" s="2" t="s">
         <v>199</v>
       </c>
@@ -10457,7 +10460,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="138" spans="1:4" ht="17.25" customHeight="1">
+    <row r="138" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A138" s="2" t="s">
         <v>200</v>
       </c>
@@ -10473,7 +10476,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="139" spans="1:4" ht="17.25" customHeight="1">
+    <row r="139" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A139" s="2" t="s">
         <v>201</v>
       </c>
@@ -10489,7 +10492,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="140" spans="1:4" ht="17.25" customHeight="1">
+    <row r="140" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A140" s="2" t="s">
         <v>202</v>
       </c>
@@ -10505,7 +10508,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="141" spans="1:4" ht="17.25" customHeight="1">
+    <row r="141" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A141" s="2" t="s">
         <v>203</v>
       </c>
@@ -10521,7 +10524,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="142" spans="1:4" ht="17.25" customHeight="1">
+    <row r="142" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A142" s="2" t="s">
         <v>205</v>
       </c>
@@ -10537,7 +10540,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:4" ht="17.25" customHeight="1">
+    <row r="143" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A143" s="2" t="s">
         <v>206</v>
       </c>
@@ -10553,20 +10556,20 @@
         <v>1</v>
       </c>
     </row>
-    <row r="144" spans="1:4" ht="17.25" customHeight="1">
+    <row r="144" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A144" s="2" t="s">
         <v>207</v>
       </c>
       <c r="B144" s="19">
         <f ca="1">TODAY()</f>
-        <v>45512</v>
+        <v>45643</v>
       </c>
       <c r="D144" s="2">
         <f ca="1">IF(ISNUMBER(B144),1,0)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="145" spans="1:4" ht="17.25" customHeight="1">
+    <row r="145" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A145" s="2" t="s">
         <v>208</v>
       </c>
@@ -10582,7 +10585,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="146" spans="1:4" ht="17.25" customHeight="1">
+    <row r="146" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A146" s="2" t="s">
         <v>210</v>
       </c>
@@ -10598,7 +10601,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="147" spans="1:4" ht="17.25" customHeight="1">
+    <row r="147" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A147" s="2" t="s">
         <v>211</v>
       </c>
@@ -10614,7 +10617,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="148" spans="1:4" ht="17.25" customHeight="1">
+    <row r="148" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A148" s="2" t="s">
         <v>213</v>
       </c>
@@ -10630,7 +10633,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="149" spans="1:4" ht="17.25" customHeight="1">
+    <row r="149" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A149" s="2" t="s">
         <v>214</v>
       </c>
@@ -10646,7 +10649,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="150" spans="1:4" ht="17.25" customHeight="1">
+    <row r="150" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A150" s="2" t="s">
         <v>215</v>
       </c>
@@ -10662,7 +10665,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="151" spans="1:4" ht="17.25" customHeight="1">
+    <row r="151" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A151" s="2" t="s">
         <v>216</v>
       </c>
@@ -10678,7 +10681,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="152" spans="1:4" ht="17.25" customHeight="1">
+    <row r="152" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A152" s="2" t="s">
         <v>217</v>
       </c>
@@ -10694,7 +10697,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="153" spans="1:4" ht="17.25" customHeight="1">
+    <row r="153" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A153" s="2" t="s">
         <v>218</v>
       </c>
@@ -10710,7 +10713,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="154" spans="1:4" ht="17.25" customHeight="1">
+    <row r="154" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A154" s="2" t="s">
         <v>219</v>
       </c>
@@ -10727,7 +10730,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="155" spans="1:4" ht="17.25" customHeight="1">
+    <row r="155" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A155" s="2" t="s">
         <v>220</v>
       </c>
@@ -10743,7 +10746,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="156" spans="1:4" ht="17.25" customHeight="1">
+    <row r="156" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A156" s="2" t="s">
         <v>221</v>
       </c>
@@ -10759,7 +10762,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="157" spans="1:4" ht="17.25" customHeight="1">
+    <row r="157" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A157" s="2" t="s">
         <v>222</v>
       </c>
@@ -10775,7 +10778,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="158" spans="1:4" ht="17.25" customHeight="1">
+    <row r="158" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A158" s="2" t="s">
         <v>223</v>
       </c>
@@ -10791,7 +10794,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="159" spans="1:4" ht="17.25" customHeight="1">
+    <row r="159" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A159" s="2" t="s">
         <v>224</v>
       </c>
@@ -10807,7 +10810,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="160" spans="1:4" ht="17.25" customHeight="1">
+    <row r="160" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A160" s="2" t="s">
         <v>225</v>
       </c>
@@ -10823,7 +10826,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="161" spans="1:4" ht="17.25" customHeight="1">
+    <row r="161" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A161" s="2" t="s">
         <v>226</v>
       </c>
@@ -10839,7 +10842,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="162" spans="1:4" ht="17.25" customHeight="1">
+    <row r="162" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A162" s="2" t="s">
         <v>227</v>
       </c>
@@ -10855,7 +10858,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="163" spans="1:4" ht="17.25" customHeight="1">
+    <row r="163" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A163" s="2" t="s">
         <v>229</v>
       </c>
@@ -10873,10 +10876,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="D1:D180">
-    <cfRule type="cellIs" dxfId="42" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="24" priority="1" operator="equal">
       <formula>1</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="41" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="23" priority="2" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10890,7 +10893,7 @@
     <outlinePr summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:R18"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" outlineLevelRow="2" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" outlineLevelRow="2" outlineLevelCol="2" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="0" hidden="1" customWidth="1"/>
     <col min="6" max="6" width="14.28515625" customWidth="1"/>
@@ -10900,17 +10903,17 @@
     <col min="15" max="18" width="9.140625" outlineLevel="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>230</v>
       </c>
       <c r="C1" t="s">
         <v>231</v>
       </c>
-      <c r="D1" s="109" t="s">
+      <c r="D1" s="110" t="s">
         <v>232</v>
       </c>
-      <c r="E1" s="109"/>
+      <c r="E1" s="110"/>
       <c r="F1" t="s">
         <v>233</v>
       </c>
@@ -10918,19 +10921,19 @@
         <v>234</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2">
         <f>SUM(A1)</f>
         <v>0</v>
       </c>
-      <c r="D2" s="109"/>
-      <c r="E2" s="109"/>
+      <c r="D2" s="110"/>
+      <c r="E2" s="110"/>
       <c r="H2" t="str">
         <f>[1]Feuil1!$A$1</f>
         <v>referenced string</v>
       </c>
     </row>
-    <row r="3" spans="1:8">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="D3" s="86" t="s">
         <v>235</v>
       </c>
@@ -10938,25 +10941,25 @@
         <v>236</v>
       </c>
     </row>
-    <row r="4" spans="1:8" hidden="1">
+    <row r="4" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="75" customHeight="1">
+    <row r="5" spans="1:8" ht="75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="10" spans="1:8" outlineLevel="1"/>
-    <row r="11" spans="1:8" outlineLevel="1"/>
-    <row r="12" spans="1:8" hidden="1" outlineLevel="2"/>
-    <row r="13" spans="1:8" hidden="1" outlineLevel="2"/>
-    <row r="14" spans="1:8" hidden="1" outlineLevel="2"/>
-    <row r="15" spans="1:8" outlineLevel="1" collapsed="1"/>
-    <row r="16" spans="1:8" outlineLevel="1"/>
-    <row r="17" outlineLevel="1"/>
-    <row r="18" outlineLevel="1"/>
+    <row r="10" spans="1:8" outlineLevel="1" x14ac:dyDescent="0.2"/>
+    <row r="11" spans="1:8" outlineLevel="1" x14ac:dyDescent="0.2"/>
+    <row r="12" spans="1:8" hidden="1" outlineLevel="2" x14ac:dyDescent="0.2"/>
+    <row r="13" spans="1:8" hidden="1" outlineLevel="2" x14ac:dyDescent="0.2"/>
+    <row r="14" spans="1:8" hidden="1" outlineLevel="2" x14ac:dyDescent="0.2"/>
+    <row r="15" spans="1:8" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.2"/>
+    <row r="16" spans="1:8" outlineLevel="1" x14ac:dyDescent="0.2"/>
+    <row r="17" outlineLevel="1" x14ac:dyDescent="0.2"/>
+    <row r="18" outlineLevel="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="D1:E2"/>
@@ -10973,14 +10976,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF68F2C0-1053-4FB6-BD74-8A11B0CAF123}">
   <dimension ref="A1:M30"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="17.7109375" customWidth="1"/>
     <col min="5" max="5" width="18.28515625" customWidth="1"/>
     <col min="13" max="13" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="13.5" thickBot="1">
+    <row r="1" spans="1:13" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="69" t="s">
         <v>239</v>
       </c>
@@ -11002,7 +11005,7 @@
       </c>
       <c r="M1" s="37"/>
     </row>
-    <row r="2" spans="1:13">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" s="41" t="s">
         <v>245</v>
       </c>
@@ -11028,7 +11031,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:13">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" s="42" t="s">
         <v>252</v>
       </c>
@@ -11051,7 +11054,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="15">
+    <row r="4" spans="1:13" ht="15" x14ac:dyDescent="0.3">
       <c r="A4" s="43" t="s">
         <v>256</v>
       </c>
@@ -11077,7 +11080,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:13">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" s="44" t="s">
         <v>262</v>
       </c>
@@ -11097,7 +11100,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:13">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" s="45" t="s">
         <v>266</v>
       </c>
@@ -11120,7 +11123,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="15.75">
+    <row r="7" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="46" t="s">
         <v>271</v>
       </c>
@@ -11140,7 +11143,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="21">
+    <row r="8" spans="1:13" ht="21" x14ac:dyDescent="0.35">
       <c r="A8" s="47" t="s">
         <v>275</v>
       </c>
@@ -11163,7 +11166,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:13">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="48" t="s">
         <v>280</v>
       </c>
@@ -11180,7 +11183,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:13">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="49" t="s">
         <v>283</v>
       </c>
@@ -11188,7 +11191,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="13.5" thickBot="1">
+    <row r="11" spans="1:13" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="50" t="s">
         <v>285</v>
       </c>
@@ -11197,7 +11200,7 @@
       </c>
       <c r="F11" s="37"/>
     </row>
-    <row r="12" spans="1:13" ht="18.75" customHeight="1">
+    <row r="12" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="51" t="s">
         <v>287</v>
       </c>
@@ -11211,7 +11214,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="18.75" customHeight="1" thickBot="1">
+    <row r="13" spans="1:13" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A13" s="52" t="s">
         <v>290</v>
       </c>
@@ -11222,7 +11225,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="18.75" customHeight="1" thickBot="1">
+    <row r="14" spans="1:13" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A14" s="53" t="s">
         <v>291</v>
       </c>
@@ -11236,7 +11239,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="18.75" customHeight="1" thickBot="1">
+    <row r="15" spans="1:13" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A15" s="54" t="s">
         <v>293</v>
       </c>
@@ -11247,7 +11250,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="16" spans="1:13" ht="19.5" customHeight="1" thickBot="1">
+    <row r="16" spans="1:13" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A16" s="55" t="s">
         <v>294</v>
       </c>
@@ -11261,12 +11264,12 @@
         <v>248</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="13.5" thickBot="1">
+    <row r="17" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A17" s="56" t="s">
         <v>296</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="13.5" thickBot="1">
+    <row r="18" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A18" s="75" t="s">
         <v>297</v>
       </c>
@@ -11278,7 +11281,7 @@
       </c>
       <c r="F18" s="37"/>
     </row>
-    <row r="19" spans="1:6" ht="13.5" thickBot="1">
+    <row r="19" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A19" s="76" t="s">
         <v>300</v>
       </c>
@@ -11289,7 +11292,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="51.75" thickBot="1">
+    <row r="20" spans="1:6" ht="51.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A20" s="77" t="s">
         <v>303</v>
       </c>
@@ -11303,12 +11306,12 @@
         <v>302</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="13.5" thickBot="1">
+    <row r="21" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A21" s="78" t="s">
         <v>306</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="13.5" thickBot="1">
+    <row r="22" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A22" s="79" t="s">
         <v>307</v>
       </c>
@@ -11317,13 +11320,13 @@
       </c>
       <c r="E22" s="22"/>
     </row>
-    <row r="23" spans="1:6" ht="13.5" thickBot="1">
+    <row r="23" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A23" s="80" t="s">
         <v>309</v>
       </c>
       <c r="E23" s="22"/>
     </row>
-    <row r="24" spans="1:6" ht="14.25" thickTop="1" thickBot="1">
+    <row r="24" spans="1:6" ht="14.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A24" s="81" t="s">
         <v>310</v>
       </c>
@@ -11332,20 +11335,20 @@
       </c>
       <c r="E24" s="22"/>
     </row>
-    <row r="25" spans="1:6" ht="14.25" thickTop="1" thickBot="1"/>
-    <row r="26" spans="1:6" ht="14.25" thickTop="1" thickBot="1">
+    <row r="25" spans="1:6" ht="14.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="1:6" ht="14.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="C26" s="68" t="s">
         <v>312</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="14.25" thickTop="1" thickBot="1"/>
-    <row r="28" spans="1:6" ht="14.25" thickTop="1" thickBot="1">
+    <row r="27" spans="1:6" ht="14.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="28" spans="1:6" ht="14.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="C28" s="89" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="13.5" thickTop="1"/>
-    <row r="30" spans="1:6">
+    <row r="29" spans="1:6" ht="13.5" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="C30" s="88" t="s">
         <v>314</v>
       </c>
@@ -11359,13 +11362,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D919E811-4385-4D35-A19E-3B7E0E659A89}">
   <dimension ref="A1:L39"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.140625" customWidth="1"/>
     <col min="7" max="7" width="15.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="13.5" thickBot="1">
+    <row r="1" spans="1:10" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="38" t="s">
         <v>315</v>
       </c>
@@ -11382,7 +11385,7 @@
       <c r="I1" s="37"/>
       <c r="J1" s="37"/>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="39" t="s">
         <v>319</v>
       </c>
@@ -11405,7 +11408,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" s="39" t="s">
         <v>321</v>
       </c>
@@ -11428,7 +11431,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" s="39" t="s">
         <v>325</v>
       </c>
@@ -11448,7 +11451,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="39" t="s">
         <v>328</v>
       </c>
@@ -11472,7 +11475,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" s="39" t="s">
         <v>330</v>
       </c>
@@ -11495,7 +11498,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" s="39" t="s">
         <v>333</v>
       </c>
@@ -11521,7 +11524,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" s="39" t="s">
         <v>337</v>
       </c>
@@ -11532,7 +11535,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" s="39" t="s">
         <v>339</v>
       </c>
@@ -11541,7 +11544,7 @@
       </c>
       <c r="C9" s="22"/>
     </row>
-    <row r="10" spans="1:10" ht="13.5" thickBot="1">
+    <row r="10" spans="1:10" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="39" t="s">
         <v>340</v>
       </c>
@@ -11559,7 +11562,7 @@
       <c r="I10" s="37"/>
       <c r="J10" s="37"/>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" s="39" t="s">
         <v>342</v>
       </c>
@@ -11582,13 +11585,13 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" s="39" t="s">
         <v>344</v>
       </c>
       <c r="B12" s="40">
         <f ca="1">TODAY()</f>
-        <v>45512</v>
+        <v>45643</v>
       </c>
       <c r="C12" s="40">
         <f>DATE(2010,10,2)</f>
@@ -11607,7 +11610,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:10">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" s="39" t="s">
         <v>346</v>
       </c>
@@ -11630,7 +11633,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:10">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" s="39" t="s">
         <v>348</v>
       </c>
@@ -11656,7 +11659,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:10">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" s="39" t="s">
         <v>350</v>
       </c>
@@ -11676,7 +11679,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:10">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" s="39" t="s">
         <v>352</v>
       </c>
@@ -11699,7 +11702,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:12">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" s="39" t="s">
         <v>354</v>
       </c>
@@ -11722,7 +11725,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:12">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" s="39" t="s">
         <v>356</v>
       </c>
@@ -11745,7 +11748,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:12">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" s="39" t="s">
         <v>358</v>
       </c>
@@ -11768,7 +11771,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:12">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20" s="39" t="s">
         <v>360</v>
       </c>
@@ -11791,7 +11794,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:12">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21" s="39" t="s">
         <v>362</v>
       </c>
@@ -11817,7 +11820,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:12">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22" s="39" t="s">
         <v>364</v>
       </c>
@@ -11843,7 +11846,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="1:12">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23" s="39" t="s">
         <v>366</v>
       </c>
@@ -11869,7 +11872,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="24" spans="1:12">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="G24" s="35" t="s">
         <v>368</v>
       </c>
@@ -11886,7 +11889,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="25" spans="1:12">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" s="39" t="s">
         <v>369</v>
       </c>
@@ -11912,7 +11915,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="1:12">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
       <c r="G26" s="35" t="s">
         <v>371</v>
       </c>
@@ -11932,7 +11935,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:12">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A27" s="22" t="s">
         <v>372</v>
       </c>
@@ -11958,7 +11961,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:12">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="G28" s="35" t="s">
         <v>374</v>
       </c>
@@ -11978,7 +11981,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:12">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
       <c r="G29" s="35" t="s">
         <v>375</v>
       </c>
@@ -11998,7 +12001,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:12">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
       <c r="G30" s="35" t="s">
         <v>376</v>
       </c>
@@ -12018,7 +12021,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:12" ht="13.5" thickBot="1">
+    <row r="31" spans="1:12" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="G31" s="36" t="s">
         <v>377</v>
       </c>
@@ -12032,7 +12035,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:12">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
       <c r="G32" s="35" t="s">
         <v>378</v>
       </c>
@@ -12046,7 +12049,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="7:10">
+    <row r="33" spans="7:10" x14ac:dyDescent="0.2">
       <c r="G33" s="35" t="s">
         <v>379</v>
       </c>
@@ -12060,7 +12063,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="7:10">
+    <row r="34" spans="7:10" x14ac:dyDescent="0.2">
       <c r="G34" s="35" t="s">
         <v>380</v>
       </c>
@@ -12074,7 +12077,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="7:10">
+    <row r="35" spans="7:10" x14ac:dyDescent="0.2">
       <c r="G35" s="35" t="s">
         <v>381</v>
       </c>
@@ -12088,7 +12091,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="7:10">
+    <row r="36" spans="7:10" x14ac:dyDescent="0.2">
       <c r="G36" s="35" t="s">
         <v>382</v>
       </c>
@@ -12102,7 +12105,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="7:10">
+    <row r="37" spans="7:10" x14ac:dyDescent="0.2">
       <c r="G37" s="35" t="s">
         <v>383</v>
       </c>
@@ -12116,110 +12119,110 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="7:10">
+    <row r="39" spans="7:10" x14ac:dyDescent="0.2">
       <c r="G39" s="35"/>
     </row>
   </sheetData>
   <phoneticPr fontId="21" type="noConversion"/>
   <conditionalFormatting sqref="B15">
-    <cfRule type="expression" dxfId="40" priority="58">
+    <cfRule type="expression" dxfId="22" priority="58">
       <formula>ODD(B15)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B26:B27">
-    <cfRule type="cellIs" dxfId="39" priority="46" operator="equal">
+    <cfRule type="cellIs" dxfId="21" priority="46" operator="equal">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B2:C2">
-    <cfRule type="aboveAverage" dxfId="38" priority="114"/>
+    <cfRule type="aboveAverage" dxfId="20" priority="114"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:C3">
-    <cfRule type="beginsWith" dxfId="37" priority="73" operator="beginsWith" text="rule">
+    <cfRule type="beginsWith" dxfId="19" priority="73" operator="beginsWith" text="rule">
       <formula>LEFT(B3,LEN("rule"))="rule"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B4:C4">
-    <cfRule type="containsBlanks" dxfId="36" priority="71">
+    <cfRule type="containsBlanks" dxfId="18" priority="71">
       <formula>LEN(TRIM(B4))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B5:C5">
-    <cfRule type="containsErrors" dxfId="35" priority="70">
+    <cfRule type="containsErrors" dxfId="17" priority="70">
       <formula>ISERROR(B5)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:C6">
-    <cfRule type="containsText" dxfId="34" priority="69" operator="containsText" text="rule">
+    <cfRule type="containsText" dxfId="16" priority="69" operator="containsText" text="rule">
       <formula>NOT(ISERROR(SEARCH("rule",B6)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8:C8">
-    <cfRule type="endsWith" dxfId="33" priority="67" operator="endsWith" text="rule">
+    <cfRule type="endsWith" dxfId="15" priority="67" operator="endsWith" text="rule">
       <formula>RIGHT(B8,LEN("rule"))="rule"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B9:C9">
-    <cfRule type="notContainsBlanks" dxfId="32" priority="66">
+    <cfRule type="notContainsBlanks" dxfId="14" priority="66">
       <formula>LEN(TRIM(B9))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B10:C10">
-    <cfRule type="notContainsErrors" dxfId="31" priority="65">
+    <cfRule type="notContainsErrors" dxfId="13" priority="65">
       <formula>NOT(ISERROR(B10))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B11:C11">
-    <cfRule type="notContainsText" dxfId="30" priority="64" operator="notContains" text="rule">
+    <cfRule type="notContainsText" dxfId="12" priority="64" operator="notContains" text="rule">
       <formula>ISERROR(SEARCH("rule",B11))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12:C12">
-    <cfRule type="timePeriod" dxfId="29" priority="63" timePeriod="today">
+    <cfRule type="timePeriod" dxfId="11" priority="63" timePeriod="today">
       <formula>FLOOR(B12,1)=TODAY()</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B13:C13">
-    <cfRule type="top10" dxfId="28" priority="115" rank="1"/>
+    <cfRule type="top10" dxfId="10" priority="115" rank="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B16:C16">
-    <cfRule type="cellIs" dxfId="27" priority="45" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="45" operator="equal">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B17:C17">
-    <cfRule type="cellIs" dxfId="26" priority="56" operator="notEqual">
+    <cfRule type="cellIs" dxfId="8" priority="56" operator="notEqual">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B18:C18">
-    <cfRule type="cellIs" dxfId="25" priority="6" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="7" priority="6" operator="greaterThan">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B19:C19">
-    <cfRule type="cellIs" dxfId="24" priority="5" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="6" priority="5" operator="greaterThanOrEqual">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B20:C20">
-    <cfRule type="cellIs" dxfId="23" priority="4" operator="lessThan">
+    <cfRule type="cellIs" dxfId="5" priority="4" operator="lessThan">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B21:C21">
-    <cfRule type="cellIs" dxfId="22" priority="3" operator="lessThanOrEqual">
+    <cfRule type="cellIs" dxfId="4" priority="3" operator="lessThanOrEqual">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B22:C22">
-    <cfRule type="cellIs" dxfId="21" priority="2" operator="between">
+    <cfRule type="cellIs" dxfId="3" priority="2" operator="between">
       <formula>2</formula>
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B23:C23">
-    <cfRule type="cellIs" dxfId="20" priority="1" operator="notBetween">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="notBetween">
       <formula>2</formula>
       <formula>4</formula>
     </cfRule>
@@ -12253,10 +12256,10 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7:D7">
-    <cfRule type="duplicateValues" dxfId="19" priority="82"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="82"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B14:D14">
-    <cfRule type="uniqueValues" dxfId="18" priority="96"/>
+    <cfRule type="uniqueValues" dxfId="0" priority="96"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:J2">
     <cfRule type="colorScale" priority="44">
@@ -12679,7 +12682,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5CCC4B1-5C65-4837-AA26-56CCF06B63BB}">
   <dimension ref="A1:J34"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="17.28515625" customWidth="1"/>
     <col min="4" max="4" width="9.5703125" customWidth="1"/>
@@ -12691,12 +12694,12 @@
     <col min="10" max="10" width="17.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>384</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="15">
+    <row r="3" spans="1:10" ht="15" x14ac:dyDescent="0.2">
       <c r="C3" s="18" t="s">
         <v>35</v>
       </c>
@@ -12722,7 +12725,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="C4" s="2" t="s">
         <v>42</v>
       </c>
@@ -12753,7 +12756,7 @@
         <v>Rank</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="C5" s="2" t="s">
         <v>44</v>
       </c>
@@ -12784,7 +12787,7 @@
         <v>Rank</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="C6" s="2" t="s">
         <v>391</v>
       </c>
@@ -12817,7 +12820,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B8" t="s">
         <v>392</v>
       </c>
@@ -12828,7 +12831,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="C9">
         <v>3</v>
       </c>
@@ -12836,7 +12839,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B11" t="s">
         <v>393</v>
       </c>
@@ -12847,7 +12850,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="C12">
         <v>3</v>
       </c>
@@ -12855,7 +12858,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:10">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B14" t="s">
         <v>396</v>
       </c>
@@ -12866,7 +12869,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:10">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="C15">
         <v>3</v>
       </c>
@@ -12874,7 +12877,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="2:4">
+    <row r="17" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B17" t="s">
         <v>397</v>
       </c>
@@ -12885,7 +12888,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="2:4">
+    <row r="18" spans="2:4" x14ac:dyDescent="0.2">
       <c r="C18">
         <v>3</v>
       </c>
@@ -12893,7 +12896,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="20" spans="2:4">
+    <row r="20" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B20" t="s">
         <v>398</v>
       </c>
@@ -12904,7 +12907,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="2:4">
+    <row r="21" spans="2:4" x14ac:dyDescent="0.2">
       <c r="C21">
         <v>3</v>
       </c>
@@ -12912,7 +12915,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="23" spans="2:4">
+    <row r="23" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B23" t="s">
         <v>399</v>
       </c>
@@ -12923,7 +12926,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="24" spans="2:4">
+    <row r="24" spans="2:4" x14ac:dyDescent="0.2">
       <c r="C24">
         <v>3</v>
       </c>
@@ -12931,7 +12934,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="26" spans="2:4">
+    <row r="26" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B26" t="s">
         <v>400</v>
       </c>
@@ -12942,7 +12945,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="27" spans="2:4">
+    <row r="27" spans="2:4" x14ac:dyDescent="0.2">
       <c r="C27">
         <v>3</v>
       </c>
@@ -12950,7 +12953,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="28" spans="2:4">
+    <row r="28" spans="2:4" x14ac:dyDescent="0.2">
       <c r="C28" t="s">
         <v>391</v>
       </c>
@@ -12959,7 +12962,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="30" spans="2:4">
+    <row r="30" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B30" t="s">
         <v>401</v>
       </c>
@@ -12970,7 +12973,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="31" spans="2:4" hidden="1">
+    <row r="31" spans="2:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="C31" t="s">
         <v>404</v>
       </c>
@@ -12978,7 +12981,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="32" spans="2:4">
+    <row r="32" spans="2:4" x14ac:dyDescent="0.2">
       <c r="C32" t="s">
         <v>405</v>
       </c>
@@ -12986,7 +12989,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="34" spans="2:2">
+    <row r="34" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B34" t="s">
         <v>406</v>
       </c>
@@ -13011,7 +13014,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE9224F2-4D06-4586-886C-E51F5EBCA7B0}">
   <dimension ref="A1:L21"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="13.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.5703125" bestFit="1" customWidth="1"/>
@@ -13032,7 +13035,7 @@
     <col min="21" max="21" width="19.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="15">
+    <row r="1" spans="1:12" ht="15" x14ac:dyDescent="0.2">
       <c r="A1" s="93" t="s">
         <v>407</v>
       </c>
@@ -13042,7 +13045,7 @@
       <c r="E1" s="18"/>
       <c r="F1" s="18"/>
     </row>
-    <row r="2" spans="1:12">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -13050,7 +13053,7 @@
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
     </row>
-    <row r="3" spans="1:12">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="90" t="s">
@@ -13060,7 +13063,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="4" spans="1:12">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="90" t="s">
@@ -13094,7 +13097,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="5" spans="1:12">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="91" t="s">
@@ -13107,7 +13110,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:12">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="92">
@@ -13120,7 +13123,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:12">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="91" t="s">
@@ -13133,7 +13136,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:12">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="92">
@@ -13146,7 +13149,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:12">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="91" t="s">
@@ -13159,7 +13162,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:12">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="92">
@@ -13172,7 +13175,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:12">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="C11" s="91" t="s">
         <v>44</v>
       </c>
@@ -13183,7 +13186,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="12" spans="1:12">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="C12" s="92">
         <v>23000</v>
       </c>
@@ -13194,7 +13197,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:12">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="C13" s="91" t="s">
         <v>50</v>
       </c>
@@ -13205,7 +13208,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:12">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="C14" s="92">
         <v>2</v>
       </c>
@@ -13216,7 +13219,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:12">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="C15" s="91" t="s">
         <v>48</v>
       </c>
@@ -13227,7 +13230,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="16" spans="1:12">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="C16" s="92">
         <v>50024</v>
       </c>
@@ -13238,7 +13241,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="3:12">
+    <row r="17" spans="3:12" x14ac:dyDescent="0.2">
       <c r="C17" s="91" t="s">
         <v>53</v>
       </c>
@@ -13249,7 +13252,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="18" spans="3:12">
+    <row r="18" spans="3:12" x14ac:dyDescent="0.2">
       <c r="C18" s="92">
         <v>189576</v>
       </c>
@@ -13260,7 +13263,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="19" spans="3:12">
+    <row r="19" spans="3:12" x14ac:dyDescent="0.2">
       <c r="C19" s="91" t="s">
         <v>57</v>
       </c>
@@ -13271,7 +13274,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="20" spans="3:12">
+    <row r="20" spans="3:12" x14ac:dyDescent="0.2">
       <c r="C20" s="92">
         <v>5000</v>
       </c>
@@ -13282,7 +13285,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="21" spans="3:12">
+    <row r="21" spans="3:12" x14ac:dyDescent="0.2">
       <c r="C21" s="91" t="s">
         <v>411</v>
       </c>
@@ -13323,29 +13326,29 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C47BF70-BA80-4124-B359-67CBCB635390}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="65.140625" customWidth="1"/>
     <col min="2" max="26" width="13.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>412</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>413</v>
       </c>
       <c r="B2" s="2"/>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>414</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>415</v>
       </c>
@@ -13358,12 +13361,15 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FE31E21-0350-44E7-AF13-4CA140505B30}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:1" ht="38.25">
+    <row r="1" spans="1:2" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A1" s="100" t="s">
         <v>416</v>
+      </c>
+      <c r="B1" t="s">
+        <v>417</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[IMP] chart: support import/export of dataset trendlines
This commit introduces the ability to import and export trendlines
associated with datasets in chart configurations.

Task: 4319957
</commit_message>
<xml_diff>
--- a/tests/__xlsx__/xlsx_demo_data.xlsx
+++ b/tests/__xlsx__/xlsx_demo_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28318"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Adrien\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BA4A409-66E7-4CFC-A548-ECD1D6D1B504}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0CDD9BA5-D2AB-4895-AC80-1F8DA821EE27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23295" yWindow="195" windowWidth="21600" windowHeight="11385" firstSheet="13" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23295" yWindow="195" windowWidth="21600" windowHeight="11385" firstSheet="13" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -31,9 +31,9 @@
   <externalReferences>
     <externalReference r:id="rId15"/>
   </externalReferences>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191028" calcCompleted="0"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId16"/>
+    <pivotCache cacheId="1350" r:id="rId16"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -1372,7 +1372,7 @@
     <numFmt numFmtId="168" formatCode="#,##0&quot; EUR €&quot;"/>
     <numFmt numFmtId="169" formatCode="&quot;€&quot;#,##0.00\ &quot;€&quot;"/>
   </numFmts>
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="26">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -2372,7 +2372,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -2385,6 +2384,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
@@ -2392,6 +2392,157 @@
     <cellStyle name="Normal 2" xfId="1" xr:uid="{1493241F-B85D-4F84-BBA0-86191B8FD032}"/>
   </cellStyles>
   <dxfs count="46">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+        <strike/>
+        <u/>
+        <color theme="7"/>
+      </font>
+      <numFmt numFmtId="170" formatCode="dd/mm/yyyy"/>
+      <fill>
+        <patternFill patternType="lightTrellis">
+          <fgColor theme="4"/>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE06666"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFB6D7A8"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -2798,157 +2949,6 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-        <strike/>
-        <u/>
-        <color theme="7"/>
-      </font>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <fill>
-        <patternFill patternType="lightTrellis">
-          <fgColor theme="4"/>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE06666"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFB6D7A8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor theme="4"/>
         </patternFill>
       </fill>
@@ -3048,7 +3048,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="fr-FR"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -3099,6 +3099,22 @@
               <a:effectLst/>
             </c:spPr>
           </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="6350" cap="rnd" cmpd="sng" algn="ctr">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+                <a:round/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="poly"/>
+            <c:order val="2"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
           <c:cat>
             <c:strRef>
               <c:f>Sheet1!$A$27:$A$35</c:f>
@@ -3370,7 +3386,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="fr-FR"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -3403,7 +3419,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="fr-FR"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="88853993"/>
@@ -3474,7 +3490,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="fr-FR"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -3507,7 +3523,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="fr-FR"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="17781237"/>
@@ -3551,7 +3567,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="fr-FR"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:legend>
@@ -3579,7 +3595,7 @@
       <a:pPr>
         <a:defRPr/>
       </a:pPr>
-      <a:endParaRPr lang="fr-FR"/>
+      <a:endParaRPr lang="en-US"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
@@ -3642,6 +3658,11 @@
             </a:ln>
           </c:spPr>
           <c:invertIfNegative val="1"/>
+          <c:trendline>
+            <c:trendlineType val="exp"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
           <c:cat>
             <c:strRef>
               <c:f>Sheet1!$A$27:$A$35</c:f>
@@ -3906,7 +3927,7 @@
                 <a:latin typeface="+mn-lt"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="fr-FR"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="88853993"/>
@@ -3968,7 +3989,7 @@
                 <a:latin typeface="+mn-lt"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="fr-FR"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="17781237"/>
@@ -3996,7 +4017,7 @@
               <a:latin typeface="+mn-lt"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="fr-FR"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:legend>
@@ -4614,7 +4635,7 @@
               <a:latin typeface="+mn-lt"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="fr-FR"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:legend>
@@ -4980,7 +5001,7 @@
               <a:latin typeface="+mn-lt"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="fr-FR"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:legend>
@@ -5050,6 +5071,11 @@
               <a:noFill/>
             </a:ln>
           </c:spPr>
+          <c:trendline>
+            <c:trendlineType val="log"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
           <c:xVal>
             <c:numRef>
               <c:f>Sheet1!$B$27:$B$35</c:f>
@@ -5192,7 +5218,7 @@
                 <a:latin typeface="+mn-lt"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="fr-FR"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="88853993"/>
@@ -5251,7 +5277,7 @@
                 <a:latin typeface="+mn-lt"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="fr-FR"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="17781237"/>
@@ -5279,7 +5305,7 @@
               <a:latin typeface="+mn-lt"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="fr-FR"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:legend>
@@ -5363,6 +5389,12 @@
             </a:ln>
           </c:spPr>
           <c:invertIfNegative val="1"/>
+          <c:trendline>
+            <c:trendlineType val="movingAvg"/>
+            <c:period val="3"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
           <c:cat>
             <c:strRef>
               <c:f>Sheet1!$A$27:$A$35</c:f>
@@ -5625,7 +5657,7 @@
                 <a:latin typeface="+mn-lt"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="fr-FR"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="88853993"/>
@@ -5687,7 +5719,7 @@
                 <a:latin typeface="+mn-lt"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="fr-FR"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="17781237"/>
@@ -5715,7 +5747,7 @@
               <a:latin typeface="+mn-lt"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="fr-FR"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:legend>
@@ -6027,7 +6059,7 @@
                 <a:latin typeface="+mn-lt"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="fr-FR"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="88853993"/>
@@ -6089,7 +6121,7 @@
                 <a:latin typeface="+mn-lt"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="fr-FR"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="17781237"/>
@@ -6117,7 +6149,7 @@
               <a:latin typeface="+mn-lt"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="fr-FR"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:legend>
@@ -6444,7 +6476,7 @@
                 <a:latin typeface="+mn-lt"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="fr-FR"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="344680958"/>
@@ -6520,7 +6552,7 @@
                 <a:latin typeface="+mn-lt"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="fr-FR"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="998664793"/>
@@ -6543,7 +6575,7 @@
               <a:latin typeface="+mn-lt"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="fr-FR"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:legend>
@@ -7572,7 +7604,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9B3CE3F5-58D8-48A3-B9C6-24D1506C9F5C}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9B3CE3F5-58D8-48A3-B9C6-24D1506C9F5C}" name="PivotTable1" cacheId="1350" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="C3:L21" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="5">
     <pivotField axis="axisRow" showAll="0">
@@ -7722,7 +7754,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{09C35CC7-7259-4A97-8FEA-EDB47375DF08}" name="Table3" displayName="Table3" ref="C3:J6" totalsRowCount="1" headerRowDxfId="43" dataDxfId="42">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{09C35CC7-7259-4A97-8FEA-EDB47375DF08}" name="Table3" displayName="Table3" ref="C3:J6" totalsRowCount="1" headerRowDxfId="17" dataDxfId="16">
   <autoFilter ref="C3:J5" xr:uid="{09C35CC7-7259-4A97-8FEA-EDB47375DF08}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -7734,22 +7766,22 @@
     <filterColumn colId="7" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{C4EE018E-238B-42BA-9035-DB01FA5420D3}" name="Name" totalsRowLabel="Total" dataDxfId="41" totalsRowDxfId="40"/>
-    <tableColumn id="2" xr3:uid="{C1F6911F-9482-4C98-BBFB-21D9CAA66DA4}" name="Age" totalsRowFunction="sum" dataDxfId="39" totalsRowDxfId="38"/>
-    <tableColumn id="5" xr3:uid="{3CE9F5DA-0A57-4696-B4E0-53601C3B7798}" name="Rank" totalsRowFunction="sum" dataDxfId="37" totalsRowDxfId="36"/>
-    <tableColumn id="6" xr3:uid="{34912838-665C-4472-B558-25990E5B148D}" name="Rank+Age =E4+D4" totalsRowFunction="sum" dataDxfId="35" totalsRowDxfId="34">
+    <tableColumn id="1" xr3:uid="{C4EE018E-238B-42BA-9035-DB01FA5420D3}" name="Name" totalsRowLabel="Total" dataDxfId="14" totalsRowDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{C1F6911F-9482-4C98-BBFB-21D9CAA66DA4}" name="Age" totalsRowFunction="sum" dataDxfId="12" totalsRowDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{3CE9F5DA-0A57-4696-B4E0-53601C3B7798}" name="Rank" totalsRowFunction="sum" dataDxfId="10" totalsRowDxfId="11"/>
+    <tableColumn id="6" xr3:uid="{34912838-665C-4472-B558-25990E5B148D}" name="Rank+Age =E4+D4" totalsRowFunction="sum" dataDxfId="8" totalsRowDxfId="9">
       <calculatedColumnFormula>Table3[[#This Row],[Rank]]+Table3[[#This Row],[Age]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{89D90022-7073-4067-BAF8-1587D27C4AFB}" name="Data =SUM(E4:E5)" totalsRowFunction="sum" dataDxfId="33" totalsRowDxfId="32">
+    <tableColumn id="7" xr3:uid="{89D90022-7073-4067-BAF8-1587D27C4AFB}" name="Data =SUM(E4:E5)" totalsRowFunction="sum" dataDxfId="6" totalsRowDxfId="7">
       <calculatedColumnFormula>SUM(Table3[Rank])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{B2A7E5BB-A379-492B-9484-72F2FD1FF3A0}" name="All =SUM(E3:E6)" totalsRowFunction="sum" dataDxfId="31" totalsRowDxfId="30">
+    <tableColumn id="8" xr3:uid="{B2A7E5BB-A379-492B-9484-72F2FD1FF3A0}" name="All =SUM(E3:E6)" totalsRowFunction="sum" dataDxfId="4" totalsRowDxfId="5">
       <calculatedColumnFormula>SUM(Table3[[#All],[Rank]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{3C532A69-E4BC-4A20-A922-4BCAA0D3FEC9}" name="Totals =E6" totalsRowFunction="sum" dataDxfId="29" totalsRowDxfId="28">
+    <tableColumn id="9" xr3:uid="{3C532A69-E4BC-4A20-A922-4BCAA0D3FEC9}" name="Totals =E6" totalsRowFunction="sum" dataDxfId="2" totalsRowDxfId="3">
       <calculatedColumnFormula>Table3[[#Totals],[Rank]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{35E9E9C3-9148-468A-85B6-19290CEB6F00}" name="Headers =E3" totalsRowFunction="sum" dataDxfId="27" totalsRowDxfId="26">
+    <tableColumn id="10" xr3:uid="{35E9E9C3-9148-468A-85B6-19290CEB6F00}" name="Headers =E3" totalsRowFunction="sum" dataDxfId="0" totalsRowDxfId="1">
       <calculatedColumnFormula>Table3[[#Headers],[Rank]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -7859,9 +7891,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -7899,7 +7931,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -8005,7 +8037,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -8147,7 +8179,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -8159,7 +8191,7 @@
     <tabColor rgb="FF00FF00"/>
   </sheetPr>
   <dimension ref="A1:L35"/>
-  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="22.28515625" customWidth="1"/>
     <col min="2" max="2" width="13.7109375" customWidth="1"/>
@@ -8168,7 +8200,7 @@
     <col min="6" max="26" width="13.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" ht="38.25" customHeight="1">
       <c r="A1" s="21"/>
       <c r="C1" s="1" t="s">
         <v>0</v>
@@ -8177,7 +8209,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="27.75" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:12" ht="27.75">
       <c r="B2" s="22" t="s">
         <v>2</v>
       </c>
@@ -8190,25 +8222,25 @@
       <c r="H2" s="118" t="s">
         <v>4</v>
       </c>
-      <c r="I2" s="119"/>
+      <c r="I2" s="123"/>
       <c r="K2" s="3"/>
     </row>
-    <row r="3" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:12" ht="17.25" customHeight="1">
       <c r="F3" s="4" t="s">
         <v>5</v>
       </c>
       <c r="G3" s="117">
         <v>8</v>
       </c>
-      <c r="H3" s="119"/>
-      <c r="I3" s="119"/>
+      <c r="H3" s="123"/>
+      <c r="I3" s="123"/>
       <c r="J3" s="5"/>
-      <c r="K3" s="120">
+      <c r="K3" s="119">
         <v>5</v>
       </c>
       <c r="L3" s="6"/>
     </row>
-    <row r="4" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:12" ht="17.25" customHeight="1">
       <c r="B4" s="7" t="s">
         <v>6</v>
       </c>
@@ -8221,50 +8253,50 @@
       <c r="G4" s="117">
         <v>9</v>
       </c>
-      <c r="H4" s="119"/>
-      <c r="I4" s="119"/>
+      <c r="H4" s="123"/>
+      <c r="I4" s="123"/>
       <c r="J4" s="5"/>
-      <c r="K4" s="121"/>
+      <c r="K4" s="120"/>
       <c r="L4" s="6"/>
     </row>
-    <row r="5" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:12" ht="17.25" customHeight="1">
       <c r="C5" s="117">
         <v>42</v>
       </c>
       <c r="G5" s="117">
         <v>15</v>
       </c>
-      <c r="H5" s="119"/>
-      <c r="I5" s="119"/>
+      <c r="H5" s="123"/>
+      <c r="I5" s="123"/>
       <c r="J5" s="5"/>
-      <c r="K5" s="121"/>
+      <c r="K5" s="120"/>
       <c r="L5" s="6"/>
     </row>
-    <row r="6" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:12" ht="17.25" customHeight="1">
       <c r="G6" s="117">
         <v>22</v>
       </c>
       <c r="J6" s="5"/>
-      <c r="K6" s="121"/>
+      <c r="K6" s="120"/>
       <c r="L6" s="6"/>
     </row>
-    <row r="7" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:12" ht="17.25" customHeight="1">
       <c r="C7" s="117">
         <v>3</v>
       </c>
       <c r="J7" s="5"/>
-      <c r="K7" s="121"/>
+      <c r="K7" s="120"/>
       <c r="L7" s="6"/>
     </row>
-    <row r="8" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:12" ht="17.25" customHeight="1">
       <c r="G8" s="117">
         <v>30</v>
       </c>
       <c r="J8" s="5"/>
-      <c r="K8" s="122"/>
+      <c r="K8" s="121"/>
       <c r="L8" s="6"/>
     </row>
-    <row r="9" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:12" ht="17.25" customHeight="1">
       <c r="B9" s="9" t="s">
         <v>8</v>
       </c>
@@ -8274,7 +8306,7 @@
       </c>
       <c r="K9" s="10"/>
     </row>
-    <row r="10" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:12" ht="17.25" customHeight="1">
       <c r="C10" s="117">
         <f>SUM(C4:C7)</f>
         <v>57.4</v>
@@ -8283,13 +8315,13 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:12" ht="17.25" customHeight="1">
       <c r="C11" s="117">
         <f>-(3+C7*SUM(C4:C7))</f>
         <v>-175.2</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:12" ht="17.25" customHeight="1">
       <c r="C12" s="117">
         <f>SUM(C9:C11)</f>
         <v>-63.399999999999991</v>
@@ -8298,13 +8330,13 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:12" ht="17.25" customHeight="1">
       <c r="G13" s="117">
         <f>A1+A2+A3+A4+A5+A6+A7+A8+A9+A10+A11+A12+A13+A14+A15+A16+A17+A18</f>
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:12" ht="17.25" customHeight="1">
       <c r="B14" s="11" t="s">
         <v>11</v>
       </c>
@@ -8313,32 +8345,32 @@
         <v>#CYCLE</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:12" ht="17.25" customHeight="1">
       <c r="C15" s="117" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:12" ht="17.25" customHeight="1">
       <c r="C16" s="117" t="str">
         <f>C15</f>
         <v>=(+</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:9" ht="17.25" customHeight="1">
       <c r="C17" s="117" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:9" ht="17.25" customHeight="1">
       <c r="C18" s="117" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:9" ht="17.25" customHeight="1">
       <c r="E19" s="3"/>
       <c r="G19" s="3"/>
     </row>
-    <row r="20" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:9" ht="17.25" customHeight="1">
       <c r="B20" s="5"/>
       <c r="C20" s="6" t="s">
         <v>15</v>
@@ -8352,7 +8384,7 @@
       </c>
       <c r="H20" s="6"/>
     </row>
-    <row r="21" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:9" ht="17.25" customHeight="1">
       <c r="A21" s="13" t="s">
         <v>18</v>
       </c>
@@ -8362,7 +8394,7 @@
       </c>
       <c r="G21" s="10"/>
     </row>
-    <row r="23" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:9" ht="17.25" customHeight="1">
       <c r="A23" s="13" t="s">
         <v>19</v>
       </c>
@@ -8376,7 +8408,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:9" ht="17.25" customHeight="1">
       <c r="C24" s="16">
         <v>10</v>
       </c>
@@ -8387,7 +8419,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:9" ht="17.25" customHeight="1">
       <c r="C25" s="16">
         <v>10.122999999999999</v>
       </c>
@@ -8398,7 +8430,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:9" ht="17.25" customHeight="1">
       <c r="B26" s="117" t="s">
         <v>20</v>
       </c>
@@ -8412,7 +8444,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:9" ht="17.25" customHeight="1">
       <c r="A27" s="117" t="s">
         <v>22</v>
       </c>
@@ -8429,7 +8461,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:9" ht="17.25" customHeight="1">
       <c r="A28" s="117" t="s">
         <v>23</v>
       </c>
@@ -8446,7 +8478,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:9" ht="17.25" customHeight="1">
       <c r="A29" s="117" t="s">
         <v>24</v>
       </c>
@@ -8463,7 +8495,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:9" ht="17.25" customHeight="1">
       <c r="A30" s="117" t="s">
         <v>25</v>
       </c>
@@ -8480,7 +8512,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:9" ht="17.25" customHeight="1">
       <c r="A31" s="117" t="s">
         <v>26</v>
       </c>
@@ -8497,7 +8529,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:9" ht="17.25" customHeight="1">
       <c r="A32" s="117" t="s">
         <v>27</v>
       </c>
@@ -8514,7 +8546,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:9" ht="17.25" customHeight="1">
       <c r="A33" s="117" t="s">
         <v>28</v>
       </c>
@@ -8531,7 +8563,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:9" ht="17.25" customHeight="1">
       <c r="A34" s="117" t="s">
         <v>29</v>
       </c>
@@ -8542,7 +8574,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="35" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:9" ht="17.25" customHeight="1">
       <c r="A35" s="117" t="s">
         <v>30</v>
       </c>
@@ -8559,7 +8591,7 @@
     <mergeCell ref="K3:K8"/>
   </mergeCells>
   <conditionalFormatting sqref="C1:C100 B21">
-    <cfRule type="cellIs" dxfId="25" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="43" priority="1" operator="equal">
       <formula>42</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8604,7 +8636,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F7A934C-2218-4A12-8B75-EE28D615D774}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="12.75"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -8613,7 +8645,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96301BE1-D86D-4D45-870D-85A75D53FC99}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -8622,7 +8654,7 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B10A8834-0E20-4F80-8813-3ACA5527B377}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="65.140625" customWidth="1"/>
     <col min="2" max="26" width="13.7109375" customWidth="1"/>
@@ -8639,7 +8671,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8649,7 +8681,7 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{025F2510-D243-4DA1-81DE-BBDDA9BC3681}">
   <dimension ref="A1:I6"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="3" max="4" width="14.28515625" customWidth="1"/>
     <col min="5" max="5" width="14.7109375" customWidth="1"/>
@@ -8658,7 +8690,7 @@
     <col min="9" max="9" width="17.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9">
       <c r="A1" s="114" t="s">
         <v>417</v>
       </c>
@@ -8687,7 +8719,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9">
       <c r="A2" s="104">
         <v>4</v>
       </c>
@@ -8716,7 +8748,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9">
       <c r="A3" s="104">
         <v>3</v>
       </c>
@@ -8745,7 +8777,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9">
       <c r="A4" s="104">
         <v>9</v>
       </c>
@@ -8774,7 +8806,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9">
       <c r="A5" s="104">
         <v>5</v>
       </c>
@@ -8803,7 +8835,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9">
       <c r="A6" s="109">
         <v>7</v>
       </c>
@@ -8876,12 +8908,12 @@
     <tabColor theme="9"/>
   </sheetPr>
   <dimension ref="A1:R163"/>
-  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="26" width="13.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:18" ht="17.25" customHeight="1">
       <c r="A1" s="117" t="s">
         <v>31</v>
       </c>
@@ -8916,7 +8948,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:18" ht="17.25" customHeight="1">
       <c r="A2" s="117" t="s">
         <v>41</v>
       </c>
@@ -8962,7 +8994,7 @@
         <v>1230.7</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:18" ht="17.25" customHeight="1">
       <c r="A3" s="117" t="s">
         <v>43</v>
       </c>
@@ -9008,7 +9040,7 @@
         <v>1217.7</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:18" ht="17.25" customHeight="1">
       <c r="A4" s="117" t="s">
         <v>45</v>
       </c>
@@ -9054,7 +9086,7 @@
         <v>1230.7</v>
       </c>
     </row>
-    <row r="5" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:18" ht="17.25" customHeight="1">
       <c r="A5" s="117" t="s">
         <v>47</v>
       </c>
@@ -9100,7 +9132,7 @@
         <v>1246.7</v>
       </c>
     </row>
-    <row r="6" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:18" ht="17.25" customHeight="1">
       <c r="A6" s="117" t="s">
         <v>49</v>
       </c>
@@ -9146,7 +9178,7 @@
         <v>1213.7</v>
       </c>
     </row>
-    <row r="7" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:18" ht="17.25" customHeight="1">
       <c r="A7" s="117" t="s">
         <v>52</v>
       </c>
@@ -9180,7 +9212,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:18" ht="17.25" customHeight="1">
       <c r="A8" s="117" t="s">
         <v>54</v>
       </c>
@@ -9214,7 +9246,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:18" ht="17.25" customHeight="1">
       <c r="A9" s="117" t="s">
         <v>56</v>
       </c>
@@ -9245,7 +9277,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:18" ht="17.25" customHeight="1">
       <c r="A10" s="117" t="s">
         <v>58</v>
       </c>
@@ -9261,7 +9293,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:18" ht="17.25" customHeight="1">
       <c r="A11" s="117" t="s">
         <v>59</v>
       </c>
@@ -9280,7 +9312,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="12" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:18" ht="17.25" customHeight="1">
       <c r="A12" s="117" t="s">
         <v>61</v>
       </c>
@@ -9311,7 +9343,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="13" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:18" ht="17.25" customHeight="1">
       <c r="A13" s="117" t="s">
         <v>62</v>
       </c>
@@ -9342,7 +9374,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="14" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:18" ht="17.25" customHeight="1">
       <c r="A14" s="117" t="s">
         <v>67</v>
       </c>
@@ -9358,7 +9390,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:18" ht="17.25" customHeight="1">
       <c r="A15" s="117" t="s">
         <v>68</v>
       </c>
@@ -9374,7 +9406,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:18" ht="17.25" customHeight="1">
       <c r="A16" s="117" t="s">
         <v>69</v>
       </c>
@@ -9390,7 +9422,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" ht="17.25" customHeight="1">
       <c r="A17" s="117" t="s">
         <v>70</v>
       </c>
@@ -9406,7 +9438,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4" ht="17.25" customHeight="1">
       <c r="A18" s="117" t="s">
         <v>71</v>
       </c>
@@ -9422,7 +9454,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:4" ht="17.25" customHeight="1">
       <c r="A19" s="117" t="s">
         <v>72</v>
       </c>
@@ -9438,7 +9470,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4" ht="17.25" customHeight="1">
       <c r="A20" s="117" t="s">
         <v>73</v>
       </c>
@@ -9454,7 +9486,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:4" ht="17.25" customHeight="1">
       <c r="A21" s="117" t="s">
         <v>74</v>
       </c>
@@ -9470,7 +9502,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:4" ht="17.25" customHeight="1">
       <c r="A22" s="117" t="s">
         <v>76</v>
       </c>
@@ -9486,7 +9518,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:4" ht="17.25" customHeight="1">
       <c r="A23" s="117" t="s">
         <v>77</v>
       </c>
@@ -9502,7 +9534,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:4" ht="17.25" customHeight="1">
       <c r="A24" s="117" t="s">
         <v>78</v>
       </c>
@@ -9519,7 +9551,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:4" ht="17.25" customHeight="1">
       <c r="A25" s="117" t="s">
         <v>79</v>
       </c>
@@ -9535,7 +9567,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:4" ht="17.25" customHeight="1">
       <c r="A26" s="117" t="s">
         <v>81</v>
       </c>
@@ -9551,7 +9583,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:4" ht="17.25" customHeight="1">
       <c r="A27" s="117" t="s">
         <v>82</v>
       </c>
@@ -9567,7 +9599,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:4" ht="17.25" customHeight="1">
       <c r="A28" s="117" t="s">
         <v>83</v>
       </c>
@@ -9584,7 +9616,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:4" ht="17.25" customHeight="1">
       <c r="A29" s="117" t="s">
         <v>84</v>
       </c>
@@ -9600,7 +9632,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:4" ht="17.25" customHeight="1">
       <c r="A30" s="117" t="s">
         <v>85</v>
       </c>
@@ -9616,7 +9648,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:4" ht="17.25" customHeight="1">
       <c r="A31" s="117" t="s">
         <v>86</v>
       </c>
@@ -9632,7 +9664,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:4" ht="17.25" customHeight="1">
       <c r="A32" s="117" t="s">
         <v>87</v>
       </c>
@@ -9648,7 +9680,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:4" ht="17.25" customHeight="1">
       <c r="A33" s="117" t="s">
         <v>88</v>
       </c>
@@ -9664,7 +9696,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:4" ht="17.25" customHeight="1">
       <c r="A34" s="117" t="s">
         <v>89</v>
       </c>
@@ -9680,7 +9712,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:4" ht="17.25" customHeight="1">
       <c r="A35" s="117" t="s">
         <v>90</v>
       </c>
@@ -9696,7 +9728,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:4" ht="17.25" customHeight="1">
       <c r="A36" s="117" t="s">
         <v>91</v>
       </c>
@@ -9712,7 +9744,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:4" ht="17.25" customHeight="1">
       <c r="A37" s="117" t="s">
         <v>92</v>
       </c>
@@ -9728,7 +9760,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:4" ht="17.25" customHeight="1">
       <c r="A38" s="117" t="s">
         <v>93</v>
       </c>
@@ -9745,7 +9777,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:4" ht="17.25" customHeight="1">
       <c r="A39" s="117" t="s">
         <v>94</v>
       </c>
@@ -9761,7 +9793,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:4" ht="17.25" customHeight="1">
       <c r="A40" s="117" t="s">
         <v>95</v>
       </c>
@@ -9777,7 +9809,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:4" ht="17.25" customHeight="1">
       <c r="A41" s="117" t="s">
         <v>96</v>
       </c>
@@ -9793,7 +9825,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:4" ht="17.25" customHeight="1">
       <c r="A42" s="117" t="s">
         <v>97</v>
       </c>
@@ -9809,7 +9841,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:4" ht="17.25" customHeight="1">
       <c r="A43" s="117" t="s">
         <v>98</v>
       </c>
@@ -9825,7 +9857,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:4" ht="17.25" customHeight="1">
       <c r="A44" s="117" t="s">
         <v>99</v>
       </c>
@@ -9841,7 +9873,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:4" ht="17.25" customHeight="1">
       <c r="A45" s="117" t="s">
         <v>100</v>
       </c>
@@ -9857,7 +9889,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:4" ht="17.25" customHeight="1">
       <c r="A46" s="117" t="s">
         <v>101</v>
       </c>
@@ -9873,7 +9905,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:4" ht="17.25" customHeight="1">
       <c r="A47" s="117" t="s">
         <v>102</v>
       </c>
@@ -9889,7 +9921,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:4" ht="17.25" customHeight="1">
       <c r="A48" s="117" t="s">
         <v>103</v>
       </c>
@@ -9905,7 +9937,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:4" ht="17.25" customHeight="1">
       <c r="A49" s="117" t="s">
         <v>104</v>
       </c>
@@ -9921,7 +9953,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:4" ht="17.25" customHeight="1">
       <c r="A50" s="117" t="s">
         <v>105</v>
       </c>
@@ -9938,7 +9970,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:4" ht="17.25" customHeight="1">
       <c r="A51" s="117" t="s">
         <v>106</v>
       </c>
@@ -9955,7 +9987,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:4" ht="17.25" customHeight="1">
       <c r="A52" s="117" t="s">
         <v>107</v>
       </c>
@@ -9971,7 +10003,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:4" ht="17.25" customHeight="1">
       <c r="A53" s="117" t="s">
         <v>108</v>
       </c>
@@ -9987,7 +10019,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:4" ht="17.25" customHeight="1">
       <c r="A54" s="117" t="s">
         <v>109</v>
       </c>
@@ -10003,7 +10035,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:4" ht="17.25" customHeight="1">
       <c r="A55" s="117" t="s">
         <v>110</v>
       </c>
@@ -10019,7 +10051,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:4" ht="17.25" customHeight="1">
       <c r="A56" s="117" t="s">
         <v>111</v>
       </c>
@@ -10035,7 +10067,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:4" ht="17.25" customHeight="1">
       <c r="A57" s="117" t="s">
         <v>112</v>
       </c>
@@ -10051,7 +10083,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:4" ht="17.25" customHeight="1">
       <c r="A58" s="117" t="s">
         <v>113</v>
       </c>
@@ -10067,7 +10099,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:4" ht="17.25" customHeight="1">
       <c r="A59" s="117" t="s">
         <v>114</v>
       </c>
@@ -10083,7 +10115,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:4" ht="17.25" customHeight="1">
       <c r="A60" s="117" t="s">
         <v>115</v>
       </c>
@@ -10099,7 +10131,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:4" ht="17.25" customHeight="1">
       <c r="A61" s="117" t="s">
         <v>116</v>
       </c>
@@ -10115,7 +10147,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:4" ht="17.25" customHeight="1">
       <c r="A62" s="117" t="s">
         <v>117</v>
       </c>
@@ -10131,7 +10163,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:4" ht="17.25" customHeight="1">
       <c r="A63" s="117" t="s">
         <v>118</v>
       </c>
@@ -10147,7 +10179,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:4" ht="17.25" customHeight="1">
       <c r="A64" s="117" t="s">
         <v>119</v>
       </c>
@@ -10163,7 +10195,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:4" ht="17.25" customHeight="1">
       <c r="A65" s="117" t="s">
         <v>120</v>
       </c>
@@ -10179,7 +10211,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:4" ht="17.25" customHeight="1">
       <c r="A66" s="117" t="s">
         <v>121</v>
       </c>
@@ -10195,7 +10227,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:4" ht="17.25" customHeight="1">
       <c r="A67" s="117" t="s">
         <v>122</v>
       </c>
@@ -10211,7 +10243,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:4" ht="17.25" customHeight="1">
       <c r="A68" s="117" t="s">
         <v>123</v>
       </c>
@@ -10227,7 +10259,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:4" ht="17.25" customHeight="1">
       <c r="A69" s="117" t="s">
         <v>125</v>
       </c>
@@ -10243,7 +10275,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:4" ht="17.25" customHeight="1">
       <c r="A70" s="117" t="s">
         <v>127</v>
       </c>
@@ -10259,7 +10291,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:4" ht="17.25" customHeight="1">
       <c r="A71" s="117" t="s">
         <v>129</v>
       </c>
@@ -10275,7 +10307,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:4" ht="17.25" customHeight="1">
       <c r="A72" s="117" t="s">
         <v>130</v>
       </c>
@@ -10291,7 +10323,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:4" ht="17.25" customHeight="1">
       <c r="A73" s="117" t="s">
         <v>131</v>
       </c>
@@ -10307,7 +10339,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:4" ht="17.25" customHeight="1">
       <c r="A74" s="117" t="s">
         <v>132</v>
       </c>
@@ -10323,7 +10355,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:4" ht="17.25" customHeight="1">
       <c r="A75" s="117" t="s">
         <v>133</v>
       </c>
@@ -10339,7 +10371,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:4" ht="17.25" customHeight="1">
       <c r="A76" s="117" t="s">
         <v>134</v>
       </c>
@@ -10355,7 +10387,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:4" ht="17.25" customHeight="1">
       <c r="A77" s="117" t="s">
         <v>135</v>
       </c>
@@ -10371,7 +10403,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="78" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:4" ht="17.25" customHeight="1">
       <c r="A78" s="117" t="s">
         <v>136</v>
       </c>
@@ -10387,7 +10419,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:4" ht="17.25" customHeight="1">
       <c r="A79" s="117" t="s">
         <v>137</v>
       </c>
@@ -10403,7 +10435,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:4" ht="17.25" customHeight="1">
       <c r="A80" s="117" t="s">
         <v>138</v>
       </c>
@@ -10419,7 +10451,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:4" ht="17.25" customHeight="1">
       <c r="A81" s="117" t="s">
         <v>139</v>
       </c>
@@ -10435,7 +10467,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:4" ht="17.25" customHeight="1">
       <c r="A82" s="117" t="s">
         <v>141</v>
       </c>
@@ -10451,7 +10483,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:4" ht="17.25" customHeight="1">
       <c r="A83" s="117" t="s">
         <v>142</v>
       </c>
@@ -10467,7 +10499,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:4" ht="17.25" customHeight="1">
       <c r="A84" s="117" t="s">
         <v>143</v>
       </c>
@@ -10483,7 +10515,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:4" ht="17.25" customHeight="1">
       <c r="A85" s="117" t="s">
         <v>144</v>
       </c>
@@ -10499,7 +10531,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="86" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:4" ht="17.25" customHeight="1">
       <c r="A86" s="117" t="s">
         <v>146</v>
       </c>
@@ -10515,7 +10547,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:4" ht="17.25" customHeight="1">
       <c r="A87" s="117" t="s">
         <v>147</v>
       </c>
@@ -10531,7 +10563,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:4" ht="17.25" customHeight="1">
       <c r="A88" s="117" t="s">
         <v>148</v>
       </c>
@@ -10547,7 +10579,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:4" ht="17.25" customHeight="1">
       <c r="A89" s="117" t="s">
         <v>149</v>
       </c>
@@ -10563,7 +10595,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="90" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:4" ht="17.25" customHeight="1">
       <c r="A90" s="117" t="s">
         <v>150</v>
       </c>
@@ -10579,7 +10611,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:4" ht="17.25" customHeight="1">
       <c r="A91" s="117" t="s">
         <v>151</v>
       </c>
@@ -10595,7 +10627,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:4" ht="17.25" customHeight="1">
       <c r="A92" s="117" t="s">
         <v>152</v>
       </c>
@@ -10611,7 +10643,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:4" ht="17.25" customHeight="1">
       <c r="A93" s="117" t="s">
         <v>153</v>
       </c>
@@ -10627,7 +10659,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="94" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:4" ht="17.25" customHeight="1">
       <c r="A94" s="117" t="s">
         <v>154</v>
       </c>
@@ -10643,7 +10675,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="95" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:4" ht="17.25" customHeight="1">
       <c r="A95" s="117" t="s">
         <v>155</v>
       </c>
@@ -10659,7 +10691,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="96" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:4" ht="17.25" customHeight="1">
       <c r="A96" s="117" t="s">
         <v>156</v>
       </c>
@@ -10675,7 +10707,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="97" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:4" ht="17.25" customHeight="1">
       <c r="A97" s="117" t="s">
         <v>157</v>
       </c>
@@ -10691,7 +10723,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="98" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:4" ht="17.25" customHeight="1">
       <c r="A98" s="117" t="s">
         <v>158</v>
       </c>
@@ -10707,7 +10739,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="99" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:4" ht="17.25" customHeight="1">
       <c r="A99" s="117" t="s">
         <v>159</v>
       </c>
@@ -10723,20 +10755,20 @@
         <v>1</v>
       </c>
     </row>
-    <row r="100" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:4" ht="17.25" customHeight="1">
       <c r="A100" s="117" t="s">
         <v>160</v>
       </c>
       <c r="B100" s="19">
         <f ca="1">NOW()</f>
-        <v>45594.46900636574</v>
+        <v>45631.469745023147</v>
       </c>
       <c r="D100" s="117">
         <f ca="1">IF(ISNUMBER(B100),1,0)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="101" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:4" ht="17.25" customHeight="1">
       <c r="A101" s="117" t="s">
         <v>161</v>
       </c>
@@ -10752,7 +10784,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="102" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:4" ht="17.25" customHeight="1">
       <c r="A102" s="117" t="s">
         <v>162</v>
       </c>
@@ -10768,7 +10800,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="103" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:4" ht="17.25" customHeight="1">
       <c r="A103" s="117" t="s">
         <v>163</v>
       </c>
@@ -10784,7 +10816,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="104" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:4" ht="17.25" customHeight="1">
       <c r="A104" s="117" t="s">
         <v>164</v>
       </c>
@@ -10800,7 +10832,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="105" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:4" ht="17.25" customHeight="1">
       <c r="A105" s="117" t="s">
         <v>165</v>
       </c>
@@ -10816,7 +10848,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="106" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:4" ht="17.25" customHeight="1">
       <c r="A106" s="117" t="s">
         <v>166</v>
       </c>
@@ -10832,7 +10864,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="107" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:4" ht="17.25" customHeight="1">
       <c r="A107" s="117" t="s">
         <v>167</v>
       </c>
@@ -10848,7 +10880,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:4" ht="17.25" customHeight="1">
       <c r="A108" s="117" t="s">
         <v>168</v>
       </c>
@@ -10864,7 +10896,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="109" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:4" ht="17.25" customHeight="1">
       <c r="A109" s="117" t="s">
         <v>169</v>
       </c>
@@ -10880,7 +10912,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="110" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:4" ht="17.25" customHeight="1">
       <c r="A110" s="117" t="s">
         <v>170</v>
       </c>
@@ -10896,7 +10928,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="111" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:4" ht="17.25" customHeight="1">
       <c r="A111" s="117" t="s">
         <v>171</v>
       </c>
@@ -10912,12 +10944,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="112" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:4" ht="17.25" customHeight="1">
       <c r="A112" s="117"/>
       <c r="B112" s="117"/>
       <c r="D112" s="117"/>
     </row>
-    <row r="113" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:4" ht="17.25" customHeight="1">
       <c r="A113" s="117" t="s">
         <v>172</v>
       </c>
@@ -10933,7 +10965,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="114" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:4" ht="17.25" customHeight="1">
       <c r="A114" s="117" t="s">
         <v>173</v>
       </c>
@@ -10949,7 +10981,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="115" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:4" ht="17.25" customHeight="1">
       <c r="A115" s="117" t="s">
         <v>175</v>
       </c>
@@ -10965,7 +10997,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="116" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:4" ht="17.25" customHeight="1">
       <c r="A116" s="117" t="s">
         <v>177</v>
       </c>
@@ -10981,7 +11013,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="117" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:4" ht="17.25" customHeight="1">
       <c r="A117" s="117" t="s">
         <v>178</v>
       </c>
@@ -10997,7 +11029,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="118" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:4" ht="17.25" customHeight="1">
       <c r="A118" s="117" t="s">
         <v>179</v>
       </c>
@@ -11013,7 +11045,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="119" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:4" ht="17.25" customHeight="1">
       <c r="A119" s="117" t="s">
         <v>180</v>
       </c>
@@ -11029,7 +11061,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="120" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:4" ht="17.25" customHeight="1">
       <c r="A120" s="117" t="s">
         <v>181</v>
       </c>
@@ -11045,7 +11077,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="121" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:4" ht="17.25" customHeight="1">
       <c r="A121" s="117" t="s">
         <v>182</v>
       </c>
@@ -11061,7 +11093,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="122" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:4" ht="17.25" customHeight="1">
       <c r="A122" s="117" t="s">
         <v>183</v>
       </c>
@@ -11077,7 +11109,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="123" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:4" ht="17.25" customHeight="1">
       <c r="A123" s="117" t="s">
         <v>184</v>
       </c>
@@ -11093,7 +11125,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="124" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:4" ht="17.25" customHeight="1">
       <c r="A124" s="117" t="s">
         <v>185</v>
       </c>
@@ -11109,7 +11141,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="125" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:4" ht="17.25" customHeight="1">
       <c r="A125" s="117" t="s">
         <v>186</v>
       </c>
@@ -11125,7 +11157,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="126" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:4" ht="17.25" customHeight="1">
       <c r="A126" s="117" t="s">
         <v>187</v>
       </c>
@@ -11141,7 +11173,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="127" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:4" ht="17.25" customHeight="1">
       <c r="A127" s="117" t="s">
         <v>188</v>
       </c>
@@ -11157,7 +11189,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="128" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:4" ht="17.25" customHeight="1">
       <c r="A128" s="117" t="s">
         <v>189</v>
       </c>
@@ -11173,7 +11205,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="129" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:4" ht="17.25" customHeight="1">
       <c r="A129" s="117" t="s">
         <v>190</v>
       </c>
@@ -11189,7 +11221,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="130" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:4" ht="17.25" customHeight="1">
       <c r="A130" s="117" t="s">
         <v>191</v>
       </c>
@@ -11205,7 +11237,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="131" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:4" ht="17.25" customHeight="1">
       <c r="A131" s="117" t="s">
         <v>192</v>
       </c>
@@ -11221,7 +11253,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="132" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:4" ht="17.25" customHeight="1">
       <c r="A132" s="117" t="s">
         <v>193</v>
       </c>
@@ -11237,7 +11269,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="133" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:4" ht="17.25" customHeight="1">
       <c r="A133" s="117" t="s">
         <v>194</v>
       </c>
@@ -11253,7 +11285,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="134" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:4" ht="17.25" customHeight="1">
       <c r="A134" s="117" t="s">
         <v>195</v>
       </c>
@@ -11269,7 +11301,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="135" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:4" ht="17.25" customHeight="1">
       <c r="A135" s="117" t="s">
         <v>196</v>
       </c>
@@ -11285,7 +11317,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="136" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:4" ht="17.25" customHeight="1">
       <c r="A136" s="117" t="s">
         <v>198</v>
       </c>
@@ -11301,7 +11333,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="137" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:4" ht="17.25" customHeight="1">
       <c r="A137" s="117" t="s">
         <v>199</v>
       </c>
@@ -11317,7 +11349,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="138" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:4" ht="17.25" customHeight="1">
       <c r="A138" s="117" t="s">
         <v>200</v>
       </c>
@@ -11333,7 +11365,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="139" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:4" ht="17.25" customHeight="1">
       <c r="A139" s="117" t="s">
         <v>201</v>
       </c>
@@ -11349,7 +11381,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="140" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:4" ht="17.25" customHeight="1">
       <c r="A140" s="117" t="s">
         <v>202</v>
       </c>
@@ -11365,7 +11397,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="141" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:4" ht="17.25" customHeight="1">
       <c r="A141" s="117" t="s">
         <v>203</v>
       </c>
@@ -11381,7 +11413,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="142" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:4" ht="17.25" customHeight="1">
       <c r="A142" s="117" t="s">
         <v>205</v>
       </c>
@@ -11397,7 +11429,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:4" ht="17.25" customHeight="1">
       <c r="A143" s="117" t="s">
         <v>206</v>
       </c>
@@ -11413,20 +11445,20 @@
         <v>1</v>
       </c>
     </row>
-    <row r="144" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:4" ht="17.25" customHeight="1">
       <c r="A144" s="117" t="s">
         <v>207</v>
       </c>
       <c r="B144" s="18">
         <f ca="1">TODAY()</f>
-        <v>45594</v>
+        <v>45631</v>
       </c>
       <c r="D144" s="117">
         <f ca="1">IF(ISNUMBER(B144),1,0)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="145" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:4" ht="17.25" customHeight="1">
       <c r="A145" s="117" t="s">
         <v>208</v>
       </c>
@@ -11442,7 +11474,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="146" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:4" ht="17.25" customHeight="1">
       <c r="A146" s="117" t="s">
         <v>210</v>
       </c>
@@ -11458,7 +11490,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="147" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:4" ht="17.25" customHeight="1">
       <c r="A147" s="117" t="s">
         <v>211</v>
       </c>
@@ -11474,7 +11506,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="148" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:4" ht="17.25" customHeight="1">
       <c r="A148" s="117" t="s">
         <v>213</v>
       </c>
@@ -11490,7 +11522,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="149" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:4" ht="17.25" customHeight="1">
       <c r="A149" s="117" t="s">
         <v>214</v>
       </c>
@@ -11506,7 +11538,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="150" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:4" ht="17.25" customHeight="1">
       <c r="A150" s="117" t="s">
         <v>215</v>
       </c>
@@ -11522,7 +11554,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="151" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:4" ht="17.25" customHeight="1">
       <c r="A151" s="117" t="s">
         <v>216</v>
       </c>
@@ -11538,7 +11570,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="152" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:4" ht="17.25" customHeight="1">
       <c r="A152" s="117" t="s">
         <v>217</v>
       </c>
@@ -11554,7 +11586,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="153" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:4" ht="17.25" customHeight="1">
       <c r="A153" s="117" t="s">
         <v>218</v>
       </c>
@@ -11570,7 +11602,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="154" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:4" ht="17.25" customHeight="1">
       <c r="A154" s="117" t="s">
         <v>219</v>
       </c>
@@ -11587,7 +11619,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="155" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:4" ht="17.25" customHeight="1">
       <c r="A155" s="117" t="s">
         <v>220</v>
       </c>
@@ -11603,7 +11635,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="156" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:4" ht="17.25" customHeight="1">
       <c r="A156" s="117" t="s">
         <v>221</v>
       </c>
@@ -11619,7 +11651,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="157" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:4" ht="17.25" customHeight="1">
       <c r="A157" s="117" t="s">
         <v>222</v>
       </c>
@@ -11635,7 +11667,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="158" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:4" ht="17.25" customHeight="1">
       <c r="A158" s="117" t="s">
         <v>223</v>
       </c>
@@ -11651,7 +11683,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="159" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:4" ht="17.25" customHeight="1">
       <c r="A159" s="117" t="s">
         <v>224</v>
       </c>
@@ -11667,7 +11699,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="160" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:4" ht="17.25" customHeight="1">
       <c r="A160" s="117" t="s">
         <v>225</v>
       </c>
@@ -11683,7 +11715,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="161" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:4" ht="17.25" customHeight="1">
       <c r="A161" s="117" t="s">
         <v>226</v>
       </c>
@@ -11699,7 +11731,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="162" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:4" ht="17.25" customHeight="1">
       <c r="A162" s="117" t="s">
         <v>227</v>
       </c>
@@ -11715,7 +11747,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="163" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:4" ht="17.25" customHeight="1">
       <c r="A163" s="117" t="s">
         <v>229</v>
       </c>
@@ -11733,10 +11765,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="D1:D180">
-    <cfRule type="cellIs" dxfId="24" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="42" priority="1" operator="equal">
       <formula>1</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="23" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="41" priority="2" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11751,7 +11783,7 @@
     <outlinePr summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:R18"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" outlineLevelRow="2" outlineLevelCol="2" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" outlineLevelRow="2" outlineLevelCol="2"/>
   <cols>
     <col min="3" max="3" width="0" hidden="1" customWidth="1"/>
     <col min="6" max="6" width="14.28515625" customWidth="1"/>
@@ -11761,17 +11793,17 @@
     <col min="15" max="18" width="9.140625" outlineLevel="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8">
       <c r="A1" t="s">
         <v>230</v>
       </c>
       <c r="C1" t="s">
         <v>231</v>
       </c>
-      <c r="D1" s="123" t="s">
+      <c r="D1" s="122" t="s">
         <v>232</v>
       </c>
-      <c r="E1" s="123"/>
+      <c r="E1" s="122"/>
       <c r="F1" t="s">
         <v>233</v>
       </c>
@@ -11779,19 +11811,19 @@
         <v>234</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8">
       <c r="A2">
         <f>SUM(A1)</f>
         <v>0</v>
       </c>
-      <c r="D2" s="123"/>
-      <c r="E2" s="123"/>
+      <c r="D2" s="122"/>
+      <c r="E2" s="122"/>
       <c r="H2" t="str">
         <f>[1]Feuil1!$A$1</f>
         <v>referenced string</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8">
       <c r="D3" s="85" t="s">
         <v>235</v>
       </c>
@@ -11799,25 +11831,25 @@
         <v>236</v>
       </c>
     </row>
-    <row r="4" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" hidden="1">
       <c r="A4" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" ht="75" customHeight="1">
       <c r="A5" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="10" spans="1:8" outlineLevel="1" x14ac:dyDescent="0.2"/>
-    <row r="11" spans="1:8" outlineLevel="1" x14ac:dyDescent="0.2"/>
-    <row r="12" spans="1:8" hidden="1" outlineLevel="2" x14ac:dyDescent="0.2"/>
-    <row r="13" spans="1:8" hidden="1" outlineLevel="2" x14ac:dyDescent="0.2"/>
-    <row r="14" spans="1:8" hidden="1" outlineLevel="2" x14ac:dyDescent="0.2"/>
-    <row r="15" spans="1:8" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.2"/>
-    <row r="16" spans="1:8" outlineLevel="1" x14ac:dyDescent="0.2"/>
-    <row r="17" outlineLevel="1" x14ac:dyDescent="0.2"/>
-    <row r="18" outlineLevel="1" x14ac:dyDescent="0.2"/>
+    <row r="10" spans="1:8" outlineLevel="1"/>
+    <row r="11" spans="1:8" outlineLevel="1"/>
+    <row r="12" spans="1:8" hidden="1" outlineLevel="2"/>
+    <row r="13" spans="1:8" hidden="1" outlineLevel="2"/>
+    <row r="14" spans="1:8" hidden="1" outlineLevel="2"/>
+    <row r="15" spans="1:8" outlineLevel="1" collapsed="1"/>
+    <row r="16" spans="1:8" outlineLevel="1"/>
+    <row r="17" outlineLevel="1"/>
+    <row r="18" outlineLevel="1"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="D1:E2"/>
@@ -11834,14 +11866,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF68F2C0-1053-4FB6-BD74-8A11B0CAF123}">
   <dimension ref="A1:M30"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75"/>
   <cols>
     <col min="3" max="3" width="17.7109375" customWidth="1"/>
     <col min="5" max="5" width="18.28515625" customWidth="1"/>
     <col min="13" max="13" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="13.5" thickBot="1">
       <c r="A1" s="68" t="s">
         <v>239</v>
       </c>
@@ -11863,7 +11895,7 @@
       </c>
       <c r="M1" s="36"/>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13">
       <c r="A2" s="40" t="s">
         <v>245</v>
       </c>
@@ -11889,7 +11921,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:13">
       <c r="A3" s="41" t="s">
         <v>252</v>
       </c>
@@ -11912,7 +11944,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="15" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" ht="15">
       <c r="A4" s="42" t="s">
         <v>256</v>
       </c>
@@ -11938,7 +11970,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:13">
       <c r="A5" s="43" t="s">
         <v>262</v>
       </c>
@@ -11958,7 +11990,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13">
       <c r="A6" s="44" t="s">
         <v>266</v>
       </c>
@@ -11981,7 +12013,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" ht="15.75">
       <c r="A7" s="45" t="s">
         <v>271</v>
       </c>
@@ -12001,7 +12033,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="21" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:13" ht="21">
       <c r="A8" s="46" t="s">
         <v>275</v>
       </c>
@@ -12024,7 +12056,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:13">
       <c r="A9" s="47" t="s">
         <v>280</v>
       </c>
@@ -12041,7 +12073,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:13">
       <c r="A10" s="48" t="s">
         <v>283</v>
       </c>
@@ -12049,7 +12081,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" ht="13.5" thickBot="1">
       <c r="A11" s="49" t="s">
         <v>285</v>
       </c>
@@ -12058,7 +12090,7 @@
       </c>
       <c r="F11" s="36"/>
     </row>
-    <row r="12" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:13" ht="18.75" customHeight="1">
       <c r="A12" s="50" t="s">
         <v>287</v>
       </c>
@@ -12072,7 +12104,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" ht="18.75" customHeight="1" thickBot="1">
       <c r="A13" s="51" t="s">
         <v>290</v>
       </c>
@@ -12083,7 +12115,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" ht="18.75" customHeight="1" thickBot="1">
       <c r="A14" s="52" t="s">
         <v>291</v>
       </c>
@@ -12097,7 +12129,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" ht="18.75" customHeight="1" thickBot="1">
       <c r="A15" s="53" t="s">
         <v>293</v>
       </c>
@@ -12108,7 +12140,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="16" spans="1:13" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" ht="19.5" customHeight="1" thickBot="1">
       <c r="A16" s="54" t="s">
         <v>294</v>
       </c>
@@ -12122,12 +12154,12 @@
         <v>248</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" ht="13.5" thickBot="1">
       <c r="A17" s="55" t="s">
         <v>296</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" ht="13.5" thickBot="1">
       <c r="A18" s="74" t="s">
         <v>297</v>
       </c>
@@ -12139,7 +12171,7 @@
       </c>
       <c r="F18" s="36"/>
     </row>
-    <row r="19" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" ht="13.5" thickBot="1">
       <c r="A19" s="75" t="s">
         <v>300</v>
       </c>
@@ -12150,7 +12182,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="51.75" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" ht="51.75" thickBot="1">
       <c r="A20" s="76" t="s">
         <v>303</v>
       </c>
@@ -12164,12 +12196,12 @@
         <v>302</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" ht="13.5" thickBot="1">
       <c r="A21" s="77" t="s">
         <v>306</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" ht="13.5" thickBot="1">
       <c r="A22" s="78" t="s">
         <v>307</v>
       </c>
@@ -12178,13 +12210,13 @@
       </c>
       <c r="E22" s="21"/>
     </row>
-    <row r="23" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" ht="13.5" thickBot="1">
       <c r="A23" s="79" t="s">
         <v>309</v>
       </c>
       <c r="E23" s="21"/>
     </row>
-    <row r="24" spans="1:6" ht="14.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" ht="14.25" thickTop="1" thickBot="1">
       <c r="A24" s="80" t="s">
         <v>310</v>
       </c>
@@ -12193,20 +12225,20 @@
       </c>
       <c r="E24" s="21"/>
     </row>
-    <row r="25" spans="1:6" ht="14.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="26" spans="1:6" ht="14.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" ht="14.25" thickTop="1" thickBot="1"/>
+    <row r="26" spans="1:6" ht="14.25" thickTop="1" thickBot="1">
       <c r="C26" s="67" t="s">
         <v>312</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="14.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="1:6" ht="14.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" ht="14.25" thickTop="1" thickBot="1"/>
+    <row r="28" spans="1:6" ht="14.25" thickTop="1" thickBot="1">
       <c r="C28" s="88" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="13.5" thickTop="1" x14ac:dyDescent="0.2"/>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:6" ht="13.5" thickTop="1"/>
+    <row r="30" spans="1:6">
       <c r="C30" s="87" t="s">
         <v>314</v>
       </c>
@@ -12220,13 +12252,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D919E811-4385-4D35-A19E-3B7E0E659A89}">
   <dimension ref="A1:L39"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="19.140625" customWidth="1"/>
     <col min="7" max="7" width="15.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="13.5" thickBot="1">
       <c r="A1" s="37" t="s">
         <v>315</v>
       </c>
@@ -12243,7 +12275,7 @@
       <c r="I1" s="36"/>
       <c r="J1" s="36"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10">
       <c r="A2" s="38" t="s">
         <v>319</v>
       </c>
@@ -12266,7 +12298,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10">
       <c r="A3" s="38" t="s">
         <v>321</v>
       </c>
@@ -12289,7 +12321,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10">
       <c r="A4" s="38" t="s">
         <v>325</v>
       </c>
@@ -12309,7 +12341,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10">
       <c r="A5" s="38" t="s">
         <v>328</v>
       </c>
@@ -12333,7 +12365,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10">
       <c r="A6" s="38" t="s">
         <v>330</v>
       </c>
@@ -12356,7 +12388,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:10">
       <c r="A7" s="38" t="s">
         <v>333</v>
       </c>
@@ -12382,7 +12414,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:10">
       <c r="A8" s="38" t="s">
         <v>337</v>
       </c>
@@ -12393,7 +12425,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10">
       <c r="A9" s="38" t="s">
         <v>339</v>
       </c>
@@ -12402,7 +12434,7 @@
       </c>
       <c r="C9" s="21"/>
     </row>
-    <row r="10" spans="1:10" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" ht="13.5" thickBot="1">
       <c r="A10" s="38" t="s">
         <v>340</v>
       </c>
@@ -12420,7 +12452,7 @@
       <c r="I10" s="36"/>
       <c r="J10" s="36"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:10">
       <c r="A11" s="38" t="s">
         <v>342</v>
       </c>
@@ -12443,13 +12475,13 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:10">
       <c r="A12" s="38" t="s">
         <v>344</v>
       </c>
       <c r="B12" s="39">
         <f ca="1">TODAY()</f>
-        <v>45594</v>
+        <v>45631</v>
       </c>
       <c r="C12" s="39">
         <f>DATE(2010,10,2)</f>
@@ -12468,7 +12500,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:10">
       <c r="A13" s="38" t="s">
         <v>346</v>
       </c>
@@ -12491,7 +12523,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:10">
       <c r="A14" s="38" t="s">
         <v>348</v>
       </c>
@@ -12517,7 +12549,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:10">
       <c r="A15" s="38" t="s">
         <v>350</v>
       </c>
@@ -12537,7 +12569,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:10">
       <c r="A16" s="38" t="s">
         <v>352</v>
       </c>
@@ -12560,7 +12592,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:12">
       <c r="A17" s="38" t="s">
         <v>354</v>
       </c>
@@ -12583,7 +12615,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:12">
       <c r="A18" s="38" t="s">
         <v>356</v>
       </c>
@@ -12606,7 +12638,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:12">
       <c r="A19" s="38" t="s">
         <v>358</v>
       </c>
@@ -12629,7 +12661,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:12">
       <c r="A20" s="38" t="s">
         <v>360</v>
       </c>
@@ -12652,7 +12684,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:12">
       <c r="A21" s="38" t="s">
         <v>362</v>
       </c>
@@ -12678,7 +12710,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:12">
       <c r="A22" s="38" t="s">
         <v>364</v>
       </c>
@@ -12704,7 +12736,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:12">
       <c r="A23" s="38" t="s">
         <v>366</v>
       </c>
@@ -12730,7 +12762,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:12">
       <c r="G24" s="34" t="s">
         <v>368</v>
       </c>
@@ -12747,7 +12779,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:12">
       <c r="A25" s="38" t="s">
         <v>369</v>
       </c>
@@ -12773,7 +12805,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:12">
       <c r="G26" s="34" t="s">
         <v>371</v>
       </c>
@@ -12793,7 +12825,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:12">
       <c r="A27" s="21" t="s">
         <v>372</v>
       </c>
@@ -12819,7 +12851,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:12">
       <c r="G28" s="34" t="s">
         <v>374</v>
       </c>
@@ -12839,7 +12871,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:12">
       <c r="G29" s="34" t="s">
         <v>375</v>
       </c>
@@ -12859,7 +12891,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:12">
       <c r="G30" s="34" t="s">
         <v>376</v>
       </c>
@@ -12879,7 +12911,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:12" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:12" ht="13.5" thickBot="1">
       <c r="G31" s="35" t="s">
         <v>377</v>
       </c>
@@ -12893,7 +12925,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:12">
       <c r="G32" s="34" t="s">
         <v>378</v>
       </c>
@@ -12907,7 +12939,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="7:10" x14ac:dyDescent="0.2">
+    <row r="33" spans="7:10">
       <c r="G33" s="34" t="s">
         <v>379</v>
       </c>
@@ -12921,7 +12953,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="7:10" x14ac:dyDescent="0.2">
+    <row r="34" spans="7:10">
       <c r="G34" s="34" t="s">
         <v>380</v>
       </c>
@@ -12935,7 +12967,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="7:10" x14ac:dyDescent="0.2">
+    <row r="35" spans="7:10">
       <c r="G35" s="34" t="s">
         <v>381</v>
       </c>
@@ -12949,7 +12981,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="7:10" x14ac:dyDescent="0.2">
+    <row r="36" spans="7:10">
       <c r="G36" s="34" t="s">
         <v>382</v>
       </c>
@@ -12963,7 +12995,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="7:10" x14ac:dyDescent="0.2">
+    <row r="37" spans="7:10">
       <c r="G37" s="34" t="s">
         <v>383</v>
       </c>
@@ -12977,110 +13009,110 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="7:10" x14ac:dyDescent="0.2">
+    <row r="39" spans="7:10">
       <c r="G39" s="34"/>
     </row>
   </sheetData>
   <phoneticPr fontId="21" type="noConversion"/>
   <conditionalFormatting sqref="B15">
-    <cfRule type="expression" dxfId="22" priority="58">
+    <cfRule type="expression" dxfId="40" priority="58">
       <formula>ODD(B15)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B26:B27">
-    <cfRule type="cellIs" dxfId="21" priority="46" operator="equal">
+    <cfRule type="cellIs" dxfId="39" priority="46" operator="equal">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B2:C2">
-    <cfRule type="aboveAverage" dxfId="20" priority="114"/>
+    <cfRule type="aboveAverage" dxfId="38" priority="114"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:C3">
-    <cfRule type="beginsWith" dxfId="19" priority="73" operator="beginsWith" text="rule">
+    <cfRule type="beginsWith" dxfId="37" priority="73" operator="beginsWith" text="rule">
       <formula>LEFT(B3,LEN("rule"))="rule"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B4:C4">
-    <cfRule type="containsBlanks" dxfId="18" priority="71">
+    <cfRule type="containsBlanks" dxfId="36" priority="71">
       <formula>LEN(TRIM(B4))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B5:C5">
-    <cfRule type="containsErrors" dxfId="17" priority="70">
+    <cfRule type="containsErrors" dxfId="35" priority="70">
       <formula>ISERROR(B5)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:C6">
-    <cfRule type="containsText" dxfId="16" priority="69" operator="containsText" text="rule">
+    <cfRule type="containsText" dxfId="34" priority="69" operator="containsText" text="rule">
       <formula>NOT(ISERROR(SEARCH("rule",B6)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8:C8">
-    <cfRule type="endsWith" dxfId="15" priority="67" operator="endsWith" text="rule">
+    <cfRule type="endsWith" dxfId="33" priority="67" operator="endsWith" text="rule">
       <formula>RIGHT(B8,LEN("rule"))="rule"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B9:C9">
-    <cfRule type="notContainsBlanks" dxfId="14" priority="66">
+    <cfRule type="notContainsBlanks" dxfId="32" priority="66">
       <formula>LEN(TRIM(B9))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B10:C10">
-    <cfRule type="notContainsErrors" dxfId="13" priority="65">
+    <cfRule type="notContainsErrors" dxfId="31" priority="65">
       <formula>NOT(ISERROR(B10))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B11:C11">
-    <cfRule type="notContainsText" dxfId="12" priority="64" operator="notContains" text="rule">
+    <cfRule type="notContainsText" dxfId="30" priority="64" operator="notContains" text="rule">
       <formula>ISERROR(SEARCH("rule",B11))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12:C12">
-    <cfRule type="timePeriod" dxfId="11" priority="63" timePeriod="today">
+    <cfRule type="timePeriod" dxfId="29" priority="63" timePeriod="today">
       <formula>FLOOR(B12,1)=TODAY()</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B13:C13">
-    <cfRule type="top10" dxfId="10" priority="115" rank="1"/>
+    <cfRule type="top10" dxfId="28" priority="115" rank="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B16:C16">
-    <cfRule type="cellIs" dxfId="9" priority="45" operator="equal">
+    <cfRule type="cellIs" dxfId="27" priority="45" operator="equal">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B17:C17">
-    <cfRule type="cellIs" dxfId="8" priority="56" operator="notEqual">
+    <cfRule type="cellIs" dxfId="26" priority="56" operator="notEqual">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B18:C18">
-    <cfRule type="cellIs" dxfId="7" priority="6" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="25" priority="6" operator="greaterThan">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B19:C19">
-    <cfRule type="cellIs" dxfId="6" priority="5" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="24" priority="5" operator="greaterThanOrEqual">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B20:C20">
-    <cfRule type="cellIs" dxfId="5" priority="4" operator="lessThan">
+    <cfRule type="cellIs" dxfId="23" priority="4" operator="lessThan">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B21:C21">
-    <cfRule type="cellIs" dxfId="4" priority="3" operator="lessThanOrEqual">
+    <cfRule type="cellIs" dxfId="22" priority="3" operator="lessThanOrEqual">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B22:C22">
-    <cfRule type="cellIs" dxfId="3" priority="2" operator="between">
+    <cfRule type="cellIs" dxfId="21" priority="2" operator="between">
       <formula>2</formula>
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B23:C23">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="notBetween">
+    <cfRule type="cellIs" dxfId="20" priority="1" operator="notBetween">
       <formula>2</formula>
       <formula>4</formula>
     </cfRule>
@@ -13114,10 +13146,10 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7:D7">
-    <cfRule type="duplicateValues" dxfId="1" priority="82"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="82"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B14:D14">
-    <cfRule type="uniqueValues" dxfId="0" priority="96"/>
+    <cfRule type="uniqueValues" dxfId="18" priority="96"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:J2">
     <cfRule type="colorScale" priority="44">
@@ -13540,7 +13572,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5CCC4B1-5C65-4837-AA26-56CCF06B63BB}">
   <dimension ref="A1:J34"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75"/>
   <cols>
     <col min="3" max="3" width="17.28515625" customWidth="1"/>
     <col min="4" max="4" width="9.5703125" customWidth="1"/>
@@ -13552,12 +13584,12 @@
     <col min="10" max="10" width="17.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10">
       <c r="A1" t="s">
         <v>384</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" ht="15">
       <c r="C3" s="17" t="s">
         <v>35</v>
       </c>
@@ -13583,7 +13615,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10">
       <c r="C4" s="117" t="s">
         <v>42</v>
       </c>
@@ -13614,7 +13646,7 @@
         <v>Rank</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10">
       <c r="C5" s="117" t="s">
         <v>44</v>
       </c>
@@ -13645,7 +13677,7 @@
         <v>Rank</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10">
       <c r="C6" s="117" t="s">
         <v>391</v>
       </c>
@@ -13678,7 +13710,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:10">
       <c r="B8" t="s">
         <v>392</v>
       </c>
@@ -13689,7 +13721,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10">
       <c r="C9">
         <v>3</v>
       </c>
@@ -13697,7 +13729,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:10">
       <c r="B11" t="s">
         <v>393</v>
       </c>
@@ -13708,7 +13740,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:10">
       <c r="C12">
         <v>3</v>
       </c>
@@ -13716,7 +13748,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:10">
       <c r="B14" t="s">
         <v>396</v>
       </c>
@@ -13727,7 +13759,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:10">
       <c r="C15">
         <v>3</v>
       </c>
@@ -13735,7 +13767,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:4">
       <c r="B17" t="s">
         <v>397</v>
       </c>
@@ -13746,7 +13778,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:4">
       <c r="C18">
         <v>3</v>
       </c>
@@ -13754,7 +13786,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:4">
       <c r="B20" t="s">
         <v>398</v>
       </c>
@@ -13765,7 +13797,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:4">
       <c r="C21">
         <v>3</v>
       </c>
@@ -13773,7 +13805,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:4">
       <c r="B23" t="s">
         <v>399</v>
       </c>
@@ -13784,7 +13816,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="24" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:4">
       <c r="C24">
         <v>3</v>
       </c>
@@ -13792,7 +13824,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="26" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="26" spans="2:4">
       <c r="B26" t="s">
         <v>400</v>
       </c>
@@ -13803,7 +13835,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="27" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="27" spans="2:4">
       <c r="C27">
         <v>3</v>
       </c>
@@ -13811,7 +13843,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="28" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="28" spans="2:4">
       <c r="C28" t="s">
         <v>391</v>
       </c>
@@ -13820,7 +13852,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="30" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:4">
       <c r="B30" t="s">
         <v>401</v>
       </c>
@@ -13831,7 +13863,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="31" spans="2:4" hidden="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="2:4" hidden="1">
       <c r="C31" t="s">
         <v>404</v>
       </c>
@@ -13839,7 +13871,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="32" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="32" spans="2:4">
       <c r="C32" t="s">
         <v>405</v>
       </c>
@@ -13847,7 +13879,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="34" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="34" spans="2:2">
       <c r="B34" t="s">
         <v>406</v>
       </c>
@@ -13872,7 +13904,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE9224F2-4D06-4586-886C-E51F5EBCA7B0}">
   <dimension ref="A1:L21"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75"/>
   <cols>
     <col min="3" max="3" width="13.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.5703125" bestFit="1" customWidth="1"/>
@@ -13893,7 +13925,7 @@
     <col min="21" max="21" width="19.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" ht="15">
       <c r="A1" s="92" t="s">
         <v>407</v>
       </c>
@@ -13903,7 +13935,7 @@
       <c r="E1" s="17"/>
       <c r="F1" s="17"/>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:12">
       <c r="A2" s="117"/>
       <c r="B2" s="117"/>
       <c r="C2" s="117"/>
@@ -13911,7 +13943,7 @@
       <c r="E2" s="117"/>
       <c r="F2" s="117"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:12">
       <c r="A3" s="117"/>
       <c r="B3" s="117"/>
       <c r="C3" s="89" t="s">
@@ -13921,7 +13953,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:12">
       <c r="A4" s="117"/>
       <c r="B4" s="117"/>
       <c r="C4" s="89" t="s">
@@ -13955,7 +13987,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:12">
       <c r="A5" s="117"/>
       <c r="B5" s="117"/>
       <c r="C5" s="90" t="s">
@@ -13968,7 +14000,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:12">
       <c r="A6" s="117"/>
       <c r="B6" s="117"/>
       <c r="C6" s="91">
@@ -13981,7 +14013,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:12">
       <c r="A7" s="117"/>
       <c r="B7" s="117"/>
       <c r="C7" s="90" t="s">
@@ -13994,7 +14026,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:12">
       <c r="A8" s="117"/>
       <c r="B8" s="117"/>
       <c r="C8" s="91">
@@ -14007,7 +14039,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:12">
       <c r="A9" s="117"/>
       <c r="B9" s="117"/>
       <c r="C9" s="90" t="s">
@@ -14020,7 +14052,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:12">
       <c r="A10" s="117"/>
       <c r="B10" s="117"/>
       <c r="C10" s="91">
@@ -14033,7 +14065,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:12">
       <c r="C11" s="90" t="s">
         <v>44</v>
       </c>
@@ -14044,7 +14076,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:12">
       <c r="C12" s="91">
         <v>23000</v>
       </c>
@@ -14055,7 +14087,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:12">
       <c r="C13" s="90" t="s">
         <v>50</v>
       </c>
@@ -14066,7 +14098,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:12">
       <c r="C14" s="91">
         <v>2</v>
       </c>
@@ -14077,7 +14109,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:12">
       <c r="C15" s="90" t="s">
         <v>48</v>
       </c>
@@ -14088,7 +14120,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:12">
       <c r="C16" s="91">
         <v>50024</v>
       </c>
@@ -14099,7 +14131,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="17" spans="3:12">
       <c r="C17" s="90" t="s">
         <v>53</v>
       </c>
@@ -14110,7 +14142,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="18" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="18" spans="3:12">
       <c r="C18" s="91">
         <v>189576</v>
       </c>
@@ -14121,7 +14153,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="19" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="19" spans="3:12">
       <c r="C19" s="90" t="s">
         <v>57</v>
       </c>
@@ -14132,7 +14164,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="20" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="20" spans="3:12">
       <c r="C20" s="91">
         <v>5000</v>
       </c>
@@ -14143,7 +14175,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="21" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="21" spans="3:12">
       <c r="C21" s="90" t="s">
         <v>411</v>
       </c>
@@ -14184,29 +14216,29 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C47BF70-BA80-4124-B359-67CBCB635390}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="65.140625" customWidth="1"/>
     <col min="2" max="26" width="13.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2">
       <c r="A1" t="s">
         <v>412</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2">
       <c r="A2" t="s">
         <v>413</v>
       </c>
       <c r="B2" s="117"/>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2">
       <c r="A3" t="s">
         <v>414</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2">
       <c r="A4" t="s">
         <v>415</v>
       </c>
@@ -14220,9 +14252,9 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FE31E21-0350-44E7-AF13-4CA140505B30}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="12.75"/>
   <sheetData>
-    <row r="1" spans="1:1" ht="51" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:1" ht="51">
       <c r="A1" s="99" t="s">
         <v>416</v>
       </c>

</xml_diff>

<commit_message>
[IMP] xlsx: support import/export of doughnut,pyramid & horizontal bar charts
This commit adds support for exporting & importing the charts mentioned above.
Pyramid charts are not supported in Excel, therefore, we do a best effort by
exporting them as horizontal bar charts.

Task: 3978237
</commit_message>
<xml_diff>
--- a/tests/__xlsx__/xlsx_demo_data.xlsx
+++ b/tests/__xlsx__/xlsx_demo_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28507"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Adrien\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{157AC437-DB84-431C-BDD0-6A0421B0B149}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7A0F40E7-3C8A-4E57-BEF5-0AD89070EFA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23295" yWindow="195" windowWidth="21600" windowHeight="11385" firstSheet="13" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23295" yWindow="195" windowWidth="21600" windowHeight="11385" firstSheet="8" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
   </externalReferences>
   <calcPr calcId="191028" calcCompleted="0"/>
   <pivotCaches>
-    <pivotCache cacheId="3563" r:id="rId16"/>
+    <pivotCache cacheId="4689" r:id="rId16"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -2375,6 +2375,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -2387,7 +2388,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
@@ -3593,6 +3593,422 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart10.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="1"/>
+  <c:style val="2"/>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$B$26</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>first dataset</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="4472C4"/>
+            </a:solidFill>
+            <a:ln cmpd="sng">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="1"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet1!$A$27:$A$35</c:f>
+              <c:strCache>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>Emily Anderson (Emmy)</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Sophie Allen (Saffi)</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Chloe Adams</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Megan Alexander (Meg)</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Lucy Arnold (Lulu)</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Hannah Alvarez</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Jessica Alcock (Jess)</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Charlotte Anaya</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Lauren Anthony</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$B$27:$B$35</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>48</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>31</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>16</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{6F2FDCE9-48DA-4B69-8628-5D25D57E5C99}">
+              <c14:invertSolidFillFmt>
+                <c14:spPr xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart">
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                  <a:ln cmpd="sng">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                  </a:ln>
+                </c14:spPr>
+              </c14:invertSolidFillFmt>
+            </c:ext>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-D94B-45A0-8AD6-3E4F4E7665C2}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$C$26</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>second dataset</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="ED7D31"/>
+            </a:solidFill>
+            <a:ln cmpd="sng">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="1"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet1!$A$27:$A$35</c:f>
+              <c:strCache>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>Emily Anderson (Emmy)</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Sophie Allen (Saffi)</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Chloe Adams</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Megan Alexander (Meg)</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Lucy Arnold (Lulu)</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Hannah Alvarez</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Jessica Alcock (Jess)</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Charlotte Anaya</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Lauren Anthony</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$C$27:$C$35</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>27</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>43</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>16</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{6F2FDCE9-48DA-4B69-8628-5D25D57E5C99}">
+              <c14:invertSolidFillFmt>
+                <c14:spPr xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart">
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                  <a:ln cmpd="sng">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                  </a:ln>
+                </c14:spPr>
+              </c14:invertSolidFillFmt>
+            </c:ext>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-D94B-45A0-8AD6-3E4F4E7665C2}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="150"/>
+        <c:axId val="998664793"/>
+        <c:axId val="344680958"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="998664793"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr lvl="0">
+                  <a:defRPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr lvl="0">
+              <a:defRPr b="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="fr-FR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="344680958"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="1"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="344680958"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="B7B7B7"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:minorGridlines>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC">
+                  <a:alpha val="0"/>
+                </a:srgbClr>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:minorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr lvl="0">
+                  <a:defRPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr lvl="0">
+              <a:defRPr b="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="fr-FR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="998664793"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr lvl="0">
+            <a:defRPr b="0">
+              <a:solidFill>
+                <a:srgbClr val="1A1A1A"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="fr-FR"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="zero"/>
+    <c:showDLblsOverMax val="1"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
@@ -6150,38 +6566,58 @@
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
-  <c:roundedCorners val="1"/>
-  <c:style val="2"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
   <c:chart>
-    <c:autoTitleDeleted val="1"/>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr lvl="0">
+              <a:defRPr b="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="2200"/>
+              <a:t>horizontal bar chart</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
     <c:plotArea>
       <c:layout/>
       <c:barChart>
-        <c:barDir val="col"/>
+        <c:barDir val="bar"/>
         <c:grouping val="clustered"/>
-        <c:varyColors val="1"/>
+        <c:varyColors val="0"/>
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>Sheet1!$B$26</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>first dataset</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="4472C4"/>
+              <a:srgbClr val="7030A0"/>
             </a:solidFill>
-            <a:ln cmpd="sng">
+            <a:ln>
               <a:solidFill>
-                <a:srgbClr val="000000"/>
+                <a:srgbClr val="7030A0"/>
               </a:solidFill>
+              <a:prstDash val="solid"/>
             </a:ln>
           </c:spPr>
           <c:invertIfNegative val="1"/>
@@ -6263,41 +6699,32 @@
                   <a:solidFill>
                     <a:srgbClr val="FFFFFF"/>
                   </a:solidFill>
-                  <a:ln cmpd="sng">
+                  <a:ln>
                     <a:solidFill>
-                      <a:srgbClr val="000000"/>
+                      <a:srgbClr val="7030A0"/>
                     </a:solidFill>
+                    <a:prstDash val="solid"/>
                   </a:ln>
                 </c14:spPr>
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-D94B-45A0-8AD6-3E4F4E7665C2}"/>
+              <c16:uniqueId val="{00000000-F453-4C27-9300-76287E40C06A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="1"/>
           <c:order val="1"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>Sheet1!$C$26</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>second dataset</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="ED7D31"/>
+              <a:srgbClr val="C65911"/>
             </a:solidFill>
-            <a:ln cmpd="sng">
+            <a:ln>
               <a:solidFill>
-                <a:srgbClr val="000000"/>
+                <a:srgbClr val="C65911"/>
               </a:solidFill>
+              <a:prstDash val="solid"/>
             </a:ln>
           </c:spPr>
           <c:invertIfNegative val="1"/>
@@ -6379,16 +6806,17 @@
                   <a:solidFill>
                     <a:srgbClr val="FFFFFF"/>
                   </a:solidFill>
-                  <a:ln cmpd="sng">
+                  <a:ln>
                     <a:solidFill>
-                      <a:srgbClr val="000000"/>
+                      <a:srgbClr val="C65911"/>
                     </a:solidFill>
+                    <a:prstDash val="solid"/>
                   </a:ln>
                 </c14:spPr>
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-D94B-45A0-8AD6-3E4F4E7665C2}"/>
+              <c16:uniqueId val="{00000001-F453-4C27-9300-76287E40C06A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6400,17 +6828,26 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:gapWidth val="150"/>
-        <c:axId val="998664793"/>
-        <c:axId val="344680958"/>
+        <c:gapWidth val="70"/>
+        <c:axId val="17781237"/>
+        <c:axId val="88853993"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="998664793"/>
+        <c:axId val="17781237"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
-        <c:axPos val="b"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln cmpd="sng">
+              <a:solidFill>
+                <a:srgbClr val="B7B7B7"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
         <c:title>
           <c:tx>
             <c:rich>
@@ -6425,14 +6862,14 @@
                     <a:latin typeface="+mn-lt"/>
                   </a:defRPr>
                 </a:pPr>
-                <a:endParaRPr/>
+                <a:endParaRPr lang="en-US"/>
               </a:p>
             </c:rich>
           </c:tx>
-          <c:overlay val="0"/>
+          <c:overlay val="1"/>
         </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
+        <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:txPr>
@@ -6440,7 +6877,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr lvl="0">
-              <a:defRPr b="0">
+              <a:defRPr sz="1000" b="0" i="0">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
@@ -6450,7 +6887,7 @@
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="344680958"/>
+        <c:crossAx val="88853993"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -6458,32 +6895,21 @@
         <c:noMultiLvlLbl val="1"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="344680958"/>
+        <c:axId val="88853993"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
-        <c:axPos val="l"/>
+        <c:axPos val="b"/>
         <c:majorGridlines>
           <c:spPr>
-            <a:ln>
+            <a:ln cmpd="sng">
               <a:solidFill>
                 <a:srgbClr val="B7B7B7"/>
               </a:solidFill>
             </a:ln>
           </c:spPr>
         </c:majorGridlines>
-        <c:minorGridlines>
-          <c:spPr>
-            <a:ln>
-              <a:solidFill>
-                <a:srgbClr val="CCCCCC">
-                  <a:alpha val="0"/>
-                </a:srgbClr>
-              </a:solidFill>
-            </a:ln>
-          </c:spPr>
-        </c:minorGridlines>
         <c:title>
           <c:tx>
             <c:rich>
@@ -6498,25 +6924,22 @@
                     <a:latin typeface="+mn-lt"/>
                   </a:defRPr>
                 </a:pPr>
-                <a:endParaRPr/>
+                <a:endParaRPr lang="en-US"/>
               </a:p>
             </c:rich>
           </c:tx>
-          <c:overlay val="0"/>
+          <c:overlay val="1"/>
         </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
+        <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:ln/>
-        </c:spPr>
         <c:txPr>
           <a:bodyPr/>
           <a:lstStyle/>
           <a:p>
             <a:pPr lvl="0">
-              <a:defRPr b="0">
+              <a:defRPr sz="1000" b="0" i="0">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
@@ -6526,22 +6949,27 @@
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="998664793"/>
+        <c:crossAx val="17781237"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
+      <c:spPr>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+      </c:spPr>
     </c:plotArea>
     <c:legend>
-      <c:legendPos val="r"/>
+      <c:legendPos val="t"/>
       <c:overlay val="0"/>
       <c:txPr>
         <a:bodyPr/>
         <a:lstStyle/>
         <a:p>
           <a:pPr lvl="0">
-            <a:defRPr b="0">
+            <a:defRPr sz="1000" b="0" i="0">
               <a:solidFill>
-                <a:srgbClr val="1A1A1A"/>
+                <a:srgbClr val="000000"/>
               </a:solidFill>
               <a:latin typeface="+mn-lt"/>
             </a:defRPr>
@@ -6554,6 +6982,380 @@
     <c:dispBlanksAs val="zero"/>
     <c:showDLblsOverMax val="1"/>
   </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln cmpd="sng">
+      <a:solidFill>
+        <a:srgbClr val="000000"/>
+      </a:solidFill>
+    </a:ln>
+  </c:spPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr lvl="0">
+              <a:defRPr b="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="2200"/>
+              <a:t>single dataset doughnut chart</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US" sz="2400"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:doughnutChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$B$26</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>first dataset</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="1F77B4"/>
+              </a:solidFill>
+              <a:ln w="14288" cmpd="sng">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-0405-4A2D-A579-D08CD080C2D2}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FF7F0E"/>
+              </a:solidFill>
+              <a:ln w="14288" cmpd="sng">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-0405-4A2D-A579-D08CD080C2D2}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="AEC7E8"/>
+              </a:solidFill>
+              <a:ln w="14288" cmpd="sng">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-0405-4A2D-A579-D08CD080C2D2}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="3"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FFBB78"/>
+              </a:solidFill>
+              <a:ln w="14288" cmpd="sng">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000007-0405-4A2D-A579-D08CD080C2D2}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="4"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="2CA02C"/>
+              </a:solidFill>
+              <a:ln w="14288" cmpd="sng">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000009-0405-4A2D-A579-D08CD080C2D2}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="5"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="98DF8A"/>
+              </a:solidFill>
+              <a:ln w="14288" cmpd="sng">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000000B-0405-4A2D-A579-D08CD080C2D2}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="6"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="D62728"/>
+              </a:solidFill>
+              <a:ln w="14288" cmpd="sng">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000000D-0405-4A2D-A579-D08CD080C2D2}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="7"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FF9896"/>
+              </a:solidFill>
+              <a:ln w="14288" cmpd="sng">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000000F-0405-4A2D-A579-D08CD080C2D2}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="8"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="9467BD"/>
+              </a:solidFill>
+              <a:ln w="14288" cmpd="sng">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000011-0405-4A2D-A579-D08CD080C2D2}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet1!$A$27:$A$35</c:f>
+              <c:strCache>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>Emily Anderson (Emmy)</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Sophie Allen (Saffi)</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Chloe Adams</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Megan Alexander (Meg)</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Lucy Arnold (Lulu)</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Hannah Alvarez</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Jessica Alcock (Jess)</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Charlotte Anaya</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Lauren Anthony</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$B$27:$B$35</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>48</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>31</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>16</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000012-0405-4A2D-A579-D08CD080C2D2}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="1"/>
+        </c:dLbls>
+        <c:firstSliceAng val="0"/>
+        <c:holeSize val="50"/>
+      </c:doughnutChart>
+      <c:spPr>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="t"/>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr lvl="0">
+            <a:defRPr sz="1000" b="0" i="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="fr-FR"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="zero"/>
+    <c:showDLblsOverMax val="1"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln cmpd="sng">
+      <a:solidFill>
+        <a:srgbClr val="000000"/>
+      </a:solidFill>
+    </a:ln>
+  </c:spPr>
   <c:printSettings>
     <c:headerFooter/>
     <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
@@ -7316,6 +8118,88 @@
     </xdr:graphicFrame>
     <xdr:clientData fLocksWithSheet="0"/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>161925</xdr:colOff>
+      <xdr:row>45</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="9" name="Chart 8" title="Chart">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5814E5DD-0992-44E8-87F0-31C94A544112}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{E2B20B98-FA84-44C9-8DBB-5852658E9967}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId8"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>895350</xdr:colOff>
+      <xdr:row>71</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>333375</xdr:colOff>
+      <xdr:row>89</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="10" name="Chart 9" title="Chart">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DD226922-C98E-43FE-A6FF-0C6686AB1592}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{5814E5DD-0992-44E8-87F0-31C94A544112}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -7575,7 +8459,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9B3CE3F5-58D8-48A3-B9C6-24D1506C9F5C}" name="PivotTable1" cacheId="3563" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9B3CE3F5-58D8-48A3-B9C6-24D1506C9F5C}" name="PivotTable1" cacheId="4689" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="C3:L21" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="5">
     <pivotField axis="axisRow" showAll="0">
@@ -8193,7 +9077,7 @@
       <c r="H2" s="118" t="s">
         <v>4</v>
       </c>
-      <c r="I2" s="123"/>
+      <c r="I2" s="119"/>
       <c r="K2" s="3"/>
     </row>
     <row r="3" spans="1:12" ht="17.25" customHeight="1">
@@ -8203,10 +9087,10 @@
       <c r="G3" s="117">
         <v>8</v>
       </c>
-      <c r="H3" s="123"/>
-      <c r="I3" s="123"/>
+      <c r="H3" s="119"/>
+      <c r="I3" s="119"/>
       <c r="J3" s="5"/>
-      <c r="K3" s="119">
+      <c r="K3" s="120">
         <v>5</v>
       </c>
       <c r="L3" s="6"/>
@@ -8224,10 +9108,10 @@
       <c r="G4" s="117">
         <v>9</v>
       </c>
-      <c r="H4" s="123"/>
-      <c r="I4" s="123"/>
+      <c r="H4" s="119"/>
+      <c r="I4" s="119"/>
       <c r="J4" s="5"/>
-      <c r="K4" s="120"/>
+      <c r="K4" s="121"/>
       <c r="L4" s="6"/>
     </row>
     <row r="5" spans="1:12" ht="17.25" customHeight="1">
@@ -8237,10 +9121,10 @@
       <c r="G5" s="117">
         <v>15</v>
       </c>
-      <c r="H5" s="123"/>
-      <c r="I5" s="123"/>
+      <c r="H5" s="119"/>
+      <c r="I5" s="119"/>
       <c r="J5" s="5"/>
-      <c r="K5" s="120"/>
+      <c r="K5" s="121"/>
       <c r="L5" s="6"/>
     </row>
     <row r="6" spans="1:12" ht="17.25" customHeight="1">
@@ -8248,7 +9132,7 @@
         <v>22</v>
       </c>
       <c r="J6" s="5"/>
-      <c r="K6" s="120"/>
+      <c r="K6" s="121"/>
       <c r="L6" s="6"/>
     </row>
     <row r="7" spans="1:12" ht="17.25" customHeight="1">
@@ -8256,7 +9140,7 @@
         <v>3</v>
       </c>
       <c r="J7" s="5"/>
-      <c r="K7" s="120"/>
+      <c r="K7" s="121"/>
       <c r="L7" s="6"/>
     </row>
     <row r="8" spans="1:12" ht="17.25" customHeight="1">
@@ -8264,7 +9148,7 @@
         <v>30</v>
       </c>
       <c r="J8" s="5"/>
-      <c r="K8" s="121"/>
+      <c r="K8" s="122"/>
       <c r="L8" s="6"/>
     </row>
     <row r="9" spans="1:12" ht="17.25" customHeight="1">
@@ -10732,7 +11616,7 @@
       </c>
       <c r="B100" s="19">
         <f ca="1">NOW()</f>
-        <v>45663.51402037037</v>
+        <v>45667.778077893519</v>
       </c>
       <c r="D100" s="117">
         <f ca="1">IF(ISNUMBER(B100),1,0)</f>
@@ -11422,7 +12306,7 @@
       </c>
       <c r="B144" s="18">
         <f ca="1">TODAY()</f>
-        <v>45663</v>
+        <v>45667</v>
       </c>
       <c r="D144" s="117">
         <f ca="1">IF(ISNUMBER(B144),1,0)</f>
@@ -11771,10 +12655,10 @@
       <c r="C1" t="s">
         <v>231</v>
       </c>
-      <c r="D1" s="122" t="s">
+      <c r="D1" s="123" t="s">
         <v>232</v>
       </c>
-      <c r="E1" s="122"/>
+      <c r="E1" s="123"/>
       <c r="F1" t="s">
         <v>233</v>
       </c>
@@ -11787,8 +12671,8 @@
         <f>SUM(A1)</f>
         <v>0</v>
       </c>
-      <c r="D2" s="122"/>
-      <c r="E2" s="122"/>
+      <c r="D2" s="123"/>
+      <c r="E2" s="123"/>
       <c r="H2" t="str">
         <f>[1]Feuil1!$A$1</f>
         <v>referenced string</v>
@@ -12452,7 +13336,7 @@
       </c>
       <c r="B12" s="39">
         <f ca="1">TODAY()</f>
-        <v>45663</v>
+        <v>45667</v>
       </c>
       <c r="C12" s="39">
         <f>DATE(2010,10,2)</f>

</xml_diff>

<commit_message>
[IMP] xlsx: support import/export of doughnut, pyramid & horizontal bar charts
This commit adds support for exporting & importing the charts mentioned above.
Pyramid charts are not supported in Excel, therefore, we do a best effort by
exporting them as horizontal bar charts.

Task: 3978237
</commit_message>
<xml_diff>
--- a/tests/__xlsx__/xlsx_demo_data.xlsx
+++ b/tests/__xlsx__/xlsx_demo_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28715"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28724"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Odoo\spreadsheet\tests\__xlsx__\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4ABEBB5E-CC42-4D3F-B076-13470D76BC9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F0F3413D-2983-43BC-B7D9-48EACAB90F26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,9 +31,14 @@
   <externalReferences>
     <externalReference r:id="rId15"/>
   </externalReferences>
+  <definedNames>
+    <definedName name="_xlchart.v1.0" hidden="1">Sheet1!$A$27:$A$35</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">Sheet1!$B$26</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">Sheet1!$B$27:$B$35</definedName>
+  </definedNames>
   <calcPr calcId="191028" calcCompleted="0"/>
   <pivotCaches>
-    <pivotCache cacheId="3062" r:id="rId16"/>
+    <pivotCache cacheId="1259" r:id="rId16"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -3608,6 +3613,793 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart10.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr lvl="0">
+              <a:defRPr b="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="2200"/>
+              <a:t>doughnut chart with hole</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.30285577409492809"/>
+          <c:y val="1.397398743755821E-2"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:doughnutChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$B$26</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>first dataset</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="1F77B4"/>
+              </a:solidFill>
+              <a:ln w="14288" cmpd="sng">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000014-D17F-47AA-A8EC-52019D60CBD0}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FF7F0E"/>
+              </a:solidFill>
+              <a:ln w="14288" cmpd="sng">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000016-D17F-47AA-A8EC-52019D60CBD0}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="AEC7E8"/>
+              </a:solidFill>
+              <a:ln w="14288" cmpd="sng">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000018-D17F-47AA-A8EC-52019D60CBD0}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="3"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FFBB78"/>
+              </a:solidFill>
+              <a:ln w="14288" cmpd="sng">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000001A-D17F-47AA-A8EC-52019D60CBD0}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="4"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="2CA02C"/>
+              </a:solidFill>
+              <a:ln w="14288" cmpd="sng">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000001C-D17F-47AA-A8EC-52019D60CBD0}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="5"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="98DF8A"/>
+              </a:solidFill>
+              <a:ln w="14288" cmpd="sng">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000001E-D17F-47AA-A8EC-52019D60CBD0}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="6"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="D62728"/>
+              </a:solidFill>
+              <a:ln w="14288" cmpd="sng">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000020-D17F-47AA-A8EC-52019D60CBD0}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="7"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FF9896"/>
+              </a:solidFill>
+              <a:ln w="14288" cmpd="sng">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000022-D17F-47AA-A8EC-52019D60CBD0}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="8"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="9467BD"/>
+              </a:solidFill>
+              <a:ln w="14288" cmpd="sng">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000024-D17F-47AA-A8EC-52019D60CBD0}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet1!$A$27:$A$35</c:f>
+              <c:strCache>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>Emily Anderson (Emmy)</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Sophie Allen (Saffi)</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Chloe Adams</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Megan Alexander (Meg)</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Lucy Arnold (Lulu)</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Hannah Alvarez</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Jessica Alcock (Jess)</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Charlotte Anaya</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Lauren Anthony</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$B$27:$B$35</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>48</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>31</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>16</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000025-D17F-47AA-A8EC-52019D60CBD0}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="1"/>
+        </c:dLbls>
+        <c:firstSliceAng val="0"/>
+        <c:holeSize val="50"/>
+      </c:doughnutChart>
+      <c:spPr>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="t"/>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr lvl="0">
+            <a:defRPr sz="1000" b="0" i="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="fr-FR"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="zero"/>
+    <c:showDLblsOverMax val="1"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln cmpd="sng">
+      <a:solidFill>
+        <a:srgbClr val="000000"/>
+      </a:solidFill>
+    </a:ln>
+  </c:spPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart11.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="1"/>
+  <c:style val="2"/>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$B$26</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>first dataset</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="4472C4"/>
+            </a:solidFill>
+            <a:ln cmpd="sng">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="1"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet1!$A$27:$A$35</c:f>
+              <c:strCache>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>Emily Anderson (Emmy)</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Sophie Allen (Saffi)</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Chloe Adams</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Megan Alexander (Meg)</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Lucy Arnold (Lulu)</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Hannah Alvarez</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Jessica Alcock (Jess)</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Charlotte Anaya</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Lauren Anthony</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$B$27:$B$35</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>48</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>31</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>16</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{6F2FDCE9-48DA-4B69-8628-5D25D57E5C99}">
+              <c14:invertSolidFillFmt>
+                <c14:spPr xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart">
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                  <a:ln cmpd="sng">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                  </a:ln>
+                </c14:spPr>
+              </c14:invertSolidFillFmt>
+            </c:ext>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-D94B-45A0-8AD6-3E4F4E7665C2}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$C$26</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>second dataset</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="ED7D31"/>
+            </a:solidFill>
+            <a:ln cmpd="sng">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="1"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet1!$A$27:$A$35</c:f>
+              <c:strCache>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>Emily Anderson (Emmy)</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Sophie Allen (Saffi)</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Chloe Adams</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Megan Alexander (Meg)</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Lucy Arnold (Lulu)</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Hannah Alvarez</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Jessica Alcock (Jess)</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Charlotte Anaya</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Lauren Anthony</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$C$27:$C$35</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>27</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>43</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>16</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{6F2FDCE9-48DA-4B69-8628-5D25D57E5C99}">
+              <c14:invertSolidFillFmt>
+                <c14:spPr xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart">
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                  <a:ln cmpd="sng">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                  </a:ln>
+                </c14:spPr>
+              </c14:invertSolidFillFmt>
+            </c:ext>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-D94B-45A0-8AD6-3E4F4E7665C2}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="150"/>
+        <c:axId val="998664793"/>
+        <c:axId val="344680958"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="998664793"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr lvl="0">
+                  <a:defRPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr lvl="0">
+              <a:defRPr b="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="fr-FR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="344680958"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="1"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="344680958"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="B7B7B7"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:minorGridlines>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="CCCCCC">
+                  <a:alpha val="0"/>
+                </a:srgbClr>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:minorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr lvl="0">
+                  <a:defRPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr lvl="0">
+              <a:defRPr b="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="fr-FR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="998664793"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr lvl="0">
+            <a:defRPr b="0">
+              <a:solidFill>
+                <a:srgbClr val="1A1A1A"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="fr-FR"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="zero"/>
+    <c:showDLblsOverMax val="1"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
@@ -6436,38 +7228,58 @@
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
-  <c:roundedCorners val="1"/>
-  <c:style val="2"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
   <c:chart>
-    <c:autoTitleDeleted val="1"/>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr lvl="0">
+              <a:defRPr b="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="2200"/>
+              <a:t>horizontal bar chart</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
     <c:plotArea>
       <c:layout/>
       <c:barChart>
-        <c:barDir val="col"/>
+        <c:barDir val="bar"/>
         <c:grouping val="clustered"/>
-        <c:varyColors val="1"/>
+        <c:varyColors val="0"/>
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>Sheet1!$B$26</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>first dataset</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="4472C4"/>
+              <a:srgbClr val="7030A0"/>
             </a:solidFill>
-            <a:ln cmpd="sng">
+            <a:ln>
               <a:solidFill>
-                <a:srgbClr val="000000"/>
+                <a:srgbClr val="7030A0"/>
               </a:solidFill>
+              <a:prstDash val="solid"/>
             </a:ln>
           </c:spPr>
           <c:invertIfNegative val="1"/>
@@ -6549,41 +7361,32 @@
                   <a:solidFill>
                     <a:srgbClr val="FFFFFF"/>
                   </a:solidFill>
-                  <a:ln cmpd="sng">
+                  <a:ln>
                     <a:solidFill>
-                      <a:srgbClr val="000000"/>
+                      <a:srgbClr val="7030A0"/>
                     </a:solidFill>
+                    <a:prstDash val="solid"/>
                   </a:ln>
                 </c14:spPr>
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-D94B-45A0-8AD6-3E4F4E7665C2}"/>
+              <c16:uniqueId val="{00000000-2AE2-4EDC-856C-ECBD6B1ECD21}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="1"/>
           <c:order val="1"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>Sheet1!$C$26</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>second dataset</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="ED7D31"/>
+              <a:srgbClr val="C65911"/>
             </a:solidFill>
-            <a:ln cmpd="sng">
+            <a:ln>
               <a:solidFill>
-                <a:srgbClr val="000000"/>
+                <a:srgbClr val="C65911"/>
               </a:solidFill>
+              <a:prstDash val="solid"/>
             </a:ln>
           </c:spPr>
           <c:invertIfNegative val="1"/>
@@ -6665,16 +7468,17 @@
                   <a:solidFill>
                     <a:srgbClr val="FFFFFF"/>
                   </a:solidFill>
-                  <a:ln cmpd="sng">
+                  <a:ln>
                     <a:solidFill>
-                      <a:srgbClr val="000000"/>
+                      <a:srgbClr val="C65911"/>
                     </a:solidFill>
+                    <a:prstDash val="solid"/>
                   </a:ln>
                 </c14:spPr>
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-D94B-45A0-8AD6-3E4F4E7665C2}"/>
+              <c16:uniqueId val="{00000001-2AE2-4EDC-856C-ECBD6B1ECD21}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6686,17 +7490,26 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:gapWidth val="150"/>
-        <c:axId val="998664793"/>
-        <c:axId val="344680958"/>
+        <c:gapWidth val="70"/>
+        <c:axId val="17781237"/>
+        <c:axId val="88853993"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="998664793"/>
+        <c:axId val="17781237"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
-        <c:axPos val="b"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln cmpd="sng">
+              <a:solidFill>
+                <a:srgbClr val="B7B7B7"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
         <c:title>
           <c:tx>
             <c:rich>
@@ -6711,14 +7524,14 @@
                     <a:latin typeface="+mn-lt"/>
                   </a:defRPr>
                 </a:pPr>
-                <a:endParaRPr/>
+                <a:endParaRPr lang="en-US"/>
               </a:p>
             </c:rich>
           </c:tx>
-          <c:overlay val="0"/>
+          <c:overlay val="1"/>
         </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
+        <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:txPr>
@@ -6726,7 +7539,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr lvl="0">
-              <a:defRPr b="0">
+              <a:defRPr sz="1000" b="0" i="0">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
@@ -6736,7 +7549,7 @@
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="344680958"/>
+        <c:crossAx val="88853993"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -6744,32 +7557,21 @@
         <c:noMultiLvlLbl val="1"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="344680958"/>
+        <c:axId val="88853993"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
-        <c:axPos val="l"/>
+        <c:axPos val="b"/>
         <c:majorGridlines>
           <c:spPr>
-            <a:ln>
+            <a:ln cmpd="sng">
               <a:solidFill>
                 <a:srgbClr val="B7B7B7"/>
               </a:solidFill>
             </a:ln>
           </c:spPr>
         </c:majorGridlines>
-        <c:minorGridlines>
-          <c:spPr>
-            <a:ln>
-              <a:solidFill>
-                <a:srgbClr val="CCCCCC">
-                  <a:alpha val="0"/>
-                </a:srgbClr>
-              </a:solidFill>
-            </a:ln>
-          </c:spPr>
-        </c:minorGridlines>
         <c:title>
           <c:tx>
             <c:rich>
@@ -6784,25 +7586,22 @@
                     <a:latin typeface="+mn-lt"/>
                   </a:defRPr>
                 </a:pPr>
-                <a:endParaRPr/>
+                <a:endParaRPr lang="en-US"/>
               </a:p>
             </c:rich>
           </c:tx>
-          <c:overlay val="0"/>
+          <c:overlay val="1"/>
         </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
+        <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:ln/>
-        </c:spPr>
         <c:txPr>
           <a:bodyPr/>
           <a:lstStyle/>
           <a:p>
             <a:pPr lvl="0">
-              <a:defRPr b="0">
+              <a:defRPr sz="1000" b="0" i="0">
                 <a:solidFill>
                   <a:srgbClr val="000000"/>
                 </a:solidFill>
@@ -6812,10 +7611,15 @@
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="998664793"/>
+        <c:crossAx val="17781237"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
+      <c:spPr>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+      </c:spPr>
     </c:plotArea>
     <c:legend>
       <c:legendPos val="r"/>
@@ -6825,9 +7629,9 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr lvl="0">
-            <a:defRPr b="0">
+            <a:defRPr sz="1000" b="0" i="0">
               <a:solidFill>
-                <a:srgbClr val="1A1A1A"/>
+                <a:srgbClr val="000000"/>
               </a:solidFill>
               <a:latin typeface="+mn-lt"/>
             </a:defRPr>
@@ -6840,12 +7644,163 @@
     <c:dispBlanksAs val="zero"/>
     <c:showDLblsOverMax val="1"/>
   </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln cmpd="sng">
+      <a:solidFill>
+        <a:srgbClr val="000000"/>
+      </a:solidFill>
+    </a:ln>
+  </c:spPr>
   <c:printSettings>
     <c:headerFooter/>
     <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
+</file>
+
+<file path=xl/charts/chartEx1.xml><?xml version="1.0" encoding="utf-8"?>
+<cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
+  <cx:chartData>
+    <cx:data id="0">
+      <cx:strDim type="cat">
+        <cx:f>_xlchart.v1.0</cx:f>
+      </cx:strDim>
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.2</cx:f>
+      </cx:numDim>
+    </cx:data>
+  </cx:chartData>
+  <cx:chart>
+    <cx:title pos="t" align="ctr" overlay="0">
+      <cx:tx>
+        <cx:txData>
+          <cx:v>Chart Title</cx:v>
+        </cx:txData>
+      </cx:tx>
+      <cx:txPr>
+        <a:bodyPr vertOverflow="overflow" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr" rtl="0">
+            <a:defRPr sz="1400" b="0" i="0">
+              <a:solidFill>
+                <a:srgbClr val="7F7F7F"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:r>
+            <a:t>Chart Title</a:t>
+          </a:r>
+        </a:p>
+      </cx:txPr>
+    </cx:title>
+    <cx:plotArea>
+      <cx:plotAreaRegion>
+        <cx:series layoutId="waterfall" uniqueId="{5051EC33-743B-4C68-89C0-7179D8BFE55F}">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.1</cx:f>
+              <cx:v>first dataset</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataLabels pos="outEnd">
+            <cx:txPr>
+              <a:bodyPr vertOverflow="overflow" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr algn="ctr" rtl="0">
+                  <a:defRPr sz="1200" b="0" i="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+                    <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+                    <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr/>
+              </a:p>
+            </cx:txPr>
+            <cx:visibility seriesName="0" categoryName="0" value="1"/>
+          </cx:dataLabels>
+          <cx:dataId val="0"/>
+          <cx:layoutPr>
+            <cx:subtotals/>
+          </cx:layoutPr>
+        </cx:series>
+      </cx:plotAreaRegion>
+      <cx:axis id="0">
+        <cx:catScaling gapWidth="0.5"/>
+        <cx:tickLabels/>
+        <cx:txPr>
+          <a:bodyPr vertOverflow="overflow" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr" rtl="0">
+              <a:defRPr sz="1200" b="0" i="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+                <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+                <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr/>
+          </a:p>
+        </cx:txPr>
+      </cx:axis>
+      <cx:axis id="1">
+        <cx:valScaling/>
+        <cx:majorGridlines/>
+        <cx:tickLabels/>
+        <cx:txPr>
+          <a:bodyPr vertOverflow="overflow" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr" rtl="0">
+              <a:defRPr sz="1200" b="0" i="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+                <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+                <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr/>
+          </a:p>
+        </cx:txPr>
+      </cx:axis>
+    </cx:plotArea>
+    <cx:legend pos="t" align="ctr" overlay="0">
+      <cx:txPr>
+        <a:bodyPr vertOverflow="overflow" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr" rtl="0">
+            <a:defRPr sz="1200" b="0" i="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr/>
+        </a:p>
+      </cx:txPr>
+    </cx:legend>
+  </cx:chart>
+</cx:chartSpace>
 </file>
 
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6888,7 +7843,555 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="395">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat">
+        <a:solidFill>
+          <a:srgbClr val="D9D9D9"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="2">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -7324,6 +8827,89 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>657225</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>180975</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>619125</xdr:colOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" Requires="cx1">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="2" name="Chart 1">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CB44F912-9067-8FA7-675B-52C07F194DE5}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2014/chartex">
+              <cx:chart xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr sz="1100"/>
+                <a:t>This chart isn't available in your version of Excel.
+Editing this shape or saving this workbook into a different file format will permanently break the chart.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>76200</xdr:colOff>
       <xdr:row>4</xdr:row>
@@ -7643,10 +9229,92 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>152400</xdr:colOff>
+      <xdr:row>55</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="10" name="Chart 9" title="Chart">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B187E09F-172F-47EE-A6CD-3039B7DE0CE4}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{5D2716A1-A175-44F9-BBD0-26D27F88F15C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>781050</xdr:colOff>
+      <xdr:row>71</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>161925</xdr:colOff>
+      <xdr:row>89</xdr:row>
+      <xdr:rowOff>104775</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="11" name="Chart 10" title="Chart">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{89D5E293-E7D5-4DCE-B066-872C6428DD51}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{B187E09F-172F-47EE-A6CD-3039B7DE0CE4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId10"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
@@ -7694,7 +9362,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor>
     <xdr:from>
@@ -7902,7 +9570,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9B3CE3F5-58D8-48A3-B9C6-24D1506C9F5C}" name="PivotTable1" cacheId="3062" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9B3CE3F5-58D8-48A3-B9C6-24D1506C9F5C}" name="PivotTable1" cacheId="1259" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="C3:L21" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="5">
     <pivotField axis="axisRow" showAll="0">
@@ -8939,6 +10607,7 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+  <drawing r:id="rId3"/>
 </worksheet>
 </file>
 
@@ -11070,7 +12739,7 @@
       </c>
       <c r="B100" s="19">
         <f ca="1">NOW()</f>
-        <v>45736.475918171294</v>
+        <v>45748.695485300923</v>
       </c>
       <c r="D100" s="117">
         <f ca="1">IF(ISNUMBER(B100),1,0)</f>
@@ -11760,7 +13429,7 @@
       </c>
       <c r="B144" s="18">
         <f ca="1">TODAY()</f>
-        <v>45736</v>
+        <v>45748</v>
       </c>
       <c r="D144" s="117">
         <f ca="1">IF(ISNUMBER(B144),1,0)</f>
@@ -12790,7 +14459,7 @@
       </c>
       <c r="B12" s="39">
         <f ca="1">TODAY()</f>
-        <v>45736</v>
+        <v>45748</v>
       </c>
       <c r="C12" s="39">
         <f>DATE(2010,10,2)</f>

</xml_diff>

<commit_message>
[IMP] SheetProtection: introducing the sheet protection
This revisions adds a (naive) protection for the full sheet.
The ability to block specific modifications (style, grid structure, etc)
is not strictly compatible with our collaborative approach as the server
is never aware of the current state of the spreadsheet.

Task: 5103728
</commit_message>
<xml_diff>
--- a/tests/__xlsx__/xlsx_demo_data.xlsx
+++ b/tests/__xlsx__/xlsx_demo_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\odoo\spreadsheet\tests\__xlsx__\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rar/rar-workspace/os2/tests/__xlsx__/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A476F739-B139-4713-A5CB-3C0E11EABA6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6DD048F-3D20-334B-864B-CDAF5F5A5BDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="680" windowWidth="29040" windowHeight="15840" firstSheet="4" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,13 +27,15 @@
     <sheet name="jestImages" sheetId="15" r:id="rId12"/>
     <sheet name="jestOneCellAnchor" sheetId="16" r:id="rId13"/>
     <sheet name="jestDataValidations" sheetId="17" r:id="rId14"/>
+    <sheet name="jestLocked" sheetId="18" r:id="rId15"/>
+    <sheet name="jestPartiallyLocked" sheetId="19" r:id="rId16"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId15"/>
+    <externalReference r:id="rId17"/>
   </externalReferences>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="1" r:id="rId16"/>
+    <pivotCache cacheId="5" r:id="rId18"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -2372,7 +2374,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{1493241F-B85D-4F84-BBA0-86191B8FD032}"/>
   </cellStyles>
-  <dxfs count="71">
+  <dxfs count="47">
     <dxf>
       <font>
         <b val="0"/>
@@ -2584,194 +2586,6 @@
         <outline val="0"/>
         <shadow val="0"/>
         <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
         <sz val="10"/>
         <color rgb="FF000000"/>
         <name val="Arial"/>
@@ -2783,207 +2597,6 @@
           <bgColor theme="9"/>
         </patternFill>
       </fill>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -3344,8 +2957,8 @@
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="Table Style 1" pivot="0" count="2" xr9:uid="{33B8EB55-D8D8-4B00-B5CF-C84A8AC9E775}">
-      <tableStyleElement type="wholeTable" dxfId="70"/>
-      <tableStyleElement type="firstRowStripe" dxfId="69"/>
+      <tableStyleElement type="wholeTable" dxfId="46"/>
+      <tableStyleElement type="firstRowStripe" dxfId="45"/>
     </tableStyle>
   </tableStyles>
   <colors>
@@ -3373,7 +2986,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="en-GB"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -3990,7 +3603,7 @@
 <file path=xl/charts/chart10.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="en-GB"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -4353,7 +3966,7 @@
 <file path=xl/charts/chart11.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="en-GB"/>
   <c:roundedCorners val="1"/>
   <c:style val="2"/>
   <c:chart>
@@ -4769,7 +4382,7 @@
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="en-GB"/>
   <c:roundedCorners val="0"/>
   <c:style val="2"/>
   <c:chart>
@@ -5214,7 +4827,7 @@
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="en-GB"/>
   <c:roundedCorners val="0"/>
   <c:style val="2"/>
   <c:chart>
@@ -5832,7 +5445,7 @@
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="en-GB"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -6198,7 +5811,7 @@
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="en-GB"/>
   <c:roundedCorners val="1"/>
   <c:style val="2"/>
   <c:chart>
@@ -6510,7 +6123,7 @@
 <file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="en-GB"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -6941,7 +6554,7 @@
 <file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="en-GB"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -7343,7 +6956,7 @@
 <file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="en-GB"/>
   <c:roundedCorners val="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -7646,7 +7259,7 @@
 <file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="en-GB"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -9230,7 +8843,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9B3CE3F5-58D8-48A3-B9C6-24D1506C9F5C}" name="PivotTable1" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9B3CE3F5-58D8-48A3-B9C6-24D1506C9F5C}" name="PivotTable1" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="C3:L21" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="5">
     <pivotField axis="axisRow" showAll="0">
@@ -9380,7 +8993,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{09C35CC7-7259-4A97-8FEA-EDB47375DF08}" name="Table3" displayName="Table3" ref="C3:J6" totalsRowCount="1" headerRowDxfId="68" dataDxfId="67">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{09C35CC7-7259-4A97-8FEA-EDB47375DF08}" name="Table3" displayName="Table3" ref="C3:J6" totalsRowCount="1" headerRowDxfId="44" dataDxfId="43">
   <autoFilter ref="C3:J5" xr:uid="{09C35CC7-7259-4A97-8FEA-EDB47375DF08}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -9392,22 +9005,22 @@
     <filterColumn colId="7" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{C4EE018E-238B-42BA-9035-DB01FA5420D3}" name="Name" totalsRowLabel="Total" dataDxfId="66" totalsRowDxfId="65"/>
-    <tableColumn id="2" xr3:uid="{C1F6911F-9482-4C98-BBFB-21D9CAA66DA4}" name="Age" totalsRowFunction="sum" dataDxfId="64" totalsRowDxfId="63"/>
-    <tableColumn id="5" xr3:uid="{3CE9F5DA-0A57-4696-B4E0-53601C3B7798}" name="Rank" totalsRowFunction="sum" dataDxfId="62" totalsRowDxfId="61"/>
-    <tableColumn id="6" xr3:uid="{34912838-665C-4472-B558-25990E5B148D}" name="Rank+Age =E4+D4" totalsRowFunction="sum" dataDxfId="60" totalsRowDxfId="59">
+    <tableColumn id="1" xr3:uid="{C4EE018E-238B-42BA-9035-DB01FA5420D3}" name="Name" totalsRowLabel="Total" dataDxfId="42" totalsRowDxfId="41"/>
+    <tableColumn id="2" xr3:uid="{C1F6911F-9482-4C98-BBFB-21D9CAA66DA4}" name="Age" totalsRowFunction="sum" dataDxfId="40" totalsRowDxfId="39"/>
+    <tableColumn id="5" xr3:uid="{3CE9F5DA-0A57-4696-B4E0-53601C3B7798}" name="Rank" totalsRowFunction="sum" dataDxfId="38" totalsRowDxfId="37"/>
+    <tableColumn id="6" xr3:uid="{34912838-665C-4472-B558-25990E5B148D}" name="Rank+Age =E4+D4" totalsRowFunction="sum" dataDxfId="36" totalsRowDxfId="35">
       <calculatedColumnFormula>Table3[[#This Row],[Rank]]+Table3[[#This Row],[Age]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{89D90022-7073-4067-BAF8-1587D27C4AFB}" name="Data =SUM(E4:E5)" totalsRowFunction="sum" dataDxfId="58" totalsRowDxfId="57">
+    <tableColumn id="7" xr3:uid="{89D90022-7073-4067-BAF8-1587D27C4AFB}" name="Data =SUM(E4:E5)" totalsRowFunction="sum" dataDxfId="34" totalsRowDxfId="33">
       <calculatedColumnFormula>SUM(Table3[Rank])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{B2A7E5BB-A379-492B-9484-72F2FD1FF3A0}" name="All =SUM(E3:E6)" totalsRowFunction="sum" dataDxfId="56" totalsRowDxfId="55">
+    <tableColumn id="8" xr3:uid="{B2A7E5BB-A379-492B-9484-72F2FD1FF3A0}" name="All =SUM(E3:E6)" totalsRowFunction="sum" dataDxfId="32" totalsRowDxfId="31">
       <calculatedColumnFormula>SUM(Table3[[#All],[Rank]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{3C532A69-E4BC-4A20-A922-4BCAA0D3FEC9}" name="Totals =E6" totalsRowFunction="sum" dataDxfId="54" totalsRowDxfId="53">
+    <tableColumn id="9" xr3:uid="{3C532A69-E4BC-4A20-A922-4BCAA0D3FEC9}" name="Totals =E6" totalsRowFunction="sum" dataDxfId="30" totalsRowDxfId="29">
       <calculatedColumnFormula>Table3[[#Totals],[Rank]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{35E9E9C3-9148-468A-85B6-19290CEB6F00}" name="Headers =E3" totalsRowFunction="sum" dataDxfId="52" totalsRowDxfId="51">
+    <tableColumn id="10" xr3:uid="{35E9E9C3-9148-468A-85B6-19290CEB6F00}" name="Headers =E3" totalsRowFunction="sum" dataDxfId="28" totalsRowDxfId="27">
       <calculatedColumnFormula>Table3[[#Headers],[Rank]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -9828,13 +9441,13 @@
     <tabColor rgb="FF00FF00"/>
   </sheetPr>
   <dimension ref="A1:L35"/>
-  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="13.796875" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="22.28515625" customWidth="1"/>
-    <col min="2" max="2" width="13.7109375" customWidth="1"/>
-    <col min="3" max="3" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="14.28515625" customWidth="1"/>
-    <col min="6" max="26" width="13.7109375" customWidth="1"/>
+    <col min="1" max="1" width="22.19921875" customWidth="1"/>
+    <col min="2" max="2" width="13.796875" customWidth="1"/>
+    <col min="3" max="3" width="13.796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="14.19921875" customWidth="1"/>
+    <col min="6" max="26" width="13.796875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -9846,7 +9459,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="27.75" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:12" ht="28" x14ac:dyDescent="0.2">
       <c r="B2" s="22" t="s">
         <v>2</v>
       </c>
@@ -10228,7 +9841,7 @@
     <mergeCell ref="K3:K8"/>
   </mergeCells>
   <conditionalFormatting sqref="C1:C100 B21">
-    <cfRule type="cellIs" dxfId="50" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="26" priority="1" operator="equal">
       <formula>42</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10273,7 +9886,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F7A934C-2218-4A12-8B75-EE28D615D774}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.796875" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -10282,7 +9895,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96301BE1-D86D-4D45-870D-85A75D53FC99}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.3984375" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -10291,10 +9904,10 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B10A8834-0E20-4F80-8813-3ACA5527B377}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="13.796875" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="65.140625" customWidth="1"/>
-    <col min="2" max="26" width="13.7109375" customWidth="1"/>
+    <col min="1" max="1" width="65.19921875" customWidth="1"/>
+    <col min="2" max="26" width="13.796875" customWidth="1"/>
   </cols>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -10308,7 +9921,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="14.3984375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10318,13 +9931,13 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{025F2510-D243-4DA1-81DE-BBDDA9BC3681}">
   <dimension ref="A1:J6"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="4" width="14.28515625" customWidth="1"/>
-    <col min="5" max="5" width="14.7109375" customWidth="1"/>
-    <col min="7" max="7" width="14.28515625" customWidth="1"/>
-    <col min="8" max="8" width="20.28515625" customWidth="1"/>
-    <col min="9" max="9" width="17.28515625" customWidth="1"/>
+    <col min="3" max="4" width="14.19921875" customWidth="1"/>
+    <col min="5" max="5" width="14.796875" customWidth="1"/>
+    <col min="7" max="7" width="14.19921875" customWidth="1"/>
+    <col min="8" max="8" width="20.19921875" customWidth="1"/>
+    <col min="9" max="9" width="17.19921875" customWidth="1"/>
     <col min="10" max="10" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -10562,15 +10175,35 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{827A154B-649F-9248-B45E-D1F5000EB396}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="1" selectUnlockedCells="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75E9A493-0805-C541-B367-D56900C82F13}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0630FA18-71FC-4ACD-8379-39A3603D1DD6}">
   <sheetPr>
     <tabColor theme="9"/>
   </sheetPr>
   <dimension ref="A1:R163"/>
-  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="13.796875" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="26" width="13.7109375" customWidth="1"/>
+    <col min="1" max="26" width="13.796875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -12421,7 +12054,7 @@
       </c>
       <c r="B100" s="19">
         <f ca="1">NOW()</f>
-        <v>45989.427180092593</v>
+        <v>46028.934024074071</v>
       </c>
       <c r="D100" s="104">
         <f ca="1">IF(ISNUMBER(B100),1,0)</f>
@@ -13111,7 +12744,7 @@
       </c>
       <c r="B144" s="18">
         <f ca="1">TODAY()</f>
-        <v>45989</v>
+        <v>46028</v>
       </c>
       <c r="D144" s="104">
         <f ca="1">IF(ISNUMBER(B144),1,0)</f>
@@ -13425,10 +13058,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="D1:D180">
-    <cfRule type="cellIs" dxfId="49" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="25" priority="1" operator="equal">
       <formula>1</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="48" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="24" priority="2" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -13443,14 +13076,14 @@
     <outlinePr summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:R31"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" outlineLevelRow="2" outlineLevelCol="2" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.19921875" defaultRowHeight="14" outlineLevelRow="2" outlineLevelCol="2" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="0" hidden="1" customWidth="1"/>
-    <col min="6" max="6" width="14.28515625" customWidth="1"/>
-    <col min="10" max="10" width="9.140625" outlineLevel="1"/>
-    <col min="11" max="11" width="9.140625" outlineLevel="1" collapsed="1"/>
+    <col min="6" max="6" width="14.19921875" customWidth="1"/>
+    <col min="10" max="10" width="9.19921875" outlineLevel="1"/>
+    <col min="11" max="11" width="9.19921875" outlineLevel="1" collapsed="1"/>
     <col min="12" max="14" width="0" hidden="1" outlineLevel="2"/>
-    <col min="15" max="18" width="9.140625" outlineLevel="1"/>
+    <col min="15" max="18" width="9.19921875" outlineLevel="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
@@ -13513,21 +13146,21 @@
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" cm="1">
         <f t="array" aca="1" ref="A30:B31" ca="1">_xlfn.RANDARRAY(2,2)</f>
-        <v>0.38411710219623751</v>
+        <v>0.69450535790710388</v>
       </c>
       <c r="B30">
         <f ca="1"/>
-        <v>9.794149803384844E-2</v>
+        <v>0.36697595067154309</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31">
         <f ca="1"/>
-        <v>0.66351595791263507</v>
+        <v>5.6962617314857855E-2</v>
       </c>
       <c r="B31">
         <f ca="1"/>
-        <v>5.0911295821026714E-2</v>
+        <v>4.4896354655804327E-2</v>
       </c>
     </row>
   </sheetData>
@@ -13546,14 +13179,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF68F2C0-1053-4FB6-BD74-8A11B0CAF123}">
   <dimension ref="A1:M30"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.19921875" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="17.7109375" customWidth="1"/>
-    <col min="5" max="5" width="18.28515625" customWidth="1"/>
-    <col min="13" max="13" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.796875" customWidth="1"/>
+    <col min="5" max="5" width="18.19921875" customWidth="1"/>
+    <col min="13" max="13" width="10.3984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="68" t="s">
         <v>239</v>
       </c>
@@ -13624,7 +13257,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="15" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" ht="16" x14ac:dyDescent="0.25">
       <c r="A4" s="42" t="s">
         <v>256</v>
       </c>
@@ -13693,7 +13326,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="45" t="s">
         <v>271</v>
       </c>
@@ -13713,7 +13346,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="21" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:13" ht="21" x14ac:dyDescent="0.25">
       <c r="A8" s="46" t="s">
         <v>275</v>
       </c>
@@ -13736,7 +13369,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:13" ht="15" x14ac:dyDescent="0.2">
       <c r="A9" s="47" t="s">
         <v>280</v>
       </c>
@@ -13761,7 +13394,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="49" t="s">
         <v>285</v>
       </c>
@@ -13834,12 +13467,12 @@
         <v>248</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A17" s="55" t="s">
         <v>296</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A18" s="74" t="s">
         <v>297</v>
       </c>
@@ -13851,7 +13484,7 @@
       </c>
       <c r="F18" s="36"/>
     </row>
-    <row r="19" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A19" s="75" t="s">
         <v>300</v>
       </c>
@@ -13862,7 +13495,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="51.75" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" ht="61" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A20" s="76" t="s">
         <v>303</v>
       </c>
@@ -13876,12 +13509,12 @@
         <v>302</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A21" s="77" t="s">
         <v>306</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A22" s="78" t="s">
         <v>307</v>
       </c>
@@ -13890,13 +13523,13 @@
       </c>
       <c r="E22" s="21"/>
     </row>
-    <row r="23" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A23" s="79" t="s">
         <v>309</v>
       </c>
       <c r="E23" s="21"/>
     </row>
-    <row r="24" spans="1:6" ht="14.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" ht="16" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A24" s="80" t="s">
         <v>310</v>
       </c>
@@ -13905,19 +13538,19 @@
       </c>
       <c r="E24" s="21"/>
     </row>
-    <row r="25" spans="1:6" ht="14.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="26" spans="1:6" ht="14.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" ht="16" thickTop="1" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="1:6" ht="16" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="C26" s="67" t="s">
         <v>312</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="14.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="1:6" ht="14.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" ht="16" thickTop="1" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="28" spans="1:6" ht="16" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="C28" s="88" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="13.5" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="29" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.2"/>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="C30" s="87" t="s">
         <v>314</v>
@@ -13932,13 +13565,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D919E811-4385-4D35-A19E-3B7E0E659A89}">
   <dimension ref="A1:L39"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.3984375" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.140625" customWidth="1"/>
-    <col min="7" max="7" width="15.85546875" customWidth="1"/>
+    <col min="1" max="1" width="19.19921875" customWidth="1"/>
+    <col min="7" max="7" width="15.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
         <v>315</v>
       </c>
@@ -14114,7 +13747,7 @@
       </c>
       <c r="C9" s="21"/>
     </row>
-    <row r="10" spans="1:10" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="38" t="s">
         <v>340</v>
       </c>
@@ -14161,7 +13794,7 @@
       </c>
       <c r="B12" s="39">
         <f ca="1">TODAY()</f>
-        <v>45989</v>
+        <v>46028</v>
       </c>
       <c r="C12" s="39">
         <f>DATE(2010,10,2)</f>
@@ -14600,7 +14233,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:12" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="G31" s="35" t="s">
         <v>377</v>
       </c>
@@ -14704,104 +14337,104 @@
   </sheetData>
   <phoneticPr fontId="21" type="noConversion"/>
   <conditionalFormatting sqref="B15">
-    <cfRule type="expression" dxfId="47" priority="59">
+    <cfRule type="expression" dxfId="23" priority="59">
       <formula>ODD(B15)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B26:B27">
-    <cfRule type="cellIs" dxfId="46" priority="47" operator="equal">
+    <cfRule type="cellIs" dxfId="22" priority="47" operator="equal">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B2:C2">
-    <cfRule type="aboveAverage" dxfId="45" priority="115"/>
+    <cfRule type="aboveAverage" dxfId="21" priority="115"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:C3">
-    <cfRule type="beginsWith" dxfId="44" priority="74" operator="beginsWith" text="rule">
+    <cfRule type="beginsWith" dxfId="20" priority="74" operator="beginsWith" text="rule">
       <formula>LEFT(B3,LEN("rule"))="rule"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B4:C4">
-    <cfRule type="containsBlanks" dxfId="43" priority="72">
+    <cfRule type="containsBlanks" dxfId="19" priority="72">
       <formula>LEN(TRIM(B4))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B5:C5">
-    <cfRule type="containsErrors" dxfId="42" priority="71">
+    <cfRule type="containsErrors" dxfId="18" priority="71">
       <formula>ISERROR(B5)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:C6">
-    <cfRule type="containsText" dxfId="41" priority="70" operator="containsText" text="rule">
+    <cfRule type="containsText" dxfId="17" priority="70" operator="containsText" text="rule">
       <formula>NOT(ISERROR(SEARCH("rule",B6)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8:C8">
-    <cfRule type="endsWith" dxfId="40" priority="68" operator="endsWith" text="rule">
+    <cfRule type="endsWith" dxfId="16" priority="68" operator="endsWith" text="rule">
       <formula>RIGHT(B8,LEN("rule"))="rule"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B9:C9">
-    <cfRule type="notContainsBlanks" dxfId="39" priority="67">
+    <cfRule type="notContainsBlanks" dxfId="15" priority="67">
       <formula>LEN(TRIM(B9))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B10:C10">
-    <cfRule type="notContainsErrors" dxfId="38" priority="66">
+    <cfRule type="notContainsErrors" dxfId="14" priority="66">
       <formula>NOT(ISERROR(B10))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B11:C11">
-    <cfRule type="notContainsText" dxfId="37" priority="65" operator="notContains" text="rule">
+    <cfRule type="notContainsText" dxfId="13" priority="65" operator="notContains" text="rule">
       <formula>ISERROR(SEARCH("rule",B11))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12:C12">
-    <cfRule type="timePeriod" dxfId="36" priority="64" timePeriod="today">
+    <cfRule type="timePeriod" dxfId="12" priority="64" timePeriod="today">
       <formula>FLOOR(B12,1)=TODAY()</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B13:C13">
-    <cfRule type="top10" dxfId="24" priority="116" percent="1" bottom="1" rank="50"/>
+    <cfRule type="top10" dxfId="11" priority="116" percent="1" bottom="1" rank="50"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B16:C16">
-    <cfRule type="cellIs" dxfId="35" priority="46" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="46" operator="equal">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B17:C17">
-    <cfRule type="cellIs" dxfId="34" priority="57" operator="notEqual">
+    <cfRule type="cellIs" dxfId="9" priority="57" operator="notEqual">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B18:C18">
-    <cfRule type="cellIs" dxfId="33" priority="7" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="8" priority="7" operator="greaterThan">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B19:C19">
-    <cfRule type="cellIs" dxfId="32" priority="6" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="7" priority="6" operator="greaterThanOrEqual">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B20:C20">
-    <cfRule type="cellIs" dxfId="31" priority="5" operator="lessThan">
+    <cfRule type="cellIs" dxfId="6" priority="5" operator="lessThan">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B21:C21">
-    <cfRule type="cellIs" dxfId="30" priority="4" operator="lessThanOrEqual">
+    <cfRule type="cellIs" dxfId="5" priority="4" operator="lessThanOrEqual">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B22:C22">
-    <cfRule type="cellIs" dxfId="29" priority="3" operator="between">
+    <cfRule type="cellIs" dxfId="4" priority="3" operator="between">
       <formula>2</formula>
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B23:C23">
-    <cfRule type="cellIs" dxfId="28" priority="2" operator="notBetween">
+    <cfRule type="cellIs" dxfId="3" priority="2" operator="notBetween">
       <formula>2</formula>
       <formula>4</formula>
     </cfRule>
@@ -14835,16 +14468,16 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B29:C29">
-    <cfRule type="cellIs" dxfId="27" priority="1" operator="between">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="between">
       <formula>$B$23</formula>
       <formula>2+2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7:D7">
-    <cfRule type="duplicateValues" dxfId="26" priority="83"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="83"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B14:D14">
-    <cfRule type="uniqueValues" dxfId="25" priority="97"/>
+    <cfRule type="uniqueValues" dxfId="0" priority="97"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:J2">
     <cfRule type="colorScale" priority="45">
@@ -15267,16 +14900,16 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5CCC4B1-5C65-4837-AA26-56CCF06B63BB}">
   <dimension ref="A1:J34"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.19921875" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="17.28515625" customWidth="1"/>
-    <col min="4" max="4" width="9.5703125" customWidth="1"/>
-    <col min="5" max="5" width="26.42578125" customWidth="1"/>
-    <col min="6" max="6" width="27.5703125" customWidth="1"/>
-    <col min="7" max="7" width="23.5703125" customWidth="1"/>
-    <col min="8" max="8" width="16.28515625" customWidth="1"/>
-    <col min="9" max="9" width="18.85546875" customWidth="1"/>
-    <col min="10" max="10" width="17.28515625" customWidth="1"/>
+    <col min="3" max="3" width="17.19921875" customWidth="1"/>
+    <col min="4" max="4" width="9.59765625" customWidth="1"/>
+    <col min="5" max="5" width="26.3984375" customWidth="1"/>
+    <col min="6" max="6" width="27.59765625" customWidth="1"/>
+    <col min="7" max="7" width="23.59765625" customWidth="1"/>
+    <col min="8" max="8" width="16.19921875" customWidth="1"/>
+    <col min="9" max="9" width="18.796875" customWidth="1"/>
+    <col min="10" max="10" width="17.19921875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
@@ -15284,7 +14917,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="C3" s="17" t="s">
         <v>35</v>
       </c>
@@ -15634,28 +15267,28 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE9224F2-4D06-4586-886C-E51F5EBCA7B0}">
   <dimension ref="A1:L21"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.19921875" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.19921875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.59765625" bestFit="1" customWidth="1"/>
     <col min="5" max="6" width="6" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="7" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="5" bestFit="1" customWidth="1"/>
     <col min="9" max="10" width="7" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="6" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="10" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.796875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.796875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.796875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.796875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="14.796875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.796875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="14.796875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="14.19921875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="19.19921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" s="92" t="s">
         <v>412</v>
       </c>
@@ -15946,10 +15579,10 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C47BF70-BA80-4124-B359-67CBCB635390}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="13.796875" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="65.140625" customWidth="1"/>
-    <col min="2" max="26" width="13.7109375" customWidth="1"/>
+    <col min="1" max="1" width="65.19921875" customWidth="1"/>
+    <col min="2" max="26" width="13.796875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
@@ -15982,9 +15615,9 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FE31E21-0350-44E7-AF13-4CA140505B30}">
   <dimension ref="A1:B12"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.796875" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:2" ht="51" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" ht="60" x14ac:dyDescent="0.2">
       <c r="A1" s="99" t="s">
         <v>421</v>
       </c>

</xml_diff>

<commit_message>
[IMP] cf: add top10 conditional formatting operator
This commits adds the "top10" conditional formatting operator, which
highlights the top or bottom N values in a selected range.

Task: 5367065
</commit_message>
<xml_diff>
--- a/tests/__xlsx__/xlsx_demo_data.xlsx
+++ b/tests/__xlsx__/xlsx_demo_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Odoo\spreadsheet\tests\__xlsx__\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\odoo\spreadsheet\tests\__xlsx__\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F832354-F3E9-4BC5-A260-88E8A391D52D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A476F739-B139-4713-A5CB-3C0E11EABA6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="4" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
   </externalReferences>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId16"/>
+    <pivotCache cacheId="1" r:id="rId16"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -1563,6 +1563,7 @@
       <sz val="10"/>
       <color theme="10"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1581,6 +1582,7 @@
       <sz val="10"/>
       <color theme="0"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="29">
@@ -2151,7 +2153,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="118">
+  <cellXfs count="116">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -2335,6 +2337,19 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="28" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="28" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="28" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -2351,28 +2366,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="28" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="28" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="28" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{1493241F-B85D-4F84-BBA0-86191B8FD032}"/>
   </cellStyles>
-  <dxfs count="47">
+  <dxfs count="71">
     <dxf>
       <font>
         <b val="0"/>
@@ -2553,6 +2553,399 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -2951,8 +3344,8 @@
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="Table Style 1" pivot="0" count="2" xr9:uid="{33B8EB55-D8D8-4B00-B5CF-C84A8AC9E775}">
-      <tableStyleElement type="wholeTable" dxfId="46"/>
-      <tableStyleElement type="firstRowStripe" dxfId="45"/>
+      <tableStyleElement type="wholeTable" dxfId="70"/>
+      <tableStyleElement type="firstRowStripe" dxfId="69"/>
     </tableStyle>
   </tableStyles>
   <colors>
@@ -8837,7 +9230,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9B3CE3F5-58D8-48A3-B9C6-24D1506C9F5C}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9B3CE3F5-58D8-48A3-B9C6-24D1506C9F5C}" name="PivotTable1" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="C3:L21" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="5">
     <pivotField axis="axisRow" showAll="0">
@@ -8987,7 +9380,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{09C35CC7-7259-4A97-8FEA-EDB47375DF08}" name="Table3" displayName="Table3" ref="C3:J6" totalsRowCount="1" headerRowDxfId="44" dataDxfId="43">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{09C35CC7-7259-4A97-8FEA-EDB47375DF08}" name="Table3" displayName="Table3" ref="C3:J6" totalsRowCount="1" headerRowDxfId="68" dataDxfId="67">
   <autoFilter ref="C3:J5" xr:uid="{09C35CC7-7259-4A97-8FEA-EDB47375DF08}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -8999,22 +9392,22 @@
     <filterColumn colId="7" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{C4EE018E-238B-42BA-9035-DB01FA5420D3}" name="Name" totalsRowLabel="Total" dataDxfId="42" totalsRowDxfId="41"/>
-    <tableColumn id="2" xr3:uid="{C1F6911F-9482-4C98-BBFB-21D9CAA66DA4}" name="Age" totalsRowFunction="sum" dataDxfId="40" totalsRowDxfId="39"/>
-    <tableColumn id="5" xr3:uid="{3CE9F5DA-0A57-4696-B4E0-53601C3B7798}" name="Rank" totalsRowFunction="sum" dataDxfId="38" totalsRowDxfId="37"/>
-    <tableColumn id="6" xr3:uid="{34912838-665C-4472-B558-25990E5B148D}" name="Rank+Age =E4+D4" totalsRowFunction="sum" dataDxfId="36" totalsRowDxfId="35">
+    <tableColumn id="1" xr3:uid="{C4EE018E-238B-42BA-9035-DB01FA5420D3}" name="Name" totalsRowLabel="Total" dataDxfId="66" totalsRowDxfId="65"/>
+    <tableColumn id="2" xr3:uid="{C1F6911F-9482-4C98-BBFB-21D9CAA66DA4}" name="Age" totalsRowFunction="sum" dataDxfId="64" totalsRowDxfId="63"/>
+    <tableColumn id="5" xr3:uid="{3CE9F5DA-0A57-4696-B4E0-53601C3B7798}" name="Rank" totalsRowFunction="sum" dataDxfId="62" totalsRowDxfId="61"/>
+    <tableColumn id="6" xr3:uid="{34912838-665C-4472-B558-25990E5B148D}" name="Rank+Age =E4+D4" totalsRowFunction="sum" dataDxfId="60" totalsRowDxfId="59">
       <calculatedColumnFormula>Table3[[#This Row],[Rank]]+Table3[[#This Row],[Age]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{89D90022-7073-4067-BAF8-1587D27C4AFB}" name="Data =SUM(E4:E5)" totalsRowFunction="sum" dataDxfId="34" totalsRowDxfId="33">
+    <tableColumn id="7" xr3:uid="{89D90022-7073-4067-BAF8-1587D27C4AFB}" name="Data =SUM(E4:E5)" totalsRowFunction="sum" dataDxfId="58" totalsRowDxfId="57">
       <calculatedColumnFormula>SUM(Table3[Rank])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{B2A7E5BB-A379-492B-9484-72F2FD1FF3A0}" name="All =SUM(E3:E6)" totalsRowFunction="sum" dataDxfId="32" totalsRowDxfId="31">
+    <tableColumn id="8" xr3:uid="{B2A7E5BB-A379-492B-9484-72F2FD1FF3A0}" name="All =SUM(E3:E6)" totalsRowFunction="sum" dataDxfId="56" totalsRowDxfId="55">
       <calculatedColumnFormula>SUM(Table3[[#All],[Rank]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{3C532A69-E4BC-4A20-A922-4BCAA0D3FEC9}" name="Totals =E6" totalsRowFunction="sum" dataDxfId="30" totalsRowDxfId="29">
+    <tableColumn id="9" xr3:uid="{3C532A69-E4BC-4A20-A922-4BCAA0D3FEC9}" name="Totals =E6" totalsRowFunction="sum" dataDxfId="54" totalsRowDxfId="53">
       <calculatedColumnFormula>Table3[[#Totals],[Rank]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{35E9E9C3-9148-468A-85B6-19290CEB6F00}" name="Headers =E3" totalsRowFunction="sum" dataDxfId="28" totalsRowDxfId="27">
+    <tableColumn id="10" xr3:uid="{35E9E9C3-9148-468A-85B6-19290CEB6F00}" name="Headers =E3" totalsRowFunction="sum" dataDxfId="52" totalsRowDxfId="51">
       <calculatedColumnFormula>Table3[[#Headers],[Rank]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -9463,10 +9856,10 @@
       <c r="G2" s="104">
         <v>5</v>
       </c>
-      <c r="H2" s="105" t="s">
+      <c r="H2" s="110" t="s">
         <v>4</v>
       </c>
-      <c r="I2" s="106"/>
+      <c r="I2" s="111"/>
       <c r="K2" s="3"/>
     </row>
     <row r="3" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -9476,10 +9869,10 @@
       <c r="G3" s="104">
         <v>8</v>
       </c>
-      <c r="H3" s="106"/>
-      <c r="I3" s="106"/>
+      <c r="H3" s="111"/>
+      <c r="I3" s="111"/>
       <c r="J3" s="5"/>
-      <c r="K3" s="107">
+      <c r="K3" s="112">
         <v>5</v>
       </c>
       <c r="L3" s="6"/>
@@ -9497,10 +9890,10 @@
       <c r="G4" s="104">
         <v>9</v>
       </c>
-      <c r="H4" s="106"/>
-      <c r="I4" s="106"/>
+      <c r="H4" s="111"/>
+      <c r="I4" s="111"/>
       <c r="J4" s="5"/>
-      <c r="K4" s="108"/>
+      <c r="K4" s="113"/>
       <c r="L4" s="6"/>
     </row>
     <row r="5" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -9510,10 +9903,10 @@
       <c r="G5" s="104">
         <v>15</v>
       </c>
-      <c r="H5" s="106"/>
-      <c r="I5" s="106"/>
+      <c r="H5" s="111"/>
+      <c r="I5" s="111"/>
       <c r="J5" s="5"/>
-      <c r="K5" s="108"/>
+      <c r="K5" s="113"/>
       <c r="L5" s="6"/>
     </row>
     <row r="6" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -9521,7 +9914,7 @@
         <v>22</v>
       </c>
       <c r="J6" s="5"/>
-      <c r="K6" s="108"/>
+      <c r="K6" s="113"/>
       <c r="L6" s="6"/>
     </row>
     <row r="7" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -9529,7 +9922,7 @@
         <v>3</v>
       </c>
       <c r="J7" s="5"/>
-      <c r="K7" s="108"/>
+      <c r="K7" s="113"/>
       <c r="L7" s="6"/>
     </row>
     <row r="8" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -9537,7 +9930,7 @@
         <v>30</v>
       </c>
       <c r="J8" s="5"/>
-      <c r="K8" s="109"/>
+      <c r="K8" s="114"/>
       <c r="L8" s="6"/>
     </row>
     <row r="9" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -9835,7 +10228,7 @@
     <mergeCell ref="K3:K8"/>
   </mergeCells>
   <conditionalFormatting sqref="C1:C100 B21">
-    <cfRule type="cellIs" dxfId="26" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="50" priority="1" operator="equal">
       <formula>42</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9936,63 +10329,63 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A1" s="112" t="s">
+      <c r="A1" s="106" t="s">
         <v>423</v>
       </c>
-      <c r="B1" s="113" t="s">
+      <c r="B1" s="107" t="s">
         <v>424</v>
       </c>
-      <c r="C1" s="113" t="s">
+      <c r="C1" s="107" t="s">
         <v>425</v>
       </c>
-      <c r="D1" s="113" t="s">
+      <c r="D1" s="107" t="s">
         <v>426</v>
       </c>
-      <c r="E1" s="113" t="s">
+      <c r="E1" s="107" t="s">
         <v>427</v>
       </c>
-      <c r="F1" s="113" t="s">
+      <c r="F1" s="107" t="s">
         <v>428</v>
       </c>
-      <c r="G1" s="113" t="s">
+      <c r="G1" s="107" t="s">
         <v>429</v>
       </c>
-      <c r="H1" s="113" t="s">
+      <c r="H1" s="107" t="s">
         <v>430</v>
       </c>
-      <c r="I1" s="114" t="s">
+      <c r="I1" s="108" t="s">
         <v>431</v>
       </c>
-      <c r="J1" s="111" t="s">
+      <c r="J1" s="105" t="s">
         <v>441</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" s="115">
+      <c r="A2">
         <v>4</v>
       </c>
-      <c r="B2" s="115">
+      <c r="B2">
         <v>99.5</v>
       </c>
-      <c r="C2" s="115">
-        <v>1</v>
-      </c>
-      <c r="D2" s="115" t="s">
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
         <v>432</v>
       </c>
-      <c r="E2" s="116">
+      <c r="E2" s="39">
         <v>45575</v>
       </c>
-      <c r="F2" s="117">
+      <c r="F2" s="109">
         <v>0.64583333333333337</v>
       </c>
-      <c r="G2" s="117" t="s">
+      <c r="G2" s="109" t="s">
         <v>433</v>
       </c>
-      <c r="H2" s="116">
+      <c r="H2" s="39">
         <v>45292</v>
       </c>
-      <c r="I2" s="115">
+      <c r="I2">
         <v>4</v>
       </c>
       <c r="J2">
@@ -10000,31 +10393,31 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" s="115">
+      <c r="A3">
         <v>3</v>
       </c>
-      <c r="B3" s="115">
+      <c r="B3">
         <v>40</v>
       </c>
-      <c r="C3" s="115">
+      <c r="C3">
         <v>2</v>
       </c>
-      <c r="D3" s="115" t="s">
+      <c r="D3" t="s">
         <v>434</v>
       </c>
-      <c r="E3" s="116">
+      <c r="E3" s="39">
         <v>45576</v>
       </c>
-      <c r="F3" s="117">
+      <c r="F3" s="109">
         <v>0.57638888888888884</v>
       </c>
-      <c r="G3" s="117" t="s">
+      <c r="G3" s="109" t="s">
         <v>435</v>
       </c>
-      <c r="H3" s="116">
+      <c r="H3" s="39">
         <v>45231</v>
       </c>
-      <c r="I3" s="115" t="s">
+      <c r="I3" t="s">
         <v>433</v>
       </c>
       <c r="J3">
@@ -10032,31 +10425,31 @@
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="115">
+      <c r="A4">
         <v>9</v>
       </c>
-      <c r="B4" s="115">
+      <c r="B4">
         <v>0</v>
       </c>
-      <c r="C4" s="115">
+      <c r="C4">
         <v>3</v>
       </c>
-      <c r="D4" s="115" t="s">
+      <c r="D4" t="s">
         <v>436</v>
       </c>
-      <c r="E4" s="116">
+      <c r="E4" s="39">
         <v>45574</v>
       </c>
-      <c r="F4" s="117">
+      <c r="F4" s="109">
         <v>0.73958333333333337</v>
       </c>
-      <c r="G4" s="117" t="s">
+      <c r="G4" s="109" t="s">
         <v>437</v>
       </c>
-      <c r="H4" s="116">
+      <c r="H4" s="39">
         <v>45325</v>
       </c>
-      <c r="I4" s="115">
+      <c r="I4">
         <v>3</v>
       </c>
       <c r="J4">
@@ -10064,31 +10457,31 @@
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" s="115">
+      <c r="A5">
         <v>5</v>
       </c>
-      <c r="B5" s="115">
+      <c r="B5">
         <v>120</v>
       </c>
-      <c r="C5" s="115">
+      <c r="C5">
         <v>4</v>
       </c>
-      <c r="D5" s="115" t="s">
+      <c r="D5" t="s">
         <v>434</v>
       </c>
-      <c r="E5" s="116">
+      <c r="E5" s="39">
         <v>45573</v>
       </c>
-      <c r="F5" s="117">
+      <c r="F5" s="109">
         <v>0.66666666666666663</v>
       </c>
-      <c r="G5" s="115" t="s">
+      <c r="G5" t="s">
         <v>438</v>
       </c>
-      <c r="H5" s="116">
+      <c r="H5" s="39">
         <v>45084</v>
       </c>
-      <c r="I5" s="115">
+      <c r="I5">
         <v>3</v>
       </c>
       <c r="J5">
@@ -10096,31 +10489,31 @@
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" s="115">
+      <c r="A6">
         <v>7</v>
       </c>
-      <c r="B6" s="115">
+      <c r="B6">
         <v>12</v>
       </c>
-      <c r="C6" s="115">
+      <c r="C6">
         <v>5</v>
       </c>
-      <c r="D6" s="115" t="s">
+      <c r="D6" t="s">
         <v>436</v>
       </c>
-      <c r="E6" s="116">
+      <c r="E6" s="39">
         <v>45566</v>
       </c>
-      <c r="F6" s="117">
+      <c r="F6" s="109">
         <v>0.5229166666666667</v>
       </c>
-      <c r="G6" s="115" t="s">
+      <c r="G6" t="s">
         <v>439</v>
       </c>
-      <c r="H6" s="116">
+      <c r="H6" s="39">
         <v>45420</v>
       </c>
-      <c r="I6" s="115" t="s">
+      <c r="I6" t="s">
         <v>438</v>
       </c>
       <c r="J6">
@@ -12028,7 +12421,7 @@
       </c>
       <c r="B100" s="19">
         <f ca="1">NOW()</f>
-        <v>45938.493500231481</v>
+        <v>45989.427180092593</v>
       </c>
       <c r="D100" s="104">
         <f ca="1">IF(ISNUMBER(B100),1,0)</f>
@@ -12718,7 +13111,7 @@
       </c>
       <c r="B144" s="18">
         <f ca="1">TODAY()</f>
-        <v>45938</v>
+        <v>45989</v>
       </c>
       <c r="D144" s="104">
         <f ca="1">IF(ISNUMBER(B144),1,0)</f>
@@ -13032,10 +13425,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="D1:D180">
-    <cfRule type="cellIs" dxfId="25" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="49" priority="1" operator="equal">
       <formula>1</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="48" priority="2" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -13067,10 +13460,10 @@
       <c r="C1" t="s">
         <v>231</v>
       </c>
-      <c r="D1" s="110" t="s">
+      <c r="D1" s="115" t="s">
         <v>232</v>
       </c>
-      <c r="E1" s="110"/>
+      <c r="E1" s="115"/>
       <c r="F1" t="s">
         <v>233</v>
       </c>
@@ -13083,8 +13476,8 @@
         <f>SUM(A1)</f>
         <v>0</v>
       </c>
-      <c r="D2" s="110"/>
-      <c r="E2" s="110"/>
+      <c r="D2" s="115"/>
+      <c r="E2" s="115"/>
       <c r="H2" t="str">
         <f>[1]Feuil1!$A$1</f>
         <v>referenced string</v>
@@ -13120,21 +13513,21 @@
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" cm="1">
         <f t="array" aca="1" ref="A30:B31" ca="1">_xlfn.RANDARRAY(2,2)</f>
-        <v>0.7272925709748963</v>
+        <v>0.38411710219623751</v>
       </c>
       <c r="B30">
         <f ca="1"/>
-        <v>0.95782684877879687</v>
+        <v>9.794149803384844E-2</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31">
         <f ca="1"/>
-        <v>0.31704384406036645</v>
+        <v>0.66351595791263507</v>
       </c>
       <c r="B31">
         <f ca="1"/>
-        <v>8.7112099778747121E-2</v>
+        <v>5.0911295821026714E-2</v>
       </c>
     </row>
   </sheetData>
@@ -13768,7 +14161,7 @@
       </c>
       <c r="B12" s="39">
         <f ca="1">TODAY()</f>
-        <v>45938</v>
+        <v>45989</v>
       </c>
       <c r="C12" s="39">
         <f>DATE(2010,10,2)</f>
@@ -14311,104 +14704,104 @@
   </sheetData>
   <phoneticPr fontId="21" type="noConversion"/>
   <conditionalFormatting sqref="B15">
-    <cfRule type="expression" dxfId="23" priority="59">
+    <cfRule type="expression" dxfId="47" priority="59">
       <formula>ODD(B15)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B26:B27">
-    <cfRule type="cellIs" dxfId="22" priority="47" operator="equal">
+    <cfRule type="cellIs" dxfId="46" priority="47" operator="equal">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B2:C2">
-    <cfRule type="aboveAverage" dxfId="21" priority="115"/>
+    <cfRule type="aboveAverage" dxfId="45" priority="115"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:C3">
-    <cfRule type="beginsWith" dxfId="20" priority="74" operator="beginsWith" text="rule">
+    <cfRule type="beginsWith" dxfId="44" priority="74" operator="beginsWith" text="rule">
       <formula>LEFT(B3,LEN("rule"))="rule"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B4:C4">
-    <cfRule type="containsBlanks" dxfId="19" priority="72">
+    <cfRule type="containsBlanks" dxfId="43" priority="72">
       <formula>LEN(TRIM(B4))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B5:C5">
-    <cfRule type="containsErrors" dxfId="18" priority="71">
+    <cfRule type="containsErrors" dxfId="42" priority="71">
       <formula>ISERROR(B5)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:C6">
-    <cfRule type="containsText" dxfId="17" priority="70" operator="containsText" text="rule">
+    <cfRule type="containsText" dxfId="41" priority="70" operator="containsText" text="rule">
       <formula>NOT(ISERROR(SEARCH("rule",B6)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8:C8">
-    <cfRule type="endsWith" dxfId="16" priority="68" operator="endsWith" text="rule">
+    <cfRule type="endsWith" dxfId="40" priority="68" operator="endsWith" text="rule">
       <formula>RIGHT(B8,LEN("rule"))="rule"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B9:C9">
-    <cfRule type="notContainsBlanks" dxfId="15" priority="67">
+    <cfRule type="notContainsBlanks" dxfId="39" priority="67">
       <formula>LEN(TRIM(B9))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B10:C10">
-    <cfRule type="notContainsErrors" dxfId="14" priority="66">
+    <cfRule type="notContainsErrors" dxfId="38" priority="66">
       <formula>NOT(ISERROR(B10))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B11:C11">
-    <cfRule type="notContainsText" dxfId="13" priority="65" operator="notContains" text="rule">
+    <cfRule type="notContainsText" dxfId="37" priority="65" operator="notContains" text="rule">
       <formula>ISERROR(SEARCH("rule",B11))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12:C12">
-    <cfRule type="timePeriod" dxfId="12" priority="64" timePeriod="today">
+    <cfRule type="timePeriod" dxfId="36" priority="64" timePeriod="today">
       <formula>FLOOR(B12,1)=TODAY()</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B13:C13">
-    <cfRule type="top10" dxfId="11" priority="116" rank="1"/>
+    <cfRule type="top10" dxfId="24" priority="116" percent="1" bottom="1" rank="50"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B16:C16">
-    <cfRule type="cellIs" dxfId="10" priority="46" operator="equal">
+    <cfRule type="cellIs" dxfId="35" priority="46" operator="equal">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B17:C17">
-    <cfRule type="cellIs" dxfId="9" priority="57" operator="notEqual">
+    <cfRule type="cellIs" dxfId="34" priority="57" operator="notEqual">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B18:C18">
-    <cfRule type="cellIs" dxfId="8" priority="7" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="33" priority="7" operator="greaterThan">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B19:C19">
-    <cfRule type="cellIs" dxfId="7" priority="6" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="32" priority="6" operator="greaterThanOrEqual">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B20:C20">
-    <cfRule type="cellIs" dxfId="6" priority="5" operator="lessThan">
+    <cfRule type="cellIs" dxfId="31" priority="5" operator="lessThan">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B21:C21">
-    <cfRule type="cellIs" dxfId="5" priority="4" operator="lessThanOrEqual">
+    <cfRule type="cellIs" dxfId="30" priority="4" operator="lessThanOrEqual">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B22:C22">
-    <cfRule type="cellIs" dxfId="4" priority="3" operator="between">
+    <cfRule type="cellIs" dxfId="29" priority="3" operator="between">
       <formula>2</formula>
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B23:C23">
-    <cfRule type="cellIs" dxfId="3" priority="2" operator="notBetween">
+    <cfRule type="cellIs" dxfId="28" priority="2" operator="notBetween">
       <formula>2</formula>
       <formula>4</formula>
     </cfRule>
@@ -14442,16 +14835,16 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B29:C29">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="between">
+    <cfRule type="cellIs" dxfId="27" priority="1" operator="between">
       <formula>$B$23</formula>
       <formula>2+2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7:D7">
-    <cfRule type="duplicateValues" dxfId="1" priority="83"/>
+    <cfRule type="duplicateValues" dxfId="26" priority="83"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B14:D14">
-    <cfRule type="uniqueValues" dxfId="0" priority="97"/>
+    <cfRule type="uniqueValues" dxfId="25" priority="97"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:J2">
     <cfRule type="colorScale" priority="45">

</xml_diff>

<commit_message>
[IMP] charts: showValues is now exported in Excel
We can setup each chart dataset and add the value as a label, this option can now be exported and imported from excel.

Task: 5213598
</commit_message>
<xml_diff>
--- a/tests/__xlsx__/xlsx_demo_data.xlsx
+++ b/tests/__xlsx__/xlsx_demo_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Odoo\spreadsheet\tests\__xlsx__\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F832354-F3E9-4BC5-A260-88E8A391D52D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2566513C-8E6E-494F-AFB8-1020D2EDD842}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="4" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="13" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -31,9 +31,9 @@
   <externalReferences>
     <externalReference r:id="rId15"/>
   </externalReferences>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028" calcCompleted="0"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId16"/>
+    <pivotCache cacheId="9922" r:id="rId16"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -1204,6 +1204,9 @@
     <t>5Rating</t>
   </si>
   <si>
+    <t>CF with formulas</t>
+  </si>
+  <si>
     <t>5Quarters</t>
   </si>
   <si>
@@ -1376,6 +1379,9 @@
     <t>Custom Formula</t>
   </si>
   <si>
+    <t>Decimal with formula</t>
+  </si>
+  <si>
     <t>option1</t>
   </si>
   <si>
@@ -1398,12 +1404,6 @@
   </si>
   <si>
     <t>A1234556</t>
-  </si>
-  <si>
-    <t>CF with formulas</t>
-  </si>
-  <si>
-    <t>Decimal with formula</t>
   </si>
 </sst>
 </file>
@@ -1418,7 +1418,7 @@
     <numFmt numFmtId="168" formatCode="#,##0&quot; EUR €&quot;"/>
     <numFmt numFmtId="169" formatCode="&quot;€&quot;#,##0.00\ &quot;€&quot;"/>
   </numFmts>
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="26">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -2151,7 +2151,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="118">
+  <cellXfs count="116">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -2335,10 +2335,22 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="28" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="28" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="28" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -2351,28 +2363,165 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="28" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="28" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="28" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="3">
-    <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
+    <cellStyle name="Lien hypertexte" xfId="2" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{1493241F-B85D-4F84-BBA0-86191B8FD032}"/>
   </cellStyles>
   <dxfs count="47">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+        <strike/>
+        <u/>
+        <color theme="7"/>
+      </font>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <fill>
+        <patternFill patternType="lightTrellis">
+          <fgColor theme="4"/>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE06666"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFB6D7A8"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -2786,157 +2935,6 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-        <strike/>
-        <u/>
-        <color theme="7"/>
-      </font>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <fill>
-        <patternFill patternType="lightTrellis">
-          <fgColor theme="4"/>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE06666"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFB6D7A8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor theme="4"/>
         </patternFill>
       </fill>
@@ -2980,7 +2978,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="fr-FR"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -3597,7 +3595,7 @@
 <file path=xl/charts/chart10.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="fr-FR"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -3960,7 +3958,7 @@
 <file path=xl/charts/chart11.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="fr-FR"/>
   <c:roundedCorners val="1"/>
   <c:style val="2"/>
   <c:chart>
@@ -4376,7 +4374,7 @@
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="fr-FR"/>
   <c:roundedCorners val="0"/>
   <c:style val="2"/>
   <c:chart>
@@ -4425,6 +4423,27 @@
             </a:ln>
           </c:spPr>
           <c:invertIfNegative val="1"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
           <c:trendline>
             <c:spPr>
               <a:ln>
@@ -4821,7 +4840,7 @@
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="fr-FR"/>
   <c:roundedCorners val="0"/>
   <c:style val="2"/>
   <c:chart>
@@ -5439,7 +5458,7 @@
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="fr-FR"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -5805,7 +5824,7 @@
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="fr-FR"/>
   <c:roundedCorners val="1"/>
   <c:style val="2"/>
   <c:chart>
@@ -6117,7 +6136,7 @@
 <file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="fr-FR"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -6548,7 +6567,7 @@
 <file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="fr-FR"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -6950,7 +6969,7 @@
 <file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="fr-FR"/>
   <c:roundedCorners val="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -7253,7 +7272,7 @@
 <file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="fr-FR"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -7309,6 +7328,27 @@
             </a:ln>
           </c:spPr>
           <c:invertIfNegative val="1"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
           <c:trendline>
             <c:spPr>
               <a:ln>
@@ -7429,6 +7469,27 @@
             </a:ln>
           </c:spPr>
           <c:invertIfNegative val="1"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
           <c:cat>
             <c:strRef>
               <c:f>Sheet1!$A$27:$A$35</c:f>
@@ -8837,7 +8898,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9B3CE3F5-58D8-48A3-B9C6-24D1506C9F5C}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9B3CE3F5-58D8-48A3-B9C6-24D1506C9F5C}" name="PivotTable1" cacheId="9922" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="C3:L21" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="5">
     <pivotField axis="axisRow" showAll="0">
@@ -8987,7 +9048,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{09C35CC7-7259-4A97-8FEA-EDB47375DF08}" name="Table3" displayName="Table3" ref="C3:J6" totalsRowCount="1" headerRowDxfId="44" dataDxfId="43">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{09C35CC7-7259-4A97-8FEA-EDB47375DF08}" name="Table3" displayName="Table3" ref="C3:J6" totalsRowCount="1" headerRowDxfId="17" dataDxfId="16">
   <autoFilter ref="C3:J5" xr:uid="{09C35CC7-7259-4A97-8FEA-EDB47375DF08}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -8999,22 +9060,22 @@
     <filterColumn colId="7" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{C4EE018E-238B-42BA-9035-DB01FA5420D3}" name="Name" totalsRowLabel="Total" dataDxfId="42" totalsRowDxfId="41"/>
-    <tableColumn id="2" xr3:uid="{C1F6911F-9482-4C98-BBFB-21D9CAA66DA4}" name="Age" totalsRowFunction="sum" dataDxfId="40" totalsRowDxfId="39"/>
-    <tableColumn id="5" xr3:uid="{3CE9F5DA-0A57-4696-B4E0-53601C3B7798}" name="Rank" totalsRowFunction="sum" dataDxfId="38" totalsRowDxfId="37"/>
-    <tableColumn id="6" xr3:uid="{34912838-665C-4472-B558-25990E5B148D}" name="Rank+Age =E4+D4" totalsRowFunction="sum" dataDxfId="36" totalsRowDxfId="35">
+    <tableColumn id="1" xr3:uid="{C4EE018E-238B-42BA-9035-DB01FA5420D3}" name="Name" totalsRowLabel="Total" dataDxfId="14" totalsRowDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{C1F6911F-9482-4C98-BBFB-21D9CAA66DA4}" name="Age" totalsRowFunction="sum" dataDxfId="12" totalsRowDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{3CE9F5DA-0A57-4696-B4E0-53601C3B7798}" name="Rank" totalsRowFunction="sum" dataDxfId="10" totalsRowDxfId="11"/>
+    <tableColumn id="6" xr3:uid="{34912838-665C-4472-B558-25990E5B148D}" name="Rank+Age =E4+D4" totalsRowFunction="sum" dataDxfId="8" totalsRowDxfId="9">
       <calculatedColumnFormula>Table3[[#This Row],[Rank]]+Table3[[#This Row],[Age]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{89D90022-7073-4067-BAF8-1587D27C4AFB}" name="Data =SUM(E4:E5)" totalsRowFunction="sum" dataDxfId="34" totalsRowDxfId="33">
+    <tableColumn id="7" xr3:uid="{89D90022-7073-4067-BAF8-1587D27C4AFB}" name="Data =SUM(E4:E5)" totalsRowFunction="sum" dataDxfId="6" totalsRowDxfId="7">
       <calculatedColumnFormula>SUM(Table3[Rank])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{B2A7E5BB-A379-492B-9484-72F2FD1FF3A0}" name="All =SUM(E3:E6)" totalsRowFunction="sum" dataDxfId="32" totalsRowDxfId="31">
+    <tableColumn id="8" xr3:uid="{B2A7E5BB-A379-492B-9484-72F2FD1FF3A0}" name="All =SUM(E3:E6)" totalsRowFunction="sum" dataDxfId="4" totalsRowDxfId="5">
       <calculatedColumnFormula>SUM(Table3[[#All],[Rank]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{3C532A69-E4BC-4A20-A922-4BCAA0D3FEC9}" name="Totals =E6" totalsRowFunction="sum" dataDxfId="30" totalsRowDxfId="29">
+    <tableColumn id="9" xr3:uid="{3C532A69-E4BC-4A20-A922-4BCAA0D3FEC9}" name="Totals =E6" totalsRowFunction="sum" dataDxfId="2" totalsRowDxfId="3">
       <calculatedColumnFormula>Table3[[#Totals],[Rank]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{35E9E9C3-9148-468A-85B6-19290CEB6F00}" name="Headers =E3" totalsRowFunction="sum" dataDxfId="28" totalsRowDxfId="27">
+    <tableColumn id="10" xr3:uid="{35E9E9C3-9148-468A-85B6-19290CEB6F00}" name="Headers =E3" totalsRowFunction="sum" dataDxfId="0" totalsRowDxfId="1">
       <calculatedColumnFormula>Table3[[#Headers],[Rank]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -9135,9 +9196,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -9175,7 +9236,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -9281,7 +9342,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -9423,7 +9484,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -9435,7 +9496,7 @@
     <tabColor rgb="FF00FF00"/>
   </sheetPr>
   <dimension ref="A1:L35"/>
-  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="22.28515625" customWidth="1"/>
     <col min="2" max="2" width="13.7109375" customWidth="1"/>
@@ -9444,7 +9505,7 @@
     <col min="6" max="26" width="13.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" ht="38.25" customHeight="1">
       <c r="A1" s="21"/>
       <c r="C1" s="1" t="s">
         <v>0</v>
@@ -9453,7 +9514,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="27.75" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:12" ht="27.75">
       <c r="B2" s="22" t="s">
         <v>2</v>
       </c>
@@ -9463,28 +9524,28 @@
       <c r="G2" s="104">
         <v>5</v>
       </c>
-      <c r="H2" s="105" t="s">
+      <c r="H2" s="110" t="s">
         <v>4</v>
       </c>
-      <c r="I2" s="106"/>
+      <c r="I2" s="115"/>
       <c r="K2" s="3"/>
     </row>
-    <row r="3" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:12" ht="17.25" customHeight="1">
       <c r="F3" s="4" t="s">
         <v>5</v>
       </c>
       <c r="G3" s="104">
         <v>8</v>
       </c>
-      <c r="H3" s="106"/>
-      <c r="I3" s="106"/>
+      <c r="H3" s="115"/>
+      <c r="I3" s="115"/>
       <c r="J3" s="5"/>
-      <c r="K3" s="107">
+      <c r="K3" s="111">
         <v>5</v>
       </c>
       <c r="L3" s="6"/>
     </row>
-    <row r="4" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:12" ht="17.25" customHeight="1">
       <c r="B4" s="7" t="s">
         <v>6</v>
       </c>
@@ -9497,50 +9558,50 @@
       <c r="G4" s="104">
         <v>9</v>
       </c>
-      <c r="H4" s="106"/>
-      <c r="I4" s="106"/>
+      <c r="H4" s="115"/>
+      <c r="I4" s="115"/>
       <c r="J4" s="5"/>
-      <c r="K4" s="108"/>
+      <c r="K4" s="112"/>
       <c r="L4" s="6"/>
     </row>
-    <row r="5" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:12" ht="17.25" customHeight="1">
       <c r="C5" s="104">
         <v>42</v>
       </c>
       <c r="G5" s="104">
         <v>15</v>
       </c>
-      <c r="H5" s="106"/>
-      <c r="I5" s="106"/>
+      <c r="H5" s="115"/>
+      <c r="I5" s="115"/>
       <c r="J5" s="5"/>
-      <c r="K5" s="108"/>
+      <c r="K5" s="112"/>
       <c r="L5" s="6"/>
     </row>
-    <row r="6" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:12" ht="17.25" customHeight="1">
       <c r="G6" s="104">
         <v>22</v>
       </c>
       <c r="J6" s="5"/>
-      <c r="K6" s="108"/>
+      <c r="K6" s="112"/>
       <c r="L6" s="6"/>
     </row>
-    <row r="7" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:12" ht="17.25" customHeight="1">
       <c r="C7" s="104">
         <v>3</v>
       </c>
       <c r="J7" s="5"/>
-      <c r="K7" s="108"/>
+      <c r="K7" s="112"/>
       <c r="L7" s="6"/>
     </row>
-    <row r="8" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:12" ht="17.25" customHeight="1">
       <c r="G8" s="104">
         <v>30</v>
       </c>
       <c r="J8" s="5"/>
-      <c r="K8" s="109"/>
+      <c r="K8" s="113"/>
       <c r="L8" s="6"/>
     </row>
-    <row r="9" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:12" ht="17.25" customHeight="1">
       <c r="B9" s="9" t="s">
         <v>8</v>
       </c>
@@ -9550,7 +9611,7 @@
       </c>
       <c r="K9" s="10"/>
     </row>
-    <row r="10" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:12" ht="17.25" customHeight="1">
       <c r="C10" s="104">
         <f>SUM(C4:C7)</f>
         <v>57.4</v>
@@ -9559,13 +9620,13 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:12" ht="17.25" customHeight="1">
       <c r="C11" s="104">
         <f>-(3+C7*SUM(C4:C7))</f>
         <v>-175.2</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:12" ht="17.25" customHeight="1">
       <c r="C12" s="104">
         <f>SUM(C9:C11)</f>
         <v>-63.399999999999991</v>
@@ -9574,13 +9635,13 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:12" ht="17.25" customHeight="1">
       <c r="G13" s="104">
         <f>A1+A2+A3+A4+A5+A6+A7+A8+A9+A10+A11+A12+A13+A14+A15+A16+A17+A18</f>
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:12" ht="17.25" customHeight="1">
       <c r="B14" s="11" t="s">
         <v>11</v>
       </c>
@@ -9589,32 +9650,32 @@
         <v>#CYCLE</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:12" ht="17.25" customHeight="1">
       <c r="C15" s="104" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:12" ht="17.25" customHeight="1">
       <c r="C16" s="104" t="str">
         <f>C15</f>
         <v>=(+</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:9" ht="17.25" customHeight="1">
       <c r="C17" s="104" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:9" ht="17.25" customHeight="1">
       <c r="C18" s="104" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:9" ht="17.25" customHeight="1">
       <c r="E19" s="3"/>
       <c r="G19" s="3"/>
     </row>
-    <row r="20" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:9" ht="17.25" customHeight="1">
       <c r="B20" s="5"/>
       <c r="C20" s="6" t="s">
         <v>15</v>
@@ -9628,7 +9689,7 @@
       </c>
       <c r="H20" s="6"/>
     </row>
-    <row r="21" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:9" ht="17.25" customHeight="1">
       <c r="A21" s="13" t="s">
         <v>18</v>
       </c>
@@ -9638,7 +9699,7 @@
       </c>
       <c r="G21" s="10"/>
     </row>
-    <row r="23" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:9" ht="17.25" customHeight="1">
       <c r="A23" s="13" t="s">
         <v>19</v>
       </c>
@@ -9652,7 +9713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:9" ht="17.25" customHeight="1">
       <c r="C24" s="16">
         <v>10</v>
       </c>
@@ -9663,7 +9724,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:9" ht="17.25" customHeight="1">
       <c r="C25" s="16">
         <v>10.122999999999999</v>
       </c>
@@ -9674,7 +9735,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:9" ht="17.25" customHeight="1">
       <c r="B26" s="104" t="s">
         <v>20</v>
       </c>
@@ -9688,7 +9749,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:9" ht="17.25" customHeight="1">
       <c r="A27" s="104" t="s">
         <v>22</v>
       </c>
@@ -9705,7 +9766,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:9" ht="17.25" customHeight="1">
       <c r="A28" s="104" t="s">
         <v>23</v>
       </c>
@@ -9722,7 +9783,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:9" ht="17.25" customHeight="1">
       <c r="A29" s="104" t="s">
         <v>24</v>
       </c>
@@ -9739,7 +9800,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:9" ht="17.25" customHeight="1">
       <c r="A30" s="104" t="s">
         <v>25</v>
       </c>
@@ -9756,7 +9817,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:9" ht="17.25" customHeight="1">
       <c r="A31" s="104" t="s">
         <v>26</v>
       </c>
@@ -9773,7 +9834,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:9" ht="17.25" customHeight="1">
       <c r="A32" s="104" t="s">
         <v>27</v>
       </c>
@@ -9790,7 +9851,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:9" ht="17.25" customHeight="1">
       <c r="A33" s="104" t="s">
         <v>28</v>
       </c>
@@ -9807,7 +9868,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:9" ht="17.25" customHeight="1">
       <c r="A34" s="104" t="s">
         <v>29</v>
       </c>
@@ -9818,7 +9879,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="35" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:9" ht="17.25" customHeight="1">
       <c r="A35" s="104" t="s">
         <v>30</v>
       </c>
@@ -9835,7 +9896,7 @@
     <mergeCell ref="K3:K8"/>
   </mergeCells>
   <conditionalFormatting sqref="C1:C100 B21">
-    <cfRule type="cellIs" dxfId="26" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="44" priority="1" operator="equal">
       <formula>42</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9880,7 +9941,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F7A934C-2218-4A12-8B75-EE28D615D774}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="12.75"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -9889,7 +9950,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96301BE1-D86D-4D45-870D-85A75D53FC99}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -9898,7 +9959,7 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B10A8834-0E20-4F80-8813-3ACA5527B377}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="65.140625" customWidth="1"/>
     <col min="2" max="26" width="13.7109375" customWidth="1"/>
@@ -9915,7 +9976,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9925,7 +9986,7 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{025F2510-D243-4DA1-81DE-BBDDA9BC3681}">
   <dimension ref="A1:J6"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="3" max="4" width="14.28515625" customWidth="1"/>
     <col min="5" max="5" width="14.7109375" customWidth="1"/>
@@ -9935,193 +9996,193 @@
     <col min="10" max="10" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A1" s="112" t="s">
-        <v>423</v>
-      </c>
-      <c r="B1" s="113" t="s">
+    <row r="1" spans="1:10">
+      <c r="A1" s="106" t="s">
         <v>424</v>
       </c>
-      <c r="C1" s="113" t="s">
+      <c r="B1" s="107" t="s">
         <v>425</v>
       </c>
-      <c r="D1" s="113" t="s">
+      <c r="C1" s="107" t="s">
         <v>426</v>
       </c>
-      <c r="E1" s="113" t="s">
+      <c r="D1" s="107" t="s">
         <v>427</v>
       </c>
-      <c r="F1" s="113" t="s">
+      <c r="E1" s="107" t="s">
         <v>428</v>
       </c>
-      <c r="G1" s="113" t="s">
+      <c r="F1" s="107" t="s">
         <v>429</v>
       </c>
-      <c r="H1" s="113" t="s">
+      <c r="G1" s="107" t="s">
         <v>430</v>
       </c>
-      <c r="I1" s="114" t="s">
+      <c r="H1" s="107" t="s">
         <v>431</v>
       </c>
-      <c r="J1" s="111" t="s">
-        <v>441</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" s="115">
+      <c r="I1" s="108" t="s">
+        <v>432</v>
+      </c>
+      <c r="J1" s="105" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="A2">
         <v>4</v>
       </c>
-      <c r="B2" s="115">
+      <c r="B2">
         <v>99.5</v>
       </c>
-      <c r="C2" s="115">
-        <v>1</v>
-      </c>
-      <c r="D2" s="115" t="s">
-        <v>432</v>
-      </c>
-      <c r="E2" s="116">
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>434</v>
+      </c>
+      <c r="E2" s="39">
         <v>45575</v>
       </c>
-      <c r="F2" s="117">
+      <c r="F2" s="109">
         <v>0.64583333333333337</v>
       </c>
-      <c r="G2" s="117" t="s">
-        <v>433</v>
-      </c>
-      <c r="H2" s="116">
+      <c r="G2" s="109" t="s">
+        <v>435</v>
+      </c>
+      <c r="H2" s="39">
         <v>45292</v>
       </c>
-      <c r="I2" s="115">
+      <c r="I2">
         <v>4</v>
       </c>
       <c r="J2">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" s="115">
+    <row r="3" spans="1:10">
+      <c r="A3">
         <v>3</v>
       </c>
-      <c r="B3" s="115">
+      <c r="B3">
         <v>40</v>
       </c>
-      <c r="C3" s="115">
+      <c r="C3">
         <v>2</v>
       </c>
-      <c r="D3" s="115" t="s">
-        <v>434</v>
-      </c>
-      <c r="E3" s="116">
+      <c r="D3" t="s">
+        <v>436</v>
+      </c>
+      <c r="E3" s="39">
         <v>45576</v>
       </c>
-      <c r="F3" s="117">
+      <c r="F3" s="109">
         <v>0.57638888888888884</v>
       </c>
-      <c r="G3" s="117" t="s">
+      <c r="G3" s="109" t="s">
+        <v>437</v>
+      </c>
+      <c r="H3" s="39">
+        <v>45231</v>
+      </c>
+      <c r="I3" t="s">
         <v>435</v>
-      </c>
-      <c r="H3" s="116">
-        <v>45231</v>
-      </c>
-      <c r="I3" s="115" t="s">
-        <v>433</v>
       </c>
       <c r="J3">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="115">
+    <row r="4" spans="1:10">
+      <c r="A4">
         <v>9</v>
       </c>
-      <c r="B4" s="115">
+      <c r="B4">
         <v>0</v>
       </c>
-      <c r="C4" s="115">
+      <c r="C4">
         <v>3</v>
       </c>
-      <c r="D4" s="115" t="s">
-        <v>436</v>
-      </c>
-      <c r="E4" s="116">
+      <c r="D4" t="s">
+        <v>438</v>
+      </c>
+      <c r="E4" s="39">
         <v>45574</v>
       </c>
-      <c r="F4" s="117">
+      <c r="F4" s="109">
         <v>0.73958333333333337</v>
       </c>
-      <c r="G4" s="117" t="s">
-        <v>437</v>
-      </c>
-      <c r="H4" s="116">
+      <c r="G4" s="109" t="s">
+        <v>439</v>
+      </c>
+      <c r="H4" s="39">
         <v>45325</v>
       </c>
-      <c r="I4" s="115">
+      <c r="I4">
         <v>3</v>
       </c>
       <c r="J4">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" s="115">
+    <row r="5" spans="1:10">
+      <c r="A5">
         <v>5</v>
       </c>
-      <c r="B5" s="115">
+      <c r="B5">
         <v>120</v>
       </c>
-      <c r="C5" s="115">
+      <c r="C5">
         <v>4</v>
       </c>
-      <c r="D5" s="115" t="s">
-        <v>434</v>
-      </c>
-      <c r="E5" s="116">
+      <c r="D5" t="s">
+        <v>436</v>
+      </c>
+      <c r="E5" s="39">
         <v>45573</v>
       </c>
-      <c r="F5" s="117">
+      <c r="F5" s="109">
         <v>0.66666666666666663</v>
       </c>
-      <c r="G5" s="115" t="s">
-        <v>438</v>
-      </c>
-      <c r="H5" s="116">
+      <c r="G5" t="s">
+        <v>440</v>
+      </c>
+      <c r="H5" s="39">
         <v>45084</v>
       </c>
-      <c r="I5" s="115">
+      <c r="I5">
         <v>3</v>
       </c>
       <c r="J5">
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" s="115">
+    <row r="6" spans="1:10">
+      <c r="A6">
         <v>7</v>
       </c>
-      <c r="B6" s="115">
+      <c r="B6">
         <v>12</v>
       </c>
-      <c r="C6" s="115">
+      <c r="C6">
         <v>5</v>
       </c>
-      <c r="D6" s="115" t="s">
-        <v>436</v>
-      </c>
-      <c r="E6" s="116">
+      <c r="D6" t="s">
+        <v>438</v>
+      </c>
+      <c r="E6" s="39">
         <v>45566</v>
       </c>
-      <c r="F6" s="117">
+      <c r="F6" s="109">
         <v>0.5229166666666667</v>
       </c>
-      <c r="G6" s="115" t="s">
-        <v>439</v>
-      </c>
-      <c r="H6" s="116">
+      <c r="G6" t="s">
+        <v>441</v>
+      </c>
+      <c r="H6" s="39">
         <v>45420</v>
       </c>
-      <c r="I6" s="115" t="s">
-        <v>438</v>
+      <c r="I6" t="s">
+        <v>440</v>
       </c>
       <c r="J6">
         <v>15</v>
@@ -10175,12 +10236,12 @@
     <tabColor theme="9"/>
   </sheetPr>
   <dimension ref="A1:R163"/>
-  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="26" width="13.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:18" ht="17.25" customHeight="1">
       <c r="A1" s="104" t="s">
         <v>31</v>
       </c>
@@ -10215,7 +10276,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:18" ht="17.25" customHeight="1">
       <c r="A2" s="104" t="s">
         <v>41</v>
       </c>
@@ -10261,7 +10322,7 @@
         <v>1230.7</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:18" ht="17.25" customHeight="1">
       <c r="A3" s="104" t="s">
         <v>43</v>
       </c>
@@ -10307,7 +10368,7 @@
         <v>1217.7</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:18" ht="17.25" customHeight="1">
       <c r="A4" s="104" t="s">
         <v>45</v>
       </c>
@@ -10353,7 +10414,7 @@
         <v>1230.7</v>
       </c>
     </row>
-    <row r="5" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:18" ht="17.25" customHeight="1">
       <c r="A5" s="104" t="s">
         <v>47</v>
       </c>
@@ -10399,7 +10460,7 @@
         <v>1246.7</v>
       </c>
     </row>
-    <row r="6" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:18" ht="17.25" customHeight="1">
       <c r="A6" s="104" t="s">
         <v>49</v>
       </c>
@@ -10445,7 +10506,7 @@
         <v>1213.7</v>
       </c>
     </row>
-    <row r="7" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:18" ht="17.25" customHeight="1">
       <c r="A7" s="104" t="s">
         <v>52</v>
       </c>
@@ -10479,7 +10540,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:18" ht="17.25" customHeight="1">
       <c r="A8" s="104" t="s">
         <v>54</v>
       </c>
@@ -10513,7 +10574,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:18" ht="17.25" customHeight="1">
       <c r="A9" s="104" t="s">
         <v>56</v>
       </c>
@@ -10544,7 +10605,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:18" ht="17.25" customHeight="1">
       <c r="A10" s="104" t="s">
         <v>58</v>
       </c>
@@ -10560,7 +10621,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:18" ht="17.25" customHeight="1">
       <c r="A11" s="104" t="s">
         <v>59</v>
       </c>
@@ -10579,7 +10640,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="12" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:18" ht="17.25" customHeight="1">
       <c r="A12" s="104" t="s">
         <v>61</v>
       </c>
@@ -10610,7 +10671,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="13" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:18" ht="17.25" customHeight="1">
       <c r="A13" s="104" t="s">
         <v>62</v>
       </c>
@@ -10641,7 +10702,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="14" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:18" ht="17.25" customHeight="1">
       <c r="A14" s="104" t="s">
         <v>67</v>
       </c>
@@ -10657,7 +10718,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:18" ht="17.25" customHeight="1">
       <c r="A15" s="104" t="s">
         <v>68</v>
       </c>
@@ -10673,7 +10734,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:18" ht="17.25" customHeight="1">
       <c r="A16" s="104" t="s">
         <v>69</v>
       </c>
@@ -10689,7 +10750,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" ht="17.25" customHeight="1">
       <c r="A17" s="104" t="s">
         <v>70</v>
       </c>
@@ -10705,7 +10766,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4" ht="17.25" customHeight="1">
       <c r="A18" s="104" t="s">
         <v>71</v>
       </c>
@@ -10721,7 +10782,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:4" ht="17.25" customHeight="1">
       <c r="A19" s="104" t="s">
         <v>72</v>
       </c>
@@ -10737,7 +10798,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4" ht="17.25" customHeight="1">
       <c r="A20" s="104" t="s">
         <v>73</v>
       </c>
@@ -10753,7 +10814,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:4" ht="17.25" customHeight="1">
       <c r="A21" s="104" t="s">
         <v>74</v>
       </c>
@@ -10769,7 +10830,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:4" ht="17.25" customHeight="1">
       <c r="A22" s="104" t="s">
         <v>76</v>
       </c>
@@ -10785,7 +10846,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:4" ht="17.25" customHeight="1">
       <c r="A23" s="104" t="s">
         <v>77</v>
       </c>
@@ -10801,7 +10862,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:4" ht="17.25" customHeight="1">
       <c r="A24" s="104" t="s">
         <v>78</v>
       </c>
@@ -10818,7 +10879,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:4" ht="17.25" customHeight="1">
       <c r="A25" s="104" t="s">
         <v>79</v>
       </c>
@@ -10834,7 +10895,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:4" ht="17.25" customHeight="1">
       <c r="A26" s="104" t="s">
         <v>81</v>
       </c>
@@ -10850,7 +10911,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:4" ht="17.25" customHeight="1">
       <c r="A27" s="104" t="s">
         <v>82</v>
       </c>
@@ -10866,7 +10927,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:4" ht="17.25" customHeight="1">
       <c r="A28" s="104" t="s">
         <v>83</v>
       </c>
@@ -10883,7 +10944,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:4" ht="17.25" customHeight="1">
       <c r="A29" s="104" t="s">
         <v>84</v>
       </c>
@@ -10899,7 +10960,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:4" ht="17.25" customHeight="1">
       <c r="A30" s="104" t="s">
         <v>85</v>
       </c>
@@ -10915,7 +10976,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:4" ht="17.25" customHeight="1">
       <c r="A31" s="104" t="s">
         <v>86</v>
       </c>
@@ -10931,7 +10992,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:4" ht="17.25" customHeight="1">
       <c r="A32" s="104" t="s">
         <v>87</v>
       </c>
@@ -10947,7 +11008,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:4" ht="17.25" customHeight="1">
       <c r="A33" s="104" t="s">
         <v>88</v>
       </c>
@@ -10963,7 +11024,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:4" ht="17.25" customHeight="1">
       <c r="A34" s="104" t="s">
         <v>89</v>
       </c>
@@ -10979,7 +11040,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:4" ht="17.25" customHeight="1">
       <c r="A35" s="104" t="s">
         <v>90</v>
       </c>
@@ -10995,7 +11056,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:4" ht="17.25" customHeight="1">
       <c r="A36" s="104" t="s">
         <v>91</v>
       </c>
@@ -11011,7 +11072,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:4" ht="17.25" customHeight="1">
       <c r="A37" s="104" t="s">
         <v>92</v>
       </c>
@@ -11027,7 +11088,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:4" ht="17.25" customHeight="1">
       <c r="A38" s="104" t="s">
         <v>93</v>
       </c>
@@ -11044,7 +11105,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:4" ht="17.25" customHeight="1">
       <c r="A39" s="104" t="s">
         <v>94</v>
       </c>
@@ -11060,7 +11121,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:4" ht="17.25" customHeight="1">
       <c r="A40" s="104" t="s">
         <v>95</v>
       </c>
@@ -11076,7 +11137,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:4" ht="17.25" customHeight="1">
       <c r="A41" s="104" t="s">
         <v>96</v>
       </c>
@@ -11092,7 +11153,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:4" ht="17.25" customHeight="1">
       <c r="A42" s="104" t="s">
         <v>97</v>
       </c>
@@ -11108,7 +11169,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:4" ht="17.25" customHeight="1">
       <c r="A43" s="104" t="s">
         <v>98</v>
       </c>
@@ -11124,7 +11185,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:4" ht="17.25" customHeight="1">
       <c r="A44" s="104" t="s">
         <v>99</v>
       </c>
@@ -11140,7 +11201,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:4" ht="17.25" customHeight="1">
       <c r="A45" s="104" t="s">
         <v>100</v>
       </c>
@@ -11156,7 +11217,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:4" ht="17.25" customHeight="1">
       <c r="A46" s="104" t="s">
         <v>101</v>
       </c>
@@ -11172,7 +11233,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:4" ht="17.25" customHeight="1">
       <c r="A47" s="104" t="s">
         <v>102</v>
       </c>
@@ -11188,7 +11249,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:4" ht="17.25" customHeight="1">
       <c r="A48" s="104" t="s">
         <v>103</v>
       </c>
@@ -11204,7 +11265,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:4" ht="17.25" customHeight="1">
       <c r="A49" s="104" t="s">
         <v>104</v>
       </c>
@@ -11220,7 +11281,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:4" ht="17.25" customHeight="1">
       <c r="A50" s="104" t="s">
         <v>105</v>
       </c>
@@ -11237,7 +11298,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:4" ht="17.25" customHeight="1">
       <c r="A51" s="104" t="s">
         <v>106</v>
       </c>
@@ -11254,7 +11315,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:4" ht="17.25" customHeight="1">
       <c r="A52" s="104" t="s">
         <v>107</v>
       </c>
@@ -11270,7 +11331,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:4" ht="17.25" customHeight="1">
       <c r="A53" s="104" t="s">
         <v>108</v>
       </c>
@@ -11286,7 +11347,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:4" ht="17.25" customHeight="1">
       <c r="A54" s="104" t="s">
         <v>109</v>
       </c>
@@ -11302,7 +11363,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:4" ht="17.25" customHeight="1">
       <c r="A55" s="104" t="s">
         <v>110</v>
       </c>
@@ -11318,7 +11379,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:4" ht="17.25" customHeight="1">
       <c r="A56" s="104" t="s">
         <v>111</v>
       </c>
@@ -11334,7 +11395,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:4" ht="17.25" customHeight="1">
       <c r="A57" s="104" t="s">
         <v>112</v>
       </c>
@@ -11350,7 +11411,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:4" ht="17.25" customHeight="1">
       <c r="A58" s="104" t="s">
         <v>113</v>
       </c>
@@ -11366,7 +11427,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:4" ht="17.25" customHeight="1">
       <c r="A59" s="104" t="s">
         <v>114</v>
       </c>
@@ -11382,7 +11443,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:4" ht="17.25" customHeight="1">
       <c r="A60" s="104" t="s">
         <v>115</v>
       </c>
@@ -11398,7 +11459,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:4" ht="17.25" customHeight="1">
       <c r="A61" s="104" t="s">
         <v>116</v>
       </c>
@@ -11414,7 +11475,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:4" ht="17.25" customHeight="1">
       <c r="A62" s="104" t="s">
         <v>117</v>
       </c>
@@ -11430,7 +11491,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:4" ht="17.25" customHeight="1">
       <c r="A63" s="104" t="s">
         <v>118</v>
       </c>
@@ -11446,7 +11507,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:4" ht="17.25" customHeight="1">
       <c r="A64" s="104" t="s">
         <v>119</v>
       </c>
@@ -11462,7 +11523,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:4" ht="17.25" customHeight="1">
       <c r="A65" s="104" t="s">
         <v>120</v>
       </c>
@@ -11478,7 +11539,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:4" ht="17.25" customHeight="1">
       <c r="A66" s="104" t="s">
         <v>121</v>
       </c>
@@ -11494,7 +11555,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:4" ht="17.25" customHeight="1">
       <c r="A67" s="104" t="s">
         <v>122</v>
       </c>
@@ -11510,7 +11571,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:4" ht="17.25" customHeight="1">
       <c r="A68" s="104" t="s">
         <v>123</v>
       </c>
@@ -11526,7 +11587,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:4" ht="17.25" customHeight="1">
       <c r="A69" s="104" t="s">
         <v>125</v>
       </c>
@@ -11542,7 +11603,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:4" ht="17.25" customHeight="1">
       <c r="A70" s="104" t="s">
         <v>127</v>
       </c>
@@ -11558,7 +11619,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:4" ht="17.25" customHeight="1">
       <c r="A71" s="104" t="s">
         <v>129</v>
       </c>
@@ -11574,7 +11635,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:4" ht="17.25" customHeight="1">
       <c r="A72" s="104" t="s">
         <v>130</v>
       </c>
@@ -11590,7 +11651,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:4" ht="17.25" customHeight="1">
       <c r="A73" s="104" t="s">
         <v>131</v>
       </c>
@@ -11606,7 +11667,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:4" ht="17.25" customHeight="1">
       <c r="A74" s="104" t="s">
         <v>132</v>
       </c>
@@ -11622,7 +11683,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:4" ht="17.25" customHeight="1">
       <c r="A75" s="104" t="s">
         <v>133</v>
       </c>
@@ -11638,7 +11699,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:4" ht="17.25" customHeight="1">
       <c r="A76" s="104" t="s">
         <v>134</v>
       </c>
@@ -11654,7 +11715,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:4" ht="17.25" customHeight="1">
       <c r="A77" s="104" t="s">
         <v>135</v>
       </c>
@@ -11670,7 +11731,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="78" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:4" ht="17.25" customHeight="1">
       <c r="A78" s="104" t="s">
         <v>136</v>
       </c>
@@ -11686,7 +11747,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:4" ht="17.25" customHeight="1">
       <c r="A79" s="104" t="s">
         <v>137</v>
       </c>
@@ -11702,7 +11763,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:4" ht="17.25" customHeight="1">
       <c r="A80" s="104" t="s">
         <v>138</v>
       </c>
@@ -11718,7 +11779,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:4" ht="17.25" customHeight="1">
       <c r="A81" s="104" t="s">
         <v>139</v>
       </c>
@@ -11734,7 +11795,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:4" ht="17.25" customHeight="1">
       <c r="A82" s="104" t="s">
         <v>141</v>
       </c>
@@ -11750,7 +11811,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:4" ht="17.25" customHeight="1">
       <c r="A83" s="104" t="s">
         <v>142</v>
       </c>
@@ -11766,7 +11827,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:4" ht="17.25" customHeight="1">
       <c r="A84" s="104" t="s">
         <v>143</v>
       </c>
@@ -11782,7 +11843,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:4" ht="17.25" customHeight="1">
       <c r="A85" s="104" t="s">
         <v>144</v>
       </c>
@@ -11798,7 +11859,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="86" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:4" ht="17.25" customHeight="1">
       <c r="A86" s="104" t="s">
         <v>146</v>
       </c>
@@ -11814,7 +11875,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:4" ht="17.25" customHeight="1">
       <c r="A87" s="104" t="s">
         <v>147</v>
       </c>
@@ -11830,7 +11891,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:4" ht="17.25" customHeight="1">
       <c r="A88" s="104" t="s">
         <v>148</v>
       </c>
@@ -11846,7 +11907,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:4" ht="17.25" customHeight="1">
       <c r="A89" s="104" t="s">
         <v>149</v>
       </c>
@@ -11862,7 +11923,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="90" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:4" ht="17.25" customHeight="1">
       <c r="A90" s="104" t="s">
         <v>150</v>
       </c>
@@ -11878,7 +11939,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:4" ht="17.25" customHeight="1">
       <c r="A91" s="104" t="s">
         <v>151</v>
       </c>
@@ -11894,7 +11955,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:4" ht="17.25" customHeight="1">
       <c r="A92" s="104" t="s">
         <v>152</v>
       </c>
@@ -11910,7 +11971,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:4" ht="17.25" customHeight="1">
       <c r="A93" s="104" t="s">
         <v>153</v>
       </c>
@@ -11926,7 +11987,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="94" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:4" ht="17.25" customHeight="1">
       <c r="A94" s="104" t="s">
         <v>154</v>
       </c>
@@ -11942,7 +12003,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="95" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:4" ht="17.25" customHeight="1">
       <c r="A95" s="104" t="s">
         <v>155</v>
       </c>
@@ -11958,7 +12019,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="96" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:4" ht="17.25" customHeight="1">
       <c r="A96" s="104" t="s">
         <v>156</v>
       </c>
@@ -11974,7 +12035,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="97" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:4" ht="17.25" customHeight="1">
       <c r="A97" s="104" t="s">
         <v>157</v>
       </c>
@@ -11990,7 +12051,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="98" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:4" ht="17.25" customHeight="1">
       <c r="A98" s="104" t="s">
         <v>158</v>
       </c>
@@ -12006,7 +12067,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="99" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:4" ht="17.25" customHeight="1">
       <c r="A99" s="104" t="s">
         <v>159</v>
       </c>
@@ -12022,20 +12083,20 @@
         <v>1</v>
       </c>
     </row>
-    <row r="100" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:4" ht="17.25" customHeight="1">
       <c r="A100" s="104" t="s">
         <v>160</v>
       </c>
       <c r="B100" s="19">
         <f ca="1">NOW()</f>
-        <v>45938.493500231481</v>
+        <v>45995.606012037038</v>
       </c>
       <c r="D100" s="104">
         <f ca="1">IF(ISNUMBER(B100),1,0)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="101" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:4" ht="17.25" customHeight="1">
       <c r="A101" s="104" t="s">
         <v>161</v>
       </c>
@@ -12051,7 +12112,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="102" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:4" ht="17.25" customHeight="1">
       <c r="A102" s="104" t="s">
         <v>162</v>
       </c>
@@ -12067,7 +12128,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="103" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:4" ht="17.25" customHeight="1">
       <c r="A103" s="104" t="s">
         <v>163</v>
       </c>
@@ -12083,7 +12144,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="104" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:4" ht="17.25" customHeight="1">
       <c r="A104" s="104" t="s">
         <v>164</v>
       </c>
@@ -12099,7 +12160,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="105" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:4" ht="17.25" customHeight="1">
       <c r="A105" s="104" t="s">
         <v>165</v>
       </c>
@@ -12115,7 +12176,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="106" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:4" ht="17.25" customHeight="1">
       <c r="A106" s="104" t="s">
         <v>166</v>
       </c>
@@ -12131,7 +12192,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="107" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:4" ht="17.25" customHeight="1">
       <c r="A107" s="104" t="s">
         <v>167</v>
       </c>
@@ -12147,7 +12208,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:4" ht="17.25" customHeight="1">
       <c r="A108" s="104" t="s">
         <v>168</v>
       </c>
@@ -12163,7 +12224,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="109" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:4" ht="17.25" customHeight="1">
       <c r="A109" s="104" t="s">
         <v>169</v>
       </c>
@@ -12179,7 +12240,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="110" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:4" ht="17.25" customHeight="1">
       <c r="A110" s="104" t="s">
         <v>170</v>
       </c>
@@ -12195,7 +12256,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="111" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:4" ht="17.25" customHeight="1">
       <c r="A111" s="104" t="s">
         <v>171</v>
       </c>
@@ -12211,12 +12272,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="112" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:4" ht="17.25" customHeight="1">
       <c r="A112" s="104"/>
       <c r="B112" s="104"/>
       <c r="D112" s="104"/>
     </row>
-    <row r="113" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:4" ht="17.25" customHeight="1">
       <c r="A113" s="104" t="s">
         <v>172</v>
       </c>
@@ -12232,7 +12293,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="114" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:4" ht="17.25" customHeight="1">
       <c r="A114" s="104" t="s">
         <v>173</v>
       </c>
@@ -12248,7 +12309,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="115" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:4" ht="17.25" customHeight="1">
       <c r="A115" s="104" t="s">
         <v>175</v>
       </c>
@@ -12264,7 +12325,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="116" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:4" ht="17.25" customHeight="1">
       <c r="A116" s="104" t="s">
         <v>177</v>
       </c>
@@ -12280,7 +12341,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="117" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:4" ht="17.25" customHeight="1">
       <c r="A117" s="104" t="s">
         <v>178</v>
       </c>
@@ -12296,7 +12357,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="118" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:4" ht="17.25" customHeight="1">
       <c r="A118" s="104" t="s">
         <v>179</v>
       </c>
@@ -12312,7 +12373,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="119" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:4" ht="17.25" customHeight="1">
       <c r="A119" s="104" t="s">
         <v>180</v>
       </c>
@@ -12328,7 +12389,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="120" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:4" ht="17.25" customHeight="1">
       <c r="A120" s="104" t="s">
         <v>181</v>
       </c>
@@ -12344,7 +12405,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="121" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:4" ht="17.25" customHeight="1">
       <c r="A121" s="104" t="s">
         <v>182</v>
       </c>
@@ -12360,7 +12421,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="122" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:4" ht="17.25" customHeight="1">
       <c r="A122" s="104" t="s">
         <v>183</v>
       </c>
@@ -12376,7 +12437,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="123" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:4" ht="17.25" customHeight="1">
       <c r="A123" s="104" t="s">
         <v>184</v>
       </c>
@@ -12392,7 +12453,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="124" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:4" ht="17.25" customHeight="1">
       <c r="A124" s="104" t="s">
         <v>185</v>
       </c>
@@ -12408,7 +12469,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="125" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:4" ht="17.25" customHeight="1">
       <c r="A125" s="104" t="s">
         <v>186</v>
       </c>
@@ -12424,7 +12485,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="126" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:4" ht="17.25" customHeight="1">
       <c r="A126" s="104" t="s">
         <v>187</v>
       </c>
@@ -12440,7 +12501,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="127" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:4" ht="17.25" customHeight="1">
       <c r="A127" s="104" t="s">
         <v>188</v>
       </c>
@@ -12456,7 +12517,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="128" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:4" ht="17.25" customHeight="1">
       <c r="A128" s="104" t="s">
         <v>189</v>
       </c>
@@ -12472,7 +12533,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="129" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:4" ht="17.25" customHeight="1">
       <c r="A129" s="104" t="s">
         <v>190</v>
       </c>
@@ -12488,7 +12549,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="130" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:4" ht="17.25" customHeight="1">
       <c r="A130" s="104" t="s">
         <v>191</v>
       </c>
@@ -12504,7 +12565,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="131" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:4" ht="17.25" customHeight="1">
       <c r="A131" s="104" t="s">
         <v>192</v>
       </c>
@@ -12520,7 +12581,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="132" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:4" ht="17.25" customHeight="1">
       <c r="A132" s="104" t="s">
         <v>193</v>
       </c>
@@ -12536,7 +12597,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="133" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:4" ht="17.25" customHeight="1">
       <c r="A133" s="104" t="s">
         <v>194</v>
       </c>
@@ -12552,7 +12613,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="134" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:4" ht="17.25" customHeight="1">
       <c r="A134" s="104" t="s">
         <v>195</v>
       </c>
@@ -12568,7 +12629,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="135" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:4" ht="17.25" customHeight="1">
       <c r="A135" s="104" t="s">
         <v>196</v>
       </c>
@@ -12584,7 +12645,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="136" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:4" ht="17.25" customHeight="1">
       <c r="A136" s="104" t="s">
         <v>198</v>
       </c>
@@ -12600,7 +12661,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="137" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:4" ht="17.25" customHeight="1">
       <c r="A137" s="104" t="s">
         <v>199</v>
       </c>
@@ -12616,7 +12677,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="138" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:4" ht="17.25" customHeight="1">
       <c r="A138" s="104" t="s">
         <v>200</v>
       </c>
@@ -12632,7 +12693,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="139" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:4" ht="17.25" customHeight="1">
       <c r="A139" s="104" t="s">
         <v>201</v>
       </c>
@@ -12648,7 +12709,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="140" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:4" ht="17.25" customHeight="1">
       <c r="A140" s="104" t="s">
         <v>202</v>
       </c>
@@ -12664,7 +12725,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="141" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:4" ht="17.25" customHeight="1">
       <c r="A141" s="104" t="s">
         <v>203</v>
       </c>
@@ -12680,7 +12741,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="142" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:4" ht="17.25" customHeight="1">
       <c r="A142" s="104" t="s">
         <v>205</v>
       </c>
@@ -12696,7 +12757,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:4" ht="17.25" customHeight="1">
       <c r="A143" s="104" t="s">
         <v>206</v>
       </c>
@@ -12712,20 +12773,20 @@
         <v>1</v>
       </c>
     </row>
-    <row r="144" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:4" ht="17.25" customHeight="1">
       <c r="A144" s="104" t="s">
         <v>207</v>
       </c>
       <c r="B144" s="18">
         <f ca="1">TODAY()</f>
-        <v>45938</v>
+        <v>45995</v>
       </c>
       <c r="D144" s="104">
         <f ca="1">IF(ISNUMBER(B144),1,0)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="145" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:4" ht="17.25" customHeight="1">
       <c r="A145" s="104" t="s">
         <v>208</v>
       </c>
@@ -12741,7 +12802,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="146" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:4" ht="17.25" customHeight="1">
       <c r="A146" s="104" t="s">
         <v>210</v>
       </c>
@@ -12757,7 +12818,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="147" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:4" ht="17.25" customHeight="1">
       <c r="A147" s="104" t="s">
         <v>211</v>
       </c>
@@ -12773,7 +12834,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="148" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:4" ht="17.25" customHeight="1">
       <c r="A148" s="104" t="s">
         <v>213</v>
       </c>
@@ -12789,7 +12850,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="149" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:4" ht="17.25" customHeight="1">
       <c r="A149" s="104" t="s">
         <v>214</v>
       </c>
@@ -12805,7 +12866,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="150" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:4" ht="17.25" customHeight="1">
       <c r="A150" s="104" t="s">
         <v>215</v>
       </c>
@@ -12821,7 +12882,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="151" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:4" ht="17.25" customHeight="1">
       <c r="A151" s="104" t="s">
         <v>216</v>
       </c>
@@ -12837,7 +12898,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="152" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:4" ht="17.25" customHeight="1">
       <c r="A152" s="104" t="s">
         <v>217</v>
       </c>
@@ -12853,7 +12914,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="153" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:4" ht="17.25" customHeight="1">
       <c r="A153" s="104" t="s">
         <v>218</v>
       </c>
@@ -12869,7 +12930,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="154" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:4" ht="17.25" customHeight="1">
       <c r="A154" s="104" t="s">
         <v>219</v>
       </c>
@@ -12886,7 +12947,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="155" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:4" ht="17.25" customHeight="1">
       <c r="A155" s="104" t="s">
         <v>220</v>
       </c>
@@ -12902,7 +12963,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="156" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:4" ht="17.25" customHeight="1">
       <c r="A156" s="104" t="s">
         <v>221</v>
       </c>
@@ -12918,7 +12979,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="157" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:4" ht="17.25" customHeight="1">
       <c r="A157" s="104" t="s">
         <v>222</v>
       </c>
@@ -12934,7 +12995,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="158" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:4" ht="17.25" customHeight="1">
       <c r="A158" s="104" t="s">
         <v>223</v>
       </c>
@@ -12950,7 +13011,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="159" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:4" ht="17.25" customHeight="1">
       <c r="A159" s="104" t="s">
         <v>224</v>
       </c>
@@ -12966,7 +13027,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="160" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:4" ht="17.25" customHeight="1">
       <c r="A160" s="104" t="s">
         <v>225</v>
       </c>
@@ -12982,7 +13043,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="161" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:4" ht="17.25" customHeight="1">
       <c r="A161" s="104" t="s">
         <v>226</v>
       </c>
@@ -12998,7 +13059,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="162" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:4" ht="17.25" customHeight="1">
       <c r="A162" s="104" t="s">
         <v>227</v>
       </c>
@@ -13014,7 +13075,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="163" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:4" ht="17.25" customHeight="1">
       <c r="A163" s="104" t="s">
         <v>229</v>
       </c>
@@ -13032,10 +13093,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="D1:D180">
-    <cfRule type="cellIs" dxfId="25" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="43" priority="1" operator="equal">
       <formula>1</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="42" priority="2" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -13050,7 +13111,7 @@
     <outlinePr summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:R31"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" outlineLevelRow="2" outlineLevelCol="2" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" outlineLevelRow="2" outlineLevelCol="2"/>
   <cols>
     <col min="3" max="3" width="0" hidden="1" customWidth="1"/>
     <col min="6" max="6" width="14.28515625" customWidth="1"/>
@@ -13060,17 +13121,17 @@
     <col min="15" max="18" width="9.140625" outlineLevel="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8">
       <c r="A1" t="s">
         <v>230</v>
       </c>
       <c r="C1" t="s">
         <v>231</v>
       </c>
-      <c r="D1" s="110" t="s">
+      <c r="D1" s="114" t="s">
         <v>232</v>
       </c>
-      <c r="E1" s="110"/>
+      <c r="E1" s="114"/>
       <c r="F1" t="s">
         <v>233</v>
       </c>
@@ -13078,19 +13139,19 @@
         <v>234</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8">
       <c r="A2">
         <f>SUM(A1)</f>
         <v>0</v>
       </c>
-      <c r="D2" s="110"/>
-      <c r="E2" s="110"/>
+      <c r="D2" s="114"/>
+      <c r="E2" s="114"/>
       <c r="H2" t="str">
         <f>[1]Feuil1!$A$1</f>
         <v>referenced string</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8">
       <c r="D3" s="85" t="s">
         <v>235</v>
       </c>
@@ -13098,43 +13159,43 @@
         <v>236</v>
       </c>
     </row>
-    <row r="4" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" hidden="1">
       <c r="A4" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" ht="75" customHeight="1">
       <c r="A5" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="10" spans="1:8" outlineLevel="1" x14ac:dyDescent="0.2"/>
-    <row r="11" spans="1:8" outlineLevel="1" x14ac:dyDescent="0.2"/>
-    <row r="12" spans="1:8" hidden="1" outlineLevel="2" x14ac:dyDescent="0.2"/>
-    <row r="13" spans="1:8" hidden="1" outlineLevel="2" x14ac:dyDescent="0.2"/>
-    <row r="14" spans="1:8" hidden="1" outlineLevel="2" x14ac:dyDescent="0.2"/>
-    <row r="15" spans="1:8" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.2"/>
-    <row r="16" spans="1:8" outlineLevel="1" x14ac:dyDescent="0.2"/>
-    <row r="17" spans="1:2" outlineLevel="1" x14ac:dyDescent="0.2"/>
-    <row r="18" spans="1:2" outlineLevel="1" x14ac:dyDescent="0.2"/>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" outlineLevel="1"/>
+    <row r="11" spans="1:8" outlineLevel="1"/>
+    <row r="12" spans="1:8" hidden="1" outlineLevel="2"/>
+    <row r="13" spans="1:8" hidden="1" outlineLevel="2"/>
+    <row r="14" spans="1:8" hidden="1" outlineLevel="2"/>
+    <row r="15" spans="1:8" outlineLevel="1" collapsed="1"/>
+    <row r="16" spans="1:8" outlineLevel="1"/>
+    <row r="17" spans="1:2" outlineLevel="1"/>
+    <row r="18" spans="1:2" outlineLevel="1"/>
+    <row r="30" spans="1:2">
       <c r="A30" cm="1">
         <f t="array" aca="1" ref="A30:B31" ca="1">_xlfn.RANDARRAY(2,2)</f>
-        <v>0.7272925709748963</v>
+        <v>0.71838237714175435</v>
       </c>
       <c r="B30">
         <f ca="1"/>
-        <v>0.95782684877879687</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+        <v>0.36236179614680708</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2">
       <c r="A31">
         <f ca="1"/>
-        <v>0.31704384406036645</v>
+        <v>0.40388442517560574</v>
       </c>
       <c r="B31">
         <f ca="1"/>
-        <v>8.7112099778747121E-2</v>
+        <v>0.47343726914281192</v>
       </c>
     </row>
   </sheetData>
@@ -13153,14 +13214,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF68F2C0-1053-4FB6-BD74-8A11B0CAF123}">
   <dimension ref="A1:M30"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75"/>
   <cols>
     <col min="3" max="3" width="17.7109375" customWidth="1"/>
     <col min="5" max="5" width="18.28515625" customWidth="1"/>
     <col min="13" max="13" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="13.5" thickBot="1">
       <c r="A1" s="68" t="s">
         <v>239</v>
       </c>
@@ -13182,7 +13243,7 @@
       </c>
       <c r="M1" s="36"/>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13">
       <c r="A2" s="40" t="s">
         <v>245</v>
       </c>
@@ -13208,7 +13269,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:13">
       <c r="A3" s="41" t="s">
         <v>252</v>
       </c>
@@ -13231,7 +13292,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="15" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" ht="15">
       <c r="A4" s="42" t="s">
         <v>256</v>
       </c>
@@ -13257,7 +13318,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:13">
       <c r="A5" s="43" t="s">
         <v>262</v>
       </c>
@@ -13277,7 +13338,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13">
       <c r="A6" s="44" t="s">
         <v>266</v>
       </c>
@@ -13300,7 +13361,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" ht="15.75">
       <c r="A7" s="45" t="s">
         <v>271</v>
       </c>
@@ -13320,7 +13381,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="21" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:13" ht="21">
       <c r="A8" s="46" t="s">
         <v>275</v>
       </c>
@@ -13343,7 +13404,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:13">
       <c r="A9" s="47" t="s">
         <v>280</v>
       </c>
@@ -13360,7 +13421,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:13">
       <c r="A10" s="48" t="s">
         <v>283</v>
       </c>
@@ -13368,7 +13429,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" ht="13.5" thickBot="1">
       <c r="A11" s="49" t="s">
         <v>285</v>
       </c>
@@ -13377,7 +13438,7 @@
       </c>
       <c r="F11" s="36"/>
     </row>
-    <row r="12" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:13" ht="18.75" customHeight="1">
       <c r="A12" s="50" t="s">
         <v>287</v>
       </c>
@@ -13391,7 +13452,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" ht="18.75" customHeight="1" thickBot="1">
       <c r="A13" s="51" t="s">
         <v>290</v>
       </c>
@@ -13402,7 +13463,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" ht="18.75" customHeight="1" thickBot="1">
       <c r="A14" s="52" t="s">
         <v>291</v>
       </c>
@@ -13416,7 +13477,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" ht="18.75" customHeight="1" thickBot="1">
       <c r="A15" s="53" t="s">
         <v>293</v>
       </c>
@@ -13427,7 +13488,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="16" spans="1:13" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" ht="19.5" customHeight="1" thickBot="1">
       <c r="A16" s="54" t="s">
         <v>294</v>
       </c>
@@ -13441,12 +13502,12 @@
         <v>248</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" ht="13.5" thickBot="1">
       <c r="A17" s="55" t="s">
         <v>296</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" ht="13.5" thickBot="1">
       <c r="A18" s="74" t="s">
         <v>297</v>
       </c>
@@ -13458,7 +13519,7 @@
       </c>
       <c r="F18" s="36"/>
     </row>
-    <row r="19" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" ht="13.5" thickBot="1">
       <c r="A19" s="75" t="s">
         <v>300</v>
       </c>
@@ -13469,7 +13530,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="51.75" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" ht="51.75" thickBot="1">
       <c r="A20" s="76" t="s">
         <v>303</v>
       </c>
@@ -13483,12 +13544,12 @@
         <v>302</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" ht="13.5" thickBot="1">
       <c r="A21" s="77" t="s">
         <v>306</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" ht="13.5" thickBot="1">
       <c r="A22" s="78" t="s">
         <v>307</v>
       </c>
@@ -13497,13 +13558,13 @@
       </c>
       <c r="E22" s="21"/>
     </row>
-    <row r="23" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" ht="13.5" thickBot="1">
       <c r="A23" s="79" t="s">
         <v>309</v>
       </c>
       <c r="E23" s="21"/>
     </row>
-    <row r="24" spans="1:6" ht="14.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" ht="14.25" thickTop="1" thickBot="1">
       <c r="A24" s="80" t="s">
         <v>310</v>
       </c>
@@ -13512,20 +13573,20 @@
       </c>
       <c r="E24" s="21"/>
     </row>
-    <row r="25" spans="1:6" ht="14.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="26" spans="1:6" ht="14.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" ht="14.25" thickTop="1" thickBot="1"/>
+    <row r="26" spans="1:6" ht="14.25" thickTop="1" thickBot="1">
       <c r="C26" s="67" t="s">
         <v>312</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="14.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="1:6" ht="14.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" ht="14.25" thickTop="1" thickBot="1"/>
+    <row r="28" spans="1:6" ht="14.25" thickTop="1" thickBot="1">
       <c r="C28" s="88" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="13.5" thickTop="1" x14ac:dyDescent="0.2"/>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:6" ht="13.5" thickTop="1"/>
+    <row r="30" spans="1:6">
       <c r="C30" s="87" t="s">
         <v>314</v>
       </c>
@@ -13539,13 +13600,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D919E811-4385-4D35-A19E-3B7E0E659A89}">
   <dimension ref="A1:L39"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="19.140625" customWidth="1"/>
     <col min="7" max="7" width="15.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="13.5" thickBot="1">
       <c r="A1" s="37" t="s">
         <v>315</v>
       </c>
@@ -13562,7 +13623,7 @@
       <c r="I1" s="36"/>
       <c r="J1" s="36"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10">
       <c r="A2" s="38" t="s">
         <v>319</v>
       </c>
@@ -13585,7 +13646,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10">
       <c r="A3" s="38" t="s">
         <v>321</v>
       </c>
@@ -13608,7 +13669,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10">
       <c r="A4" s="38" t="s">
         <v>325</v>
       </c>
@@ -13628,7 +13689,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10">
       <c r="A5" s="38" t="s">
         <v>328</v>
       </c>
@@ -13652,7 +13713,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10">
       <c r="A6" s="38" t="s">
         <v>330</v>
       </c>
@@ -13675,7 +13736,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:10">
       <c r="A7" s="38" t="s">
         <v>333</v>
       </c>
@@ -13701,7 +13762,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:10">
       <c r="A8" s="38" t="s">
         <v>337</v>
       </c>
@@ -13712,7 +13773,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10">
       <c r="A9" s="38" t="s">
         <v>339</v>
       </c>
@@ -13721,7 +13782,7 @@
       </c>
       <c r="C9" s="21"/>
     </row>
-    <row r="10" spans="1:10" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" ht="13.5" thickBot="1">
       <c r="A10" s="38" t="s">
         <v>340</v>
       </c>
@@ -13739,7 +13800,7 @@
       <c r="I10" s="36"/>
       <c r="J10" s="36"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:10">
       <c r="A11" s="38" t="s">
         <v>342</v>
       </c>
@@ -13762,13 +13823,13 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:10">
       <c r="A12" s="38" t="s">
         <v>344</v>
       </c>
       <c r="B12" s="39">
         <f ca="1">TODAY()</f>
-        <v>45938</v>
+        <v>45995</v>
       </c>
       <c r="C12" s="39">
         <f>DATE(2010,10,2)</f>
@@ -13787,7 +13848,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:10">
       <c r="A13" s="38" t="s">
         <v>346</v>
       </c>
@@ -13810,7 +13871,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:10">
       <c r="A14" s="38" t="s">
         <v>348</v>
       </c>
@@ -13836,7 +13897,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:10">
       <c r="A15" s="38" t="s">
         <v>350</v>
       </c>
@@ -13856,7 +13917,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:10">
       <c r="A16" s="38" t="s">
         <v>352</v>
       </c>
@@ -13879,7 +13940,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:12">
       <c r="A17" s="38" t="s">
         <v>354</v>
       </c>
@@ -13902,7 +13963,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:12">
       <c r="A18" s="38" t="s">
         <v>356</v>
       </c>
@@ -13925,7 +13986,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:12">
       <c r="A19" s="38" t="s">
         <v>358</v>
       </c>
@@ -13948,7 +14009,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:12">
       <c r="A20" s="38" t="s">
         <v>360</v>
       </c>
@@ -13971,7 +14032,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:12">
       <c r="A21" s="38" t="s">
         <v>362</v>
       </c>
@@ -13997,7 +14058,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:12">
       <c r="A22" s="38" t="s">
         <v>364</v>
       </c>
@@ -14023,7 +14084,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:12">
       <c r="A23" s="38" t="s">
         <v>366</v>
       </c>
@@ -14049,7 +14110,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:12">
       <c r="G24" s="34" t="s">
         <v>368</v>
       </c>
@@ -14066,7 +14127,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:12">
       <c r="A25" s="38" t="s">
         <v>369</v>
       </c>
@@ -14092,7 +14153,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:12">
       <c r="G26" s="34" t="s">
         <v>371</v>
       </c>
@@ -14112,7 +14173,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:12">
       <c r="A27" s="21" t="s">
         <v>372</v>
       </c>
@@ -14138,7 +14199,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:12">
       <c r="G28" s="34" t="s">
         <v>374</v>
       </c>
@@ -14158,9 +14219,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:12">
       <c r="A29" s="38" t="s">
-        <v>440</v>
+        <v>375</v>
       </c>
       <c r="B29">
         <v>3</v>
@@ -14169,7 +14230,7 @@
         <v>10</v>
       </c>
       <c r="G29" s="34" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="H29">
         <v>5</v>
@@ -14187,9 +14248,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:12">
       <c r="G30" s="34" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="H30">
         <v>5</v>
@@ -14207,9 +14268,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:12" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:12" ht="13.5" thickBot="1">
       <c r="G31" s="35" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="H31" s="36">
         <v>5</v>
@@ -14221,9 +14282,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:12">
       <c r="G32" s="34" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="H32">
         <v>5</v>
@@ -14235,9 +14296,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="7:10" x14ac:dyDescent="0.2">
+    <row r="33" spans="7:10">
       <c r="G33" s="34" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="H33">
         <v>5</v>
@@ -14249,9 +14310,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="7:10" x14ac:dyDescent="0.2">
+    <row r="34" spans="7:10">
       <c r="G34" s="34" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="H34">
         <v>5</v>
@@ -14263,9 +14324,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="7:10" x14ac:dyDescent="0.2">
+    <row r="35" spans="7:10">
       <c r="G35" s="34" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="H35">
         <v>5</v>
@@ -14277,9 +14338,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="7:10" x14ac:dyDescent="0.2">
+    <row r="36" spans="7:10">
       <c r="G36" s="34" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="H36">
         <v>5</v>
@@ -14291,9 +14352,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="7:10" x14ac:dyDescent="0.2">
+    <row r="37" spans="7:10">
       <c r="G37" s="34" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="H37">
         <v>5</v>
@@ -14305,110 +14366,110 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="7:10" x14ac:dyDescent="0.2">
+    <row r="39" spans="7:10">
       <c r="G39" s="34"/>
     </row>
   </sheetData>
   <phoneticPr fontId="21" type="noConversion"/>
   <conditionalFormatting sqref="B15">
-    <cfRule type="expression" dxfId="23" priority="59">
+    <cfRule type="expression" dxfId="41" priority="59">
       <formula>ODD(B15)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B26:B27">
-    <cfRule type="cellIs" dxfId="22" priority="47" operator="equal">
+    <cfRule type="cellIs" dxfId="40" priority="47" operator="equal">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B2:C2">
-    <cfRule type="aboveAverage" dxfId="21" priority="115"/>
+    <cfRule type="aboveAverage" dxfId="39" priority="115"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:C3">
-    <cfRule type="beginsWith" dxfId="20" priority="74" operator="beginsWith" text="rule">
+    <cfRule type="beginsWith" dxfId="38" priority="74" operator="beginsWith" text="rule">
       <formula>LEFT(B3,LEN("rule"))="rule"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B4:C4">
-    <cfRule type="containsBlanks" dxfId="19" priority="72">
+    <cfRule type="containsBlanks" dxfId="37" priority="72">
       <formula>LEN(TRIM(B4))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B5:C5">
-    <cfRule type="containsErrors" dxfId="18" priority="71">
+    <cfRule type="containsErrors" dxfId="36" priority="71">
       <formula>ISERROR(B5)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:C6">
-    <cfRule type="containsText" dxfId="17" priority="70" operator="containsText" text="rule">
+    <cfRule type="containsText" dxfId="35" priority="70" operator="containsText" text="rule">
       <formula>NOT(ISERROR(SEARCH("rule",B6)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8:C8">
-    <cfRule type="endsWith" dxfId="16" priority="68" operator="endsWith" text="rule">
+    <cfRule type="endsWith" dxfId="34" priority="68" operator="endsWith" text="rule">
       <formula>RIGHT(B8,LEN("rule"))="rule"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B9:C9">
-    <cfRule type="notContainsBlanks" dxfId="15" priority="67">
+    <cfRule type="notContainsBlanks" dxfId="33" priority="67">
       <formula>LEN(TRIM(B9))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B10:C10">
-    <cfRule type="notContainsErrors" dxfId="14" priority="66">
+    <cfRule type="notContainsErrors" dxfId="32" priority="66">
       <formula>NOT(ISERROR(B10))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B11:C11">
-    <cfRule type="notContainsText" dxfId="13" priority="65" operator="notContains" text="rule">
+    <cfRule type="notContainsText" dxfId="31" priority="65" operator="notContains" text="rule">
       <formula>ISERROR(SEARCH("rule",B11))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12:C12">
-    <cfRule type="timePeriod" dxfId="12" priority="64" timePeriod="today">
+    <cfRule type="timePeriod" dxfId="30" priority="64" timePeriod="today">
       <formula>FLOOR(B12,1)=TODAY()</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B13:C13">
-    <cfRule type="top10" dxfId="11" priority="116" rank="1"/>
+    <cfRule type="top10" dxfId="29" priority="116" rank="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B16:C16">
-    <cfRule type="cellIs" dxfId="10" priority="46" operator="equal">
+    <cfRule type="cellIs" dxfId="28" priority="46" operator="equal">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B17:C17">
-    <cfRule type="cellIs" dxfId="9" priority="57" operator="notEqual">
+    <cfRule type="cellIs" dxfId="27" priority="57" operator="notEqual">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B18:C18">
-    <cfRule type="cellIs" dxfId="8" priority="7" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="26" priority="7" operator="greaterThan">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B19:C19">
-    <cfRule type="cellIs" dxfId="7" priority="6" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="25" priority="6" operator="greaterThanOrEqual">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B20:C20">
-    <cfRule type="cellIs" dxfId="6" priority="5" operator="lessThan">
+    <cfRule type="cellIs" dxfId="24" priority="5" operator="lessThan">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B21:C21">
-    <cfRule type="cellIs" dxfId="5" priority="4" operator="lessThanOrEqual">
+    <cfRule type="cellIs" dxfId="23" priority="4" operator="lessThanOrEqual">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B22:C22">
-    <cfRule type="cellIs" dxfId="4" priority="3" operator="between">
+    <cfRule type="cellIs" dxfId="22" priority="3" operator="between">
       <formula>2</formula>
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B23:C23">
-    <cfRule type="cellIs" dxfId="3" priority="2" operator="notBetween">
+    <cfRule type="cellIs" dxfId="21" priority="2" operator="notBetween">
       <formula>2</formula>
       <formula>4</formula>
     </cfRule>
@@ -14442,16 +14503,16 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B29:C29">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="between">
+    <cfRule type="cellIs" dxfId="20" priority="1" operator="between">
       <formula>$B$23</formula>
       <formula>2+2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7:D7">
-    <cfRule type="duplicateValues" dxfId="1" priority="83"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="83"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B14:D14">
-    <cfRule type="uniqueValues" dxfId="0" priority="97"/>
+    <cfRule type="uniqueValues" dxfId="18" priority="97"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:J2">
     <cfRule type="colorScale" priority="45">
@@ -14874,7 +14935,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5CCC4B1-5C65-4837-AA26-56CCF06B63BB}">
   <dimension ref="A1:J34"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75"/>
   <cols>
     <col min="3" max="3" width="17.28515625" customWidth="1"/>
     <col min="4" max="4" width="9.5703125" customWidth="1"/>
@@ -14886,12 +14947,12 @@
     <col min="10" max="10" width="17.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10">
       <c r="A1" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" ht="15" x14ac:dyDescent="0.2">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="15">
       <c r="C3" s="17" t="s">
         <v>35</v>
       </c>
@@ -14899,25 +14960,25 @@
         <v>36</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="F3" s="17" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="G3" s="17" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="H3" s="17" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="I3" s="17" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="J3" s="17" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
       <c r="C4" s="104" t="s">
         <v>42</v>
       </c>
@@ -14948,7 +15009,7 @@
         <v>Rank</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10">
       <c r="C5" s="104" t="s">
         <v>44</v>
       </c>
@@ -14979,9 +15040,9 @@
         <v>Rank</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10">
       <c r="C6" s="104" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="D6" s="104">
         <f>SUBTOTAL(109,Table3[Age])</f>
@@ -15012,9 +15073,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:10">
       <c r="B8" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -15023,22 +15084,22 @@
         <v>2</v>
       </c>
       <c r="F8" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="G8" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="H8" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="I8" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="J8" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10">
       <c r="C9">
         <v>3</v>
       </c>
@@ -15066,18 +15127,18 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:10">
       <c r="B11" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="C11" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="D11" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10">
       <c r="C12">
         <v>3</v>
       </c>
@@ -15085,9 +15146,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:10">
       <c r="B14" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="C14">
         <v>1</v>
@@ -15096,7 +15157,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:10">
       <c r="C15">
         <v>3</v>
       </c>
@@ -15104,9 +15165,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:4">
       <c r="B17" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C17">
         <v>1</v>
@@ -15115,7 +15176,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:4">
       <c r="C18">
         <v>3</v>
       </c>
@@ -15123,9 +15184,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:4">
       <c r="B20" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C20">
         <v>1</v>
@@ -15134,7 +15195,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:4">
       <c r="C21">
         <v>3</v>
       </c>
@@ -15142,9 +15203,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:4">
       <c r="B23" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="C23">
         <v>1</v>
@@ -15153,7 +15214,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="24" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:4">
       <c r="C24">
         <v>3</v>
       </c>
@@ -15161,9 +15222,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="26" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="26" spans="2:4">
       <c r="B26" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="C26">
         <v>1</v>
@@ -15172,7 +15233,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="27" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="27" spans="2:4">
       <c r="C27">
         <v>3</v>
       </c>
@@ -15180,45 +15241,45 @@
         <v>4</v>
       </c>
     </row>
-    <row r="28" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="28" spans="2:4">
       <c r="C28" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="D28">
         <f>SUBTOTAL(109,Table4910[Column2])</f>
         <v>6</v>
       </c>
     </row>
-    <row r="30" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:4">
       <c r="B30" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="C30" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="D30" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="31" spans="2:4" hidden="1" x14ac:dyDescent="0.2">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="31" spans="2:4" hidden="1">
       <c r="C31" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="D31" t="s">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="32" spans="2:4" x14ac:dyDescent="0.2">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="32" spans="2:4">
       <c r="C32" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="D32" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="34" spans="2:2" x14ac:dyDescent="0.2">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="34" spans="2:2">
       <c r="B34" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
     </row>
   </sheetData>
@@ -15241,7 +15302,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE9224F2-4D06-4586-886C-E51F5EBCA7B0}">
   <dimension ref="A1:L21"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75"/>
   <cols>
     <col min="3" max="3" width="13.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.5703125" bestFit="1" customWidth="1"/>
@@ -15262,9 +15323,9 @@
     <col min="21" max="21" width="19.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" ht="15">
       <c r="A1" s="92" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="17"/>
@@ -15272,7 +15333,7 @@
       <c r="E1" s="17"/>
       <c r="F1" s="17"/>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:12">
       <c r="A2" s="104"/>
       <c r="B2" s="104"/>
       <c r="C2" s="104"/>
@@ -15280,21 +15341,21 @@
       <c r="E2" s="104"/>
       <c r="F2" s="104"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:12">
       <c r="A3" s="104"/>
       <c r="B3" s="104"/>
       <c r="C3" s="89" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="D3" s="89" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
       <c r="A4" s="104"/>
       <c r="B4" s="104"/>
       <c r="C4" s="89" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="D4">
         <v>12.1</v>
@@ -15321,10 +15382,10 @@
         <v>12052</v>
       </c>
       <c r="L4" t="s">
-        <v>416</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
       <c r="A5" s="104"/>
       <c r="B5" s="104"/>
       <c r="C5" s="90" t="s">
@@ -15337,7 +15398,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:12">
       <c r="A6" s="104"/>
       <c r="B6" s="104"/>
       <c r="C6" s="91">
@@ -15350,7 +15411,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:12">
       <c r="A7" s="104"/>
       <c r="B7" s="104"/>
       <c r="C7" s="90" t="s">
@@ -15363,7 +15424,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:12">
       <c r="A8" s="104"/>
       <c r="B8" s="104"/>
       <c r="C8" s="91">
@@ -15376,7 +15437,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:12">
       <c r="A9" s="104"/>
       <c r="B9" s="104"/>
       <c r="C9" s="90" t="s">
@@ -15389,7 +15450,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:12">
       <c r="A10" s="104"/>
       <c r="B10" s="104"/>
       <c r="C10" s="91">
@@ -15402,7 +15463,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:12">
       <c r="C11" s="90" t="s">
         <v>44</v>
       </c>
@@ -15413,7 +15474,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:12">
       <c r="C12" s="91">
         <v>23000</v>
       </c>
@@ -15424,7 +15485,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:12">
       <c r="C13" s="90" t="s">
         <v>50</v>
       </c>
@@ -15435,7 +15496,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:12">
       <c r="C14" s="91">
         <v>2</v>
       </c>
@@ -15446,7 +15507,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:12">
       <c r="C15" s="90" t="s">
         <v>48</v>
       </c>
@@ -15457,7 +15518,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:12">
       <c r="C16" s="91">
         <v>50024</v>
       </c>
@@ -15468,7 +15529,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="17" spans="3:12">
       <c r="C17" s="90" t="s">
         <v>53</v>
       </c>
@@ -15479,7 +15540,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="18" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="18" spans="3:12">
       <c r="C18" s="91">
         <v>189576</v>
       </c>
@@ -15490,7 +15551,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="19" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="19" spans="3:12">
       <c r="C19" s="90" t="s">
         <v>57</v>
       </c>
@@ -15501,7 +15562,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="20" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="20" spans="3:12">
       <c r="C20" s="91">
         <v>5000</v>
       </c>
@@ -15512,9 +15573,9 @@
         <v>37</v>
       </c>
     </row>
-    <row r="21" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="21" spans="3:12">
       <c r="C21" s="90" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="D21">
         <v>9</v>
@@ -15553,31 +15614,31 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C47BF70-BA80-4124-B359-67CBCB635390}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="65.140625" customWidth="1"/>
     <col min="2" max="26" width="13.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="B2" s="104"/>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
     </row>
   </sheetData>
@@ -15589,25 +15650,25 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FE31E21-0350-44E7-AF13-4CA140505B30}">
   <dimension ref="A1:B12"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="12.75"/>
   <sheetData>
-    <row r="1" spans="1:2" ht="51" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" ht="51">
       <c r="A1" s="99" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="B1" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="B7" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
       <c r="A8">
         <v>1</v>
       </c>
@@ -15615,7 +15676,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:2">
       <c r="A9">
         <v>2</v>
       </c>
@@ -15623,7 +15684,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:2">
       <c r="A10">
         <v>3</v>
       </c>
@@ -15631,7 +15692,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:2">
       <c r="A11">
         <v>4</v>
       </c>
@@ -15639,7 +15700,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:2">
       <c r="A12">
         <v>5</v>
       </c>

</xml_diff>

<commit_message>
[IMP] named ranges: add support of xlsx import/export
This commit introduces the support for named ranges in the import and
export of XLSX files.

Task: 5462359
</commit_message>
<xml_diff>
--- a/tests/__xlsx__/xlsx_demo_data.xlsx
+++ b/tests/__xlsx__/xlsx_demo_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rar/rar-workspace/o-spreadsheet/tests/__xlsx__/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\odoo\spreadsheet\tests\__xlsx__\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8C7959D-379F-564A-B7D4-13925F876C7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{346363BF-6AD4-4354-A44F-43A8F3AE431A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="23400" yWindow="2720" windowWidth="29040" windowHeight="15840" firstSheet="4" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-1860" windowWidth="29040" windowHeight="18240" firstSheet="5" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,6 +33,11 @@
   <externalReferences>
     <externalReference r:id="rId17"/>
   </externalReferences>
+  <definedNames>
+    <definedName name="My_Named_Range">jestMiscTest!$A$8:$B$10</definedName>
+    <definedName name="Table_Col_Named_Range">Table10[Col1]</definedName>
+    <definedName name="Table_Named_Range">Table10[]</definedName>
+  </definedNames>
   <calcPr calcId="191028"/>
   <pivotCaches>
     <pivotCache cacheId="0" r:id="rId18"/>
@@ -2986,7 +2991,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-GB"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -3603,7 +3608,7 @@
 <file path=xl/charts/chart10.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-GB"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -3966,7 +3971,7 @@
 <file path=xl/charts/chart11.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-GB"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="1"/>
   <c:style val="2"/>
   <c:chart>
@@ -4382,7 +4387,7 @@
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-GB"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <c:style val="2"/>
   <c:chart>
@@ -4848,7 +4853,7 @@
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-GB"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <c:style val="2"/>
   <c:chart>
@@ -5466,7 +5471,7 @@
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-GB"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -5832,7 +5837,7 @@
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-GB"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="1"/>
   <c:style val="2"/>
   <c:chart>
@@ -6144,7 +6149,7 @@
 <file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-GB"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -6575,7 +6580,7 @@
 <file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-GB"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -6977,7 +6982,7 @@
 <file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-GB"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -7280,7 +7285,7 @@
 <file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-GB"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -8771,6 +8776,9 @@
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:relativeUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Feuil1"/>
     </sheetNames>
@@ -9504,13 +9512,13 @@
     <tabColor rgb="FF00FF00"/>
   </sheetPr>
   <dimension ref="A1:L35"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="13.796875" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="13.85546875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="22.19921875" customWidth="1"/>
-    <col min="2" max="2" width="13.796875" customWidth="1"/>
-    <col min="3" max="3" width="13.796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="14.19921875" customWidth="1"/>
-    <col min="6" max="26" width="13.796875" customWidth="1"/>
+    <col min="1" max="1" width="22.140625" customWidth="1"/>
+    <col min="2" max="2" width="13.85546875" customWidth="1"/>
+    <col min="3" max="3" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="14.140625" customWidth="1"/>
+    <col min="6" max="26" width="13.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -9522,7 +9530,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="28" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:12" ht="27.75" x14ac:dyDescent="0.2">
       <c r="B2" s="22" t="s">
         <v>2</v>
       </c>
@@ -9949,7 +9957,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F7A934C-2218-4A12-8B75-EE28D615D774}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.796875" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -9958,7 +9966,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96301BE1-D86D-4D45-870D-85A75D53FC99}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.3984375" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -9967,10 +9975,10 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B10A8834-0E20-4F80-8813-3ACA5527B377}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="13.796875" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="13.85546875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="65.19921875" customWidth="1"/>
-    <col min="2" max="26" width="13.796875" customWidth="1"/>
+    <col min="1" max="1" width="65.140625" customWidth="1"/>
+    <col min="2" max="26" width="13.85546875" customWidth="1"/>
   </cols>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9984,7 +9992,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="14.3984375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9994,13 +10002,13 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{025F2510-D243-4DA1-81DE-BBDDA9BC3681}">
   <dimension ref="A1:J6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="4" width="14.19921875" customWidth="1"/>
-    <col min="5" max="5" width="14.796875" customWidth="1"/>
-    <col min="7" max="7" width="14.19921875" customWidth="1"/>
-    <col min="8" max="8" width="20.19921875" customWidth="1"/>
-    <col min="9" max="9" width="17.19921875" customWidth="1"/>
+    <col min="3" max="4" width="14.140625" customWidth="1"/>
+    <col min="5" max="5" width="14.85546875" customWidth="1"/>
+    <col min="7" max="7" width="14.140625" customWidth="1"/>
+    <col min="8" max="8" width="20.140625" customWidth="1"/>
+    <col min="9" max="9" width="17.140625" customWidth="1"/>
     <col min="10" max="10" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -10241,7 +10249,7 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{175FB5D6-D3ED-FD4F-886B-71BD0CB28755}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="1" selectUnlockedCells="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -10251,7 +10259,7 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B936FE7B-5147-E945-A711-7FBABD0575D3}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -10264,9 +10272,9 @@
     <tabColor theme="9"/>
   </sheetPr>
   <dimension ref="A1:R163"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="13.796875" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="13.85546875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="26" width="13.796875" customWidth="1"/>
+    <col min="1" max="26" width="13.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -12117,7 +12125,7 @@
       </c>
       <c r="B100" s="19">
         <f ca="1">NOW()</f>
-        <v>46050.431470138887</v>
+        <v>46113.450567939813</v>
       </c>
       <c r="D100" s="104">
         <f ca="1">IF(ISNUMBER(B100),1,0)</f>
@@ -12807,7 +12815,7 @@
       </c>
       <c r="B144" s="18">
         <f ca="1">TODAY()</f>
-        <v>46050</v>
+        <v>46113</v>
       </c>
       <c r="D144" s="104">
         <f ca="1">IF(ISNUMBER(B144),1,0)</f>
@@ -13139,14 +13147,14 @@
     <outlinePr summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:R31"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.19921875" defaultRowHeight="14" outlineLevelRow="2" outlineLevelCol="2" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" outlineLevelRow="2" outlineLevelCol="2" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="0" hidden="1" customWidth="1"/>
-    <col min="6" max="6" width="14.19921875" customWidth="1"/>
-    <col min="10" max="10" width="9.19921875" outlineLevel="1"/>
-    <col min="11" max="11" width="9.19921875" outlineLevel="1" collapsed="1"/>
+    <col min="6" max="6" width="14.140625" customWidth="1"/>
+    <col min="10" max="10" width="9.140625" outlineLevel="1"/>
+    <col min="11" max="11" width="9.140625" outlineLevel="1" collapsed="1"/>
     <col min="12" max="14" width="0" hidden="1" outlineLevel="2"/>
-    <col min="15" max="18" width="9.19921875" outlineLevel="1"/>
+    <col min="15" max="18" width="9.140625" outlineLevel="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
@@ -13209,21 +13217,21 @@
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" cm="1">
         <f t="array" aca="1" ref="A30:B31" ca="1">_xlfn.RANDARRAY(2,2)</f>
-        <v>0.77093979243831789</v>
+        <v>0.46080895274950051</v>
       </c>
       <c r="B30">
         <f ca="1"/>
-        <v>0.89996963625071968</v>
+        <v>0.12189382146451888</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31">
         <f ca="1"/>
-        <v>4.753041610255937E-2</v>
+        <v>0.83857971910007767</v>
       </c>
       <c r="B31">
         <f ca="1"/>
-        <v>0.61224139121963739</v>
+        <v>0.50857115329836389</v>
       </c>
     </row>
   </sheetData>
@@ -13242,14 +13250,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF68F2C0-1053-4FB6-BD74-8A11B0CAF123}">
   <dimension ref="A1:M30"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.19921875" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="17.796875" customWidth="1"/>
-    <col min="5" max="5" width="18.19921875" customWidth="1"/>
-    <col min="13" max="13" width="10.3984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.85546875" customWidth="1"/>
+    <col min="5" max="5" width="18.140625" customWidth="1"/>
+    <col min="13" max="13" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="68" t="s">
         <v>239</v>
       </c>
@@ -13320,7 +13328,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="16" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" ht="15" x14ac:dyDescent="0.3">
       <c r="A4" s="42" t="s">
         <v>256</v>
       </c>
@@ -13389,7 +13397,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="45" t="s">
         <v>271</v>
       </c>
@@ -13409,7 +13417,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="21" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" ht="21" x14ac:dyDescent="0.35">
       <c r="A8" s="46" t="s">
         <v>275</v>
       </c>
@@ -13432,7 +13440,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:13" ht="15" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="47" t="s">
         <v>280</v>
       </c>
@@ -13457,7 +13465,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="49" t="s">
         <v>285</v>
       </c>
@@ -13530,12 +13538,12 @@
         <v>248</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A17" s="55" t="s">
         <v>296</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A18" s="74" t="s">
         <v>297</v>
       </c>
@@ -13547,7 +13555,7 @@
       </c>
       <c r="F18" s="36"/>
     </row>
-    <row r="19" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A19" s="75" t="s">
         <v>300</v>
       </c>
@@ -13558,7 +13566,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="61" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" ht="51.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A20" s="76" t="s">
         <v>303</v>
       </c>
@@ -13572,12 +13580,12 @@
         <v>302</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A21" s="77" t="s">
         <v>306</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A22" s="78" t="s">
         <v>307</v>
       </c>
@@ -13586,13 +13594,13 @@
       </c>
       <c r="E22" s="21"/>
     </row>
-    <row r="23" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A23" s="79" t="s">
         <v>309</v>
       </c>
       <c r="E23" s="21"/>
     </row>
-    <row r="24" spans="1:6" ht="16" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" ht="14.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A24" s="80" t="s">
         <v>310</v>
       </c>
@@ -13601,19 +13609,19 @@
       </c>
       <c r="E24" s="21"/>
     </row>
-    <row r="25" spans="1:6" ht="16" thickTop="1" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="26" spans="1:6" ht="16" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" ht="14.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="1:6" ht="14.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="C26" s="67" t="s">
         <v>312</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="16" thickTop="1" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="1:6" ht="16" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" ht="14.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="28" spans="1:6" ht="14.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="C28" s="88" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="29" spans="1:6" ht="13.5" thickTop="1" x14ac:dyDescent="0.2"/>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="C30" s="87" t="s">
         <v>314</v>
@@ -13628,13 +13636,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D919E811-4385-4D35-A19E-3B7E0E659A89}">
   <dimension ref="A1:L39"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.3984375" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.19921875" customWidth="1"/>
-    <col min="7" max="7" width="15.796875" customWidth="1"/>
+    <col min="1" max="1" width="19.140625" customWidth="1"/>
+    <col min="7" max="7" width="15.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="37" t="s">
         <v>315</v>
       </c>
@@ -13810,7 +13818,7 @@
       </c>
       <c r="C9" s="21"/>
     </row>
-    <row r="10" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="38" t="s">
         <v>340</v>
       </c>
@@ -13857,7 +13865,7 @@
       </c>
       <c r="B12" s="39">
         <f ca="1">TODAY()</f>
-        <v>46050</v>
+        <v>46113</v>
       </c>
       <c r="C12" s="39">
         <f>DATE(2010,10,2)</f>
@@ -14296,7 +14304,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:12" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="G31" s="35" t="s">
         <v>378</v>
       </c>
@@ -14963,16 +14971,16 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5CCC4B1-5C65-4837-AA26-56CCF06B63BB}">
   <dimension ref="A1:J34"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.19921875" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="17.19921875" customWidth="1"/>
-    <col min="4" max="4" width="9.59765625" customWidth="1"/>
-    <col min="5" max="5" width="26.3984375" customWidth="1"/>
-    <col min="6" max="6" width="27.59765625" customWidth="1"/>
-    <col min="7" max="7" width="23.59765625" customWidth="1"/>
-    <col min="8" max="8" width="16.19921875" customWidth="1"/>
-    <col min="9" max="9" width="18.796875" customWidth="1"/>
-    <col min="10" max="10" width="17.19921875" customWidth="1"/>
+    <col min="3" max="3" width="17.140625" customWidth="1"/>
+    <col min="4" max="4" width="9.5703125" customWidth="1"/>
+    <col min="5" max="5" width="26.42578125" customWidth="1"/>
+    <col min="6" max="6" width="27.5703125" customWidth="1"/>
+    <col min="7" max="7" width="23.5703125" customWidth="1"/>
+    <col min="8" max="8" width="16.140625" customWidth="1"/>
+    <col min="9" max="9" width="18.85546875" customWidth="1"/>
+    <col min="10" max="10" width="17.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
@@ -14980,7 +14988,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" ht="15" x14ac:dyDescent="0.2">
       <c r="C3" s="17" t="s">
         <v>35</v>
       </c>
@@ -15330,28 +15338,28 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE9224F2-4D06-4586-886C-E51F5EBCA7B0}">
   <dimension ref="A1:L21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.19921875" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="13.19921875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.59765625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="6" width="6" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="7" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="5" bestFit="1" customWidth="1"/>
     <col min="9" max="10" width="7" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="6" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="10" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.796875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.796875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.796875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="9.796875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="14.796875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.796875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="14.796875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="14.19921875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="19.19921875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="19.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" ht="15" x14ac:dyDescent="0.2">
       <c r="A1" s="92" t="s">
         <v>413</v>
       </c>
@@ -15361,7 +15369,7 @@
       <c r="E1" s="17"/>
       <c r="F1" s="17"/>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:12" ht="14.1" x14ac:dyDescent="0.2">
       <c r="A2" s="104"/>
       <c r="B2" s="104"/>
       <c r="C2" s="104"/>
@@ -15369,7 +15377,7 @@
       <c r="E2" s="104"/>
       <c r="F2" s="104"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:12" ht="14.1" x14ac:dyDescent="0.2">
       <c r="A3" s="104"/>
       <c r="B3" s="104"/>
       <c r="C3" s="89" t="s">
@@ -15379,7 +15387,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:12" ht="14.1" x14ac:dyDescent="0.2">
       <c r="A4" s="104"/>
       <c r="B4" s="104"/>
       <c r="C4" s="89" t="s">
@@ -15413,7 +15421,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:12" ht="14.1" x14ac:dyDescent="0.2">
       <c r="A5" s="104"/>
       <c r="B5" s="104"/>
       <c r="C5" s="90" t="s">
@@ -15426,7 +15434,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:12" ht="14.1" x14ac:dyDescent="0.2">
       <c r="A6" s="104"/>
       <c r="B6" s="104"/>
       <c r="C6" s="91">
@@ -15439,7 +15447,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:12" ht="14.1" x14ac:dyDescent="0.2">
       <c r="A7" s="104"/>
       <c r="B7" s="104"/>
       <c r="C7" s="90" t="s">
@@ -15452,7 +15460,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:12" ht="14.1" x14ac:dyDescent="0.2">
       <c r="A8" s="104"/>
       <c r="B8" s="104"/>
       <c r="C8" s="91">
@@ -15465,7 +15473,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:12" ht="14.1" x14ac:dyDescent="0.2">
       <c r="A9" s="104"/>
       <c r="B9" s="104"/>
       <c r="C9" s="90" t="s">
@@ -15478,7 +15486,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:12" ht="14.1" x14ac:dyDescent="0.2">
       <c r="A10" s="104"/>
       <c r="B10" s="104"/>
       <c r="C10" s="91">
@@ -15491,7 +15499,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:12" ht="14.1" x14ac:dyDescent="0.2">
       <c r="C11" s="90" t="s">
         <v>44</v>
       </c>
@@ -15502,7 +15510,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:12" ht="14.1" x14ac:dyDescent="0.2">
       <c r="C12" s="91">
         <v>23000</v>
       </c>
@@ -15513,7 +15521,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:12" ht="14.1" x14ac:dyDescent="0.2">
       <c r="C13" s="90" t="s">
         <v>50</v>
       </c>
@@ -15524,7 +15532,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:12" ht="14.1" x14ac:dyDescent="0.2">
       <c r="C14" s="91">
         <v>2</v>
       </c>
@@ -15535,7 +15543,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:12" ht="14.1" x14ac:dyDescent="0.2">
       <c r="C15" s="90" t="s">
         <v>48</v>
       </c>
@@ -15546,7 +15554,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:12" ht="14.1" x14ac:dyDescent="0.2">
       <c r="C16" s="91">
         <v>50024</v>
       </c>
@@ -15557,7 +15565,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="17" spans="3:12" ht="14.1" x14ac:dyDescent="0.2">
       <c r="C17" s="90" t="s">
         <v>53</v>
       </c>
@@ -15568,7 +15576,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="18" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="18" spans="3:12" ht="14.1" x14ac:dyDescent="0.2">
       <c r="C18" s="91">
         <v>189576</v>
       </c>
@@ -15579,7 +15587,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="19" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="19" spans="3:12" ht="14.1" x14ac:dyDescent="0.2">
       <c r="C19" s="90" t="s">
         <v>57</v>
       </c>
@@ -15590,7 +15598,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="20" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="20" spans="3:12" ht="14.1" x14ac:dyDescent="0.2">
       <c r="C20" s="91">
         <v>5000</v>
       </c>
@@ -15601,7 +15609,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="21" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="21" spans="3:12" ht="14.1" x14ac:dyDescent="0.2">
       <c r="C21" s="90" t="s">
         <v>417</v>
       </c>
@@ -15642,10 +15650,10 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C47BF70-BA80-4124-B359-67CBCB635390}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="13.796875" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="13.85546875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="65.19921875" customWidth="1"/>
-    <col min="2" max="26" width="13.796875" customWidth="1"/>
+    <col min="1" max="1" width="65.140625" customWidth="1"/>
+    <col min="2" max="26" width="13.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
@@ -15678,9 +15686,9 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FE31E21-0350-44E7-AF13-4CA140505B30}">
   <dimension ref="A1:B12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.796875" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:2" ht="60" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" ht="51" x14ac:dyDescent="0.2">
       <c r="A1" s="99" t="s">
         <v>422</v>
       </c>

</xml_diff>

<commit_message>
[FIX] data validation: import formula from excel
When importing a data validation rule with formulas
the "=" was missing after the import

closes odoo/o-spreadsheet#7848

Task: 4975550
Signed-off-by: Rémi Rahir (rar) <rar@odoo.com>
</commit_message>
<xml_diff>
--- a/tests/__xlsx__/xlsx_demo_data.xlsx
+++ b/tests/__xlsx__/xlsx_demo_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29816"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dhrutik Patel\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48DA6F05-B302-48AE-B11C-1FB2528D58DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1B86E9B1-DF37-4B7C-B14C-0625DAE1CA60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="4" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -31,9 +31,9 @@
   <externalReferences>
     <externalReference r:id="rId15"/>
   </externalReferences>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191028" calcCompleted="0"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId16"/>
+    <pivotCache cacheId="4560" r:id="rId16"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -46,6 +46,7 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
@@ -1203,6 +1204,9 @@
     <t>5Rating</t>
   </si>
   <si>
+    <t>CF with formulas</t>
+  </si>
+  <si>
     <t>5Quarters</t>
   </si>
   <si>
@@ -1397,9 +1401,6 @@
   </si>
   <si>
     <t>A1234556</t>
-  </si>
-  <si>
-    <t>CF with formulas</t>
   </si>
 </sst>
 </file>
@@ -1414,7 +1415,7 @@
     <numFmt numFmtId="168" formatCode="#,##0&quot; EUR €&quot;"/>
     <numFmt numFmtId="169" formatCode="&quot;€&quot;#,##0.00\ &quot;€&quot;"/>
   </numFmts>
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="26">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -2414,7 +2415,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -2427,13 +2427,165 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="3">
-    <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
+    <cellStyle name="Lien hypertexte" xfId="2" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{1493241F-B85D-4F84-BBA0-86191B8FD032}"/>
   </cellStyles>
   <dxfs count="47">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+        <strike/>
+        <u/>
+        <color theme="7"/>
+      </font>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <fill>
+        <patternFill patternType="lightTrellis">
+          <fgColor theme="4"/>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE06666"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFB6D7A8"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9900"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -2847,157 +2999,6 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-        <strike/>
-        <u/>
-        <color theme="7"/>
-      </font>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <fill>
-        <patternFill patternType="lightTrellis">
-          <fgColor theme="4"/>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE06666"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFB6D7A8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF9900"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor theme="4"/>
         </patternFill>
       </fill>
@@ -3041,7 +3042,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="fr-FR"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -3642,7 +3643,7 @@
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="fr-FR"/>
   <c:roundedCorners val="0"/>
   <c:style val="2"/>
   <c:chart>
@@ -4074,7 +4075,7 @@
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="fr-FR"/>
   <c:roundedCorners val="0"/>
   <c:style val="2"/>
   <c:chart>
@@ -4692,7 +4693,7 @@
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="fr-FR"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -5058,7 +5059,7 @@
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="fr-FR"/>
   <c:roundedCorners val="1"/>
   <c:style val="2"/>
   <c:chart>
@@ -5357,7 +5358,7 @@
 <file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="fr-FR"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -5774,7 +5775,7 @@
 <file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="fr-FR"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -6176,7 +6177,7 @@
 <file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="fr-FR"/>
   <c:roundedCorners val="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -6466,7 +6467,7 @@
 <file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="fr-FR"/>
   <c:roundedCorners val="1"/>
   <c:style val="2"/>
   <c:chart>
@@ -7798,6 +7799,9 @@
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:relativeUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Feuil1"/>
     </sheetNames>
@@ -7933,7 +7937,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9B3CE3F5-58D8-48A3-B9C6-24D1506C9F5C}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9B3CE3F5-58D8-48A3-B9C6-24D1506C9F5C}" name="PivotTable1" cacheId="4560" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="C3:L21" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="5">
     <pivotField axis="axisRow" showAll="0">
@@ -8083,7 +8087,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{09C35CC7-7259-4A97-8FEA-EDB47375DF08}" name="Table3" displayName="Table3" ref="C3:J6" totalsRowCount="1" headerRowDxfId="44" dataDxfId="43">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{09C35CC7-7259-4A97-8FEA-EDB47375DF08}" name="Table3" displayName="Table3" ref="C3:J6" totalsRowCount="1" headerRowDxfId="17" dataDxfId="16">
   <autoFilter ref="C3:J5" xr:uid="{09C35CC7-7259-4A97-8FEA-EDB47375DF08}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -8095,22 +8099,22 @@
     <filterColumn colId="7" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{C4EE018E-238B-42BA-9035-DB01FA5420D3}" name="Name" totalsRowLabel="Total" dataDxfId="42" totalsRowDxfId="41"/>
-    <tableColumn id="2" xr3:uid="{C1F6911F-9482-4C98-BBFB-21D9CAA66DA4}" name="Age" totalsRowFunction="sum" dataDxfId="40" totalsRowDxfId="39"/>
-    <tableColumn id="5" xr3:uid="{3CE9F5DA-0A57-4696-B4E0-53601C3B7798}" name="Rank" totalsRowFunction="sum" dataDxfId="38" totalsRowDxfId="37"/>
-    <tableColumn id="6" xr3:uid="{34912838-665C-4472-B558-25990E5B148D}" name="Rank+Age =E4+D4" totalsRowFunction="sum" dataDxfId="36" totalsRowDxfId="35">
+    <tableColumn id="1" xr3:uid="{C4EE018E-238B-42BA-9035-DB01FA5420D3}" name="Name" totalsRowLabel="Total" dataDxfId="14" totalsRowDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{C1F6911F-9482-4C98-BBFB-21D9CAA66DA4}" name="Age" totalsRowFunction="sum" dataDxfId="12" totalsRowDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{3CE9F5DA-0A57-4696-B4E0-53601C3B7798}" name="Rank" totalsRowFunction="sum" dataDxfId="10" totalsRowDxfId="11"/>
+    <tableColumn id="6" xr3:uid="{34912838-665C-4472-B558-25990E5B148D}" name="Rank+Age =E4+D4" totalsRowFunction="sum" dataDxfId="8" totalsRowDxfId="9">
       <calculatedColumnFormula>Table3[[#This Row],[Rank]]+Table3[[#This Row],[Age]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{89D90022-7073-4067-BAF8-1587D27C4AFB}" name="Data =SUM(E4:E5)" totalsRowFunction="sum" dataDxfId="34" totalsRowDxfId="33">
+    <tableColumn id="7" xr3:uid="{89D90022-7073-4067-BAF8-1587D27C4AFB}" name="Data =SUM(E4:E5)" totalsRowFunction="sum" dataDxfId="6" totalsRowDxfId="7">
       <calculatedColumnFormula>SUM(Table3[Rank])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{B2A7E5BB-A379-492B-9484-72F2FD1FF3A0}" name="All =SUM(E3:E6)" totalsRowFunction="sum" dataDxfId="32" totalsRowDxfId="31">
+    <tableColumn id="8" xr3:uid="{B2A7E5BB-A379-492B-9484-72F2FD1FF3A0}" name="All =SUM(E3:E6)" totalsRowFunction="sum" dataDxfId="4" totalsRowDxfId="5">
       <calculatedColumnFormula>SUM(Table3[[#All],[Rank]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{3C532A69-E4BC-4A20-A922-4BCAA0D3FEC9}" name="Totals =E6" totalsRowFunction="sum" dataDxfId="30" totalsRowDxfId="29">
+    <tableColumn id="9" xr3:uid="{3C532A69-E4BC-4A20-A922-4BCAA0D3FEC9}" name="Totals =E6" totalsRowFunction="sum" dataDxfId="2" totalsRowDxfId="3">
       <calculatedColumnFormula>Table3[[#Totals],[Rank]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{35E9E9C3-9148-468A-85B6-19290CEB6F00}" name="Headers =E3" totalsRowFunction="sum" dataDxfId="28" totalsRowDxfId="27">
+    <tableColumn id="10" xr3:uid="{35E9E9C3-9148-468A-85B6-19290CEB6F00}" name="Headers =E3" totalsRowFunction="sum" dataDxfId="0" totalsRowDxfId="1">
       <calculatedColumnFormula>Table3[[#Headers],[Rank]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -8531,7 +8535,7 @@
     <tabColor rgb="FF00FF00"/>
   </sheetPr>
   <dimension ref="A1:L35"/>
-  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="22.28515625" customWidth="1"/>
     <col min="2" max="2" width="13.7109375" customWidth="1"/>
@@ -8540,7 +8544,7 @@
     <col min="6" max="26" width="13.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" ht="38.25" customHeight="1">
       <c r="A1" s="21"/>
       <c r="C1" s="1" t="s">
         <v>0</v>
@@ -8549,7 +8553,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="27.75" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:12" ht="27.75">
       <c r="B2" s="22" t="s">
         <v>2</v>
       </c>
@@ -8562,25 +8566,25 @@
       <c r="H2" s="118" t="s">
         <v>4</v>
       </c>
-      <c r="I2" s="119"/>
+      <c r="I2" s="123"/>
       <c r="K2" s="3"/>
     </row>
-    <row r="3" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:12" ht="17.25" customHeight="1">
       <c r="F3" s="4" t="s">
         <v>5</v>
       </c>
       <c r="G3" s="117">
         <v>8</v>
       </c>
-      <c r="H3" s="119"/>
-      <c r="I3" s="119"/>
+      <c r="H3" s="123"/>
+      <c r="I3" s="123"/>
       <c r="J3" s="5"/>
-      <c r="K3" s="120">
+      <c r="K3" s="119">
         <v>5</v>
       </c>
       <c r="L3" s="6"/>
     </row>
-    <row r="4" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:12" ht="17.25" customHeight="1">
       <c r="B4" s="7" t="s">
         <v>6</v>
       </c>
@@ -8593,50 +8597,50 @@
       <c r="G4" s="117">
         <v>9</v>
       </c>
-      <c r="H4" s="119"/>
-      <c r="I4" s="119"/>
+      <c r="H4" s="123"/>
+      <c r="I4" s="123"/>
       <c r="J4" s="5"/>
-      <c r="K4" s="121"/>
+      <c r="K4" s="120"/>
       <c r="L4" s="6"/>
     </row>
-    <row r="5" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:12" ht="17.25" customHeight="1">
       <c r="C5" s="117">
         <v>42</v>
       </c>
       <c r="G5" s="117">
         <v>15</v>
       </c>
-      <c r="H5" s="119"/>
-      <c r="I5" s="119"/>
+      <c r="H5" s="123"/>
+      <c r="I5" s="123"/>
       <c r="J5" s="5"/>
-      <c r="K5" s="121"/>
+      <c r="K5" s="120"/>
       <c r="L5" s="6"/>
     </row>
-    <row r="6" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:12" ht="17.25" customHeight="1">
       <c r="G6" s="117">
         <v>22</v>
       </c>
       <c r="J6" s="5"/>
-      <c r="K6" s="121"/>
+      <c r="K6" s="120"/>
       <c r="L6" s="6"/>
     </row>
-    <row r="7" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:12" ht="17.25" customHeight="1">
       <c r="C7" s="117">
         <v>3</v>
       </c>
       <c r="J7" s="5"/>
-      <c r="K7" s="121"/>
+      <c r="K7" s="120"/>
       <c r="L7" s="6"/>
     </row>
-    <row r="8" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:12" ht="17.25" customHeight="1">
       <c r="G8" s="117">
         <v>30</v>
       </c>
       <c r="J8" s="5"/>
-      <c r="K8" s="122"/>
+      <c r="K8" s="121"/>
       <c r="L8" s="6"/>
     </row>
-    <row r="9" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:12" ht="17.25" customHeight="1">
       <c r="B9" s="9" t="s">
         <v>8</v>
       </c>
@@ -8646,7 +8650,7 @@
       </c>
       <c r="K9" s="10"/>
     </row>
-    <row r="10" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:12" ht="17.25" customHeight="1">
       <c r="C10" s="117">
         <f>SUM(C4:C7)</f>
         <v>57.4</v>
@@ -8655,13 +8659,13 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:12" ht="17.25" customHeight="1">
       <c r="C11" s="117">
         <f>-(3+C7*SUM(C4:C7))</f>
         <v>-175.2</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:12" ht="17.25" customHeight="1">
       <c r="C12" s="117">
         <f>SUM(C9:C11)</f>
         <v>-63.399999999999991</v>
@@ -8670,13 +8674,13 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:12" ht="17.25" customHeight="1">
       <c r="G13" s="117">
         <f>A1+A2+A3+A4+A5+A6+A7+A8+A9+A10+A11+A12+A13+A14+A15+A16+A17+A18</f>
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:12" ht="17.25" customHeight="1">
       <c r="B14" s="11" t="s">
         <v>11</v>
       </c>
@@ -8685,32 +8689,32 @@
         <v>#CYCLE</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:12" ht="17.25" customHeight="1">
       <c r="C15" s="117" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:12" ht="17.25" customHeight="1">
       <c r="C16" s="117" t="str">
         <f>C15</f>
         <v>=(+</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:9" ht="17.25" customHeight="1">
       <c r="C17" s="117" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:9" ht="17.25" customHeight="1">
       <c r="C18" s="117" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:9" ht="17.25" customHeight="1">
       <c r="E19" s="3"/>
       <c r="G19" s="3"/>
     </row>
-    <row r="20" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:9" ht="17.25" customHeight="1">
       <c r="B20" s="5"/>
       <c r="C20" s="6" t="s">
         <v>15</v>
@@ -8724,7 +8728,7 @@
       </c>
       <c r="H20" s="6"/>
     </row>
-    <row r="21" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:9" ht="17.25" customHeight="1">
       <c r="A21" s="13" t="s">
         <v>18</v>
       </c>
@@ -8734,7 +8738,7 @@
       </c>
       <c r="G21" s="10"/>
     </row>
-    <row r="23" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:9" ht="17.25" customHeight="1">
       <c r="A23" s="13" t="s">
         <v>19</v>
       </c>
@@ -8748,7 +8752,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:9" ht="17.25" customHeight="1">
       <c r="C24" s="16">
         <v>10</v>
       </c>
@@ -8759,7 +8763,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:9" ht="17.25" customHeight="1">
       <c r="C25" s="16">
         <v>10.122999999999999</v>
       </c>
@@ -8770,7 +8774,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:9" ht="17.25" customHeight="1">
       <c r="B26" s="117" t="s">
         <v>20</v>
       </c>
@@ -8784,7 +8788,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:9" ht="17.25" customHeight="1">
       <c r="A27" s="117" t="s">
         <v>22</v>
       </c>
@@ -8801,7 +8805,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:9" ht="17.25" customHeight="1">
       <c r="A28" s="117" t="s">
         <v>23</v>
       </c>
@@ -8818,7 +8822,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:9" ht="17.25" customHeight="1">
       <c r="A29" s="117" t="s">
         <v>24</v>
       </c>
@@ -8835,7 +8839,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:9" ht="17.25" customHeight="1">
       <c r="A30" s="117" t="s">
         <v>25</v>
       </c>
@@ -8852,7 +8856,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:9" ht="17.25" customHeight="1">
       <c r="A31" s="117" t="s">
         <v>26</v>
       </c>
@@ -8869,7 +8873,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:9" ht="17.25" customHeight="1">
       <c r="A32" s="117" t="s">
         <v>27</v>
       </c>
@@ -8886,7 +8890,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:9" ht="17.25" customHeight="1">
       <c r="A33" s="117" t="s">
         <v>28</v>
       </c>
@@ -8903,7 +8907,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:9" ht="17.25" customHeight="1">
       <c r="A34" s="117" t="s">
         <v>29</v>
       </c>
@@ -8914,7 +8918,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="35" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:9" ht="17.25" customHeight="1">
       <c r="A35" s="117" t="s">
         <v>30</v>
       </c>
@@ -8931,7 +8935,7 @@
     <mergeCell ref="K3:K8"/>
   </mergeCells>
   <conditionalFormatting sqref="C1:C100 B21">
-    <cfRule type="cellIs" dxfId="26" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="44" priority="1" operator="equal">
       <formula>42</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8976,7 +8980,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F7A934C-2218-4A12-8B75-EE28D615D774}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="12.75"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -8985,7 +8989,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96301BE1-D86D-4D45-870D-85A75D53FC99}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -8994,7 +8998,7 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B10A8834-0E20-4F80-8813-3ACA5527B377}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="65.140625" customWidth="1"/>
     <col min="2" max="26" width="13.7109375" customWidth="1"/>
@@ -9011,7 +9015,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9020,8 +9024,8 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{025F2510-D243-4DA1-81DE-BBDDA9BC3681}">
-  <dimension ref="A1:I6"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:J6"/>
+  <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="3" max="4" width="14.28515625" customWidth="1"/>
     <col min="5" max="5" width="14.7109375" customWidth="1"/>
@@ -9030,36 +9034,36 @@
     <col min="9" max="9" width="17.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10">
       <c r="A1" s="114" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="B1" s="115" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="C1" s="115" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="D1" s="115" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="E1" s="115" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="F1" s="115" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="G1" s="115" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="H1" s="115" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="I1" s="116" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
       <c r="A2" s="104">
         <v>4</v>
       </c>
@@ -9070,7 +9074,7 @@
         <v>1</v>
       </c>
       <c r="D2" s="105" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="E2" s="106">
         <v>45575</v>
@@ -9079,7 +9083,7 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="G2" s="107" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="H2" s="106">
         <v>45292</v>
@@ -9087,8 +9091,11 @@
       <c r="I2" s="108">
         <v>4</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
       <c r="A3" s="104">
         <v>3</v>
       </c>
@@ -9099,7 +9106,7 @@
         <v>2</v>
       </c>
       <c r="D3" s="105" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="E3" s="106">
         <v>45576</v>
@@ -9108,16 +9115,19 @@
         <v>0.57638888888888884</v>
       </c>
       <c r="G3" s="107" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="H3" s="106">
         <v>45231</v>
       </c>
       <c r="I3" s="108" t="s">
-        <v>433</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+        <v>434</v>
+      </c>
+      <c r="J3">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
       <c r="A4" s="104">
         <v>9</v>
       </c>
@@ -9128,7 +9138,7 @@
         <v>3</v>
       </c>
       <c r="D4" s="105" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="E4" s="106">
         <v>45574</v>
@@ -9137,7 +9147,7 @@
         <v>0.73958333333333337</v>
       </c>
       <c r="G4" s="107" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="H4" s="106">
         <v>45325</v>
@@ -9145,8 +9155,11 @@
       <c r="I4" s="108">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J4">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
       <c r="A5" s="104">
         <v>5</v>
       </c>
@@ -9157,7 +9170,7 @@
         <v>4</v>
       </c>
       <c r="D5" s="105" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="E5" s="106">
         <v>45573</v>
@@ -9166,7 +9179,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="G5" s="105" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="H5" s="106">
         <v>45084</v>
@@ -9174,8 +9187,11 @@
       <c r="I5" s="108">
         <v>3</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J5">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
       <c r="A6" s="109">
         <v>7</v>
       </c>
@@ -9186,7 +9202,7 @@
         <v>5</v>
       </c>
       <c r="D6" s="110" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="E6" s="111">
         <v>45566</v>
@@ -9195,17 +9211,20 @@
         <v>0.5229166666666667</v>
       </c>
       <c r="G6" s="110" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="H6" s="111">
         <v>45420</v>
       </c>
       <c r="I6" s="113" t="s">
-        <v>438</v>
+        <v>439</v>
+      </c>
+      <c r="J6">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="9">
+  <dataValidations count="10">
     <dataValidation type="whole" errorStyle="warning" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2:A6" xr:uid="{B9309757-E2F4-49A1-880B-2F47F04364D6}">
       <formula1>1</formula1>
       <formula2>5</formula2>
@@ -9237,6 +9256,10 @@
     <dataValidation type="list" errorStyle="warning" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D6" xr:uid="{1E18A174-B5CF-4015-B7DC-F1491351E054}">
       <formula1>"option1,option2,option3"</formula1>
     </dataValidation>
+    <dataValidation type="decimal" errorStyle="warning" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J6" xr:uid="{EAFFF3C7-1A46-48EE-850D-DE4852C6359D}">
+      <formula1>$A$2</formula1>
+      <formula2>2+10</formula2>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -9248,12 +9271,12 @@
     <tabColor theme="9"/>
   </sheetPr>
   <dimension ref="A1:R163"/>
-  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="26" width="13.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:18" ht="17.25" customHeight="1">
       <c r="A1" s="117" t="s">
         <v>31</v>
       </c>
@@ -9288,7 +9311,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:18" ht="17.25" customHeight="1">
       <c r="A2" s="117" t="s">
         <v>41</v>
       </c>
@@ -9334,7 +9357,7 @@
         <v>1230.7</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:18" ht="17.25" customHeight="1">
       <c r="A3" s="117" t="s">
         <v>43</v>
       </c>
@@ -9380,7 +9403,7 @@
         <v>1217.7</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:18" ht="17.25" customHeight="1">
       <c r="A4" s="117" t="s">
         <v>45</v>
       </c>
@@ -9426,7 +9449,7 @@
         <v>1230.7</v>
       </c>
     </row>
-    <row r="5" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:18" ht="17.25" customHeight="1">
       <c r="A5" s="117" t="s">
         <v>47</v>
       </c>
@@ -9472,7 +9495,7 @@
         <v>1246.7</v>
       </c>
     </row>
-    <row r="6" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:18" ht="17.25" customHeight="1">
       <c r="A6" s="117" t="s">
         <v>49</v>
       </c>
@@ -9518,7 +9541,7 @@
         <v>1213.7</v>
       </c>
     </row>
-    <row r="7" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:18" ht="17.25" customHeight="1">
       <c r="A7" s="117" t="s">
         <v>52</v>
       </c>
@@ -9552,7 +9575,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:18" ht="17.25" customHeight="1">
       <c r="A8" s="117" t="s">
         <v>54</v>
       </c>
@@ -9586,7 +9609,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:18" ht="17.25" customHeight="1">
       <c r="A9" s="117" t="s">
         <v>56</v>
       </c>
@@ -9617,7 +9640,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:18" ht="17.25" customHeight="1">
       <c r="A10" s="117" t="s">
         <v>58</v>
       </c>
@@ -9633,7 +9656,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:18" ht="17.25" customHeight="1">
       <c r="A11" s="117" t="s">
         <v>59</v>
       </c>
@@ -9652,7 +9675,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="12" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:18" ht="17.25" customHeight="1">
       <c r="A12" s="117" t="s">
         <v>61</v>
       </c>
@@ -9683,7 +9706,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="13" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:18" ht="17.25" customHeight="1">
       <c r="A13" s="117" t="s">
         <v>62</v>
       </c>
@@ -9714,7 +9737,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="14" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:18" ht="17.25" customHeight="1">
       <c r="A14" s="117" t="s">
         <v>67</v>
       </c>
@@ -9730,7 +9753,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:18" ht="17.25" customHeight="1">
       <c r="A15" s="117" t="s">
         <v>68</v>
       </c>
@@ -9746,7 +9769,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:18" ht="17.25" customHeight="1">
       <c r="A16" s="117" t="s">
         <v>69</v>
       </c>
@@ -9762,7 +9785,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" ht="17.25" customHeight="1">
       <c r="A17" s="117" t="s">
         <v>70</v>
       </c>
@@ -9778,7 +9801,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4" ht="17.25" customHeight="1">
       <c r="A18" s="117" t="s">
         <v>71</v>
       </c>
@@ -9794,7 +9817,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:4" ht="17.25" customHeight="1">
       <c r="A19" s="117" t="s">
         <v>72</v>
       </c>
@@ -9810,7 +9833,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4" ht="17.25" customHeight="1">
       <c r="A20" s="117" t="s">
         <v>73</v>
       </c>
@@ -9826,7 +9849,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:4" ht="17.25" customHeight="1">
       <c r="A21" s="117" t="s">
         <v>74</v>
       </c>
@@ -9842,7 +9865,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:4" ht="17.25" customHeight="1">
       <c r="A22" s="117" t="s">
         <v>76</v>
       </c>
@@ -9858,7 +9881,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:4" ht="17.25" customHeight="1">
       <c r="A23" s="117" t="s">
         <v>77</v>
       </c>
@@ -9874,7 +9897,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:4" ht="17.25" customHeight="1">
       <c r="A24" s="117" t="s">
         <v>78</v>
       </c>
@@ -9891,7 +9914,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:4" ht="17.25" customHeight="1">
       <c r="A25" s="117" t="s">
         <v>79</v>
       </c>
@@ -9907,7 +9930,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:4" ht="17.25" customHeight="1">
       <c r="A26" s="117" t="s">
         <v>81</v>
       </c>
@@ -9923,7 +9946,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:4" ht="17.25" customHeight="1">
       <c r="A27" s="117" t="s">
         <v>82</v>
       </c>
@@ -9939,7 +9962,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:4" ht="17.25" customHeight="1">
       <c r="A28" s="117" t="s">
         <v>83</v>
       </c>
@@ -9956,7 +9979,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:4" ht="17.25" customHeight="1">
       <c r="A29" s="117" t="s">
         <v>84</v>
       </c>
@@ -9972,7 +9995,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:4" ht="17.25" customHeight="1">
       <c r="A30" s="117" t="s">
         <v>85</v>
       </c>
@@ -9988,7 +10011,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:4" ht="17.25" customHeight="1">
       <c r="A31" s="117" t="s">
         <v>86</v>
       </c>
@@ -10004,7 +10027,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:4" ht="17.25" customHeight="1">
       <c r="A32" s="117" t="s">
         <v>87</v>
       </c>
@@ -10020,7 +10043,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:4" ht="17.25" customHeight="1">
       <c r="A33" s="117" t="s">
         <v>88</v>
       </c>
@@ -10036,7 +10059,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:4" ht="17.25" customHeight="1">
       <c r="A34" s="117" t="s">
         <v>89</v>
       </c>
@@ -10052,7 +10075,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:4" ht="17.25" customHeight="1">
       <c r="A35" s="117" t="s">
         <v>90</v>
       </c>
@@ -10068,7 +10091,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:4" ht="17.25" customHeight="1">
       <c r="A36" s="117" t="s">
         <v>91</v>
       </c>
@@ -10084,7 +10107,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:4" ht="17.25" customHeight="1">
       <c r="A37" s="117" t="s">
         <v>92</v>
       </c>
@@ -10100,7 +10123,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:4" ht="17.25" customHeight="1">
       <c r="A38" s="117" t="s">
         <v>93</v>
       </c>
@@ -10117,7 +10140,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:4" ht="17.25" customHeight="1">
       <c r="A39" s="117" t="s">
         <v>94</v>
       </c>
@@ -10133,7 +10156,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:4" ht="17.25" customHeight="1">
       <c r="A40" s="117" t="s">
         <v>95</v>
       </c>
@@ -10149,7 +10172,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:4" ht="17.25" customHeight="1">
       <c r="A41" s="117" t="s">
         <v>96</v>
       </c>
@@ -10165,7 +10188,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:4" ht="17.25" customHeight="1">
       <c r="A42" s="117" t="s">
         <v>97</v>
       </c>
@@ -10181,7 +10204,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:4" ht="17.25" customHeight="1">
       <c r="A43" s="117" t="s">
         <v>98</v>
       </c>
@@ -10197,7 +10220,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:4" ht="17.25" customHeight="1">
       <c r="A44" s="117" t="s">
         <v>99</v>
       </c>
@@ -10213,7 +10236,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:4" ht="17.25" customHeight="1">
       <c r="A45" s="117" t="s">
         <v>100</v>
       </c>
@@ -10229,7 +10252,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:4" ht="17.25" customHeight="1">
       <c r="A46" s="117" t="s">
         <v>101</v>
       </c>
@@ -10245,7 +10268,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:4" ht="17.25" customHeight="1">
       <c r="A47" s="117" t="s">
         <v>102</v>
       </c>
@@ -10261,7 +10284,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:4" ht="17.25" customHeight="1">
       <c r="A48" s="117" t="s">
         <v>103</v>
       </c>
@@ -10277,7 +10300,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:4" ht="17.25" customHeight="1">
       <c r="A49" s="117" t="s">
         <v>104</v>
       </c>
@@ -10293,7 +10316,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:4" ht="17.25" customHeight="1">
       <c r="A50" s="117" t="s">
         <v>105</v>
       </c>
@@ -10310,7 +10333,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:4" ht="17.25" customHeight="1">
       <c r="A51" s="117" t="s">
         <v>106</v>
       </c>
@@ -10327,7 +10350,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:4" ht="17.25" customHeight="1">
       <c r="A52" s="117" t="s">
         <v>107</v>
       </c>
@@ -10343,7 +10366,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:4" ht="17.25" customHeight="1">
       <c r="A53" s="117" t="s">
         <v>108</v>
       </c>
@@ -10359,7 +10382,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:4" ht="17.25" customHeight="1">
       <c r="A54" s="117" t="s">
         <v>109</v>
       </c>
@@ -10375,7 +10398,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:4" ht="17.25" customHeight="1">
       <c r="A55" s="117" t="s">
         <v>110</v>
       </c>
@@ -10391,7 +10414,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:4" ht="17.25" customHeight="1">
       <c r="A56" s="117" t="s">
         <v>111</v>
       </c>
@@ -10407,7 +10430,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:4" ht="17.25" customHeight="1">
       <c r="A57" s="117" t="s">
         <v>112</v>
       </c>
@@ -10423,7 +10446,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:4" ht="17.25" customHeight="1">
       <c r="A58" s="117" t="s">
         <v>113</v>
       </c>
@@ -10439,7 +10462,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:4" ht="17.25" customHeight="1">
       <c r="A59" s="117" t="s">
         <v>114</v>
       </c>
@@ -10455,7 +10478,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:4" ht="17.25" customHeight="1">
       <c r="A60" s="117" t="s">
         <v>115</v>
       </c>
@@ -10471,7 +10494,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:4" ht="17.25" customHeight="1">
       <c r="A61" s="117" t="s">
         <v>116</v>
       </c>
@@ -10487,7 +10510,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:4" ht="17.25" customHeight="1">
       <c r="A62" s="117" t="s">
         <v>117</v>
       </c>
@@ -10503,7 +10526,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:4" ht="17.25" customHeight="1">
       <c r="A63" s="117" t="s">
         <v>118</v>
       </c>
@@ -10519,7 +10542,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:4" ht="17.25" customHeight="1">
       <c r="A64" s="117" t="s">
         <v>119</v>
       </c>
@@ -10535,7 +10558,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:4" ht="17.25" customHeight="1">
       <c r="A65" s="117" t="s">
         <v>120</v>
       </c>
@@ -10551,7 +10574,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:4" ht="17.25" customHeight="1">
       <c r="A66" s="117" t="s">
         <v>121</v>
       </c>
@@ -10567,7 +10590,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:4" ht="17.25" customHeight="1">
       <c r="A67" s="117" t="s">
         <v>122</v>
       </c>
@@ -10583,7 +10606,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:4" ht="17.25" customHeight="1">
       <c r="A68" s="117" t="s">
         <v>123</v>
       </c>
@@ -10599,7 +10622,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:4" ht="17.25" customHeight="1">
       <c r="A69" s="117" t="s">
         <v>125</v>
       </c>
@@ -10615,7 +10638,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:4" ht="17.25" customHeight="1">
       <c r="A70" s="117" t="s">
         <v>127</v>
       </c>
@@ -10631,7 +10654,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:4" ht="17.25" customHeight="1">
       <c r="A71" s="117" t="s">
         <v>129</v>
       </c>
@@ -10647,7 +10670,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:4" ht="17.25" customHeight="1">
       <c r="A72" s="117" t="s">
         <v>130</v>
       </c>
@@ -10663,7 +10686,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:4" ht="17.25" customHeight="1">
       <c r="A73" s="117" t="s">
         <v>131</v>
       </c>
@@ -10679,7 +10702,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:4" ht="17.25" customHeight="1">
       <c r="A74" s="117" t="s">
         <v>132</v>
       </c>
@@ -10695,7 +10718,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:4" ht="17.25" customHeight="1">
       <c r="A75" s="117" t="s">
         <v>133</v>
       </c>
@@ -10711,7 +10734,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:4" ht="17.25" customHeight="1">
       <c r="A76" s="117" t="s">
         <v>134</v>
       </c>
@@ -10727,7 +10750,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:4" ht="17.25" customHeight="1">
       <c r="A77" s="117" t="s">
         <v>135</v>
       </c>
@@ -10743,7 +10766,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="78" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:4" ht="17.25" customHeight="1">
       <c r="A78" s="117" t="s">
         <v>136</v>
       </c>
@@ -10759,7 +10782,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:4" ht="17.25" customHeight="1">
       <c r="A79" s="117" t="s">
         <v>137</v>
       </c>
@@ -10775,7 +10798,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:4" ht="17.25" customHeight="1">
       <c r="A80" s="117" t="s">
         <v>138</v>
       </c>
@@ -10791,7 +10814,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:4" ht="17.25" customHeight="1">
       <c r="A81" s="117" t="s">
         <v>139</v>
       </c>
@@ -10807,7 +10830,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:4" ht="17.25" customHeight="1">
       <c r="A82" s="117" t="s">
         <v>141</v>
       </c>
@@ -10823,7 +10846,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:4" ht="17.25" customHeight="1">
       <c r="A83" s="117" t="s">
         <v>142</v>
       </c>
@@ -10839,7 +10862,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:4" ht="17.25" customHeight="1">
       <c r="A84" s="117" t="s">
         <v>143</v>
       </c>
@@ -10855,7 +10878,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:4" ht="17.25" customHeight="1">
       <c r="A85" s="117" t="s">
         <v>144</v>
       </c>
@@ -10871,7 +10894,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="86" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:4" ht="17.25" customHeight="1">
       <c r="A86" s="117" t="s">
         <v>146</v>
       </c>
@@ -10887,7 +10910,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:4" ht="17.25" customHeight="1">
       <c r="A87" s="117" t="s">
         <v>147</v>
       </c>
@@ -10903,7 +10926,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:4" ht="17.25" customHeight="1">
       <c r="A88" s="117" t="s">
         <v>148</v>
       </c>
@@ -10919,7 +10942,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:4" ht="17.25" customHeight="1">
       <c r="A89" s="117" t="s">
         <v>149</v>
       </c>
@@ -10935,7 +10958,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="90" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:4" ht="17.25" customHeight="1">
       <c r="A90" s="117" t="s">
         <v>150</v>
       </c>
@@ -10951,7 +10974,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:4" ht="17.25" customHeight="1">
       <c r="A91" s="117" t="s">
         <v>151</v>
       </c>
@@ -10967,7 +10990,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:4" ht="17.25" customHeight="1">
       <c r="A92" s="117" t="s">
         <v>152</v>
       </c>
@@ -10983,7 +11006,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:4" ht="17.25" customHeight="1">
       <c r="A93" s="117" t="s">
         <v>153</v>
       </c>
@@ -10999,7 +11022,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="94" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:4" ht="17.25" customHeight="1">
       <c r="A94" s="117" t="s">
         <v>154</v>
       </c>
@@ -11015,7 +11038,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="95" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:4" ht="17.25" customHeight="1">
       <c r="A95" s="117" t="s">
         <v>155</v>
       </c>
@@ -11031,7 +11054,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="96" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:4" ht="17.25" customHeight="1">
       <c r="A96" s="117" t="s">
         <v>156</v>
       </c>
@@ -11047,7 +11070,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="97" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:4" ht="17.25" customHeight="1">
       <c r="A97" s="117" t="s">
         <v>157</v>
       </c>
@@ -11063,7 +11086,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="98" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:4" ht="17.25" customHeight="1">
       <c r="A98" s="117" t="s">
         <v>158</v>
       </c>
@@ -11079,7 +11102,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="99" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:4" ht="17.25" customHeight="1">
       <c r="A99" s="117" t="s">
         <v>159</v>
       </c>
@@ -11095,20 +11118,20 @@
         <v>1</v>
       </c>
     </row>
-    <row r="100" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:4" ht="17.25" customHeight="1">
       <c r="A100" s="117" t="s">
         <v>160</v>
       </c>
       <c r="B100" s="19">
         <f ca="1">NOW()</f>
-        <v>45905.868253935187</v>
+        <v>46076.541597106479</v>
       </c>
       <c r="D100" s="117">
         <f ca="1">IF(ISNUMBER(B100),1,0)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="101" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:4" ht="17.25" customHeight="1">
       <c r="A101" s="117" t="s">
         <v>161</v>
       </c>
@@ -11124,7 +11147,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="102" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:4" ht="17.25" customHeight="1">
       <c r="A102" s="117" t="s">
         <v>162</v>
       </c>
@@ -11140,7 +11163,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="103" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:4" ht="17.25" customHeight="1">
       <c r="A103" s="117" t="s">
         <v>163</v>
       </c>
@@ -11156,7 +11179,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="104" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:4" ht="17.25" customHeight="1">
       <c r="A104" s="117" t="s">
         <v>164</v>
       </c>
@@ -11172,7 +11195,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="105" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:4" ht="17.25" customHeight="1">
       <c r="A105" s="117" t="s">
         <v>165</v>
       </c>
@@ -11188,7 +11211,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="106" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:4" ht="17.25" customHeight="1">
       <c r="A106" s="117" t="s">
         <v>166</v>
       </c>
@@ -11204,7 +11227,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="107" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:4" ht="17.25" customHeight="1">
       <c r="A107" s="117" t="s">
         <v>167</v>
       </c>
@@ -11220,7 +11243,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:4" ht="17.25" customHeight="1">
       <c r="A108" s="117" t="s">
         <v>168</v>
       </c>
@@ -11236,7 +11259,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="109" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:4" ht="17.25" customHeight="1">
       <c r="A109" s="117" t="s">
         <v>169</v>
       </c>
@@ -11252,7 +11275,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="110" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:4" ht="17.25" customHeight="1">
       <c r="A110" s="117" t="s">
         <v>170</v>
       </c>
@@ -11268,7 +11291,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="111" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:4" ht="17.25" customHeight="1">
       <c r="A111" s="117" t="s">
         <v>171</v>
       </c>
@@ -11284,12 +11307,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="112" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:4" ht="17.25" customHeight="1">
       <c r="A112" s="117"/>
       <c r="B112" s="117"/>
       <c r="D112" s="117"/>
     </row>
-    <row r="113" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:4" ht="17.25" customHeight="1">
       <c r="A113" s="117" t="s">
         <v>172</v>
       </c>
@@ -11305,7 +11328,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="114" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:4" ht="17.25" customHeight="1">
       <c r="A114" s="117" t="s">
         <v>173</v>
       </c>
@@ -11321,7 +11344,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="115" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:4" ht="17.25" customHeight="1">
       <c r="A115" s="117" t="s">
         <v>175</v>
       </c>
@@ -11337,7 +11360,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="116" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:4" ht="17.25" customHeight="1">
       <c r="A116" s="117" t="s">
         <v>177</v>
       </c>
@@ -11353,7 +11376,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="117" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:4" ht="17.25" customHeight="1">
       <c r="A117" s="117" t="s">
         <v>178</v>
       </c>
@@ -11369,7 +11392,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="118" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:4" ht="17.25" customHeight="1">
       <c r="A118" s="117" t="s">
         <v>179</v>
       </c>
@@ -11385,7 +11408,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="119" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:4" ht="17.25" customHeight="1">
       <c r="A119" s="117" t="s">
         <v>180</v>
       </c>
@@ -11401,7 +11424,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="120" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:4" ht="17.25" customHeight="1">
       <c r="A120" s="117" t="s">
         <v>181</v>
       </c>
@@ -11417,7 +11440,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="121" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:4" ht="17.25" customHeight="1">
       <c r="A121" s="117" t="s">
         <v>182</v>
       </c>
@@ -11433,7 +11456,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="122" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:4" ht="17.25" customHeight="1">
       <c r="A122" s="117" t="s">
         <v>183</v>
       </c>
@@ -11449,7 +11472,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="123" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:4" ht="17.25" customHeight="1">
       <c r="A123" s="117" t="s">
         <v>184</v>
       </c>
@@ -11465,7 +11488,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="124" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:4" ht="17.25" customHeight="1">
       <c r="A124" s="117" t="s">
         <v>185</v>
       </c>
@@ -11481,7 +11504,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="125" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:4" ht="17.25" customHeight="1">
       <c r="A125" s="117" t="s">
         <v>186</v>
       </c>
@@ -11497,7 +11520,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="126" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:4" ht="17.25" customHeight="1">
       <c r="A126" s="117" t="s">
         <v>187</v>
       </c>
@@ -11513,7 +11536,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="127" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:4" ht="17.25" customHeight="1">
       <c r="A127" s="117" t="s">
         <v>188</v>
       </c>
@@ -11529,7 +11552,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="128" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:4" ht="17.25" customHeight="1">
       <c r="A128" s="117" t="s">
         <v>189</v>
       </c>
@@ -11545,7 +11568,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="129" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:4" ht="17.25" customHeight="1">
       <c r="A129" s="117" t="s">
         <v>190</v>
       </c>
@@ -11561,7 +11584,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="130" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:4" ht="17.25" customHeight="1">
       <c r="A130" s="117" t="s">
         <v>191</v>
       </c>
@@ -11577,7 +11600,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="131" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:4" ht="17.25" customHeight="1">
       <c r="A131" s="117" t="s">
         <v>192</v>
       </c>
@@ -11593,7 +11616,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="132" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:4" ht="17.25" customHeight="1">
       <c r="A132" s="117" t="s">
         <v>193</v>
       </c>
@@ -11609,7 +11632,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="133" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:4" ht="17.25" customHeight="1">
       <c r="A133" s="117" t="s">
         <v>194</v>
       </c>
@@ -11625,7 +11648,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="134" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:4" ht="17.25" customHeight="1">
       <c r="A134" s="117" t="s">
         <v>195</v>
       </c>
@@ -11641,7 +11664,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="135" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:4" ht="17.25" customHeight="1">
       <c r="A135" s="117" t="s">
         <v>196</v>
       </c>
@@ -11657,7 +11680,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="136" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:4" ht="17.25" customHeight="1">
       <c r="A136" s="117" t="s">
         <v>198</v>
       </c>
@@ -11673,7 +11696,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="137" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:4" ht="17.25" customHeight="1">
       <c r="A137" s="117" t="s">
         <v>199</v>
       </c>
@@ -11689,7 +11712,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="138" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:4" ht="17.25" customHeight="1">
       <c r="A138" s="117" t="s">
         <v>200</v>
       </c>
@@ -11705,7 +11728,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="139" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:4" ht="17.25" customHeight="1">
       <c r="A139" s="117" t="s">
         <v>201</v>
       </c>
@@ -11721,7 +11744,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="140" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:4" ht="17.25" customHeight="1">
       <c r="A140" s="117" t="s">
         <v>202</v>
       </c>
@@ -11737,7 +11760,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="141" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:4" ht="17.25" customHeight="1">
       <c r="A141" s="117" t="s">
         <v>203</v>
       </c>
@@ -11753,7 +11776,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="142" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:4" ht="17.25" customHeight="1">
       <c r="A142" s="117" t="s">
         <v>205</v>
       </c>
@@ -11769,7 +11792,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:4" ht="17.25" customHeight="1">
       <c r="A143" s="117" t="s">
         <v>206</v>
       </c>
@@ -11785,20 +11808,20 @@
         <v>1</v>
       </c>
     </row>
-    <row r="144" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:4" ht="17.25" customHeight="1">
       <c r="A144" s="117" t="s">
         <v>207</v>
       </c>
       <c r="B144" s="18">
         <f ca="1">TODAY()</f>
-        <v>45905</v>
+        <v>46076</v>
       </c>
       <c r="D144" s="117">
         <f ca="1">IF(ISNUMBER(B144),1,0)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="145" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:4" ht="17.25" customHeight="1">
       <c r="A145" s="117" t="s">
         <v>208</v>
       </c>
@@ -11814,7 +11837,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="146" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:4" ht="17.25" customHeight="1">
       <c r="A146" s="117" t="s">
         <v>210</v>
       </c>
@@ -11830,7 +11853,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="147" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:4" ht="17.25" customHeight="1">
       <c r="A147" s="117" t="s">
         <v>211</v>
       </c>
@@ -11846,7 +11869,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="148" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:4" ht="17.25" customHeight="1">
       <c r="A148" s="117" t="s">
         <v>213</v>
       </c>
@@ -11862,7 +11885,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="149" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:4" ht="17.25" customHeight="1">
       <c r="A149" s="117" t="s">
         <v>214</v>
       </c>
@@ -11878,7 +11901,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="150" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:4" ht="17.25" customHeight="1">
       <c r="A150" s="117" t="s">
         <v>215</v>
       </c>
@@ -11894,7 +11917,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="151" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:4" ht="17.25" customHeight="1">
       <c r="A151" s="117" t="s">
         <v>216</v>
       </c>
@@ -11910,7 +11933,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="152" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:4" ht="17.25" customHeight="1">
       <c r="A152" s="117" t="s">
         <v>217</v>
       </c>
@@ -11926,7 +11949,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="153" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:4" ht="17.25" customHeight="1">
       <c r="A153" s="117" t="s">
         <v>218</v>
       </c>
@@ -11942,7 +11965,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="154" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:4" ht="17.25" customHeight="1">
       <c r="A154" s="117" t="s">
         <v>219</v>
       </c>
@@ -11959,7 +11982,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="155" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:4" ht="17.25" customHeight="1">
       <c r="A155" s="117" t="s">
         <v>220</v>
       </c>
@@ -11975,7 +11998,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="156" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:4" ht="17.25" customHeight="1">
       <c r="A156" s="117" t="s">
         <v>221</v>
       </c>
@@ -11991,7 +12014,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="157" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:4" ht="17.25" customHeight="1">
       <c r="A157" s="117" t="s">
         <v>222</v>
       </c>
@@ -12007,7 +12030,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="158" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:4" ht="17.25" customHeight="1">
       <c r="A158" s="117" t="s">
         <v>223</v>
       </c>
@@ -12023,7 +12046,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="159" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:4" ht="17.25" customHeight="1">
       <c r="A159" s="117" t="s">
         <v>224</v>
       </c>
@@ -12039,7 +12062,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="160" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:4" ht="17.25" customHeight="1">
       <c r="A160" s="117" t="s">
         <v>225</v>
       </c>
@@ -12055,7 +12078,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="161" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:4" ht="17.25" customHeight="1">
       <c r="A161" s="117" t="s">
         <v>226</v>
       </c>
@@ -12071,7 +12094,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="162" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:4" ht="17.25" customHeight="1">
       <c r="A162" s="117" t="s">
         <v>227</v>
       </c>
@@ -12087,7 +12110,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="163" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:4" ht="17.25" customHeight="1">
       <c r="A163" s="117" t="s">
         <v>229</v>
       </c>
@@ -12105,10 +12128,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="D1:D180">
-    <cfRule type="cellIs" dxfId="25" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="43" priority="1" operator="equal">
       <formula>1</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="42" priority="2" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -12123,7 +12146,7 @@
     <outlinePr summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:R30"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" outlineLevelRow="2" outlineLevelCol="2" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" outlineLevelRow="2" outlineLevelCol="2"/>
   <cols>
     <col min="3" max="3" width="0" hidden="1" customWidth="1"/>
     <col min="6" max="6" width="14.28515625" customWidth="1"/>
@@ -12133,17 +12156,17 @@
     <col min="15" max="18" width="9.140625" outlineLevel="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8">
       <c r="A1" t="s">
         <v>230</v>
       </c>
       <c r="C1" t="s">
         <v>231</v>
       </c>
-      <c r="D1" s="123" t="s">
+      <c r="D1" s="122" t="s">
         <v>232</v>
       </c>
-      <c r="E1" s="123"/>
+      <c r="E1" s="122"/>
       <c r="F1" t="s">
         <v>233</v>
       </c>
@@ -12151,19 +12174,19 @@
         <v>234</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8">
       <c r="A2">
         <f>SUM(A1)</f>
         <v>0</v>
       </c>
-      <c r="D2" s="123"/>
-      <c r="E2" s="123"/>
+      <c r="D2" s="122"/>
+      <c r="E2" s="122"/>
       <c r="H2" t="str">
         <f>[1]Feuil1!$A$1</f>
         <v>referenced string</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8">
       <c r="D3" s="85" t="s">
         <v>235</v>
       </c>
@@ -12171,26 +12194,26 @@
         <v>236</v>
       </c>
     </row>
-    <row r="4" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" hidden="1">
       <c r="A4" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" ht="75" customHeight="1">
       <c r="A5" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="10" spans="1:8" outlineLevel="1" x14ac:dyDescent="0.2"/>
-    <row r="11" spans="1:8" outlineLevel="1" x14ac:dyDescent="0.2"/>
-    <row r="12" spans="1:8" hidden="1" outlineLevel="2" x14ac:dyDescent="0.2"/>
-    <row r="13" spans="1:8" hidden="1" outlineLevel="2" x14ac:dyDescent="0.2"/>
-    <row r="14" spans="1:8" hidden="1" outlineLevel="2" x14ac:dyDescent="0.2"/>
-    <row r="15" spans="1:8" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.2"/>
-    <row r="16" spans="1:8" outlineLevel="1" x14ac:dyDescent="0.2"/>
-    <row r="17" spans="1:1" outlineLevel="1" x14ac:dyDescent="0.2"/>
-    <row r="18" spans="1:1" outlineLevel="1" x14ac:dyDescent="0.2"/>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" outlineLevel="1"/>
+    <row r="11" spans="1:8" outlineLevel="1"/>
+    <row r="12" spans="1:8" hidden="1" outlineLevel="2"/>
+    <row r="13" spans="1:8" hidden="1" outlineLevel="2"/>
+    <row r="14" spans="1:8" hidden="1" outlineLevel="2"/>
+    <row r="15" spans="1:8" outlineLevel="1" collapsed="1"/>
+    <row r="16" spans="1:8" outlineLevel="1"/>
+    <row r="17" spans="1:1" outlineLevel="1"/>
+    <row r="18" spans="1:1" outlineLevel="1"/>
+    <row r="30" spans="1:1">
       <c r="A30" t="e" cm="1">
         <f t="array" aca="1" ref="A30" ca="1">RANDARRAY(2, 2)</f>
         <v>#NAME?</v>
@@ -12212,14 +12235,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF68F2C0-1053-4FB6-BD74-8A11B0CAF123}">
   <dimension ref="A1:M30"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75"/>
   <cols>
     <col min="3" max="3" width="17.7109375" customWidth="1"/>
     <col min="5" max="5" width="18.28515625" customWidth="1"/>
     <col min="13" max="13" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="13.5" thickBot="1">
       <c r="A1" s="68" t="s">
         <v>239</v>
       </c>
@@ -12241,7 +12264,7 @@
       </c>
       <c r="M1" s="36"/>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13">
       <c r="A2" s="40" t="s">
         <v>245</v>
       </c>
@@ -12267,7 +12290,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:13">
       <c r="A3" s="41" t="s">
         <v>252</v>
       </c>
@@ -12290,7 +12313,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="15" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" ht="15">
       <c r="A4" s="42" t="s">
         <v>256</v>
       </c>
@@ -12316,7 +12339,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:13">
       <c r="A5" s="43" t="s">
         <v>262</v>
       </c>
@@ -12336,7 +12359,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13">
       <c r="A6" s="44" t="s">
         <v>266</v>
       </c>
@@ -12359,7 +12382,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" ht="15.75">
       <c r="A7" s="45" t="s">
         <v>271</v>
       </c>
@@ -12379,7 +12402,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="21" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:13" ht="21">
       <c r="A8" s="46" t="s">
         <v>275</v>
       </c>
@@ -12402,7 +12425,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:13">
       <c r="A9" s="47" t="s">
         <v>280</v>
       </c>
@@ -12419,7 +12442,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:13">
       <c r="A10" s="48" t="s">
         <v>283</v>
       </c>
@@ -12427,7 +12450,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" ht="13.5" thickBot="1">
       <c r="A11" s="49" t="s">
         <v>285</v>
       </c>
@@ -12436,7 +12459,7 @@
       </c>
       <c r="F11" s="36"/>
     </row>
-    <row r="12" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:13" ht="18.75" customHeight="1">
       <c r="A12" s="50" t="s">
         <v>287</v>
       </c>
@@ -12450,7 +12473,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" ht="18.75" customHeight="1" thickBot="1">
       <c r="A13" s="51" t="s">
         <v>290</v>
       </c>
@@ -12461,7 +12484,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" ht="18.75" customHeight="1" thickBot="1">
       <c r="A14" s="52" t="s">
         <v>291</v>
       </c>
@@ -12475,7 +12498,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" ht="18.75" customHeight="1" thickBot="1">
       <c r="A15" s="53" t="s">
         <v>293</v>
       </c>
@@ -12486,7 +12509,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="16" spans="1:13" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" ht="19.5" customHeight="1" thickBot="1">
       <c r="A16" s="54" t="s">
         <v>294</v>
       </c>
@@ -12500,12 +12523,12 @@
         <v>248</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" ht="13.5" thickBot="1">
       <c r="A17" s="55" t="s">
         <v>296</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" ht="13.5" thickBot="1">
       <c r="A18" s="74" t="s">
         <v>297</v>
       </c>
@@ -12517,7 +12540,7 @@
       </c>
       <c r="F18" s="36"/>
     </row>
-    <row r="19" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" ht="13.5" thickBot="1">
       <c r="A19" s="75" t="s">
         <v>300</v>
       </c>
@@ -12528,7 +12551,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="51.75" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" ht="51.75" thickBot="1">
       <c r="A20" s="76" t="s">
         <v>303</v>
       </c>
@@ -12542,12 +12565,12 @@
         <v>302</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" ht="13.5" thickBot="1">
       <c r="A21" s="77" t="s">
         <v>306</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" ht="13.5" thickBot="1">
       <c r="A22" s="78" t="s">
         <v>307</v>
       </c>
@@ -12556,13 +12579,13 @@
       </c>
       <c r="E22" s="21"/>
     </row>
-    <row r="23" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" ht="13.5" thickBot="1">
       <c r="A23" s="79" t="s">
         <v>309</v>
       </c>
       <c r="E23" s="21"/>
     </row>
-    <row r="24" spans="1:6" ht="14.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" ht="14.25" thickTop="1" thickBot="1">
       <c r="A24" s="80" t="s">
         <v>310</v>
       </c>
@@ -12571,20 +12594,20 @@
       </c>
       <c r="E24" s="21"/>
     </row>
-    <row r="25" spans="1:6" ht="14.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="26" spans="1:6" ht="14.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" ht="14.25" thickTop="1" thickBot="1"/>
+    <row r="26" spans="1:6" ht="14.25" thickTop="1" thickBot="1">
       <c r="C26" s="67" t="s">
         <v>312</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="14.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="1:6" ht="14.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" ht="14.25" thickTop="1" thickBot="1"/>
+    <row r="28" spans="1:6" ht="14.25" thickTop="1" thickBot="1">
       <c r="C28" s="88" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="13.5" thickTop="1" x14ac:dyDescent="0.2"/>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:6" ht="13.5" thickTop="1"/>
+    <row r="30" spans="1:6">
       <c r="C30" s="87" t="s">
         <v>314</v>
       </c>
@@ -12598,13 +12621,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D919E811-4385-4D35-A19E-3B7E0E659A89}">
   <dimension ref="A1:L39"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="19.140625" customWidth="1"/>
     <col min="7" max="7" width="15.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="13.5" thickBot="1">
       <c r="A1" s="37" t="s">
         <v>315</v>
       </c>
@@ -12621,7 +12644,7 @@
       <c r="I1" s="36"/>
       <c r="J1" s="36"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10">
       <c r="A2" s="38" t="s">
         <v>319</v>
       </c>
@@ -12644,7 +12667,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10">
       <c r="A3" s="38" t="s">
         <v>321</v>
       </c>
@@ -12667,7 +12690,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10">
       <c r="A4" s="38" t="s">
         <v>325</v>
       </c>
@@ -12687,7 +12710,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10">
       <c r="A5" s="38" t="s">
         <v>328</v>
       </c>
@@ -12711,7 +12734,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10">
       <c r="A6" s="38" t="s">
         <v>330</v>
       </c>
@@ -12734,7 +12757,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:10">
       <c r="A7" s="38" t="s">
         <v>333</v>
       </c>
@@ -12760,7 +12783,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:10">
       <c r="A8" s="38" t="s">
         <v>337</v>
       </c>
@@ -12771,7 +12794,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10">
       <c r="A9" s="38" t="s">
         <v>339</v>
       </c>
@@ -12780,7 +12803,7 @@
       </c>
       <c r="C9" s="21"/>
     </row>
-    <row r="10" spans="1:10" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" ht="13.5" thickBot="1">
       <c r="A10" s="38" t="s">
         <v>340</v>
       </c>
@@ -12798,7 +12821,7 @@
       <c r="I10" s="36"/>
       <c r="J10" s="36"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:10">
       <c r="A11" s="38" t="s">
         <v>342</v>
       </c>
@@ -12821,13 +12844,13 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:10">
       <c r="A12" s="38" t="s">
         <v>344</v>
       </c>
       <c r="B12" s="39">
         <f ca="1">TODAY()</f>
-        <v>45905</v>
+        <v>46076</v>
       </c>
       <c r="C12" s="39">
         <f>DATE(2010,10,2)</f>
@@ -12846,7 +12869,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:10">
       <c r="A13" s="38" t="s">
         <v>346</v>
       </c>
@@ -12869,7 +12892,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:10">
       <c r="A14" s="38" t="s">
         <v>348</v>
       </c>
@@ -12895,7 +12918,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:10">
       <c r="A15" s="38" t="s">
         <v>350</v>
       </c>
@@ -12915,7 +12938,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:10">
       <c r="A16" s="38" t="s">
         <v>352</v>
       </c>
@@ -12938,7 +12961,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:12">
       <c r="A17" s="38" t="s">
         <v>354</v>
       </c>
@@ -12961,7 +12984,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:12">
       <c r="A18" s="38" t="s">
         <v>356</v>
       </c>
@@ -12984,7 +13007,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:12">
       <c r="A19" s="38" t="s">
         <v>358</v>
       </c>
@@ -13007,7 +13030,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:12">
       <c r="A20" s="38" t="s">
         <v>360</v>
       </c>
@@ -13030,7 +13053,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:12">
       <c r="A21" s="38" t="s">
         <v>362</v>
       </c>
@@ -13056,7 +13079,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:12">
       <c r="A22" s="38" t="s">
         <v>364</v>
       </c>
@@ -13082,7 +13105,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:12">
       <c r="A23" s="38" t="s">
         <v>366</v>
       </c>
@@ -13108,7 +13131,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:12">
       <c r="G24" s="34" t="s">
         <v>368</v>
       </c>
@@ -13125,7 +13148,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:12">
       <c r="A25" s="38" t="s">
         <v>369</v>
       </c>
@@ -13151,7 +13174,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:12">
       <c r="G26" s="34" t="s">
         <v>371</v>
       </c>
@@ -13171,7 +13194,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:12">
       <c r="A27" s="21" t="s">
         <v>372</v>
       </c>
@@ -13197,7 +13220,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:12">
       <c r="G28" s="34" t="s">
         <v>374</v>
       </c>
@@ -13217,9 +13240,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:12">
       <c r="A29" s="38" t="s">
-        <v>440</v>
+        <v>375</v>
       </c>
       <c r="B29">
         <v>3</v>
@@ -13228,7 +13251,7 @@
         <v>10</v>
       </c>
       <c r="G29" s="34" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="H29">
         <v>5</v>
@@ -13246,9 +13269,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:12">
       <c r="G30" s="34" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="H30">
         <v>5</v>
@@ -13266,9 +13289,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:12" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:12" ht="13.5" thickBot="1">
       <c r="G31" s="35" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="H31" s="36">
         <v>5</v>
@@ -13280,9 +13303,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:12">
       <c r="G32" s="34" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="H32">
         <v>5</v>
@@ -13294,9 +13317,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="7:10" x14ac:dyDescent="0.2">
+    <row r="33" spans="7:10">
       <c r="G33" s="34" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="H33">
         <v>5</v>
@@ -13308,9 +13331,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="7:10" x14ac:dyDescent="0.2">
+    <row r="34" spans="7:10">
       <c r="G34" s="34" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="H34">
         <v>5</v>
@@ -13322,9 +13345,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="7:10" x14ac:dyDescent="0.2">
+    <row r="35" spans="7:10">
       <c r="G35" s="34" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="H35">
         <v>5</v>
@@ -13336,9 +13359,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="7:10" x14ac:dyDescent="0.2">
+    <row r="36" spans="7:10">
       <c r="G36" s="34" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="H36">
         <v>5</v>
@@ -13350,9 +13373,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="7:10" x14ac:dyDescent="0.2">
+    <row r="37" spans="7:10">
       <c r="G37" s="34" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="H37">
         <v>5</v>
@@ -13364,110 +13387,110 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="7:10" x14ac:dyDescent="0.2">
+    <row r="39" spans="7:10">
       <c r="G39" s="34"/>
     </row>
   </sheetData>
   <phoneticPr fontId="21" type="noConversion"/>
   <conditionalFormatting sqref="B15">
-    <cfRule type="expression" dxfId="23" priority="59">
+    <cfRule type="expression" dxfId="41" priority="59">
       <formula>ODD(B15)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B26:B27">
-    <cfRule type="cellIs" dxfId="22" priority="47" operator="equal">
+    <cfRule type="cellIs" dxfId="40" priority="47" operator="equal">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B2:C2">
-    <cfRule type="aboveAverage" dxfId="21" priority="115"/>
+    <cfRule type="aboveAverage" dxfId="39" priority="115"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:C3">
-    <cfRule type="beginsWith" dxfId="20" priority="74" operator="beginsWith" text="rule">
+    <cfRule type="beginsWith" dxfId="38" priority="74" operator="beginsWith" text="rule">
       <formula>LEFT(B3,LEN("rule"))="rule"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B4:C4">
-    <cfRule type="containsBlanks" dxfId="19" priority="72">
+    <cfRule type="containsBlanks" dxfId="37" priority="72">
       <formula>LEN(TRIM(B4))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B5:C5">
-    <cfRule type="containsErrors" dxfId="18" priority="71">
+    <cfRule type="containsErrors" dxfId="36" priority="71">
       <formula>ISERROR(B5)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:C6">
-    <cfRule type="containsText" dxfId="17" priority="70" operator="containsText" text="rule">
+    <cfRule type="containsText" dxfId="35" priority="70" operator="containsText" text="rule">
       <formula>NOT(ISERROR(SEARCH("rule",B6)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8:C8">
-    <cfRule type="endsWith" dxfId="16" priority="68" operator="endsWith" text="rule">
+    <cfRule type="endsWith" dxfId="34" priority="68" operator="endsWith" text="rule">
       <formula>RIGHT(B8,LEN("rule"))="rule"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B9:C9">
-    <cfRule type="notContainsBlanks" dxfId="15" priority="67">
+    <cfRule type="notContainsBlanks" dxfId="33" priority="67">
       <formula>LEN(TRIM(B9))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B10:C10">
-    <cfRule type="notContainsErrors" dxfId="14" priority="66">
+    <cfRule type="notContainsErrors" dxfId="32" priority="66">
       <formula>NOT(ISERROR(B10))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B11:C11">
-    <cfRule type="notContainsText" dxfId="13" priority="65" operator="notContains" text="rule">
+    <cfRule type="notContainsText" dxfId="31" priority="65" operator="notContains" text="rule">
       <formula>ISERROR(SEARCH("rule",B11))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12:C12">
-    <cfRule type="timePeriod" dxfId="12" priority="64" timePeriod="today">
+    <cfRule type="timePeriod" dxfId="30" priority="64" timePeriod="today">
       <formula>FLOOR(B12,1)=TODAY()</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B13:C13">
-    <cfRule type="top10" dxfId="11" priority="116" rank="1"/>
+    <cfRule type="top10" dxfId="29" priority="116" rank="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B16:C16">
-    <cfRule type="cellIs" dxfId="10" priority="46" operator="equal">
+    <cfRule type="cellIs" dxfId="28" priority="46" operator="equal">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B17:C17">
-    <cfRule type="cellIs" dxfId="9" priority="57" operator="notEqual">
+    <cfRule type="cellIs" dxfId="27" priority="57" operator="notEqual">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B18:C18">
-    <cfRule type="cellIs" dxfId="8" priority="7" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="26" priority="7" operator="greaterThan">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B19:C19">
-    <cfRule type="cellIs" dxfId="7" priority="6" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="25" priority="6" operator="greaterThanOrEqual">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B20:C20">
-    <cfRule type="cellIs" dxfId="6" priority="5" operator="lessThan">
+    <cfRule type="cellIs" dxfId="24" priority="5" operator="lessThan">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B21:C21">
-    <cfRule type="cellIs" dxfId="5" priority="4" operator="lessThanOrEqual">
+    <cfRule type="cellIs" dxfId="23" priority="4" operator="lessThanOrEqual">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B22:C22">
-    <cfRule type="cellIs" dxfId="4" priority="3" operator="between">
+    <cfRule type="cellIs" dxfId="22" priority="3" operator="between">
       <formula>2</formula>
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B23:C23">
-    <cfRule type="cellIs" dxfId="3" priority="2" operator="notBetween">
+    <cfRule type="cellIs" dxfId="21" priority="2" operator="notBetween">
       <formula>2</formula>
       <formula>4</formula>
     </cfRule>
@@ -13501,16 +13524,16 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B29:C29">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="between">
+    <cfRule type="cellIs" dxfId="20" priority="1" operator="between">
       <formula>$B$23</formula>
       <formula>2+2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7:D7">
-    <cfRule type="duplicateValues" dxfId="1" priority="83"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="83"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B14:D14">
-    <cfRule type="uniqueValues" dxfId="0" priority="97"/>
+    <cfRule type="uniqueValues" dxfId="18" priority="97"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:J2">
     <cfRule type="colorScale" priority="45">
@@ -13933,7 +13956,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5CCC4B1-5C65-4837-AA26-56CCF06B63BB}">
   <dimension ref="A1:J34"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75"/>
   <cols>
     <col min="3" max="3" width="17.28515625" customWidth="1"/>
     <col min="4" max="4" width="9.5703125" customWidth="1"/>
@@ -13945,12 +13968,12 @@
     <col min="10" max="10" width="17.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10">
       <c r="A1" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" ht="15" x14ac:dyDescent="0.2">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="15">
       <c r="C3" s="17" t="s">
         <v>35</v>
       </c>
@@ -13958,25 +13981,25 @@
         <v>36</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="F3" s="17" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="G3" s="17" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="H3" s="17" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="I3" s="17" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="J3" s="17" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
       <c r="C4" s="117" t="s">
         <v>42</v>
       </c>
@@ -14007,7 +14030,7 @@
         <v>Rank</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10">
       <c r="C5" s="117" t="s">
         <v>44</v>
       </c>
@@ -14038,9 +14061,9 @@
         <v>Rank</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10">
       <c r="C6" s="117" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="D6" s="117">
         <f>SUBTOTAL(109,Table3[Age])</f>
@@ -14071,9 +14094,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:10">
       <c r="B8" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -14082,22 +14105,22 @@
         <v>2</v>
       </c>
       <c r="F8" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="G8" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="H8" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="I8" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="J8" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10">
       <c r="C9">
         <v>3</v>
       </c>
@@ -14125,18 +14148,18 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:10">
       <c r="B11" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="C11" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="D11" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10">
       <c r="C12">
         <v>3</v>
       </c>
@@ -14144,9 +14167,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:10">
       <c r="B14" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="C14">
         <v>1</v>
@@ -14155,7 +14178,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:10">
       <c r="C15">
         <v>3</v>
       </c>
@@ -14163,9 +14186,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:4">
       <c r="B17" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C17">
         <v>1</v>
@@ -14174,7 +14197,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:4">
       <c r="C18">
         <v>3</v>
       </c>
@@ -14182,9 +14205,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:4">
       <c r="B20" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C20">
         <v>1</v>
@@ -14193,7 +14216,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:4">
       <c r="C21">
         <v>3</v>
       </c>
@@ -14201,9 +14224,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:4">
       <c r="B23" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="C23">
         <v>1</v>
@@ -14212,7 +14235,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="24" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:4">
       <c r="C24">
         <v>3</v>
       </c>
@@ -14220,9 +14243,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="26" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="26" spans="2:4">
       <c r="B26" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="C26">
         <v>1</v>
@@ -14231,7 +14254,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="27" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="27" spans="2:4">
       <c r="C27">
         <v>3</v>
       </c>
@@ -14239,45 +14262,45 @@
         <v>4</v>
       </c>
     </row>
-    <row r="28" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="28" spans="2:4">
       <c r="C28" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="D28">
         <f>SUBTOTAL(109,Table4910[Column2])</f>
         <v>6</v>
       </c>
     </row>
-    <row r="30" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:4">
       <c r="B30" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="C30" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="D30" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="31" spans="2:4" hidden="1" x14ac:dyDescent="0.2">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="31" spans="2:4" hidden="1">
       <c r="C31" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="D31" t="s">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="32" spans="2:4" x14ac:dyDescent="0.2">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="32" spans="2:4">
       <c r="C32" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="D32" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="34" spans="2:2" x14ac:dyDescent="0.2">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="34" spans="2:2">
       <c r="B34" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
     </row>
   </sheetData>
@@ -14300,7 +14323,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE9224F2-4D06-4586-886C-E51F5EBCA7B0}">
   <dimension ref="A1:L21"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75"/>
   <cols>
     <col min="3" max="3" width="13.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.5703125" bestFit="1" customWidth="1"/>
@@ -14321,9 +14344,9 @@
     <col min="21" max="21" width="19.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" ht="15">
       <c r="A1" s="92" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="17"/>
@@ -14331,7 +14354,7 @@
       <c r="E1" s="17"/>
       <c r="F1" s="17"/>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:12">
       <c r="A2" s="117"/>
       <c r="B2" s="117"/>
       <c r="C2" s="117"/>
@@ -14339,21 +14362,21 @@
       <c r="E2" s="117"/>
       <c r="F2" s="117"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:12">
       <c r="A3" s="117"/>
       <c r="B3" s="117"/>
       <c r="C3" s="89" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="D3" s="89" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
       <c r="A4" s="117"/>
       <c r="B4" s="117"/>
       <c r="C4" s="89" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="D4">
         <v>12.1</v>
@@ -14380,10 +14403,10 @@
         <v>12052</v>
       </c>
       <c r="L4" t="s">
-        <v>416</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
       <c r="A5" s="117"/>
       <c r="B5" s="117"/>
       <c r="C5" s="90" t="s">
@@ -14396,7 +14419,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:12">
       <c r="A6" s="117"/>
       <c r="B6" s="117"/>
       <c r="C6" s="91">
@@ -14409,7 +14432,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:12">
       <c r="A7" s="117"/>
       <c r="B7" s="117"/>
       <c r="C7" s="90" t="s">
@@ -14422,7 +14445,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:12">
       <c r="A8" s="117"/>
       <c r="B8" s="117"/>
       <c r="C8" s="91">
@@ -14435,7 +14458,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:12">
       <c r="A9" s="117"/>
       <c r="B9" s="117"/>
       <c r="C9" s="90" t="s">
@@ -14448,7 +14471,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:12">
       <c r="A10" s="117"/>
       <c r="B10" s="117"/>
       <c r="C10" s="91">
@@ -14461,7 +14484,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:12">
       <c r="C11" s="90" t="s">
         <v>44</v>
       </c>
@@ -14472,7 +14495,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:12">
       <c r="C12" s="91">
         <v>23000</v>
       </c>
@@ -14483,7 +14506,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:12">
       <c r="C13" s="90" t="s">
         <v>50</v>
       </c>
@@ -14494,7 +14517,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:12">
       <c r="C14" s="91">
         <v>2</v>
       </c>
@@ -14505,7 +14528,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:12">
       <c r="C15" s="90" t="s">
         <v>48</v>
       </c>
@@ -14516,7 +14539,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:12">
       <c r="C16" s="91">
         <v>50024</v>
       </c>
@@ -14527,7 +14550,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="17" spans="3:12">
       <c r="C17" s="90" t="s">
         <v>53</v>
       </c>
@@ -14538,7 +14561,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="18" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="18" spans="3:12">
       <c r="C18" s="91">
         <v>189576</v>
       </c>
@@ -14549,7 +14572,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="19" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="19" spans="3:12">
       <c r="C19" s="90" t="s">
         <v>57</v>
       </c>
@@ -14560,7 +14583,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="20" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="20" spans="3:12">
       <c r="C20" s="91">
         <v>5000</v>
       </c>
@@ -14571,9 +14594,9 @@
         <v>37</v>
       </c>
     </row>
-    <row r="21" spans="3:12" x14ac:dyDescent="0.2">
+    <row r="21" spans="3:12">
       <c r="C21" s="90" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="D21">
         <v>9</v>
@@ -14612,31 +14635,31 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C47BF70-BA80-4124-B359-67CBCB635390}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="13.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="65.140625" customWidth="1"/>
     <col min="2" max="26" width="13.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="B2" s="117"/>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
     </row>
   </sheetData>
@@ -14648,25 +14671,25 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FE31E21-0350-44E7-AF13-4CA140505B30}">
   <dimension ref="A1:B12"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="12.75"/>
   <sheetData>
-    <row r="1" spans="1:2" ht="51" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" ht="51">
       <c r="A1" s="99" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="B1" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="B7" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
       <c r="A8">
         <v>1</v>
       </c>
@@ -14674,7 +14697,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:2">
       <c r="A9">
         <v>2</v>
       </c>
@@ -14682,7 +14705,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:2">
       <c r="A10">
         <v>3</v>
       </c>
@@ -14690,7 +14713,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:2">
       <c r="A11">
         <v>4</v>
       </c>
@@ -14698,7 +14721,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:2">
       <c r="A12">
         <v>5</v>
       </c>

</xml_diff>